<commit_message>
philo Franck ,Hahn, Schlick
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="505">
   <si>
     <t xml:space="preserve">FRISE DES PHILOSOPHES ALLEMANDS MODERNES — Données source</t>
   </si>
@@ -1091,6 +1091,34 @@
     <t xml:space="preserve">philosophe germano-balte devenu philosophe voyageur connu pour son journal de voyage.</t>
   </si>
   <si>
+    <t xml:space="preserve">1882 – 1936</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moritz SCHLICK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Moritz_Schlick"  title=" Wikipedia"&gt;Moritz SCHLICK&lt;/a&gt; était un philosophe allemand, physicien de formation, et l’une des figures centrales de l’empirisme logique. Il est surtout connu comme le fondateur et le dirigeant intellectuel du Cercle de Vienne, groupe qui se réunissait autour de la philosophie des sciences dans les années 1920 et 1930. Il occupa à Vienne une chaire autrefois associée à Ernst Mach et à Ludwig Boltzmann. &lt;/p&gt; &lt;p&gt; Sa première grande œuvre est la Théorie générale de la connaissance (Allgemeine Erkenntnislehre, 1918). Dans cet ouvrage, il défend encore une forme de réalisme scientifique : le monde extérieur existe indépendamment de nous et peut être connu grâce aux sciences. Il s’oppose ainsi à l’idéalisme et à l’idée kantienne selon laquelle nous ne connaîtrions jamais les choses en elles-mêmes. Pour lui, connaître consiste notamment à coordonner des signes et des concepts avec les objets et les processus étudiés par les sciences. &lt;/p&gt; &lt;p&gt;  À partir des années 1920, son orientation évolue sous l’influence de Wittgenstein et du développement de la logique moderne. Il affirme alors que la philosophie ne doit pas construire une nouvelle vision métaphysique du monde, mais clarifier le sens des propositions. Une &lt;a href="https://encyclo-philo.fr/schlick-a"  title="l’encyclopedie philosophique : schick par encyclophilo"&gt;proposition authentiquement scientifique &lt;/a&gt; doit pouvoir être reliée à une méthode possible de vérification empirique ; les énoncés de logique et de mathématiques sont, quant à eux, analytiques ou tautologiques. Cette orientation est souvent résumée par la formule : « le sens d’une proposition est sa méthode de vérification ». &lt;/p&gt; &lt;p&gt; Il faut cependant éviter de le réduire à un vérificationnisme simpliste. Il admet qu’une proposition puisse être vérifiable en principe, même si la vérification ne peut pas être réalisée immédiatement ou matériellement. La vérification ne signifie donc pas forcément une observation actuelle, mais la possibilité de décrire une procédure permettant de déterminer si l’énoncé est vrai ou faux. Sur le plan éthique, Il ne pense pas que les jugements de valeur soient des connaissances scientifiques ; il leur accorde néanmoins une importance dans la vie humaine et dans l’analyse des motivations. &lt;/p&gt; &lt;p&gt; On peut le classer comme un philosophe des sciences, un empiriste logique, &lt;a href="https://www.youtube.com/watch?v=ESWQzsf1Fr4"  title="la fin du positivisme logique par philo analytique"&gt;un positiviste logique &lt;/a&gt; et un représentant de la philosophie analytique naissante. Il est plus central et plus systématique que Hans Hahn dans l’organisation du Cercle de Vienne, tandis que Hahn était avant tout mathématicien et philosophe des fondements des mathématiques. Sa pensée se situe à la rencontre du réalisme scientifique, de l’empirisme, de l’analyse logique du langage et de l’anti-métaphysique ; son projet fondamental était de faire de la philosophie une activité de clarification au service de la connaissance scientifique. &lt;/p&gt; 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wp5JgFBYz_Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moritz SCHLICK par VIS PHILO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.laphilo.fr/pho/mschlick-mini.webp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">logique ; epistemologie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positivisme Logique ; Analytique</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> philosophe allemand, physicien de formation, figure centrale de l’empirisme logique.</t>
+  </si>
+  <si>
     <t xml:space="preserve">1977</t>
   </si>
   <si>
@@ -1606,7 +1634,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1727,6 +1755,25 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Georgia"/>
@@ -1809,7 +1856,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1883,6 +1930,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2142,7 +2201,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.93"/>
@@ -3482,79 +3541,79 @@
         <v>330</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="206.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="297" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="n">
-        <v>1885</v>
-      </c>
-      <c r="B39" s="7" t="s">
+        <v>1882</v>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>1936</v>
+      </c>
+      <c r="C39" s="7" t="s">
         <v>331</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="D39" s="8" t="s">
         <v>332</v>
       </c>
-      <c r="D39" s="8" t="s">
+      <c r="E39" s="18" t="s">
         <v>333</v>
       </c>
-      <c r="E39" s="12" t="s">
+      <c r="F39" s="7" t="s">
         <v>334</v>
       </c>
-      <c r="F39" s="7" t="s">
+      <c r="G39" s="9" t="s">
         <v>335</v>
       </c>
-      <c r="G39" s="9" t="s">
+      <c r="H39" s="19" t="s">
         <v>336</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>337</v>
       </c>
       <c r="I39" s="7"/>
       <c r="J39" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="K39" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="K39" s="2" t="s">
+      <c r="L39" s="20" t="s">
         <v>339</v>
       </c>
-      <c r="L39" s="15" t="s">
+    </row>
+    <row r="40" customFormat="false" ht="206.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="n">
+        <v>1885</v>
+      </c>
+      <c r="B40" s="7" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="n">
-        <v>1886</v>
-      </c>
-      <c r="B40" s="7" t="s">
+      <c r="C40" s="7" t="s">
         <v>341</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="D40" s="8" t="s">
         <v>342</v>
       </c>
-      <c r="D40" s="8" t="s">
+      <c r="E40" s="12" t="s">
         <v>343</v>
       </c>
-      <c r="E40" s="11" t="s">
+      <c r="F40" s="7" t="s">
         <v>344</v>
       </c>
-      <c r="F40" s="7" t="s">
+      <c r="G40" s="9" t="s">
         <v>345</v>
       </c>
-      <c r="G40" s="9" t="s">
+      <c r="H40" s="9" t="s">
         <v>346</v>
-      </c>
-      <c r="H40" s="9" t="s">
-        <v>347</v>
       </c>
       <c r="I40" s="7"/>
       <c r="J40" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="K40" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="K40" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="L40" s="2" t="s">
+      <c r="L40" s="15" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="n">
         <v>1886</v>
       </c>
@@ -3567,7 +3626,7 @@
       <c r="D41" s="8" t="s">
         <v>352</v>
       </c>
-      <c r="E41" s="9" t="s">
+      <c r="E41" s="11" t="s">
         <v>353</v>
       </c>
       <c r="F41" s="7" t="s">
@@ -3581,10 +3640,10 @@
       </c>
       <c r="I41" s="7"/>
       <c r="J41" s="2" t="s">
-        <v>84</v>
+        <v>357</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>357</v>
+        <v>134</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>358</v>
@@ -3592,7 +3651,7 @@
     </row>
     <row r="42" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="n">
-        <v>1888</v>
+        <v>1886</v>
       </c>
       <c r="B42" s="7" t="s">
         <v>359</v>
@@ -3617,57 +3676,57 @@
       </c>
       <c r="I42" s="7"/>
       <c r="J42" s="2" t="s">
-        <v>348</v>
+        <v>84</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>320</v>
+        <v>366</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="n">
         <v>1888</v>
       </c>
-      <c r="B43" s="7" t="n">
-        <v>1973</v>
+      <c r="B43" s="7" t="s">
+        <v>368</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>368</v>
-      </c>
-      <c r="E43" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>371</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>371</v>
-      </c>
-      <c r="H43" s="11" t="s">
-        <v>372</v>
+        <v>373</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>374</v>
       </c>
       <c r="I43" s="7"/>
       <c r="J43" s="2" t="s">
-        <v>373</v>
+        <v>357</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>357</v>
+        <v>320</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="n">
-        <v>1889</v>
-      </c>
-      <c r="B44" s="7" t="s">
-        <v>375</v>
+        <v>1888</v>
+      </c>
+      <c r="B44" s="7" t="n">
+        <v>1973</v>
       </c>
       <c r="C44" s="7" t="s">
         <v>376</v>
@@ -3675,7 +3734,7 @@
       <c r="D44" s="8" t="s">
         <v>377</v>
       </c>
-      <c r="E44" s="9" t="s">
+      <c r="E44" s="11" t="s">
         <v>378</v>
       </c>
       <c r="F44" s="7" t="s">
@@ -3684,23 +3743,23 @@
       <c r="G44" s="9" t="s">
         <v>380</v>
       </c>
-      <c r="H44" s="9" t="s">
+      <c r="H44" s="11" t="s">
         <v>381</v>
       </c>
       <c r="I44" s="7"/>
       <c r="J44" s="2" t="s">
-        <v>104</v>
+        <v>382</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>382</v>
+        <v>366</v>
       </c>
       <c r="L44" s="2" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="207" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="n">
-        <v>1891</v>
+        <v>1889</v>
       </c>
       <c r="B45" s="7" t="s">
         <v>384</v>
@@ -3725,57 +3784,57 @@
       </c>
       <c r="I45" s="7"/>
       <c r="J45" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="K45" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="K45" s="2" t="s">
+      <c r="L45" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="L45" s="2" t="s">
+    </row>
+    <row r="46" customFormat="false" ht="207" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="n">
+        <v>1891</v>
+      </c>
+      <c r="B46" s="7" t="s">
         <v>393</v>
       </c>
-    </row>
-    <row r="46" customFormat="false" ht="219.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="n">
-        <v>1892</v>
-      </c>
-      <c r="B46" s="7" t="s">
+      <c r="C46" s="7" t="s">
         <v>394</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="D46" s="8" t="s">
         <v>395</v>
       </c>
-      <c r="D46" s="8" t="s">
+      <c r="E46" s="9" t="s">
         <v>396</v>
       </c>
-      <c r="E46" s="9" t="s">
+      <c r="F46" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="F46" s="7" t="s">
+      <c r="G46" s="9" t="s">
         <v>398</v>
       </c>
-      <c r="G46" s="9" t="s">
+      <c r="H46" s="9" t="s">
         <v>399</v>
-      </c>
-      <c r="H46" s="9" t="s">
-        <v>400</v>
       </c>
       <c r="I46" s="7"/>
       <c r="J46" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="K46" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="K46" s="2" t="s">
+      <c r="L46" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="L46" s="2" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="144.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="47" customFormat="false" ht="219.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="n">
         <v>1892</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>359</v>
+        <v>403</v>
       </c>
       <c r="C47" s="7" t="s">
         <v>404</v>
@@ -3797,90 +3856,90 @@
       </c>
       <c r="I47" s="7"/>
       <c r="J47" s="2" t="s">
-        <v>207</v>
+        <v>410</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>189</v>
+        <v>411</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="144.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="n">
-        <v>1893</v>
+        <v>1892</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>411</v>
+        <v>368</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>413</v>
-      </c>
-      <c r="E48" s="12" t="s">
         <v>414</v>
       </c>
+      <c r="E48" s="9" t="s">
+        <v>415</v>
+      </c>
       <c r="F48" s="7" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="I48" s="7"/>
       <c r="J48" s="2" t="s">
-        <v>418</v>
+        <v>207</v>
       </c>
       <c r="K48" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="L48" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="L48" s="15" t="s">
+    </row>
+    <row r="49" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="n">
+        <v>1893</v>
+      </c>
+      <c r="B49" s="7" t="s">
         <v>420</v>
       </c>
-    </row>
-    <row r="49" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="n">
-        <v>1895</v>
-      </c>
-      <c r="B49" s="7" t="s">
+      <c r="C49" s="7" t="s">
         <v>421</v>
       </c>
-      <c r="C49" s="7" t="s">
+      <c r="D49" s="8" t="s">
         <v>422</v>
       </c>
-      <c r="D49" s="8" t="s">
+      <c r="E49" s="12" t="s">
         <v>423</v>
       </c>
-      <c r="E49" s="9" t="s">
+      <c r="F49" s="7" t="s">
         <v>424</v>
       </c>
-      <c r="F49" s="7" t="s">
+      <c r="G49" s="9" t="s">
         <v>425</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="H49" s="9" t="s">
         <v>426</v>
-      </c>
-      <c r="H49" s="9" t="s">
-        <v>427</v>
       </c>
       <c r="I49" s="7"/>
       <c r="J49" s="2" t="s">
-        <v>123</v>
+        <v>427</v>
       </c>
       <c r="K49" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="L49" s="2" t="s">
+      <c r="L49" s="15" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="215.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="n">
-        <v>1897</v>
+        <v>1895</v>
       </c>
       <c r="B50" s="7" t="s">
         <v>430</v>
@@ -3891,7 +3950,7 @@
       <c r="D50" s="8" t="s">
         <v>432</v>
       </c>
-      <c r="E50" s="11" t="s">
+      <c r="E50" s="9" t="s">
         <v>433</v>
       </c>
       <c r="F50" s="7" t="s">
@@ -3905,21 +3964,21 @@
       </c>
       <c r="I50" s="7"/>
       <c r="J50" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="K50" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="K50" s="2" t="s">
+      <c r="L50" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="L50" s="2" t="s">
+    </row>
+    <row r="51" customFormat="false" ht="215.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="7" t="n">
+        <v>1897</v>
+      </c>
+      <c r="B51" s="7" t="s">
         <v>439</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="316.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="n">
-        <v>1899</v>
-      </c>
-      <c r="B51" s="7" t="n">
-        <v>1973</v>
       </c>
       <c r="C51" s="7" t="s">
         <v>440</v>
@@ -3927,7 +3986,7 @@
       <c r="D51" s="8" t="s">
         <v>441</v>
       </c>
-      <c r="E51" s="13" t="s">
+      <c r="E51" s="11" t="s">
         <v>442</v>
       </c>
       <c r="F51" s="7" t="s">
@@ -3936,26 +3995,26 @@
       <c r="G51" s="9" t="s">
         <v>444</v>
       </c>
-      <c r="H51" s="11" t="s">
+      <c r="H51" s="9" t="s">
         <v>445</v>
       </c>
       <c r="I51" s="7"/>
       <c r="J51" s="2" t="s">
-        <v>348</v>
+        <v>446</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="231.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="316.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="n">
-        <v>1900</v>
-      </c>
-      <c r="B52" s="7" t="s">
-        <v>448</v>
+        <v>1899</v>
+      </c>
+      <c r="B52" s="7" t="n">
+        <v>1973</v>
       </c>
       <c r="C52" s="7" t="s">
         <v>449</v>
@@ -3963,7 +4022,7 @@
       <c r="D52" s="8" t="s">
         <v>450</v>
       </c>
-      <c r="E52" s="12" t="s">
+      <c r="E52" s="13" t="s">
         <v>451</v>
       </c>
       <c r="F52" s="7" t="s">
@@ -3972,57 +4031,57 @@
       <c r="G52" s="9" t="s">
         <v>453</v>
       </c>
-      <c r="H52" s="9" t="s">
+      <c r="H52" s="11" t="s">
         <v>454</v>
       </c>
       <c r="I52" s="7"/>
       <c r="J52" s="2" t="s">
-        <v>168</v>
+        <v>357</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="L52" s="15" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="53" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="L52" s="2" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="231.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="n">
-        <v>1903</v>
+        <v>1900</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>458</v>
-      </c>
-      <c r="E53" s="9" t="s">
         <v>459</v>
       </c>
+      <c r="E53" s="12" t="s">
+        <v>460</v>
+      </c>
       <c r="F53" s="7" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="H53" s="9" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="I53" s="7"/>
       <c r="J53" s="2" t="s">
-        <v>463</v>
+        <v>168</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>428</v>
-      </c>
-      <c r="L53" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="L53" s="15" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="176.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="n">
         <v>1903</v>
       </c>
@@ -4035,7 +4094,7 @@
       <c r="D54" s="8" t="s">
         <v>467</v>
       </c>
-      <c r="E54" s="11" t="s">
+      <c r="E54" s="9" t="s">
         <v>468</v>
       </c>
       <c r="F54" s="7" t="s">
@@ -4049,121 +4108,157 @@
       </c>
       <c r="I54" s="7"/>
       <c r="J54" s="2" t="s">
-        <v>304</v>
+        <v>472</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>472</v>
+        <v>437</v>
       </c>
       <c r="L54" s="2" t="s">
         <v>473</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="195.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="176.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="n">
-        <v>1904</v>
+        <v>1903</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>375</v>
+        <v>474</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>475</v>
-      </c>
-      <c r="E55" s="12" t="s">
         <v>476</v>
       </c>
+      <c r="E55" s="11" t="s">
+        <v>477</v>
+      </c>
       <c r="F55" s="7" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="H55" s="9" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="I55" s="7"/>
       <c r="J55" s="2" t="s">
-        <v>418</v>
+        <v>304</v>
       </c>
       <c r="K55" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="195.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="7" t="n">
+        <v>1904</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>483</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>484</v>
+      </c>
+      <c r="E56" s="12" t="s">
+        <v>485</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="G56" s="9" t="s">
+        <v>487</v>
+      </c>
+      <c r="H56" s="9" t="s">
+        <v>488</v>
+      </c>
+      <c r="I56" s="7"/>
+      <c r="J56" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="K56" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="L55" s="15" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="236.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="1" t="n">
+      <c r="L56" s="15" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="236.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="n">
         <v>1929</v>
       </c>
-      <c r="B56" s="1" t="n">
+      <c r="B57" s="1" t="n">
         <v>2026</v>
       </c>
-      <c r="C56" s="1" t="s">
-        <v>481</v>
-      </c>
-      <c r="D56" s="18" t="s">
-        <v>482</v>
-      </c>
-      <c r="E56" s="17" t="s">
-        <v>483</v>
-      </c>
-      <c r="F56" s="19" t="s">
-        <v>484</v>
-      </c>
-      <c r="G56" s="10" t="s">
-        <v>485</v>
-      </c>
-      <c r="H56" s="10" t="s">
-        <v>486</v>
-      </c>
-      <c r="I56" s="10"/>
-      <c r="J56" s="2" t="s">
+      <c r="C57" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="D57" s="21" t="s">
+        <v>491</v>
+      </c>
+      <c r="E57" s="17" t="s">
+        <v>492</v>
+      </c>
+      <c r="F57" s="22" t="s">
+        <v>493</v>
+      </c>
+      <c r="G57" s="10" t="s">
+        <v>494</v>
+      </c>
+      <c r="H57" s="10" t="s">
+        <v>495</v>
+      </c>
+      <c r="I57" s="10"/>
+      <c r="J57" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="K56" s="2" t="s">
-        <v>428</v>
-      </c>
-      <c r="L56" s="2" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="183.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="7" t="n">
+      <c r="K57" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="L57" s="2" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="183.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="7" t="n">
         <v>1941</v>
       </c>
-      <c r="B57" s="7" t="n">
+      <c r="B58" s="7" t="n">
         <v>1993</v>
       </c>
-      <c r="C57" s="7" t="s">
-        <v>488</v>
-      </c>
-      <c r="D57" s="8" t="s">
-        <v>489</v>
-      </c>
-      <c r="E57" s="13" t="s">
-        <v>490</v>
-      </c>
-      <c r="F57" s="7" t="s">
-        <v>491</v>
-      </c>
-      <c r="G57" s="9" t="s">
-        <v>492</v>
-      </c>
-      <c r="H57" s="9" t="s">
-        <v>493</v>
-      </c>
-      <c r="I57" s="9"/>
-      <c r="J57" s="2" t="s">
+      <c r="C58" s="7" t="s">
+        <v>497</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>498</v>
+      </c>
+      <c r="E58" s="13" t="s">
+        <v>499</v>
+      </c>
+      <c r="F58" s="7" t="s">
+        <v>500</v>
+      </c>
+      <c r="G58" s="9" t="s">
+        <v>501</v>
+      </c>
+      <c r="H58" s="9" t="s">
+        <v>502</v>
+      </c>
+      <c r="I58" s="9"/>
+      <c r="J58" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K57" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="L57" s="2" t="s">
-        <v>495</v>
+      <c r="K58" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="L58" s="2" t="s">
+        <v>504</v>
       </c>
     </row>
   </sheetData>
@@ -4189,14 +4284,16 @@
     <hyperlink ref="E34" r:id="rId15" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Theodor_Lessing&quot; title=&quot; Wikipedia&quot;&gt;Theodor LESSING&lt;/a&gt;  était un philosophe, essayiste et publiciste allemand &lt;a href=&quot;https://www.persee.fr/doc/rjuiv_0484-8616_1996_num_155_1_2554&quot;  title=&quot;Lessing et le sionisme par persée&quot;&gt;d’origine juive, &lt;/a&gt; connu comme un penseur critique de la modernité, du nationalisme et de l’antisémitisme. &lt;/p&gt; &lt;p&gt; Il s’inscrit surtout dans une philosophie de la culture et une philosophie sociale critique. Son travail ne cherche pas à construire un système abstrait, mais à analyser les maladies de la civilisation moderne, la violence des masses, la guerre, la ville industrielle et la destruction du vivant. Sa pensée est marquée par un humanisme pessimiste et engagé qui dénoncé le militarisme, la brutalisation de la société et les dérives autoritaires de l’Allemagne de Weimar, allant jusqu’à prévoir le danger nazi avant 1933. Il fut aussi l’un des premiers à réfléchir à la condition des minorités et à ce qu’il a appelé le &lt;a href=&quot;https://www.sifriatenou.com/2020/10/20/5449/&quot;  title=&quot;lessing la haine de soi par sifriatenou&quot;&gt;« judaïsme de haine de soi »,&lt;/a&gt; pour décrire les effets psychologiques de l’antisémitisme sur les Juifs eux-mêmes. &lt;/p&gt; &lt;p&gt; Il est également une figure de la critique écologique avant l’heure. Dès les années 1930, il s’inquiète de la déforestation, de la pollution urbaine et d’un possible dérèglement du climat, ce qui le rend étonnamment actuel. Il voit la modernité technique non comme un progrès neutre, mais comme une force capable de détruire les équilibres humains et naturels. &lt;/p&gt; &lt;p&gt; Sur le plan politique, il est un intellectuel indépendant, polémique et souvent isolé, qui s’oppose à l’autoritarisme autant qu’aux conformismes de son époque. Il a &lt;a href=&quot;https://www.youtube.com/watch?v=pdcxbRYcn&quot;  title=&quot;lessing par jacques Aron et Editions harmattan&quot;&gt;fini assassiné en exil &lt;/a&gt;  à Mariánské Lázně par des nationalistes sudètes, devenant l’une des premières victimes du nazisme hors d’Allemagne. &lt;/p&gt; &#10;"/>
     <hyperlink ref="E35" r:id="rId16" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Max_Scheler&quot; title=&quot; Wikipedia&quot;&gt;Max SCHELER&lt;/a&gt;  était un philosophe allemand, figure phare de la phénoménologie et de l’anthropologie philosophique, dont l’œuvre traverse des domaines variés comme l’éthique, l’axiologie et la sociologie de la connaissance. &lt;/p&gt; &lt;p&gt; Il élabore une &lt;a href=&quot;https://www.persee.fr/doc/phlou_0776-555x_1927_num_29_14_2467&quot;  title=&quot;La philosophie de M. Scheler. Son analyse de la sympathie et de l'amour par Persée&quot;&gt;hiérarchie des valeurs &lt;/a&gt; qui va des valeurs de l’agréable et du désagréable jusqu’aux valeurs spirituelles (beau/laid, juste/injuste, connaissance, et enfin le sacré et le profane). Cette hiérarchie sert de base à une éthique et à une phénoménologie de la sensation et des sentiments qui orientent l’action humaine. Il propose une approche phénoménologique qui insiste sur &quot;l’attitude spirituelle&quot; ou &quot;l’œil vivant&quot; vers le monde, en s’opposant à une réduction purement méthodologique et en valorisant l’intuition des valeurs telles qu’elles se donnent à la conscience. &lt;/p&gt; &lt;p&gt; Il fonde l’idée d’une anthropologie philosophique qui cherche à comprendre l’homme dans le vivant et ses rapports au monde, en intégrant des connaissances des sciences naturelles et des sciences humaines. &lt;a href=&quot;https://www.youtube.com/watch?v=pPuUoTPig7w&quot; title=&quot;Le salut vient-il du travail ? - Valeur et dignité du travail selon Max SCHELER par Editions M-Editer&quot;&gt;Cette orientation &lt;/a&gt; mène plus tard à une sociologie de la connaissance. Voici ses oeuvres majeures : &lt;/p&gt; &lt;p&gt; - &quot;Die Wissensformen und die Gesellschaft&quot; paru en 1926 – synthèse de son projet de sociologie de la connaissance et jalon important de l’anthropologie philosophique et sociale. Cette œuvre est souvent citée comme fondatrice d’une approche sociologique qui rejoint les débats de Weimar.&lt;/p&gt; &lt;p&gt; - &quot;Stellung des Menschen im Kosmos&quot; paru en 1928 – portrait philosophique de l’homme dans le cadre d’un ensemble plus large d’ouvrages préfigurant l’anthropologie philosophique et son intérêt pour le positionnement de l’homme dans l’ordre du vivant. &lt;/p&gt; &lt;p&gt; Son approche personnaliste et son engagement en faveur d’une philosophie sociale et éthique centrée sur la dignité humaine, &lt;a href=&quot;https://www.youtube.com/watch?v=HHAKQrNdMYk&quot; title=&quot;&#10;Le ressentiment détruit ta vie… (Max Sheller, l'homme du ressentiment) par Timothée Delahaye&quot;&gt;le resentiment &lt;/a&gt; et les valeurs morales continuent d’être discutés dans les études contemporaines, notamment dans les analyses qui situent Scheler dans le dialogue franco-allemand et dans les traditions de philosophie sociale et morale. &lt;/p&gt; "/>
     <hyperlink ref="E38" r:id="rId17" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hermann_von_Keyserling&quot; title=&quot; Wikipedia&quot;&gt;Hermann Von KEYSERLING&lt;/a&gt;  était un philosophe  &lt;a href=&quot;https://www.persee.fr/doc/slaoc_1245-2491_1997_num_4_1_1809&quot; style=&quot;color:#88A1E9&quot; title=&quot; Hermann von Keyserling et les interférences germano-slaves par Persée&quot;&gt;germano-balte &lt;/a&gt; devenu philosophe voyageur, figure très en vue de la République de Weimar, connu pour son Journal de voyage d’un philosophe et pour son &quot;École de la sagesse&quot; à Darmstadt. &lt;/p&gt; &lt;p&gt; Il conçoit la philosophie non comme une science rigoureuse, mais comme sagesse vécue : &quot;la vie elle-même sous la forme du savoir&quot;, contre les théories objectivantes du savoir technico-scientifique. Il s’inscrit dans la philosophie de la vie, mais de façon personnelle : importance de l’intuition, de la singularité des événements et de la transformation intérieure. Son projet est une nouvelle synthèse de l’âme et de l’esprit, la pénétration réciproque de sagesse et politique, et l’idée que dans la vie déterminée par l’esprit, c’est &lt;a href=&quot;https://www.youtube.com/watch?v=Y0DY8F72114&quot; title=&quot;Eduard von Keyserling, DUMALA par Le Veilleur&quot;&gt;le Sens &lt;/a&gt; qui crée les faits plutôt que l’inverse. &lt;/p&gt; &lt;p&gt; Il  utilise très tôt le terme Führerprinzip, en liant l’idée de &quot;dirigeants nés&quot; à un élitisme spiritualiste et social-darwinien, tout en refusant par la suite d’adhérer au national-socialisme, qu’il voit comme mouvement de masses manipulées.  Le régime nazi ferme son École de la sagesse au milieu des années 1930, lui interdit de publier et de voyager, tandis que sa réputation continue de grandir à l’étranger. &lt;/p&gt;&lt;p&gt; Ses oeuvres principales sont : - &quot;Reisetagebuch eines Philosophen&quot;  paru en 1919 : récit de son tour du monde (1911-1912, Asie, Amérique, Europe du Sud) mêlant observations culturelles, méditations spirituelles et diagnostics sur les civilisations ; c’est son grand succès de librairie, largement traduit. -&quot;Das Gefüge der Welt. Versuch einer kritischen Philosophie&quot; (La Structure du monde, 1907) : tentative de &quot;philosophie critique&quot; personnelle, déjà marquée par l’idée que le savoir véritable est inséparable de la vie. - &quot;Schöpferische Erkenntnis&quot; (Connaissance créatrice) et &quot;Wiedergeburt&quot; (Renaissance) : textes doctrinaux de l’&quot;École de la sagesse&quot;, insistant sur la connaissance comme acte créateur, transformant la vie plutôt que la décrivant objectivement. &lt;/p&gt; "/>
-    <hyperlink ref="E40" r:id="rId18" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl_Korsch&quot; title=&quot; Wikipedia&quot;&gt;Karl KORDCH&lt;/a&gt;  était un philosophe marxiste allemand,  théoricien du communisme de conseils et critique du léninisme orthodoxe. Issu d'un milieu bourgeois, il évolua du réformisme social au marxisme hétérodoxe, influençant les courants ultra-gauche via son rejet du matérialisme positiviste et son insistance sur la praxis révolutionnaire historique.  Exclu du parti en 1926 pour &quot;ultra-gauchisme&quot;, il émigra après 1933 vers les USA, où il approfondit sa théorie marxiste. &lt;/p&gt; &lt;p&gt; Son œuvre majeure &quot;Marxisme et philosophie&quot; paru en 1923 marque sa rupture avec le léninisme en critiquant sa dérive scientiste. Il   &lt;a href=&quot;https://www.zones-subversives.com/article-le-marxisme-critique-de-karl-korsch-116431466.html&quot;  title=&quot;Le marxisme critique de Karl Korsch par Chroniques critiques&quot;&gt;rejette le marxisme &lt;/a&gt; comme &quot;science positive&quot; figée ou philosophie matérialiste abstraite ; il le conçoit comme une théorie historique et concrète, liée à la lutte des classes et à la dialectique hégélienne réinterprétée comme expression de la révolution bourgeoise puis prolétarienne. &lt;/p&gt; &lt;p&gt; Il  théorise les conseils comme organes centraux de la transition socialiste, via la praxis dialectique et l'auto-activité des masses, contre la socialisation étatique. Ses écrits inspirent le KAPD et l'ultra-gauche, voyant les conseils comme alternative à la bureaucratisation stalinienne. Son influence perdure chez les communistes de conseils, soulignant la conscience ouvrière spontanée pour l'émancipation réelle. &lt;/p&gt; "/>
-    <hyperlink ref="E43" r:id="rId19" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Eugen_Rosenstock-Huessy&quot; title=&quot; Wikipedia&quot;&gt;Eugen ROSENSTOCK-HUESSY&lt;/a&gt; était un penseur germano‑américain dont l'œuvre mêle philosophie sociale, histoire des idées et une théorie du langage centrée sur la parole comme acte créateur et structurant de la vie collective. Né en Allemagne, il forma des liens intellectuels avec des figures comme Franz Rosenzweig et Martin Buber, fut professeur (notamment aux États‑Unis après son exil) et créa une œuvre originale qui vise à comprendre comment les communautés se constituent et se transforment dans le temps par des échanges de parole. &lt;/p&gt; &lt;p&gt; Au  &lt;a href=&quot;https://www.en-attendant-nadeau.fr/2019/11/19/homme-quadridimensionnel-rosenstock//&quot;  title=&quot;l’homme quadridimensionnel par ean&quot;&gt;cœur de sa pensée &lt;/a&gt;  se trouve la notion de &quot;speech thinking&quot; (pensée de la parole) : il soutient que la parole n’est pas qu’un moyen descriptif, mais un acte répondant et créatif qui institue des relations sociales, forge des temporalités collectives et permet la transmission et la renouvellement des institutions humaines. Il affirme que, par le langage, les groupes deviennent « maîtres du temps » en fondant de nouveaux commencements, en rappelant le passé et en orientant l’action future — d’où son intérêt pour la densité historique de la vie sociale et le rôle des rituels, des serments et des discours publics. &lt;/p&gt; &lt;p&gt; Sur la religion et la théologie, il s’inscrit dans un courant post‑nietzschéen de renouveau religieux qui comprend Rosenzweig et Buber; il considère les énoncés religieux comme des actes de parole non‑métaphysiques qui dévoilent des dimensions de l’expérience humaine et communautaire inaccessibles aux seules sciences naturelles. Cette orientation le conduit à une pensée intégrative où philosophie, théologie et histoire participent à une réflexion pratique sur la transformation sociale et la responsabilité collective. &lt;/p&gt; &lt;p&gt; Ses livres et conférences couvrent une grande variété de thèmes — histoire des peuples, rhétorique sociale, philosophie de la loi et de l’éducation — et sa méthode combine analyses historiques, typologies du langage et propositions pour renouveler la vie civique; son influence se voit aujourd’hui dans des études sur la communication, la sociologie historique et la philosophie de la culture. &lt;/p&gt; "/>
-    <hyperlink ref="H43" r:id="rId20" display="https://www.laphilo.fr/pho/erhuessy-mini.webp"/>
-    <hyperlink ref="E50" r:id="rId21" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Gershom_Scholem&quot; title=&quot; Wikipedia&quot;&gt;Gershom SCHOLEM&lt;/a&gt; était un philosophe juif germano-israélien,  fondateur de l'étude académique moderne de la Kabbale et grand expert de  &lt;a href=&quot;https://www.nonfiction.fr/article-12478-gershom-scholem-de-berlin-a-la-palestine.htm&quot; title=&quot;Gershom Scholem : de Berlin à la Palestine  par nonfiction&quot;&gt;la mystique juive. &lt;/a&gt; Né à Berlin dans une famille assimilée, il s'est tourné vers le sionisme jeune et a immigré en Palestine en 1923, devenant professeur à l'Université hébraïque de Jérusalem. &lt;/p&gt; &lt;p&gt; Il a étudié les mathématiques, la philosophie et les langues sémitiques à Berlin, Iéna et Munich, où il a soutenu une thèse sur le &quot;Sefer ha-Bahir&quot;, un texte kabbalistique ancien. Ami proche de Walter Benjamin et correspondant de Leo Strauss, il a fui l'Europe nazie et s'est consacré à la recherche sur les manuscrits juifs pillés. &lt;/p&gt; &lt;p&gt; Il voyait  &lt;a href=&quot;https://www.youtube.com/watch?v=5HvDF8-XTjc&quot;  title=&quot;Dieu son nom et la Cabale selon Gershom Scholem  par Xavier Charles DJEBALI&quot;&gt;la Kabbale &lt;/a&gt; non comme une superstition marginale, mais au cœur de l'essence spirituelle du judaïsme, explorée via des méthodes scientifiques et historiques. Il insistait sur le rôle du messianisme et de la tradition comme forces de renouvellement, où la révélation divine est infiniment interprétable et liée à l'expérience historique du peuple juif. Pour lui, le sionisme allait au-delà de la politique : c'était un renouveau profond du judaïsme, unissant ancien et nouveau contre l'assimilation. &lt;/p&gt; &lt;p&gt; Son oeuvre majeure &quot;Les Grandes tendances de la mystique juive&quot; paru en 1941, basé sur des conférences, dédié à Benjamin, explore l'évolution de la mystique juive. Sa pensée met l'accent sur l'identité juive forgée par l'histoire, où la tradition intègre la nouveauté pour survivre aux crises. &lt;/p&gt; &lt;audio controls title=&quot;Des livres pour notre temps et les mondes à venir. 1/2 Gershom Scholem : penser dans les marges de la marge par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13094-10.11.2019-ITEMA_22199082-0.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
-    <hyperlink ref="E51" r:id="rId22" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Leo_Strauss&quot; title=&quot; Wikipedia&quot;&gt;Leo SRAUSS&lt;/a&gt; était un philosophe politique germano-américain, connu pour sa critique profonde de la modernité et pour sa relecture des grands textes de la philosophie politique classique. Sa pensée a eu une influence durable, notamment aux États‑Unis, où elle a marqué des générations d’étudiants en théorie politique. &lt;/p&gt; &lt;p&gt; Au cœur de sa philosophie se trouve l’idée que la modernité a rompu avec le droit naturel classique, c’est‑à‑dire avec la recherche de ce qui est juste par nature et non simplement selon l’histoire ou les sciences sociales. Il voit dans le positivisme, le relativisme et l’historicisme modernes une source de décadence intellectuelle, car ils empêchent de poser les questions normatives fondamentales : qu’est‑ce qu’une vie bonne, qu’est‑ce qu’un régime politique juste. Pour lui, la  &lt;a href=&quot;https://www.persee.fr/doc/rfsp_0035-2950_1985_num_35_4_394205&quot; title=&quot;philosophie et zscience politique par persée&quot;&gt;philosophie politique authentique &lt;/a&gt; doit réactiver ces questions et affronter directement les notions de meilleur régime et d’ordre politique juste, plutôt que de se contenter de descriptions neutres. &lt;/p&gt; &lt;p&gt; Cette critique le conduit à renouer avec les auteurs de l’Antiquité, en particulier Platon, Aristote et les philosophes médiévaux juifs et arabes, qu’il lit souvent contre les interprétations modernes. Il insiste sur la dimension éducative de la philosophie : il parle de « liberal education » comme d’une libération de la vulgarité, entendue comme manque d’expérience des belles choses. La fréquentation des grands textes est, pour lui, une école de modestie et d’audace intellectuelle, parce qu’elle oblige à mesurer nos catégories modernes à celles d’auteurs qui pensaient autrement le politique et le juste. &lt;/p&gt; &lt;p&gt; Célèbre pour sa thèse sur l’« écriture ésotérique » : selon lui, nombre de philosophes du passé ont écrit de manière volontairement oblique pour se protéger de la censure ou de la persécution, réservant un sens plus profond aux lecteurs attentifs. Cela l’amène à distinguer entre le message « exotérique » (apparent, destiné au grand public) et le message « ésotérique » (plus exigeant, adressé à une minorité philosophique). Cette hypothèse sur la lecture des classiques s’articule à sa conception du   &lt;a href=&quot;https://www.youtube.com/watch?v=9Vhsveytymk&quot; title=&quot;nihilisme et politique leo strauss par bildung et culture&quot;&gt;mode de vie philosophique, &lt;/a&gt; toujours exposé au risque de la tyrannie et de l’incompréhension. Ainsi, sa philosophie politique est à la fois une critique de la modernité et une tentative de redécouvrir la place de la philosophie au cœur du politique contemporain. &lt;/p&gt; &#10; &lt;audio controls title=&quot;la pensée de leon strauss par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13397-05.04.2008-ITEMA_20118283-2008C3397E0019-ITE_00016207_RSCE-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;  &#10;"/>
-    <hyperlink ref="H51" r:id="rId23" display="https://www.laphilo.fr/pho/lstrauss-mini.webp"/>
-    <hyperlink ref="E54" r:id="rId24" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hans_Jonas&quot; title=&quot; Wikipedia&quot;&gt;Hans JONAS&lt;/a&gt;  était un philosophe germano-américain connu pour ses travaux sur l'éthique de la technologie et &lt;a href=&quot;https://www.youtube.com/watch?v=NPIJHZO7hQo&quot; title=&quot; Le PRINCIPE RESPONSABILITÉ en 6 minutes ! (HANS JONAS) par Culture Philo&quot;&gt;la responsabilité&lt;/a&gt; envers les générations futures. Ses premières recherches portent sur le gnosticisme, vu comme une réponse à l'aliénation existentielle dans un monde hostile. Dans les années 1960, il développe une philosophie de la vie organique (The Phenomenon of Life), critiquant le dualisme cartésien et valorisant la nature vivante contre la technoscience destructrice. Son œuvre maîtresse &lt;a href=&quot;https://www.youtube.com/watch?v=LsIWCR9_N64&quot; style=&quot;color:#88A1E9&quot; title=&quot; Philo, Hans jonas, Le principe responsabilité, Bac philo par SOS Bac Français&quot;&gt; &quot;Le Principe responsabilité&quot;&lt;/a&gt; paru en1979, formule un impératif éthique pour l'ère technologique : &quot;Agis de façon que les effets de ton action soient compatibles avec la permanence d'une vie authentiquement humaine sur Terre&quot;. &lt;/p&gt; &lt;p&gt; Il  anticipe les crises écologiques et bioéthiques, proposant une &quot;heuristique de la peur&quot; pour guider l'action humaine face aux risques imprévisibles de la puissance technique. Influencé par sa tradition juive et Heidegger, il réconcilie existentialisme, phénoménologie et morale prophétique, impactant l'éthique environnementale contemporaine. &lt;/p&gt; &lt;p&gt; Il observe un &quot;déchaînement prométhéen&quot; : l'humanité acquiert un pouvoir inédit sur la nature via la science et la technique, capable de menacer sa propre survie et celle des générations futures. Contrairement aux éthiques classiques (kantienne ou utilitariste), limitées au présent ou aux intentions, sa réflexion intègre les conséquences à long terme, imprévisibles et collectives, sur la vie humaine et la planète. Face aux risques inconnus (nucléaire, génétique, environnementaux), il prône une &quot;heuristique de la peur&quot; : anticiper le pire scénario (in dubio pro malo) pour guider l'action, sans paralyser le progrès mais en le subordonnant à la préservation de la vie. Le savoir devient un devoir moral prioritaire, élargissant l'éthique à la nature et aux générations absentes.&lt;/p&gt;  &lt;/p&gt; &lt;p&gt;  &lt;audio controls title=&quot; Hans Jonas. Pour une éthique de la société technologique par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/22267-14.06.2021-ITEMA_22702122-2014C12410E0357.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
-    <hyperlink ref="E57" r:id="rId25" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Reiner_Sch%C3%BCrmann&quot;  title=&quot; Wikipedia&quot;&gt;Reiner SCHÜRMANN&lt;/a&gt; est un philosophe allemand d’expression française, né à Amsterdam et mort à New York, où il a enseigné à la New School for Social Research à partir de 1975. Très marqué par la phénoménologie et la pensée de Heidegger, il se distingue par une réflexion exigeante sur la métaphysique, l’histoire de la philosophie et l’agir humain, développée dans trois grands ouvrages : Maître Eckhart et la joie errante (1972), Le principe d’anarchie (1982) et Des hégémonies brisées (posthume, 1996). &lt;/p&gt;&lt;p&gt; Dans Maître Eckhart et la joie errante, Schürmann reprend la pensée du mystique allemand du XIVᵉ siècle pour explorer la possibilité d’une vie spirituelle détachée de toute identité fixe ou de tout fondement stable. Il met en avant ce qu’il appelle une « joie errante » : une forme de liberté intérieure où le sujet ne se réclame plus d’une essence, d’un Dieu garanti ou d’une identité nationale, mais accepte de vivre dans une errance originaire et sans fondement. &lt;/p&gt; &lt;p&gt; Dans Le principe d’anarchie (souvent considéré comme son chef‑d’œuvre), Schürmann interprète Heidegger comme une pensée qui conduit à la ruine de tout principe premier (« archè ») sur lequel la tradition occidentale aurait voulu fonder la connaissance, la morale et la politique. Il en tire une théorie de l’« anarchie » non pas comme désordre, mais comme conscience lucide de l’absence de fondement ultime : l’agir humain doit alors se penser comme une praxis ouverte, responsable et créative, sans recours à une règle suprême. &lt;/p&gt; &lt;p&gt; Dans Des hégémonies brisées, Schürmann entreprend une vaste reconstruction de l’histoire de la philosophie occidentale comme succession d’« hégémonies » (modèles de vérité, de métaphysique, de politique) qui s’imposent, puis se défont. Il montre comment la modernité et la déconstruction heideggérienne ont dissous les grands systèmes de pensée, ouvrant à ce qu’il nomme une « philosophie tragique » où l’être se donne comme événement contingent, marqué par une distance, une fracture intérieure, plutôt que par une harmonie ou une cohérence totale. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="E39" r:id="rId18" display="https://fr.wikipedia.org/wiki/Moritz_Schlick"/>
+    <hyperlink ref="H39" r:id="rId19" display="https://www.laphilo.fr/pho/mschlick-mini.webp"/>
+    <hyperlink ref="E41" r:id="rId20" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl_Korsch&quot; title=&quot; Wikipedia&quot;&gt;Karl KORDCH&lt;/a&gt;  était un philosophe marxiste allemand,  théoricien du communisme de conseils et critique du léninisme orthodoxe. Issu d'un milieu bourgeois, il évolua du réformisme social au marxisme hétérodoxe, influençant les courants ultra-gauche via son rejet du matérialisme positiviste et son insistance sur la praxis révolutionnaire historique.  Exclu du parti en 1926 pour &quot;ultra-gauchisme&quot;, il émigra après 1933 vers les USA, où il approfondit sa théorie marxiste. &lt;/p&gt; &lt;p&gt; Son œuvre majeure &quot;Marxisme et philosophie&quot; paru en 1923 marque sa rupture avec le léninisme en critiquant sa dérive scientiste. Il   &lt;a href=&quot;https://www.zones-subversives.com/article-le-marxisme-critique-de-karl-korsch-116431466.html&quot;  title=&quot;Le marxisme critique de Karl Korsch par Chroniques critiques&quot;&gt;rejette le marxisme &lt;/a&gt; comme &quot;science positive&quot; figée ou philosophie matérialiste abstraite ; il le conçoit comme une théorie historique et concrète, liée à la lutte des classes et à la dialectique hégélienne réinterprétée comme expression de la révolution bourgeoise puis prolétarienne. &lt;/p&gt; &lt;p&gt; Il  théorise les conseils comme organes centraux de la transition socialiste, via la praxis dialectique et l'auto-activité des masses, contre la socialisation étatique. Ses écrits inspirent le KAPD et l'ultra-gauche, voyant les conseils comme alternative à la bureaucratisation stalinienne. Son influence perdure chez les communistes de conseils, soulignant la conscience ouvrière spontanée pour l'émancipation réelle. &lt;/p&gt; "/>
+    <hyperlink ref="E44" r:id="rId21" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Eugen_Rosenstock-Huessy&quot; title=&quot; Wikipedia&quot;&gt;Eugen ROSENSTOCK-HUESSY&lt;/a&gt; était un penseur germano‑américain dont l'œuvre mêle philosophie sociale, histoire des idées et une théorie du langage centrée sur la parole comme acte créateur et structurant de la vie collective. Né en Allemagne, il forma des liens intellectuels avec des figures comme Franz Rosenzweig et Martin Buber, fut professeur (notamment aux États‑Unis après son exil) et créa une œuvre originale qui vise à comprendre comment les communautés se constituent et se transforment dans le temps par des échanges de parole. &lt;/p&gt; &lt;p&gt; Au  &lt;a href=&quot;https://www.en-attendant-nadeau.fr/2019/11/19/homme-quadridimensionnel-rosenstock//&quot;  title=&quot;l’homme quadridimensionnel par ean&quot;&gt;cœur de sa pensée &lt;/a&gt;  se trouve la notion de &quot;speech thinking&quot; (pensée de la parole) : il soutient que la parole n’est pas qu’un moyen descriptif, mais un acte répondant et créatif qui institue des relations sociales, forge des temporalités collectives et permet la transmission et la renouvellement des institutions humaines. Il affirme que, par le langage, les groupes deviennent « maîtres du temps » en fondant de nouveaux commencements, en rappelant le passé et en orientant l’action future — d’où son intérêt pour la densité historique de la vie sociale et le rôle des rituels, des serments et des discours publics. &lt;/p&gt; &lt;p&gt; Sur la religion et la théologie, il s’inscrit dans un courant post‑nietzschéen de renouveau religieux qui comprend Rosenzweig et Buber; il considère les énoncés religieux comme des actes de parole non‑métaphysiques qui dévoilent des dimensions de l’expérience humaine et communautaire inaccessibles aux seules sciences naturelles. Cette orientation le conduit à une pensée intégrative où philosophie, théologie et histoire participent à une réflexion pratique sur la transformation sociale et la responsabilité collective. &lt;/p&gt; &lt;p&gt; Ses livres et conférences couvrent une grande variété de thèmes — histoire des peuples, rhétorique sociale, philosophie de la loi et de l’éducation — et sa méthode combine analyses historiques, typologies du langage et propositions pour renouveler la vie civique; son influence se voit aujourd’hui dans des études sur la communication, la sociologie historique et la philosophie de la culture. &lt;/p&gt; "/>
+    <hyperlink ref="H44" r:id="rId22" display="https://www.laphilo.fr/pho/erhuessy-mini.webp"/>
+    <hyperlink ref="E51" r:id="rId23" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Gershom_Scholem&quot; title=&quot; Wikipedia&quot;&gt;Gershom SCHOLEM&lt;/a&gt; était un philosophe juif germano-israélien,  fondateur de l'étude académique moderne de la Kabbale et grand expert de  &lt;a href=&quot;https://www.nonfiction.fr/article-12478-gershom-scholem-de-berlin-a-la-palestine.htm&quot; title=&quot;Gershom Scholem : de Berlin à la Palestine  par nonfiction&quot;&gt;la mystique juive. &lt;/a&gt; Né à Berlin dans une famille assimilée, il s'est tourné vers le sionisme jeune et a immigré en Palestine en 1923, devenant professeur à l'Université hébraïque de Jérusalem. &lt;/p&gt; &lt;p&gt; Il a étudié les mathématiques, la philosophie et les langues sémitiques à Berlin, Iéna et Munich, où il a soutenu une thèse sur le &quot;Sefer ha-Bahir&quot;, un texte kabbalistique ancien. Ami proche de Walter Benjamin et correspondant de Leo Strauss, il a fui l'Europe nazie et s'est consacré à la recherche sur les manuscrits juifs pillés. &lt;/p&gt; &lt;p&gt; Il voyait  &lt;a href=&quot;https://www.youtube.com/watch?v=5HvDF8-XTjc&quot;  title=&quot;Dieu son nom et la Cabale selon Gershom Scholem  par Xavier Charles DJEBALI&quot;&gt;la Kabbale &lt;/a&gt; non comme une superstition marginale, mais au cœur de l'essence spirituelle du judaïsme, explorée via des méthodes scientifiques et historiques. Il insistait sur le rôle du messianisme et de la tradition comme forces de renouvellement, où la révélation divine est infiniment interprétable et liée à l'expérience historique du peuple juif. Pour lui, le sionisme allait au-delà de la politique : c'était un renouveau profond du judaïsme, unissant ancien et nouveau contre l'assimilation. &lt;/p&gt; &lt;p&gt; Son oeuvre majeure &quot;Les Grandes tendances de la mystique juive&quot; paru en 1941, basé sur des conférences, dédié à Benjamin, explore l'évolution de la mystique juive. Sa pensée met l'accent sur l'identité juive forgée par l'histoire, où la tradition intègre la nouveauté pour survivre aux crises. &lt;/p&gt; &lt;audio controls title=&quot;Des livres pour notre temps et les mondes à venir. 1/2 Gershom Scholem : penser dans les marges de la marge par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13094-10.11.2019-ITEMA_22199082-0.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
+    <hyperlink ref="E52" r:id="rId24" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Leo_Strauss&quot; title=&quot; Wikipedia&quot;&gt;Leo SRAUSS&lt;/a&gt; était un philosophe politique germano-américain, connu pour sa critique profonde de la modernité et pour sa relecture des grands textes de la philosophie politique classique. Sa pensée a eu une influence durable, notamment aux États‑Unis, où elle a marqué des générations d’étudiants en théorie politique. &lt;/p&gt; &lt;p&gt; Au cœur de sa philosophie se trouve l’idée que la modernité a rompu avec le droit naturel classique, c’est‑à‑dire avec la recherche de ce qui est juste par nature et non simplement selon l’histoire ou les sciences sociales. Il voit dans le positivisme, le relativisme et l’historicisme modernes une source de décadence intellectuelle, car ils empêchent de poser les questions normatives fondamentales : qu’est‑ce qu’une vie bonne, qu’est‑ce qu’un régime politique juste. Pour lui, la  &lt;a href=&quot;https://www.persee.fr/doc/rfsp_0035-2950_1985_num_35_4_394205&quot; title=&quot;philosophie et zscience politique par persée&quot;&gt;philosophie politique authentique &lt;/a&gt; doit réactiver ces questions et affronter directement les notions de meilleur régime et d’ordre politique juste, plutôt que de se contenter de descriptions neutres. &lt;/p&gt; &lt;p&gt; Cette critique le conduit à renouer avec les auteurs de l’Antiquité, en particulier Platon, Aristote et les philosophes médiévaux juifs et arabes, qu’il lit souvent contre les interprétations modernes. Il insiste sur la dimension éducative de la philosophie : il parle de « liberal education » comme d’une libération de la vulgarité, entendue comme manque d’expérience des belles choses. La fréquentation des grands textes est, pour lui, une école de modestie et d’audace intellectuelle, parce qu’elle oblige à mesurer nos catégories modernes à celles d’auteurs qui pensaient autrement le politique et le juste. &lt;/p&gt; &lt;p&gt; Célèbre pour sa thèse sur l’« écriture ésotérique » : selon lui, nombre de philosophes du passé ont écrit de manière volontairement oblique pour se protéger de la censure ou de la persécution, réservant un sens plus profond aux lecteurs attentifs. Cela l’amène à distinguer entre le message « exotérique » (apparent, destiné au grand public) et le message « ésotérique » (plus exigeant, adressé à une minorité philosophique). Cette hypothèse sur la lecture des classiques s’articule à sa conception du   &lt;a href=&quot;https://www.youtube.com/watch?v=9Vhsveytymk&quot; title=&quot;nihilisme et politique leo strauss par bildung et culture&quot;&gt;mode de vie philosophique, &lt;/a&gt; toujours exposé au risque de la tyrannie et de l’incompréhension. Ainsi, sa philosophie politique est à la fois une critique de la modernité et une tentative de redécouvrir la place de la philosophie au cœur du politique contemporain. &lt;/p&gt; &#10; &lt;audio controls title=&quot;la pensée de leon strauss par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13397-05.04.2008-ITEMA_20118283-2008C3397E0019-ITE_00016207_RSCE-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;  &#10;"/>
+    <hyperlink ref="H52" r:id="rId25" display="https://www.laphilo.fr/pho/lstrauss-mini.webp"/>
+    <hyperlink ref="E55" r:id="rId26" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hans_Jonas&quot; title=&quot; Wikipedia&quot;&gt;Hans JONAS&lt;/a&gt;  était un philosophe germano-américain connu pour ses travaux sur l'éthique de la technologie et &lt;a href=&quot;https://www.youtube.com/watch?v=NPIJHZO7hQo&quot; title=&quot; Le PRINCIPE RESPONSABILITÉ en 6 minutes ! (HANS JONAS) par Culture Philo&quot;&gt;la responsabilité&lt;/a&gt; envers les générations futures. Ses premières recherches portent sur le gnosticisme, vu comme une réponse à l'aliénation existentielle dans un monde hostile. Dans les années 1960, il développe une philosophie de la vie organique (The Phenomenon of Life), critiquant le dualisme cartésien et valorisant la nature vivante contre la technoscience destructrice. Son œuvre maîtresse &lt;a href=&quot;https://www.youtube.com/watch?v=LsIWCR9_N64&quot; style=&quot;color:#88A1E9&quot; title=&quot; Philo, Hans jonas, Le principe responsabilité, Bac philo par SOS Bac Français&quot;&gt; &quot;Le Principe responsabilité&quot;&lt;/a&gt; paru en1979, formule un impératif éthique pour l'ère technologique : &quot;Agis de façon que les effets de ton action soient compatibles avec la permanence d'une vie authentiquement humaine sur Terre&quot;. &lt;/p&gt; &lt;p&gt; Il  anticipe les crises écologiques et bioéthiques, proposant une &quot;heuristique de la peur&quot; pour guider l'action humaine face aux risques imprévisibles de la puissance technique. Influencé par sa tradition juive et Heidegger, il réconcilie existentialisme, phénoménologie et morale prophétique, impactant l'éthique environnementale contemporaine. &lt;/p&gt; &lt;p&gt; Il observe un &quot;déchaînement prométhéen&quot; : l'humanité acquiert un pouvoir inédit sur la nature via la science et la technique, capable de menacer sa propre survie et celle des générations futures. Contrairement aux éthiques classiques (kantienne ou utilitariste), limitées au présent ou aux intentions, sa réflexion intègre les conséquences à long terme, imprévisibles et collectives, sur la vie humaine et la planète. Face aux risques inconnus (nucléaire, génétique, environnementaux), il prône une &quot;heuristique de la peur&quot; : anticiper le pire scénario (in dubio pro malo) pour guider l'action, sans paralyser le progrès mais en le subordonnant à la préservation de la vie. Le savoir devient un devoir moral prioritaire, élargissant l'éthique à la nature et aux générations absentes.&lt;/p&gt;  &lt;/p&gt; &lt;p&gt;  &lt;audio controls title=&quot; Hans Jonas. Pour une éthique de la société technologique par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/22267-14.06.2021-ITEMA_22702122-2014C12410E0357.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
+    <hyperlink ref="E58" r:id="rId27" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Reiner_Sch%C3%BCrmann&quot;  title=&quot; Wikipedia&quot;&gt;Reiner SCHÜRMANN&lt;/a&gt; est un philosophe allemand d’expression française, né à Amsterdam et mort à New York, où il a enseigné à la New School for Social Research à partir de 1975. Très marqué par la phénoménologie et la pensée de Heidegger, il se distingue par une réflexion exigeante sur la métaphysique, l’histoire de la philosophie et l’agir humain, développée dans trois grands ouvrages : Maître Eckhart et la joie errante (1972), Le principe d’anarchie (1982) et Des hégémonies brisées (posthume, 1996). &lt;/p&gt;&lt;p&gt; Dans Maître Eckhart et la joie errante, Schürmann reprend la pensée du mystique allemand du XIVᵉ siècle pour explorer la possibilité d’une vie spirituelle détachée de toute identité fixe ou de tout fondement stable. Il met en avant ce qu’il appelle une « joie errante » : une forme de liberté intérieure où le sujet ne se réclame plus d’une essence, d’un Dieu garanti ou d’une identité nationale, mais accepte de vivre dans une errance originaire et sans fondement. &lt;/p&gt; &lt;p&gt; Dans Le principe d’anarchie (souvent considéré comme son chef‑d’œuvre), Schürmann interprète Heidegger comme une pensée qui conduit à la ruine de tout principe premier (« archè ») sur lequel la tradition occidentale aurait voulu fonder la connaissance, la morale et la politique. Il en tire une théorie de l’« anarchie » non pas comme désordre, mais comme conscience lucide de l’absence de fondement ultime : l’agir humain doit alors se penser comme une praxis ouverte, responsable et créative, sans recours à une règle suprême. &lt;/p&gt; &lt;p&gt; Dans Des hégémonies brisées, Schürmann entreprend une vaste reconstruction de l’histoire de la philosophie occidentale comme succession d’« hégémonies » (modèles de vérité, de métaphysique, de politique) qui s’imposent, puis se défont. Il montre comment la modernité et la déconstruction heideggérienne ont dissous les grands systèmes de pensée, ouvrant à ce qu’il nomme une « philosophie tragique » où l’être se donne comme événement contingent, marqué par une distance, une fracture intérieure, plutôt que par une harmonie ou une cohérence totale. &lt;/p&gt; &#10;&#10;"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Ajoute la colonne « Traditions » et la frise des philosophes juifs
- Nouvelle colonne « Traditions » dans les 12 xlsx de philosophes
  (valeurs séparées par « ; »), lue par build-data.py et exposée aux
  frises et à la recherche.
- Frise /philosophes/frise/pensee-juive-toutes-epoques/ : 100 philosophes
  juifs de toutes nationalités (marqués « juive », chaque nom vérifié sur
  Wikipédia). Pastille « Juifs » dans la recherche, lien depuis le
  cartouche de /histoire-des-philosophes/, carte dans le catalogue.
- build-data.py signale les erreurs de saisie probables (dates affichées
  incohérentes, doublons, nationalité manquante, courant inconnu).
- « HILLET Hazaken » corrigé en « HILLEL Hazaken », redirection 301.
- Dimension de feuille corrigée dans les xlsx (modernes déclarait
  1 048 576 lignes).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -758,6 +758,11 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="M3" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traditions</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="137.25" customHeight="1" s="30">
       <c r="A4" s="35" t="n">
@@ -1777,7 +1782,11 @@
           <t>philosophe prussien qui développa l'idéologie Marxiste.</t>
         </is>
       </c>
-      <c r="M21" s="29" t="n"/>
+      <c r="M21" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="213.4" customHeight="1" s="30">
       <c r="A22" s="35" t="n">
@@ -2169,6 +2178,11 @@
           <t>philosophe juif allemand fondateur de l’école de Marbourg, un courant néokantien.</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="284.25" customHeight="1" s="30">
       <c r="A29" s="35" t="n">
@@ -2451,6 +2465,11 @@
           <t>philosophe et neurologue allemand connu pour son travail sur la psychanalyse.</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="279.1" customHeight="1" s="30">
       <c r="A34" s="35" t="n">
@@ -2507,7 +2526,11 @@
           <t>philosophe prussien cofondateur de la sociologie de la modernité "sociologie formelle".</t>
         </is>
       </c>
-      <c r="M34" s="29" t="n"/>
+      <c r="M34" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="245.25" customHeight="1" s="30">
       <c r="A35" s="35" t="n">
@@ -2564,6 +2587,11 @@
       <c r="L35" s="29" t="inlineStr">
         <is>
           <t>philosophe autrichien fondateur de la phénoménologie.</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
         </is>
       </c>
     </row>
@@ -2796,6 +2824,11 @@
           <t xml:space="preserve">philosophe et essayiste allemand  penseur critique de la modernité, du nationalisme et de l’antisémitisme. </t>
         </is>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="253.5" customHeight="1" s="30">
       <c r="A40" s="35" t="n">
@@ -2910,6 +2943,11 @@
           <t>philosophe allemand  figure importante du  néokantisme.</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="227.25" customHeight="1" s="30">
       <c r="A42" s="35" t="n">
@@ -3135,6 +3173,11 @@
           <t>philosophe juif allemand rattaché au marxisme hétérodoxe et à la philosophie de l’espérance.</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="153" customHeight="1" s="30">
       <c r="A46" s="35" t="n">
@@ -3249,6 +3292,11 @@
           <t>philosophe juif allemand auteur de "L’Étoile de la rédemption".</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="203.25" customHeight="1" s="30">
       <c r="A48" s="35" t="n">
@@ -3360,6 +3408,11 @@
           <t>philosophe germano‑américain mêlant philosophie sociale &amp; histoire des idées.</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="213" customHeight="1" s="30">
       <c r="A50" s="35" t="n">
@@ -3585,6 +3638,11 @@
           <t>philosophe allemand connu pour ses réflexions marxistes, mystiques juives et esthétiques.</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="144.75" customHeight="1" s="30">
       <c r="A54" s="35" t="n">
@@ -3698,6 +3756,11 @@
           <t>philosophe allemand classé dans la sociologie de la connaissance et  compréhensive .</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="181.5" customHeight="1" s="30">
       <c r="A56" s="35" t="n">
@@ -3754,6 +3817,11 @@
           <t>philosophe allemand de l'école de Francfort associé à la Théorie critique.</t>
         </is>
       </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="215.25" customHeight="1" s="30">
       <c r="A57" s="35" t="n">
@@ -3810,6 +3878,11 @@
           <t>philosophe juif germano-israélien fondateur de l'étude académique moderne de la Kabbale.</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="316.5" customHeight="1" s="30">
       <c r="A58" s="35" t="n">
@@ -3866,6 +3939,11 @@
           <t>philosophe politique germano-américain connu pour sa critique de la modernité.</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="231.75" customHeight="1" s="30">
       <c r="A59" s="35" t="n">
@@ -3979,6 +4057,11 @@
           <t>philosophe et sociologue allemand principal représentant de l'école de Francfort.</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="176.25" customHeight="1" s="30">
       <c r="A61" s="35" t="n">
@@ -4034,6 +4117,11 @@
       <c r="L61" s="29" t="inlineStr">
         <is>
           <t>philosophe germano-américain connu pour son éthique pour l'âge technologique.</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche refaite, philosophes vivants par sujet de travail, corrections de données
Recherche : cartouches repliables en listes déroulantes (Filtres, Philosophes
d'aujourd'hui, Par tradition, Tradition des courants), barre de tri au-dessus
de la liste avec bouton de sens et réinitialisation, adaptation mobile.
Vivants : colonne Thèmes des xlsx d'actifs, huit frises vivants-<thème>.
Données : noms corrigés (Stiegler, Giordano Bruno, Felwine Sarr, Rancière…)
avec redirections 301, Kripke et Searle passés chez les Américains, PDF de
Freud restauré, vignettes du Proche-Orient ancien.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -983,7 +983,7 @@
       </c>
       <c r="E7" s="40" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Friedrich_Schleiermacher"   title=" Wikipedia"&gt;Friedrich SCHEIERMACHER&lt;/a&gt;  était un philosophe prussien,  souvent considéré comme le "père de la théologie libérale moderne". &lt;a href="https://www.persee.fr/doc/rhpr_0035-2403_2011_num_91_1_1522"  title="son apport théorique et pratique par persée"&gt;Sa philosophie &lt;/a&gt; intègre des éléments du romantisme, de l'idéalisme allemand et du piétisme, en centrant l'humain sur une conscience intuitive de l'infini. Il édita Platon, prêcha et influença le protestantisme européen sans séparer foi et culture. &lt;/p&gt; &lt;p&gt;  Il pose le sentiment religieux comme une conscience immédiate de la dépendance absolue envers l'infini (Dieu), distincte du savoir ou de la morale kantienne. L'ego est une individualisation de la  &lt;a href="https://www.youtube.com/watch?v=gvpaUR1XceM"  style="color:#88A1E9"  title="Schleiermacher: The Man Behind Protestant Liberalism par Stephen D Morrison"&gt;raison universelle, &lt;/a&gt; un microcosme où univers et individu s'unissent via la conscience de soi. Il articule individualité et communauté via la communication, honorant la finitude humaine et l'invention de soi contre l'absolutisme idéaliste. &lt;/p&gt; &lt;p&gt; Ses œuvres majeures sont "Discours sur la religion" paru en 1799 et "La foi chrétienne"  paru vers 1821, où il réconcilie rationalité et piété. Il a profondément marqué la théologie protestante moderne en introduisant une approche centrée sur le sentiment religieux et l'expérience personnelle, plutôt que sur les dogmes rigides ou la raison pure. Son idée de "dépendance absolue" envers Dieu et la relativisation des doctrines comme expressions humaines de la piété ont pavé la voie au &lt;a href="https://www.youtube.com/watch?v=1FveOtAB86s"  title="L'argument éthique de Schleiermacher en faveur de l'universalisme par Sola Media"&gt;libéralisme théologique. &lt;/a&gt;&lt;/p&gt; &lt;p&gt;  Fondateur de l'herméneutique moderne, art général d'interprétation reliant traduction, littérature et exégèse biblique, il lance l'herméneutique critique de l'Écriture et une théologie pratique pertinente pour la modernité, influençant Ritschl et l'individualisme religieux.&lt;/p&gt; </t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Friedrich_Schleiermacher"   title=" Wikipedia"&gt;Friedrich SCHLEIERMACHER&lt;/a&gt;  était un philosophe prussien,  souvent considéré comme le "père de la théologie libérale moderne". &lt;a href="https://www.persee.fr/doc/rhpr_0035-2403_2011_num_91_1_1522"  title="son apport théorique et pratique par persée"&gt;Sa philosophie &lt;/a&gt; intègre des éléments du romantisme, de l'idéalisme allemand et du piétisme, en centrant l'humain sur une conscience intuitive de l'infini. Il édita Platon, prêcha et influença le protestantisme européen sans séparer foi et culture. &lt;/p&gt; &lt;p&gt;  Il pose le sentiment religieux comme une conscience immédiate de la dépendance absolue envers l'infini (Dieu), distincte du savoir ou de la morale kantienne. L'ego est une individualisation de la  &lt;a href="https://www.youtube.com/watch?v=gvpaUR1XceM"  style="color:#88A1E9"  title="Schleiermacher: The Man Behind Protestant Liberalism par Stephen D Morrison"&gt;raison universelle, &lt;/a&gt; un microcosme où univers et individu s'unissent via la conscience de soi. Il articule individualité et communauté via la communication, honorant la finitude humaine et l'invention de soi contre l'absolutisme idéaliste. &lt;/p&gt; &lt;p&gt; Ses œuvres majeures sont "Discours sur la religion" paru en 1799 et "La foi chrétienne"  paru vers 1821, où il réconcilie rationalité et piété. Il a profondément marqué la théologie protestante moderne en introduisant une approche centrée sur le sentiment religieux et l'expérience personnelle, plutôt que sur les dogmes rigides ou la raison pure. Son idée de "dépendance absolue" envers Dieu et la relativisation des doctrines comme expressions humaines de la piété ont pavé la voie au &lt;a href="https://www.youtube.com/watch?v=1FveOtAB86s"  title="L'argument éthique de Schleiermacher en faveur de l'universalisme par Sola Media"&gt;libéralisme théologique. &lt;/a&gt;&lt;/p&gt; &lt;p&gt;  Fondateur de l'herméneutique moderne, art général d'interprétation reliant traduction, littérature et exégèse biblique, il lance l'herméneutique critique de l'Écriture et une théologie pratique pertinente pour la modernité, influençant Ritschl et l'individualisme religieux.&lt;/p&gt; </t>
         </is>
       </c>
       <c r="F7" s="35" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="E10" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Friedrich_Karl_Forberg" title=" Wikipedia"&gt;Friedrick Karl FORBERG&lt;/a&gt;  était un philosophe allemand  figure mineure mais controversée de l'idéalisme allemand post-kantien, connu pour ses liens avec Fichte et son implication dans   &lt;a href="https://laviedesidees.fr/Le-juge-et-le-policier"  style="color:#88A1E9"  title="Le juge et le policier par la vie des idées"&gt;"l'Atheismusstreit" &lt;/a&gt; (querelle de l'athéisme). Il est un l'héritier des Lumières et de Kant, influencé par Reinhold et Fichte, qu'il considère comme un maître et ami. &lt;/p&gt; &lt;p&gt; Il défend une philosophie critique et idéaliste, centrée sur l'esthétique transcendante et les fondements de l'action libre. Rationaliste protestant, il s'intéresse à l'exégèse biblique et aux langues anciennes (grec, latin), révisant des auteurs comme Aristophane ou Horace. &lt;/p&gt; &lt;p&gt; Son essai "Entwicklung des Begriffs der Religion" paru en 1798  est central : il définit la religion comme un "postulat pratique" moral, indépendant de preuves théoriques de Dieu ou d'une "ordre divin". La foi n'est pas spéculative mais un engagement éthique dans une "ordre moral du monde", sans besoin de métaphysique théiste – une position fichtéenne radicale. Il  incarne un rationalisme audacieux : lucide sur l'absence de preuves divines, il mise tout sur la moralité humaine autonome.  &lt;/p&gt; </t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Friedrich_Karl_Forberg" title=" Wikipedia"&gt;Friedrich Karl FORBERG&lt;/a&gt;  était un philosophe allemand  figure mineure mais controversée de l'idéalisme allemand post-kantien, connu pour ses liens avec Fichte et son implication dans   &lt;a href="https://laviedesidees.fr/Le-juge-et-le-policier"  style="color:#88A1E9"  title="Le juge et le policier par la vie des idées"&gt;"l'Atheismusstreit" &lt;/a&gt; (querelle de l'athéisme). Il est un l'héritier des Lumières et de Kant, influencé par Reinhold et Fichte, qu'il considère comme un maître et ami. &lt;/p&gt; &lt;p&gt; Il défend une philosophie critique et idéaliste, centrée sur l'esthétique transcendante et les fondements de l'action libre. Rationaliste protestant, il s'intéresse à l'exégèse biblique et aux langues anciennes (grec, latin), révisant des auteurs comme Aristophane ou Horace. &lt;/p&gt; &lt;p&gt; Son essai "Entwicklung des Begriffs der Religion" paru en 1798  est central : il définit la religion comme un "postulat pratique" moral, indépendant de preuves théoriques de Dieu ou d'une "ordre divin". La foi n'est pas spéculative mais un engagement éthique dans une "ordre moral du monde", sans besoin de métaphysique théiste – une position fichtéenne radicale. Il  incarne un rationalisme audacieux : lucide sur l'absence de preuves divines, il mise tout sur la moralité humaine autonome.  &lt;/p&gt; </t>
         </is>
       </c>
       <c r="F10" s="35" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Christian_Friedrich_Krause"  title=" Wikipedia"&gt;Karl Christian Friedrich KRAUSE&lt;/a&gt; était un philosophe allemand marquée par &lt;a href="https://www.youtube.com/watch?v=xEGV23CVwgc"  title="Krausism par WikiTubia"&gt;le krausisme &lt;/a&gt; dont le système a exercé une influence notable en Espagne et en Amérique latine. Il propose une forme &lt;a href="https://www.persee.fr/doc/phlou_0776-5541_1897_num_4_16_1574"  title="Quelques formes contemporaines du Panthéisme  par Persée"&gt;d’idéalisme panentéiste &lt;/a&gt; visant à réconcilier Dieu comme substance universelle avec le monde et l’humanité, et voit l’univers comme un &lt;a href="https://450.fm/2023/03/18/franc-macon-et-philosophe-du-droit-karl-krause-du-soin-divin-de-la-loi/" style="color:#88A1E9" title="Franc-maçon et philosophe du droit Karl Krause : « Du soin divin de la loi » par 450fm"&gt;organisme divin &lt;/a&gt; en développement. &lt;/p&gt; &lt;p&gt; Il soutient que Dieu est une réalité infinie et un ground de tout être et savoir, et que l’univers s’organise autour de cette essence absolue. Cette approche cherche à dépasser les limites des conceptions strictement théistes ou matérialistes en affirmant l’interpénétration de l’infini divin et du monde fini. Pour lui, le monde et l’humanité constituent un organisme qui évolue vers une unité supérieure, avec le principe du droit parfait (ou loi) comme moteur du développement moral et social. Cette idée implique une continuité entre l’individu, les groupes et l’humanité entière dans un processus d’unification spirituelle. &lt;/p&gt; &lt;p&gt; Le système Krause a donné naissance au krausisme, un courant influent dans l’orthodoxie libérale et l’éducation en Espagne et ailleurs, où ses idées ont nourri des réformes éducatives et des débats sur la tolérance, la citoyenneté et l’éthique civique. Il tenta de réconcilier la connaissance sensible et l’intuition religieuse ou morale, cherchant à montrer que la raison et la foi ne s’opposent pas mais se complètent dans la connaissance de Dieu et du monde. &lt;/p&gt; &lt;p&gt; Ses Œuvres majeures sont :  - Entwurf des Systems der Philosophie paru en 1804 , une esquisse systématique de sa philosophie.  - Vorlesungen über das System der Philosophie  en 1828, un cours sur son système philosophique. &lt;/p&gt; 
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Christian_Friedrich_Krause"  title=" Wikipedia"&gt;Karl Christian Friedrich KRAUSE&lt;/a&gt; était un philosophe allemand marqué par &lt;a href="https://www.youtube.com/watch?v=xEGV23CVwgc"  title="Krausism par WikiTubia"&gt;le krausisme &lt;/a&gt; dont le système a exercé une influence notable en Espagne et en Amérique latine. Il propose une forme &lt;a href="https://www.persee.fr/doc/phlou_0776-5541_1897_num_4_16_1574"  title="Quelques formes contemporaines du Panthéisme  par Persée"&gt;d’idéalisme panentéiste &lt;/a&gt; visant à réconcilier Dieu comme substance universelle avec le monde et l’humanité, et voit l’univers comme un &lt;a href="https://450.fm/2023/03/18/franc-macon-et-philosophe-du-droit-karl-krause-du-soin-divin-de-la-loi/" style="color:#88A1E9" title="Franc-maçon et philosophe du droit Karl Krause : « Du soin divin de la loi » par 450fm"&gt;organisme divin &lt;/a&gt; en développement. &lt;/p&gt; &lt;p&gt; Il soutient que Dieu est une réalité infinie et un ground de tout être et savoir, et que l’univers s’organise autour de cette essence absolue. Cette approche cherche à dépasser les limites des conceptions strictement théistes ou matérialistes en affirmant l’interpénétration de l’infini divin et du monde fini. Pour lui, le monde et l’humanité constituent un organisme qui évolue vers une unité supérieure, avec le principe du droit parfait (ou loi) comme moteur du développement moral et social. Cette idée implique une continuité entre l’individu, les groupes et l’humanité entière dans un processus d’unification spirituelle. &lt;/p&gt; &lt;p&gt; Le système Krause a donné naissance au krausisme, un courant influent dans l’orthodoxie libérale et l’éducation en Espagne et ailleurs, où ses idées ont nourri des réformes éducatives et des débats sur la tolérance, la citoyenneté et l’éthique civique. Il tenta de réconcilier la connaissance sensible et l’intuition religieuse ou morale, cherchant à montrer que la raison et la foi ne s’opposent pas mais se complètent dans la connaissance de Dieu et du monde. &lt;/p&gt; &lt;p&gt; Ses Œuvres majeures sont :  - Entwurf des Systems der Philosophie paru en 1804 , une esquisse systématique de sa philosophie.  - Vorlesungen über das System der Philosophie  en 1828, un cours sur son système philosophique. &lt;/p&gt; 
 </t>
         </is>
       </c>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="E33" s="40" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Sigmund_Freud"  title=" Wikipedia"&gt; Sigmund FREUD&lt;/a&gt; est un neurologue et philosophe Allemand connu pour son travail sur la Psychanalyse et son point de vue sur  &lt;a  href="https://www.youtube.com/watch?v=uYd0Xi3ACQ8&amp;t=17s&amp;ab_channel=LePr%C3%A9cepteur"  title="L'origine de la religion par Le Précepteur"&gt;la Religion&lt;/a&gt;. &lt;/p&gt; &lt;p&gt;  Et si ce n’était pas la raison et la volonté, mais l’inconscient et ses pulsions violentes et destructrices, qui étaient la grande force de l’esprit et de l’histoire ? Voilà l’hypothèse scandaleuse qui est au cœur de l’œuvre de Freud. &lt;/p&gt; &lt;p&gt; Si le concept avait été envisagée par d’autres, seul William James en 1875 organisa des travaux de psychologie à l'université d'Harward. &lt;a  href="https://www.laphilo.fr/document/le_reve_et_son_interpretation.pdf"  title="Le rêve et son interprétation en version numérique"&gt;"Le rêve et son interprétation"&lt;/a&gt;, publié en 1900, fait de l’analyse des rêves la « voie royale » pour aborder l’inconscient.&lt;/p&gt; &lt;p&gt;  Il est amené à repenser son modèle pour en accentuer la dimension conflictuelle entre ce qu’il nomme désormais &lt;a  href="https://www.youtube.com/watch?v=QO7HTLC0r6I&amp;ab_channel=Coursitout" title="Le ça, le moi et le surmoi par Coursitout"&gt;le « Ça », le « Moi » et le « Surmoi »&lt;/a&gt;. &lt;/p&gt; &lt;p&gt; Le Ça, correspondant à l’inconscient, est la partie obscure et inaccessible de notre personnalité. Le Moi, socle de la personnalité, est l’instance intermédiaire qui doit concilier les exigences contradictoires du Ça et du Surmoi. Le Surmoi, lui, est le juge intérieur qui naît de l’intériorisation des interdits sociaux. &lt;/p&gt; &lt;p&gt; Si  &lt;a  href="https://www.youtube.com/watch?v=b_v6YfaC5gU&amp;t=17s&amp;ab_channel=LePr%C3%A9cepteur"  title="L'inconscient par Le Précepteur"&gt;l’inconscient&lt;/a&gt; est ce chaos au cœur de l’individu, il devient le cœur du processus de civilisation. &lt;/p&gt; &lt;p&gt; En 1933, les œuvres de Freud sont brûlées par les Nazis mais le travail de Freud n’en reste pas moins incontournable dans l’histoire de la psychologie moderne. Sa postérité est immense. &lt;/p&gt;  &lt;audio controls title="L'Ombilic des rêves par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/19288-29.07.2018-ITEMA_21741416-2.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Sigmund_Freud"  title=" Wikipedia"&gt; Sigmund FREUD&lt;/a&gt; est un neurologue et philosophe Allemand connu pour son travail sur la Psychanalyse et son point de vue sur  &lt;a  href="https://www.youtube.com/watch?v=uYd0Xi3ACQ8&amp;t=17s&amp;ab_channel=LePr%C3%A9cepteur"  title="L'origine de la religion par Le Précepteur"&gt;la Religion&lt;/a&gt;. &lt;/p&gt; &lt;p&gt;  Et si ce n’était pas la raison et la volonté, mais l’inconscient et ses pulsions violentes et destructrices, qui étaient la grande force de l’esprit et de l’histoire ? Voilà l’hypothèse scandaleuse qui est au cœur de l’œuvre de Freud. &lt;/p&gt; &lt;p&gt; Si le concept avait été envisagée par d’autres, seul William James en 1875 organisa des travaux de psychologie à l'université d'Harvard. &lt;a  href="/document/le_reve_et_son_interpretation.pdf"  title="Le rêve et son interprétation en version numérique"&gt;"Le rêve et son interprétation"&lt;/a&gt;, publié en 1900, fait de l’analyse des rêves la « voie royale » pour aborder l’inconscient.&lt;/p&gt; &lt;p&gt;  Il est amené à repenser son modèle pour en accentuer la dimension conflictuelle entre ce qu’il nomme désormais &lt;a  href="https://www.youtube.com/watch?v=QO7HTLC0r6I&amp;ab_channel=Coursitout" title="Le ça, le moi et le surmoi par Coursitout"&gt;le « Ça », le « Moi » et le « Surmoi »&lt;/a&gt;. &lt;/p&gt; &lt;p&gt; Le Ça, correspondant à l’inconscient, est la partie obscure et inaccessible de notre personnalité. Le Moi, socle de la personnalité, est l’instance intermédiaire qui doit concilier les exigences contradictoires du Ça et du Surmoi. Le Surmoi, lui, est le juge intérieur qui naît de l’intériorisation des interdits sociaux. &lt;/p&gt; &lt;p&gt; Si  &lt;a  href="https://www.youtube.com/watch?v=b_v6YfaC5gU&amp;t=17s&amp;ab_channel=LePr%C3%A9cepteur"  title="L'inconscient par Le Précepteur"&gt;l’inconscient&lt;/a&gt; est ce chaos au cœur de l’individu, il devient le cœur du processus de civilisation. &lt;/p&gt; &lt;p&gt; En 1933, les œuvres de Freud sont brûlées par les Nazis mais le travail de Freud n’en reste pas moins incontournable dans l’histoire de la psychologie moderne. Sa postérité est immense. &lt;/p&gt;  &lt;audio controls title="L'Ombilic des rêves par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/19288-29.07.2018-ITEMA_21741416-2.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
Lot 10 : Croce, Jaspers, Teilhard de Chardin, Du Bois, Ryle, Strawson, Lakatos, Feyerabend, MacIntyre, Eco, Negri ; Leibniz et Peirce correctement orthographiés (301 depuis les anciennes adresses)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -5264,18 +5264,60 @@
       </c>
     </row>
     <row r="68" customFormat="false" ht="267.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0"/>
-      <c r="B68" s="0"/>
-      <c r="C68" s="0"/>
-      <c r="D68" s="0"/>
-      <c r="E68" s="0"/>
+      <c r="A68" s="0">
+        <v>1883</v>
+      </c>
+      <c r="B68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1969</t>
+        </is>
+      </c>
+      <c r="C68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1883 – 1969</t>
+        </is>
+      </c>
+      <c r="D68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Karl JASPERS</t>
+        </is>
+      </c>
+      <c r="E68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Jaspers" title=" Wikipedia"&gt;Karl JASPERS&lt;/a&gt; est un psychiatre et philosophe allemand, l’un des fondateurs de la philosophie de l’existence. Né à Oldenbourg, il étudie le droit puis la médecine et travaille à la clinique psychiatrique de Heidelberg. Son &lt;em&gt;Psychopathologie générale&lt;/em&gt; (1913) renouvelle la psychiatrie en distinguant ce que l’on peut « expliquer » par des causes et ce que l’on doit « comprendre » de l’intérieur, dans l’expérience du malade. Il se tourne ensuite vers la philosophie, qu’il enseigne à Heidelberg.&lt;/p&gt; &lt;p&gt;Dans sa &lt;em&gt;Philosophie&lt;/em&gt; (1932), il distingue l’existence de tout ce que la science peut connaître : ce que je suis vraiment ne se laisse pas réduire à un objet. C’est dans les « situations limites », la mort, la souffrance, la lutte, la culpabilité, que l’homme découvre qu’il ne peut rien maîtriser et s’ouvre à la « transcendance ». La communication authentique avec autrui, une « lutte aimante », est le lieu où chacun devient lui-même. Il forge aussi la notion d’« âge axial » pour désigner le moment, autour du VIe siècle avant notre ère, où naissent presque en même temps les grandes sagesses de la Chine, de l’Inde, de la Perse, d’Israël et de la Grèce.&lt;/p&gt; &lt;p&gt;Marié à une femme juive, Gertrud, il est privé d’enseignement par les nazis en 1937 et vit sous la menace de la déportation. Après la guerre, il publie &lt;em&gt;La Culpabilité allemande&lt;/em&gt; (1946), où il distingue culpabilité criminelle, politique, morale et métaphysique. Maître et ami d’&lt;a href="https://fr.wikipedia.org/wiki/Hannah_Arendt" title=" Wikipedia"&gt;Hannah Arendt&lt;/a&gt;, il s’installe à Bâle en 1948 et y meurt en 1969.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="F68" s="0"/>
       <c r="G68" s="0"/>
-      <c r="H68" s="0"/>
+      <c r="H68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/jaspers-mini.webp</t>
+        </is>
+      </c>
       <c r="I68" s="0"/>
-      <c r="J68" s="0"/>
-      <c r="K68" s="0"/>
-      <c r="L68" s="0"/>
+      <c r="J68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique ; politique</t>
+        </is>
+      </c>
+      <c r="K68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Existentialisme</t>
+        </is>
+      </c>
+      <c r="L68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">psychiatre et philosophe allemand, penseur de l’existence, des situations limites et de la culpabilité.</t>
+        </is>
+      </c>
+      <c r="N68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O68">
+        <v>3</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="0"/>

</xml_diff>

<commit_message>
Courants à un seul philosophe, lot 4 : 22 fiches nouvelles (Shang Yang, Hui Shi, Kumarila, Phule, Bernstein, Kamo no Mabuchi, Tsunetomo, Vinoba Bhave, Jayarashi, Trần Nhân Tông, Choe Si-hyeong, Ibn Abd al-Wahhab, Chamoiseau, Cratyle, Joan Robinson, Julian Huxley, Berthelot, Duhem, Davidson, Gioberti, da Costa, Collier) ; vidéo de Simón Bolívar (éditeur)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -5383,18 +5383,63 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0"/>
-      <c r="B69" s="0"/>
-      <c r="C69" s="0"/>
-      <c r="D69" s="0"/>
-      <c r="E69" s="0"/>
+      <c r="A69" s="0">
+        <v>1850</v>
+      </c>
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1932</t>
+        </is>
+      </c>
+      <c r="C69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1850 – 1932</t>
+        </is>
+      </c>
+      <c r="D69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eduard BERNSTEIN</t>
+        </is>
+      </c>
+      <c r="E69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Eduard_Bernstein" title=" Wikipedia"&gt;Eduard BERNSTEIN&lt;/a&gt; est un théoricien et homme politique allemand, le père du « révisionnisme » et l’un des fondateurs de la &lt;a href="https://fr.wikipedia.org/wiki/Social-d%C3%A9mocratie" title=" Wikipedia"&gt;social-démocratie&lt;/a&gt; moderne. Né à Berlin en 1850 dans une famille juive modeste, fils d’un mécanicien de locomotive, il est employé de banque quand il adhère en 1872 au parti social-démocrate. Les lois antisocialistes de Bismarck le contraignent à l’exil : en Suisse, où il dirige le journal du parti, puis à Londres, où il devient l’ami et le collaborateur de Friedrich Engels, qui fait de lui l’un de ses exécuteurs testamentaires.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Les Présupposés du socialisme&lt;/em&gt; (1899), il soumet le marxisme à l’épreuve des faits. Le capitalisme ne s’effondre pas, les classes moyennes ne disparaissent pas, la misère ouvrière ne s’aggrave pas : la théorie de la catastrophe finale est démentie. Le socialisme ne viendra pas d’une révolution, mais de réformes progressives, conquises par les syndicats, les coopératives et le suffrage universel. Il est l’héritier du libéralisme, et doit s’appuyer sur une éthique d’inspiration kantienne plutôt que sur une prétendue nécessité de l’histoire. « Ce qu’on appelle d’ordinaire le but final du socialisme n’est rien pour moi, le mouvement est tout. »&lt;/p&gt; &lt;p&gt;Ce « révisionnisme » déclenche une violente controverse. Karl Kautsky le combat au nom de l’orthodoxie, et &lt;a href="https://fr.wikipedia.org/wiki/Rosa_Luxemburg" title=" Wikipedia"&gt;Rosa Luxemburg&lt;/a&gt; lui répond par &lt;em&gt;Réforme sociale ou révolution ?&lt;/em&gt; (1899). Officiellement condamné par le parti, Bernstein inspire pourtant sa pratique réelle. Député au Reichstag, il vote en 1915 contre les crédits de guerre. Il meurt à Berlin en décembre 1932, peu avant l’arrivée de Hitler au pouvoir. En 1959, le programme de Bad Godesberg, par lequel le SPD renonce au marxisme, consacre ses idées.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="F69" s="0"/>
       <c r="G69" s="0"/>
-      <c r="H69" s="0"/>
+      <c r="H69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/bernstein-mini.webp</t>
+        </is>
+      </c>
       <c r="I69" s="0"/>
-      <c r="J69" s="0"/>
-      <c r="K69" s="0"/>
-      <c r="L69" s="0"/>
+      <c r="J69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">politique</t>
+        </is>
+      </c>
+      <c r="K69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Social-démocratie ; Marxisme</t>
+        </is>
+      </c>
+      <c r="L69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">théoricien socialiste allemand, père du révisionnisme et de la social-démocratie réformiste.</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
+      <c r="N69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O69"/>
       <c r="XFC69" s="0"/>
       <c r="XFD69" s="0"/>
     </row>

</xml_diff>

<commit_message>
36 fiches nouvelles (onglets « philowait ») : Fontenelle, Rosmini, Ubaghs, K. L. Michelet, Nadejdine, Darwin, Lewes, Tyndall, Mach, Clifford, Eucken, Poincaré, Léon Robin, Dupréel, R. W. Sellars, C. D. Broad, Piaget, Jakobson, Gouhier, W. Sellars, Birault, Starobinski, Gorz, Danto, Frankfurt, Alain Roger, Rabhi, Dascal, Earman, Cartwright, Loewer, Besnier, Susan Wolf, J. D. Norton, Brading, Werndl ; frise « Occident » remplacée par trois frises (Antiquité à 1700, Lumières à 1900, depuis 1900)
- Placement dans les frises vérifié pour les 252 fiches ajoutées depuis le 3 octobre :
  Newton da Costa (mort en 2024) passe chez les Américains ; Kim Yong-ok et
  Patrick Chamoiseau, vivants, passent chez les contemporains du monde ;
  Piaget et Starobinski comptés comme Suisses francophones ; Dascal hors des
  Pensées du Sud ; Gorz et Lakatos dans la pensée juive
- Dalaï-lama : vidéo INA, podcast France Culture, portrait (éditeur)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -2572,7 +2572,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD69"/>
+  <dimension ref="A1:XFD71"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.93"/>
@@ -5442,6 +5442,108 @@
       <c r="O69"/>
       <c r="XFC69" s="0"/>
       <c r="XFD69" s="0"/>
+    </row>
+    <row r="70" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0">
+        <v>1801</v>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1801 – 1893</t>
+        </is>
+      </c>
+      <c r="D70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Karl Ludwig MICHELET</t>
+        </is>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Ludwig_Michelet" title=" Wikipedia"&gt;Karl Ludwig MICHELET&lt;/a&gt; est un philosophe allemand, l’un des disciples les plus fidèles de &lt;a href="https://fr.wikipedia.org/wiki/Georg_Wilhelm_Friedrich_Hegel" title=" Wikipedia"&gt;Hegel&lt;/a&gt;. Né à Berlin en 1801 dans une famille de marchands huguenots, d’origine française, il suit les cours de Hegel et enseigne à l’université de Berlin pendant des décennies. Après la mort du maître en 1831, il fait partie du groupe d’élèves qui publient ses œuvres complètes et prépare l’édition de ses &lt;em&gt;Leçons sur l’histoire de la philosophie&lt;/em&gt;.&lt;/p&gt; &lt;p&gt;Spécialiste d’Aristote, il écrit en français un &lt;em&gt;Examen critique du livre d’Aristote intitulé Métaphysique&lt;/em&gt;, couronné en 1836 par l’Académie des sciences morales et politiques en même temps que l’essai de Félix Ravaisson. Quand l’école de Hegel se divise sur la religion et la politique, il reprend la distinction proposée par son élève David Friedrich Strauss entre une « droite », fidèle au christianisme, une « gauche », celle des &lt;a href="https://fr.wikipedia.org/wiki/Jeunes_h%C3%A9g%C3%A9liens" title=" Wikipedia"&gt;Jeunes hégéliens&lt;/a&gt;, et un « centre », auquel il se rattache. Pour lui, Dieu n’est pas une personne séparée du monde : il devient personnel dans l’esprit humain, et l’immortalité n’est pas celle de l’individu, mais celle de l’esprit qui se développe dans l’histoire.&lt;/p&gt; &lt;p&gt;En 1843, il fonde avec ses élèves la Société philosophique de Berlin, qui maintient la tradition hégélienne pendant tout le siècle. Il y défend Hegel contre la critique que lui adresse Schelling, revenu à Berlin en 1841, et publie une histoire de la philosophie allemande de Kant à Hegel, puis une philosophie du droit. Fidèle jusqu’au bout, il intitule l’un de ses derniers livres &lt;em&gt;Hegel, le philosophe universel irréfuté&lt;/em&gt; (1870). Il meurt à Berlin en 1893, à quatre-vingt-onze ans.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/klmichelet-mini.webp</t>
+        </is>
+      </c>
+      <c r="J70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique ; ethique</t>
+        </is>
+      </c>
+      <c r="K70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand</t>
+        </is>
+      </c>
+      <c r="L70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe allemand, disciple et éditeur de Hegel, chef du « centre » hégélien.</t>
+        </is>
+      </c>
+      <c r="N70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O70"/>
+    </row>
+    <row r="71" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="0">
+        <v>1846</v>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1926</t>
+        </is>
+      </c>
+      <c r="C71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1846 – 1926</t>
+        </is>
+      </c>
+      <c r="D71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rudolf EUCKEN</t>
+        </is>
+      </c>
+      <c r="E71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Rudolf_Christoph_Eucken" title=" Wikipedia"&gt;Rudolf EUCKEN&lt;/a&gt; est un philosophe allemand. Né en 1846 à Aurich, en Frise orientale, il étudie à Göttingen et à Berlin, où il suit l’enseignement de Friedrich Adolf Trendelenburg, spécialiste d’Aristote. Professeur à Bâle, puis à Iéna de 1874 à 1920, il attire des étudiants du monde entier. En 1908, il reçoit le prix Nobel de littérature, l’un des rares philosophes à l’avoir obtenu, pour « sa recherche sincère de la vérité » et sa « vision idéaliste de la vie ».&lt;/p&gt; &lt;p&gt;Sa philosophie, qu’il appelle « activisme », est une réaction contre le matérialisme et le naturalisme de son temps. Selon lui, l’être humain n’est pas seulement un produit de la nature : il participe à une « vie de l’esprit » indépendante, universelle, qui le dépasse et qu’il doit conquérir par l’effort et l’action. Le sens de la vie ne se trouve ni dans le plaisir ni dans le seul progrès technique, mais dans cette élévation de l’individu vers une vie spirituelle, où la religion, la morale et la culture trouvent leur source. Cette vie de l’esprit n’est pas donnée d’avance : chaque époque et chaque personne doivent la reconquérir contre la dispersion et la routine.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Le Sens et la valeur de la vie&lt;/em&gt; (1908) et &lt;em&gt;Les Grands Courants de la pensée contemporaine&lt;/em&gt;, il veut donner à son époque une orientation spirituelle et défendre une religion débarrassée de ses dogmes. Très lu avant 1914, traduit dans de nombreuses langues, il s’engage pendant la guerre pour la cause allemande. Son &lt;a href="https://fr.wikipedia.org/wiki/Spiritualisme_%28philosophie%29" title=" Wikipedia"&gt;spiritualisme&lt;/a&gt; tombe ensuite dans l’oubli. Il meurt à Iéna en 1926.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/eucken-mini.webp</t>
+        </is>
+      </c>
+      <c r="J71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique ; ethique ; spiritualite</t>
+        </is>
+      </c>
+      <c r="K71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spiritualisme ; Idéalisme</t>
+        </is>
+      </c>
+      <c r="L71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe allemand de la vie de l’esprit, prix Nobel de littérature en 1908.</t>
+        </is>
+      </c>
+      <c r="N71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O71"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Textes des philosophes, lots 12 à 17 : 60 fiches portées à 1 530-1 620 caractères (Forberg, d'Holbach, Alcuin, Dante, Gassendi, Lucrèce… jusqu'à Shinran, Thomas Reid, Quill Kukla) ; erreurs corrigées (Érasme, Amenhotep, Boèce, Singer, Sorai, Simone Weil, Ammonios d'Alexandrie, Siger…) ; lien du nom de Secrétan corrigé (renvoyait à Kierkegaard) ; Alcuin rangé dans les médiévaux ; « Hienrich » Rickert renommé Heinrich (301 depuis l'ancienne adresse)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -2921,8 +2921,10 @@
       <c r="D10" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>77</v>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Friedrich_Karl_Forberg" title=" Wikipedia"&gt;Friedrich Karl FORBERG&lt;/a&gt;  était un philosophe allemand  figure mineure mais controversée de l'idéalisme allemand post-kantien, connu pour ses liens avec Fichte et son implication dans   &lt;a href="https://laviedesidees.fr/Le-juge-et-le-policier"  style="color:#88A1E9"  title="Le juge et le policier par la vie des idées"&gt;"l'Atheismusstreit" &lt;/a&gt; (querelle de l'athéisme). Il est l'héritier des Lumières et de Kant, influencé par Reinhold et Fichte, qu'il considère comme un maître et ami. &lt;/p&gt; &lt;p&gt; Il défend une philosophie critique et idéaliste, centrée sur l'esthétique transcendante et les fondements de l'action libre. Rationaliste protestant, il s'intéresse à l'exégèse biblique et aux langues anciennes (grec, latin), révisant des auteurs comme Aristophane ou Horace. &lt;/p&gt; &lt;p&gt; Son essai "Entwicklung des Begriffs der Religion" paru en 1798  est central : il définit la religion comme un "postulat pratique" moral, indépendant de preuves théoriques de Dieu ou d'une "ordre divin". La foi n'est pas spéculative mais un engagement éthique dans une "ordre moral du monde", sans besoin de métaphysique théiste – une position fichtéenne radicale. Il  incarne un rationalisme audacieux : lucide sur l'absence de preuves divines, il mise tout sur la moralité humaine autonome. Son essai paraît en 1798 dans la revue dirigée par Fichte, accompagné d’un article de Fichte lui-même sur le fondement de notre croyance en un gouvernement divin du monde. Forberg y écrit que l’existence de Dieu est et reste incertaine, mais qu’on peut agir comme si un ordre moral du monde devait triompher. Accusés d’athéisme, les deux auteurs sont poursuivis, et Fichte doit quitter l’université d’Iéna en 1799. Forberg devient ensuite bibliothécaire à Cobourg.  &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F10" s="7" t="s">
         <v>78</v>
@@ -4054,11 +4056,15 @@
       <c r="C37" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="D37" s="8" t="s">
-        <v>323</v>
-      </c>
-      <c r="E37" s="9" t="s">
-        <v>324</v>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heinrich RICKERT</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Heinrich_Rickert" title=" Wikipedia"&gt;Heinrich RICKERT&lt;/a&gt; était un philosophe allemand  majeur du néokantisme, chef de file de l'école de Bade aux côtés de Wilhelm Windelband, axé sur &lt;a href="https://www.youtube.com/watch?v=-hQyRZfaCos"  title="Heinrich Rickert: Knowledge, Values, and Reality (#1349) par Philosopher Friends"&gt;une épistémologie &lt;/a&gt; distinguant les sciences nomologiques (naturelles) des sciences idiographiques (historiques et culturelles). &lt;/p&gt; &lt;p&gt; Ses oeuvres principales sont : - "Der Gegenstand der Erkenntnis" paru en 1892, réédité jusqu'en 1928 : introduction à sa philosophie transcendantale, distinguant sujet et objet épistémologiques. - "Die Grenzen der naturwissenschaftlichen Begriffsbildung" paru en 1902, plusieurs éditions : fondement de sa méthodologie, opposant généralisation scientifique et individualisation historique par des « concepts individuels », - "Allgemeine Grundlegung der Philosophie" en 1921 et "Grundprobleme der Philosophie" en 1934 : systématisation de sa théorie de la connaissance et de l'ontologie. &lt;/p&gt; &lt;p&gt;&lt;a href="https://www.youtube.com/watch?v=nLzgyLsPWeI"  title="Heinrich Rickert et le concept logique de l'historique  par Nick Nielsen"&gt; Il  oppose &lt;/a&gt;  les sciences de la nature (recherche de lois générales) aux sciences culturelles (focalisées sur l'individuel et les valeurs), introduisant la notion de « relation aux valeurs » pour fonder l'objectivité historique. Il défend un idéalisme transcendantal kantien : la connaissance valide repose sur des principes a priori, avec une "transcendance" comme cause non empirique des expériences conscientes. Pour Rickert, l’historien ne juge pas les valeurs, mais il choisit ce qui mérite d’être raconté en rapportant les faits à des valeurs reconnues par une culture. Cette idée a profondément marqué le sociologue Max Weber. Professeur à Fribourg, puis à Heidelberg, il dirige à Fribourg l’habilitation du jeune Martin Heidegger. ​&lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F37" s="7" t="s">
         <v>325</v>
@@ -4840,7 +4846,7 @@
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Helmuth_Plessner"  title=" Wikipedia"&gt;Helmuth PLESSNER&lt;/a&gt; était un philosophe allemand, fondateur clé de &lt;a href="https://publictionnaire.huma-num.fr/notice/plessner-helmuth/"   title="L’apport de l’anthropologie  par Publitionnaire"&gt;l'anthropologie philosophique &lt;/a&gt;  européenne aux côtés de figures comme Max Scheler et Arnold Gehlen. Influencé par le néokantisme, la phénoménologie et la biologie, il développa une vision de l'humain comme être "naturellement artificiel", marqué par une "positionnalité excentrique" qui le distingue des animaux. &lt;/p&gt; &lt;p&gt;  L'homme vit à distance de son corps et de son milieu, possédant simultanément un corps et étant un corps vivant. Cela génère trois lois anthropologiques : la loi de l'"excentricité", celle de la "médiation"  et celle de l'"utopie naturelle". &lt;/p&gt; &lt;p&gt; Il dépasse le dualisme nature/esprit en fondant une herméneutique biologique : la vie s'exprime via les frontières organiques, et l'intentionnalité humaine émerge de cette interaction environnementale, non d'un ego transcendantal. &lt;/p&gt; &lt;p&gt;  Dans "Rire et pleurer", il analyse ces expressions comme réponses excentriques au pathique, révélant la distance ironique de l'humain à soi. Quand à "Grenzen der Gemeinschaft"paru en 1924, il rejette le radicalisme communautaire au profit d'une sociologie de la "distance naturelle", préfigurant Habermas. &lt;/p&gt; </t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Helmuth_Plessner"  title=" Wikipedia"&gt;Helmuth PLESSNER&lt;/a&gt; était un philosophe allemand, fondateur clé de &lt;a href="https://publictionnaire.huma-num.fr/notice/plessner-helmuth/"   title="L’apport de l’anthropologie  par Publitionnaire"&gt;l'anthropologie philosophique &lt;/a&gt;  européenne aux côtés de figures comme Max Scheler et Arnold Gehlen. Influencé par le néokantisme, la phénoménologie et la biologie, il développa une vision de l'humain comme être "naturellement artificiel", marqué par une "positionnalité excentrique" qui le distingue des animaux. &lt;/p&gt; &lt;p&gt;  L'homme vit à distance de son corps et de son milieu, possédant simultanément un corps et étant un corps vivant. Cela génère trois lois anthropologiques : la loi de l'"excentricité", celle de la "médiation"  et celle de l'"utopie naturelle". &lt;/p&gt; &lt;p&gt; Il dépasse le dualisme nature/esprit en fondant une herméneutique biologique : la vie s'exprime via les frontières organiques, et l'intentionnalité humaine émerge de cette interaction environnementale, non d'un ego transcendantal. &lt;/p&gt; &lt;p&gt;  Dans "Rire et pleurer", il analyse ces expressions comme réponses excentriques au pathique, révélant la distance ironique de l'humain à soi. Quant à &lt;em&gt;Les Limites de la communauté&lt;/em&gt;, paru en 1924, il rejette le radicalisme communautaire au profit d'une sociologie de la "distance naturelle", préfigurant Habermas. Son œuvre principale, &lt;em&gt;Les Degrés de l’organique et l’homme&lt;/em&gt; (1928), décrit la vie à partir de la manière dont chaque être se rapporte à sa limite : la plante est ouverte à son milieu, l’animal est centré sur lui-même, l’homme seul peut se voir de l’extérieur. D’origine juive, Plessner doit quitter l’Allemagne en 1933 pour les Pays-Bas. Dans &lt;em&gt;La Nation retardée&lt;/em&gt;, il analyse les causes du nazisme. Revenu en 1951, il enseigne la sociologie à Göttingen. &lt;/p&gt; </t>
         </is>
       </c>
       <c r="F56" s="7" t="s">
@@ -4879,8 +4885,11 @@
       <c r="D57" s="8" t="s">
         <v>495</v>
       </c>
-      <c r="E57" s="13" t="s">
-        <v>496</v>
+      <c r="E57" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Mannheim" title=" Wikipedia"&gt;Karl MANNHEIM&lt;/a&gt;  était un philosophe allemand d'origine hongroise classé dans la sociologie de la connaissance et dans la sociologie compréhensive, à la frontière de la philosophie et des sciences sociales. Il ne sépare pas vraiment les deux domaines, car il cherche à montrer que la pensée dépend toujours d’un contexte social et historique. &lt;/p&gt; &lt;p&gt; Sa contribution la plus célèbre est  &lt;a href="https://www.youtube.com/watch?v=bBVJF4k_4-s"  title="transsiional sociologist par Socio exploration"&gt;Idéologie et utopie.&lt;/a&gt;  Dans ce livre, il explique que nos idées ne sont pas produites dans le vide: elles sont liées à notre position dans la société, à notre époque et à nos groupes d’appartenance. &lt;/p&gt; &lt;p&gt; Il  distingue notamment plusieurs formes d’idéologie et d’utopie. L’idéologie tend à justifier l’ordre existant, tandis que l’utopie ouvre la pensée vers une transformation du monde social. &lt;/p&gt; &lt;p&gt; Il défend aussi une forme de relationnisme: il ne dit pas que toute vérité est fausse, mais que les points de vue sont toujours partiels et situés. Cela lui permet de critiquer le relativisme absolu tout en reconnaissant que la connaissance humaine est historiquement conditionnée. Il  est un penseur des rapports entre   &lt;a href="https://www.youtube.com/watch?v=6R-Fre-UwgQ"  title="Sociological theory of culture  par Mannheuim"&gt;pensée, société et histoire.&lt;/a&gt;  On peut donc le ranger parmi les grands théoriciens de l’idéologie, de l’utopie et de la sociologie de la connaissance.   &lt;/p&gt; Né à Budapest en 1893, membre du cercle de Georg Lukács, il enseigne à Heidelberg puis à Francfort, avant de devoir fuir le nazisme en 1933 pour la London School of Economics. Dans un essai célèbre, il fait de la « génération » une notion sociologique : ceux qui ont vécu les mêmes événements à un âge semblable partagent une manière de voir le monde.
+</t>
+        </is>
       </c>
       <c r="F57" s="7" t="s">
         <v>497</v>

</xml_diff>

<commit_message>
Textes des philosophes, lot 18 : 10 fiches portées à 1 410-1 620 caractères (Garin, Bostrom, Chilon, Vuillemin, Mandana Misra, Beuchot, Ortega y Gasset, Spalding, Jean de Mirecourt, Sebond) ; erreurs corrigées (Spalding 1761, Primo de Rivera, argument de la simulation, « легенdaire », Index 1564) ; dates vérifiées (Yi Hwang, Hermias d'Alexandrie, Téléclès, Pierre d'Espagne, Bède, Alcuin) ; liens morts réparés : 13 titres Wikipédia, 9 identifiants YouTube, lien de Granel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -3934,7 +3934,7 @@
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Georg_Simmel" title=" Wikipedia"&gt;Georg SIMMEL&lt;/a&gt; était un philosophe du royaume de Prusse souvent considéré comme l’un des fondateurs de la sociologie de la modernité et de la   &lt;a href="https://www.youtube.com/watch?v=k2SZfvBp6H8"  title="Georg Simmel , sociologie urbaine . par PHILOVIBE"&gt;"sociologie formelle". &lt;/a&gt;  Il enseigne longtemps en marge de l’université, ce qui explique qu’il ait été moins institutionnalisé que Durkheim ou Weber, mais très influent sur eux et sur la sociologie ultérieure. &lt;/p&gt; &lt;p&gt; Il ne part pas de "la" société comme un grand tout, mais des formes d’interaction entre individus.  Il parle de sociologie formelle : les contenus (amour, travail, politique) varient, mais les formes (conflit, échange) se retrouvent partout et peuvent être étudiées en elles‑mêmes. Pour lui, la modernité se caractérise par une tension entre individu et société, entre culture subjective et culture objective.  La culture est produite par les individus mais devient ensuite une force autonome qui les dépasse, les contraint, et peut les écraser par sa complexité. &lt;/p&gt; &lt;p&gt; Il appartient au courant de la   &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_viel"  title="Philosophie de vie par Wikipedia"&gt;"philosophie de la vie" : &lt;/a&gt;  la vie est pour lui un flux créateur, mouvant, qui déborde toutes les formes fixes.  Les formes (institutions, normes, objets culturels) sont nécessaires pour donner sens au flux de la vie, mais elles se rigidifient et entrent en tension avec ce mouvement vital qui cherche toujours à se dépasser. Il  il insiste sur l’idée que la culture apparaît là où la vie rencontre des valeurs qui la transcendent (art, science, morale), mais ces valeurs finissent par se solidifier en systèmes objectifs qui peuvent aliéner l’individu. &lt;/p&gt;   &lt;audio controls title="Georg Simmel : Les grandes villes / Revue Questions internationales par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/12003-25.03.2013-ITEMA_20463123-2013C18006S0084-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Georg_Simmel" title=" Wikipedia"&gt;Georg SIMMEL&lt;/a&gt; était un philosophe du royaume de Prusse souvent considéré comme l’un des fondateurs de la sociologie de la modernité et de la   &lt;a href="https://www.youtube.com/watch?v=k2SZfvBp6H8"  title="Georg Simmel , sociologie urbaine . par PHILOVIBE"&gt;"sociologie formelle". &lt;/a&gt;  Il enseigne longtemps en marge de l’université, ce qui explique qu’il ait été moins institutionnalisé que Durkheim ou Weber, mais très influent sur eux et sur la sociologie ultérieure. &lt;/p&gt; &lt;p&gt; Il ne part pas de "la" société comme un grand tout, mais des formes d’interaction entre individus.  Il parle de sociologie formelle : les contenus (amour, travail, politique) varient, mais les formes (conflit, échange) se retrouvent partout et peuvent être étudiées en elles‑mêmes. Pour lui, la modernité se caractérise par une tension entre individu et société, entre culture subjective et culture objective.  La culture est produite par les individus mais devient ensuite une force autonome qui les dépasse, les contraint, et peut les écraser par sa complexité. &lt;/p&gt; &lt;p&gt; Il appartient au courant de la   &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_vie"  title="Philosophie de vie par Wikipedia"&gt;"philosophie de la vie" : &lt;/a&gt;  la vie est pour lui un flux créateur, mouvant, qui déborde toutes les formes fixes.  Les formes (institutions, normes, objets culturels) sont nécessaires pour donner sens au flux de la vie, mais elles se rigidifient et entrent en tension avec ce mouvement vital qui cherche toujours à se dépasser. Il  il insiste sur l’idée que la culture apparaît là où la vie rencontre des valeurs qui la transcendent (art, science, morale), mais ces valeurs finissent par se solidifier en systèmes objectifs qui peuvent aliéner l’individu. &lt;/p&gt;   &lt;audio controls title="Georg Simmel : Les grandes villes / Revue Questions internationales par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/12003-25.03.2013-ITEMA_20463123-2013C18006S0084-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
         </is>
       </c>
       <c r="F34" s="7" t="s">
@@ -4445,8 +4445,11 @@
       <c r="D46" s="8" t="s">
         <v>400</v>
       </c>
-      <c r="E46" s="13" t="s">
-        <v>401</v>
+      <c r="E46" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ernst_Bloch"  title=" Wikipedia"&gt;Ernst BLOCH&lt;/a&gt;  était un philosophe juif allemand  souvent rattaché au marxisme hétérodoxe et à la philosophie de l’espérance. Sa pensée se distingue par une défense de l’utopie comme force critique et émancipatrice, contre les lectures trop fermées ou déterministes de l’histoire. &lt;/p&gt; &lt;p&gt; Il part de l’idée que la réalité humaine n’est jamais complètement accomplie: il y a toujours du “pas encore” dans l’histoire, dans la société et dans la conscience. Il appelle cela le non-simultané ou le caractère inachevé du réel, ce qui permet de penser le futur comme ouvert plutôt que comme déjà écrit. &lt;/p&gt; &lt;p&gt; Son ouvrage majeur,  &lt;a href="https://www.youtube.com/watch?v=u-zXjE1duok"  title="Le principe de l’espérance par Culture Philo"&gt; Le Principe espérance, &lt;/a&gt; développe l’idée que l’espérance n’est pas une illusion passive, mais une énergie active qui pousse les hommes à transformer le monde. L’utopie, chez lui, n’est donc pas un rêve irréaliste: c’est une anticipation concrète de ce qui pourrait advenir. &lt;/p&gt; &lt;p&gt; Il accorde aussi une grande importance aux œuvres culturelles, à la religion, à l’art et même aux rêves éveillés, parce qu’ils contiennent des indices de possibles non réalisés. Il voit dans ces domaines des formes où s’exprime un dépassement de la situation présente, une ouverture vers un monde plus juste. &lt;/p&gt; &lt;p&gt; Sa philosophie est une pensée du possible et du futur. Elle combine critique du présent, héritage marxiste et réhabilitation de l’utopie pour montrer que l’histoire humaine peut encore être transformée. &lt;/p&gt;  &lt;audio controls title="A quoi bon espérer ? par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-27.06.2023-ITEMA_23423905-2023C48904S0178-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
+</t>
+        </is>
       </c>
       <c r="F46" s="7" t="s">
         <v>402</v>

</xml_diff>

<commit_message>
Textes des philosophes, lot 19 : 10 fiches portées à 1 420-1 620 caractères (Chevalier, Boehme, Camus, Goddard, Krishnamurti, Korsch, Cratyle, Alexandre de Hales, Regan, Kodjo-Grandvaux) ; Chevalier et Camus réécrits (rôle sous Vichy d'après Wikipédia ; absurde et révolte) ; noms corrigés KORSCH, BOEHME ; courants : liens réparés (Créolisation, Ishraqisme, Falsafa) et vidéos/textes de l'éditeur (Bouddhisme de la Terre pure, Pensée décoloniale, Yogācāra)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -4490,8 +4490,10 @@
       <c r="D47" s="8" t="s">
         <v>410</v>
       </c>
-      <c r="E47" s="12" t="s">
-        <v>411</v>
+      <c r="E47" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Korsch" title=" Wikipedia"&gt;Karl KORSCH&lt;/a&gt;  était un philosophe marxiste allemand,  théoricien du communisme de conseils et critique du léninisme orthodoxe. Issu d'un milieu bourgeois, il évolua du réformisme social au marxisme hétérodoxe, influençant les courants ultra-gauche via son rejet du matérialisme positiviste et son insistance sur la praxis révolutionnaire historique. Juriste de formation, il est en 1923 ministre de la Justice de Thuringe, puis député communiste au Reichstag.  Exclu du parti en 1926 pour "ultra-gauchisme", il émigra après 1933 vers les États-Unis, où il approfondit sa théorie marxiste. &lt;/p&gt; &lt;p&gt; Son œuvre majeure &lt;em&gt;Marxisme et philosophie&lt;/em&gt; paru en 1923 marque sa rupture avec le léninisme en critiquant sa dérive scientiste. Il   &lt;a href="https://www.zones-subversives.com/article-le-marxisme-critique-de-karl-korsch-116431466.html"  title="Le marxisme critique de Karl Korsch par Chroniques critiques"&gt;rejette le marxisme &lt;/a&gt; comme "science positive" figée ou philosophie matérialiste abstraite ; il le conçoit comme une théorie historique et concrète, liée à la lutte des classes et à la dialectique hégélienne réinterprétée comme expression de la révolution bourgeoise puis prolétarienne. &lt;/p&gt; &lt;p&gt; Il  théorise les conseils comme organes centraux de la transition socialiste, via la praxis dialectique et l'auto-activité des masses, contre la socialisation étatique. Ses écrits inspirent le KAPD et l'ultra-gauche, voyant les conseils comme alternative à la bureaucratisation stalinienne. Son influence perdure chez les communistes de conseils, soulignant la conscience ouvrière spontanée pour l'émancipation réelle. Aux États-Unis, il publie &lt;em&gt;Karl Marx&lt;/em&gt; (1938) et reste proche de Bertolt Brecht, qui le considérait comme son maître en marxisme. &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F47" s="7" t="s">
         <v>412</v>

</xml_diff>

<commit_message>
Liens morts retirés des textes en gardant les mots (21 adresses, 22 liens) : 17 vidéos YouTube supprimées (Lewis, Quine, Deleuze, Simplicius, Ficin, Grosseteste, Stuart Mill, Wittgenstein ×2, Owen, Avicenne, Nezahualcoyotl, Roy, Voltaire, Bogdanov, Pissarev, Lessing) et 5 pages disparues (Charbonneau, Bergson, B. Stiegler, Aurobindo, Tan Sitong) ; description de Pierre d'Espagne : « philosophe portugais »
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -4199,8 +4199,11 @@
       <c r="D40" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="E40" s="14" t="s">
-        <v>350</v>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Theodor_Lessing" title=" Wikipedia"&gt;Theodor LESSING&lt;/a&gt;  était un philosophe, essayiste et publiciste allemand &lt;a href="https://www.persee.fr/doc/rjuiv_0484-8616_1996_num_155_1_2554"  title="Lessing et le sionisme par persée"&gt;d’origine juive, &lt;/a&gt; connu comme un penseur critique de la modernité, du nationalisme et de l’antisémitisme. &lt;/p&gt; &lt;p&gt; Il s’inscrit surtout dans une philosophie de la culture et une philosophie sociale critique. Son travail ne cherche pas à construire un système abstrait, mais à analyser les maladies de la civilisation moderne, la violence des masses, la guerre, la ville industrielle et la destruction du vivant. Sa pensée est marquée par un humanisme pessimiste et engagé qui dénoncé le militarisme, la brutalisation de la société et les dérives autoritaires de l’Allemagne de Weimar, allant jusqu’à prévoir le danger nazi avant 1933. Il fut aussi l’un des premiers à réfléchir à la condition des minorités et à ce qu’il a appelé le &lt;a href="https://www.sifriatenou.com/2020/10/20/5449/"  title="lessing la haine de soi par sifriatenou"&gt;« judaïsme de haine de soi »,&lt;/a&gt; pour décrire les effets psychologiques de l’antisémitisme sur les Juifs eux-mêmes. &lt;/p&gt; &lt;p&gt; Il est également une figure de la critique écologique avant l’heure. Dès les années 1930, il s’inquiète de la déforestation, de la pollution urbaine et d’un possible dérèglement du climat, ce qui le rend étonnamment actuel. Il voit la modernité technique non comme un progrès neutre, mais comme une force capable de détruire les équilibres humains et naturels. &lt;/p&gt; &lt;p&gt; Sur le plan politique, il est un intellectuel indépendant, polémique et souvent isolé, qui s’oppose à l’autoritarisme autant qu’aux conformismes de son époque. Il a fini assassiné en exil   à Mariánské Lázně par des nationalistes sudètes, devenant l’une des premières victimes du nazisme hors d’Allemagne. &lt;/p&gt; 
+</t>
+        </is>
       </c>
       <c r="F40" s="7" t="s">
         <v>351</v>

</xml_diff>

<commit_message>
Fiches — 20 fiches modifiées : Friedrich SCHLEIERMACHER, Arthur SCHOPENHAUER, Karl Ludwig MICHELET, Katherine BRADING, Carrie JENKINS, PADMASAMBHAVA et 14 autre(s) ; 4 images
Publié depuis l'éditeur des fiches.
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -2786,14 +2786,16 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="n">
-        <v>1769</v>
+      <c r="A7" s="7">
+        <v>1768</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>48</v>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1768 – 1834</t>
+        </is>
       </c>
       <c r="D7" s="11" t="s">
         <v>49</v>
@@ -3094,8 +3096,7 @@
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Arthur_Schopenhauer"  title=" Wikipedia"&gt; Arthur SCHOPENHAUER&lt;/a&gt; était un philosophe allemand atypique, souvent qualifié de "philosophe du pessimisme"     avec une &lt;a  href="https://www.youtube.com/watch?v=iVkkzzxBnQ0&amp;t=10s&amp;ab_channel=LePr%C3%A9cepteur"  title="La métaphysique, l'amour, le sexe par Le Précepteur"&gt;vision anticonformiste&lt;/a&gt; du monde. Né à Dantzig dans une famille aisée, il rejette le commerce paternel pour se tourner vers la philosophie, influencé par Kant, Platon et les textes hindous comme les Upanishads. Après des études à Göttingen et Berlin, il publie sa thèse sur le principe de raison suffisante en 1813, marquant le début d'une œuvre centrée sur la "volonté" comme essence irrationnelle du monde. &lt;/p&gt; &lt;p&gt; Dans son œuvre métaphysique majeure publiée en 1818 &lt;a  href="https://www.youtube.com/watch?v=U2jxUWYr9vY&amp;ab_channel=Basileus"  title="Schopenhauer: Le Monde comme volonté et représentation par Basileus"&gt;"Le Monde comme Volonté et Représentation"&lt;/a&gt;,  distingue le monde phénoménal (représentation kantienne, soumis à l'espace, au temps et à la causalité) de la "chose en soi", identifiée à une Volonté aveugle et insatiable. Cette Volonté, principe de souffrance universelle, pousse les êtres à désirer sans fin, rendant l'existence un cycle de douleur et d'ennui. Il en tire un pessimisme radical : la vie n'a pas de sens positif, seule la négation de la volonté offre une issue. Sa vision pessimiste de la vie, selon laquelle &lt;a  href="https://www.youtube.com/watch?v=X_K4vRpp5fo&amp;t=16s&amp;ab_channel=LePr%C3%A9cepteur"   title="L'origine de notre souffrance par Le Précepteur"&gt;la souffrance&lt;/a&gt; et  &lt;a  href="https://www.youtube.com/watch?v=fNfZNj_FRHg"   title="la philosophie de schopenhauer par kosmos"&gt;le désir &lt;/a&gt;  sont inévitables et où la seule voie vers le bonheur consiste à renoncer à nos désirs et à trouver la paix intérieure. &lt;/p&gt; &lt;p&gt; Sa notion de "Volonté" est la force fondamentale qui anime tout ce qui existe dans l'univers, y compris les êtres vivants. Il la considère comme étant une puissance irrationnelle et inconsciente qui se manifeste dans notre désir de vivre et dans tous les aspects de la vie.&lt;/p&gt; &lt;p&gt;  Le monde de  la "Représentation" représente la face externe du monde, ce que nous voyons, le monde de l'espace et du temps. Nous ne pouvons pas connaître la réalité en soi, qui est inobservable et inconnaissable mais seulement les représentations que nous en avons à travers nos sens et notre esprit. &lt;/p&gt;&lt;p&gt; &lt;a  href="https://www.youtube.com/watch?v=qozOyALs6S4"   title="la philosophie de schopenhauer par parole de philosophe"&gt;Premier philosophe &lt;/a&gt; occidental à intégrer sérieusement le bouddhisme et l'hindouisme, il voit dans le nirvana ou l'ascèse une libération par l'abolition du vouloir-vivre. L'art, notamment la musique (qu'il élève au-dessus des autres arts), permet une contemplation temporaire de l'Idée platonicienne, suspendant la volonté et procurant un plaisir désintéressé. La compassion, fondement éthique, naît de la reconnaissance de l'unité de la &lt;a  href="https://www.youtube.com/watch?v=c__hjru6nwI"   title="la philosophie de schopenhauer par voyage endormis"&gt;Volonté en tous. &lt;/a&gt; &lt;/p&gt; &lt;p&gt; Il publie ensuite en 1851 "The Art of Contemplation" où il explique comment les œuvres d'Art peuvent nous aider à trouver la paix intérieure en contemplant la réalité métaphysique. Il est aussi connu pour sa rhétorique et son livre &lt;a  href="https://www.youtube.com/watch?v=HVQRjluNjLE&amp;ab_channel=LePr%C3%A9cepteur"  title=""L'art d'avoir toujours raison" par Le Précepteur"&gt;"L'art d'avoir toujours raison"&lt;/a&gt;. &lt;/p&gt;  &lt;audio controls title="L'art peut il consoler ? par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/22078-23.04.2021-ITEMA_22644473-2020C12410E0108.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
-</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Arthur_Schopenhauer" title=" Wikipedia"&gt; Arthur SCHOPENHAUER&lt;/a&gt; était un philosophe allemand atypique, souvent qualifié de "philosophe du pessimisme"     avec une &lt;a href="https://www.youtube.com/watch?v=iVkkzzxBnQ0&amp;amp;t=10s&amp;amp;ab_channel=LePr%C3%A9cepteur" title="La métaphysique, l'amour, le sexe par Le Précepteur"&gt;vision anticonformiste&lt;/a&gt; du monde. Né à Dantzig dans une famille aisée, il rejette le commerce paternel pour se tourner vers la philosophie, influencé par Kant, Platon et les textes hindous comme les Upanishads. Après des études à Göttingen et Berlin, il publie sa thèse sur le principe de raison suffisante en 1813, marquant le début d'une œuvre centrée sur la "volonté" comme essence irrationnelle du monde. &lt;/p&gt; &lt;p&gt; Dans son œuvre métaphysique majeure publiée en 1818 &lt;a href="https://www.youtube.com/watch?v=U2jxUWYr9vY&amp;amp;ab_channel=Basileus" title="Schopenhauer: Le Monde comme volonté et représentation par Basileus"&gt;"&lt;/a&gt;&lt;a href="https://www.youtube.com/watch?v=JeNhNwVV9zY" title="Le monde comme volonté et comme représentation (Schopenhauer) par GORVS S"&gt;Le Monde comme Volonté et Représentation&lt;/a&gt;", &amp;nbsp;distingue le monde phénoménal (représentation kantienne, soumis à l'espace, au temps et à la causalité) de la "chose en soi", identifiée à une Volonté aveugle et insatiable. Cette Volonté, principe de souffrance universelle, pousse les êtres à désirer sans fin, rendant l'existence un cycle de douleur et d'ennui. Il en tire un pessimisme radical : la vie n'a pas de sens positif, seule la négation de la volonté offre une issue. Sa vision pessimiste de la vie, selon laquelle &lt;a href="https://www.youtube.com/watch?v=X_K4vRpp5fo&amp;amp;t=16s&amp;amp;ab_channel=LePr%C3%A9cepteur" title="L'origine de notre souffrance par Le Précepteur"&gt;la souffrance&lt;/a&gt; et  &lt;a href="https://www.youtube.com/watch?v=fNfZNj_FRHg" title="la philosophie de schopenhauer par kosmos"&gt;le désir &lt;/a&gt;  sont inévitables et où la seule voie vers le bonheur consiste à renoncer à nos désirs et à trouver la paix intérieure. &lt;/p&gt; &lt;p&gt; Sa notion de "Volonté" est la force fondamentale qui anime tout ce qui existe dans l'univers, y compris les êtres vivants. Il la considère comme étant une puissance irrationnelle et inconsciente qui se manifeste dans notre désir de vivre et dans tous les aspects de la vie.&lt;/p&gt; &lt;p&gt;  Le monde de  la "Représentation" représente la face externe du monde, ce que nous voyons, le monde de l'espace et du temps. Nous ne pouvons pas connaître la réalité en soi, qui est inobservable et inconnaissable mais seulement les représentations que nous en avons à travers nos sens et notre esprit. &lt;/p&gt;&lt;p&gt; &lt;a href="https://www.youtube.com/watch?v=qozOyALs6S4" title="la philosophie de schopenhauer par parole de philosophe"&gt;Premier philosophe &lt;/a&gt; occidental à intégrer sérieusement le bouddhisme et l'hindouisme, il voit dans le nirvana ou l'ascèse une libération par l'abolition du vouloir-vivre. L'art, notamment la musique (qu'il élève au-dessus des autres arts), permet une contemplation temporaire de l'Idée platonicienne, suspendant la volonté et procurant un plaisir désintéressé. La compassion, fondement éthique, naît de la reconnaissance de l'unité de la &lt;a href="https://www.youtube.com/watch?v=c__hjru6nwI" title="la philosophie de schopenhauer par voyage endormis"&gt;Volonté en tous. &lt;/a&gt; &lt;/p&gt; &lt;p&gt; Il publie ensuite en 1851 "The Art of Contemplation" où il explique comment les œuvres d'Art peuvent nous aider à trouver la paix intérieure en contemplant la réalité métaphysique. Il est aussi connu pour sa rhétorique et son livre &lt;a href="https://www.youtube.com/watch?v=HVQRjluNjLE&amp;amp;ab_channel=LePr%C3%A9cepteur" title="" l'art="" d'avoir="" toujours="" raison"="" par="" le="" précepteur"=""&gt;"L'art d'avoir toujours raison"&lt;/a&gt;. &lt;/p&gt;  &lt;audio controls title="L'art peut il consoler ? par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/22078-23.04.2021-ITEMA_22644473-2020C12410E0108.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
       <c r="F14" s="7" t="s">
@@ -3168,699 +3169,721 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="n">
-        <v>1804</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="G16" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="I16" s="7"/>
-      <c r="J16" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Matérialisme ; Humanisme ; Jeunes hégéliens ; Athéisme</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="N16" s="0" t="s">
-        <v>27</v>
-      </c>
+    <row r="16" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0">
+        <v>1801</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1801 – 1893</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Karl Ludwig MICHELET</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Ludwig_Michelet" title=" Wikipedia"&gt;Karl Ludwig MICHELET&lt;/a&gt; est un philosophe allemand, l’un des disciples les plus fidèles de &lt;a href="https://fr.wikipedia.org/wiki/Georg_Wilhelm_Friedrich_Hegel" title=" Wikipedia"&gt;Hegel&lt;/a&gt;. Né à Berlin en 1801 dans une famille de marchands huguenots, d’origine française, il suit les cours de Hegel et enseigne à l’université de Berlin pendant des décennies. Après la mort du maître en 1831, il fait partie du groupe d’élèves qui publient ses œuvres complètes et prépare l’édition de ses &lt;em&gt;Leçons sur l’histoire de la philosophie&lt;/em&gt;.&lt;/p&gt; &lt;p&gt;Spécialiste d’Aristote, il écrit en français un &lt;em&gt;Examen critique du livre d’Aristote intitulé Métaphysique&lt;/em&gt;, couronné en 1836 par l’Académie des sciences morales et politiques en même temps que l’essai de Félix Ravaisson. Quand l’école de Hegel se divise sur la religion et la politique, il reprend la distinction proposée par son élève David Friedrich Strauss entre une « droite », fidèle au christianisme, une « gauche », celle des &lt;a href="https://fr.wikipedia.org/wiki/Jeunes_h%C3%A9g%C3%A9liens" title=" Wikipedia"&gt;Jeunes hégéliens&lt;/a&gt;, et un « centre », auquel il se rattache. Pour lui, Dieu n’est pas une personne séparée du monde : il devient personnel dans l’esprit humain, et l’immortalité n’est pas celle de l’individu, mais celle de l’esprit qui se développe dans l’histoire.&lt;/p&gt; &lt;p&gt;En 1843, il fonde avec ses élèves la Société philosophique de Berlin, qui maintient la tradition hégélienne pendant tout le siècle. Il y défend Hegel contre la critique que lui adresse Schelling, revenu à Berlin en 1841, et publie une histoire de la philosophie allemande de Kant à Hegel, puis une philosophie du droit. Fidèle jusqu’au bout, il intitule l’un de ses derniers livres &lt;em&gt;Hegel, le philosophe universel irréfuté&lt;/em&gt; (1870). Il meurt à Berlin en 1893, à quatre-vingt-onze ans.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fjxyOTDwZic</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"FOREWORD to HEGEL'S PHILOSOPHY OF NATURE by KARL LUDWIG MICHELET" par The Spirit of Hegel</t>
+        </is>
+      </c>
+      <c r="H16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/klmichelet-mini.webp</t>
+        </is>
+      </c>
+      <c r="J16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique ; ethique</t>
+        </is>
+      </c>
+      <c r="K16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand</t>
+        </is>
+      </c>
+      <c r="L16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe allemand, disciple et éditeur de Hegel, chef du « centre » hégélien.</t>
+        </is>
+      </c>
+      <c r="N16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O16"/>
     </row>
     <row r="17" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="n">
-        <v>1806</v>
+        <v>1804</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="I17" s="7"/>
       <c r="J17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matérialisme ; Humanisme ; Jeunes hégéliens ; Athéisme</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="N17" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="n">
+        <v>1806</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="I18" s="7"/>
+      <c r="J18" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Nihilisme ; Anarchisme ; Jeunes hégéliens ; Individualisme</t>
         </is>
       </c>
-      <c r="L17" s="2" t="s">
+      <c r="L18" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="N17" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="236.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="n">
+      <c r="N18" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="236.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="n">
         <v>1808</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B19" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C19" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D19" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E19" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F19" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G19" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="H19" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="I18" s="9"/>
-      <c r="J18" s="2" t="s">
+      <c r="I19" s="9"/>
+      <c r="J19" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Herméneutique ; Jeunes hégéliens</t>
         </is>
       </c>
-      <c r="L18" s="2" t="s">
+      <c r="L19" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="n">
+      <c r="M19" s="2"/>
+      <c r="N19" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="n">
         <v>1809</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B20" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C20" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D20" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bruno_Bauer" title=" Wikipedia"&gt;Bruno BAUER&lt;/a&gt; était unthéologien, philosophe et historien allemand, figure majeure des Jeunes Hégéliens et précurseur de la critique radicale de la religion. Initialement hégélien de droite, il évolua vers une gauche radicale dans les années 1840, développant une philosophie centrée sur la "conscience de soi infinie" comme force motrice de l'histoire et de la critique des institutions. &lt;/p&gt; &lt;p&gt; Élève de Hegel à Berlin, il enseigna à Bonn et Berlin jusqu'à son renvoi en 1842 pour ses idées athées. Il critiqua violemment la religion chrétienne et l'État prussien, influençant Marx et Engels (qu'il inspira puis critiqua). Après 1848, déçu par les révolutions, il adopta une posture conservatrice soutenant Bismarck. &lt;/p&gt; &lt;p&gt; Il  théorise la "conscience de soi infinie" comme activité critique infinie qui nie toute "positivité". La religion est une aliénation où l'humain projette ses pouvoirs sur un Dieu extérieur, devant être vaincue par la critique rationnelle et la praxis révolutionnaire. &lt;/p&gt; &lt;p&gt;  Dans son ouvrage  &lt;a href="https://www.youtube.com/watch?v=1huRf1-2d5Q"  title="Bruno BAUER - KARL MARX : La QUESTION JUIVE  par Frère Ismaêl"&gt;"La Question juive" &lt;/a&gt;  paru en 1843, il refuse l'émancipation politique des Juifs en tant que groupe religieux au sein de l'État chrétien prussien. Il exige leur renoncement préalable à la religion juive, voyant l'émancipation universelle comme conditionnée par l'abolition de toute religion et la réalisation de l'autonomie critique de la conscience humaine. L'émancipation politique générale (allemande) précède toute émancipation spécifique ; les Juifs doivent d'abord s'émanciper eux-mêmes en tant qu'humains par la critique radicale de la religion, transformant l'opposition théologique en liberté universelle. Marx critiquera Bauer sur cette question.&lt;/p&gt; </t>
         </is>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F20" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G20" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H20" s="9" t="s">
         <v>165</v>
-      </c>
-      <c r="I19" s="7"/>
-      <c r="J19" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Marxisme ; Jeunes hégéliens</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="N19" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="246" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="n">
-        <v>1817</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="H20" s="9" t="s">
-        <v>175</v>
       </c>
       <c r="I20" s="7"/>
       <c r="J20" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marxisme ; Jeunes hégéliens</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="N20" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="246" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="n">
+        <v>1817</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="I21" s="7"/>
+      <c r="J21" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="K20" s="2" t="s">
+      <c r="K21" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="L20" s="2" t="s">
+      <c r="L21" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="N20" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="292.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="n">
+      <c r="N21" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="292.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="n">
         <v>1818</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B22" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C22" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D22" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Marx"  title=" Wikipedia"&gt;Karl MARX&lt;/a&gt; était un philosophe, économiste et révolutionnaire allemand né à Trèves, est le fondateur  &lt;a href="https://www.youtube.com/watch?v=W_ZwUjnl4W4"  title="La philosophie de Karl Marx par Parole de philosophe"&gt;du marxisme &lt;/a&gt; avec Friedrich Engels. Issu d'une famille juive convertie au protestantisme, il étudie le droit et la philosophie à Bonn, Berlin et Iéna, où il est influencé par Hegel et les jeunes hégéliens comme David Strauss, dont il critique les idées religieuses dans sa jeunesse. Exilé en France puis en Angleterre après les révolutions de 1848, il vit dans la précarité à Londres, soutenu par Engels, et milite au sein de l'Internationale ouvrière. Son portrait de 1875 le montre barbu, pensif, incarnation du penseur engagé.   &lt;/p&gt; &lt;p&gt;    Sa philosophie repose sur le matérialisme historique et dialectique, voyant l'histoire comme une succession de modes de production (esclavagiste, féodal, capitaliste) mue par  &lt;a href="https://www.youtube.com/watch?v=1pYmqDnvTh8"  title="Les classes sociales par DigiSchool Lycee "&gt;la lutte des classes &lt;/a&gt; entre exploiteurs et exploités. Dans  &lt;a href="https://www.youtube.com/watch?v=jb-5oSF2dpU&amp;ab_channel=TanguyLacroix"  title="Le Manifeste du Parti Communiste par Tanguy Lacroix "&gt;"Le Manifeste communiste  &lt;/a&gt; (1848), coécrit avec Engels, il appelle le prolétariat à abolir la propriété privée des moyens de production pour instaurer une société sans classes. Le Capital (1867-1883) analyse le capitalisme comme un système d'exploitation via la plus-value extraite du travail   &lt;a href="https://www.youtube.com/watch?v=rEAxxsX_um0&amp;t=4s&amp;ab_channel=LePr%C3%A9cepteur"  title="L'Aliénation par le Précepteur "&gt;salarié aliéné, &lt;/a&gt;  prédisant sa chute par ses contradictions internes. &lt;/p&gt; &lt;p&gt;  Il rejette la religion comme « opium du peuple », outil d'aliénation masquant l'exploitation réelle, et prône la praxis révolutionnaire : transformer le monde par l'action collective des travailleurs. Critiquant le libéralisme et le socialisme utopique, il envisage une dictature du prolétariat transitoire menant au communisme, où l'État dépérit et les besoins sont satisfaits selon les capacités. Ses idées opposent radicalement celles de Donoso Cortés, qui y voyait un aboutissement satanique du libéralisme. &lt;/p&gt; &lt;p&gt; Sa contribution la plus importante à la théorie politique est sa conception du  &lt;a href="https://fr.wikipedia.org/wiki/Mat%C3%A9rialisme_dialectique"  title="Le Marxisme Dialectique par Wikipedia "&gt;"matérialisme dialectique"&lt;/a&gt;, qui est l'idée que le changement historique est motivé par des conflits entre des classes sociales opposées et que ces conflits sont finalement résolus par la révolution. &lt;/p&gt; &lt;p&gt; Il a également écrit abondamment sur l'économie, en particulier sur la théorie de la valeur-travail, qui postule que la valeur d'un bien ou d'un service est basée sur la quantité de travail nécessaire pour le produire. &lt;/p&gt; &lt;p&gt;     Son influence sur le XXe siècle est immense : révolutions bolchevique, chinoise, mouvements ouvriers mondiaux, et disciplines comme la sociologie ou l'économie. Malgré les échecs des régimes « marxistes », sa critique du capitalisme reste débattue aujourd'hui. &lt;/p&gt;    &lt;audio controls title="Pour l'avenir par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-26.09.2020-ITEMA_22438423-2020C40092E0005-1779455909.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
         </is>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F22" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">"Karl Marx" par The School of Life</t>
         </is>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="H22" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="I21" s="9"/>
-      <c r="J21" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Marxisme ; Jeunes hégéliens</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="N21" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O21" s="2" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="n">
-        <v>1820</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="E22" s="12" t="s">
-        <v>190</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="G22" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="H22" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="I22" s="7"/>
+      <c r="I22" s="9"/>
       <c r="J22" s="2" t="s">
         <v>166</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Marxisme ; Jeunes hégéliens</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="n">
+        <v>1820</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="I23" s="7"/>
+      <c r="J23" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Marxisme ; Matérialisme ; Jeunes hégéliens</t>
         </is>
       </c>
-      <c r="L22" s="2" t="s">
+      <c r="L23" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="N22" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="272.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="n">
-        <v>1832</v>
-      </c>
-      <c r="B23" s="7" t="n">
-        <v>1888</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="E23" s="14" t="s">
-        <v>198</v>
-      </c>
-      <c r="F23" s="7"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="12" t="s">
-        <v>199</v>
-      </c>
-      <c r="I23" s="16" t="s">
-        <v>200</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="L23" s="17" t="s">
-        <v>202</v>
-      </c>
       <c r="N23" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="306.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="272.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="n">
         <v>1832</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="7" t="n">
+        <v>1888</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="F24" s="7"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="I24" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="L24" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="N24" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="306.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="n">
+        <v>1832</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C25" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D25" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="E25" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Wilhelm_Wundt"  title=" Wikipedia"&gt;Wilhelm WUNDT&lt;/a&gt;  était un physiologiste et philosophe allemand, souvent considéré comme le père de la psychologie expérimentale moderne. Né près de Mannheim dans une famille de pasteurs luthériens, il étudie la médecine à Tübingen, Heidelberg et Berlin, où il se forme à la physiologie auprès de figures comme Helmholtz. Après son doctorat en 1856, il devient assistant en physiologie et publie en 1874 ses  &lt;a href="https://www.youtube.com/watch?v=-7f525JhOCE" title=" psycholoie par coursitout"&gt;Principes de psychologie &lt;/a&gt; physiologique, un ouvrage fondateur qui pose les bases scientifiques de la psychologie en s'appuyant sur des méthodes expérimentales inspirées des sciences naturelles. &lt;/p&gt; &lt;p&gt; En 1879, il fonde à l'université de Leipzig le premier laboratoire de psychologie expérimentale au monde, marquant la naissance officielle de la psychologie comme discipline autonome, séparée de la philosophie. Ce laboratoire attire des étudiants du monde entier, dont 186 doctorants, et devient un centre d'observation des processus mentaux via l'introspection contrôlée – une méthode rigoureuse où des sujets entraînés analysent leurs sensations, émotions et idées sous conditions expérimentales précises. Il crée aussi en 1881 le premier journal de psychologie, Philosophische Studien. &lt;/p&gt; &lt;p&gt;  Il développe  &lt;a href="https://fr.wikipedia.org/wiki/Volontarisme_(courant_politique)" title=" volontarisme par wikipedia"&gt;le voluntarisme, &lt;/a&gt; une école qui étudie la conscience comme un flux organisé par la volonté, décomposant les expériences en éléments de base : sensations, sentiments et images mentales. Ses recherches portent sur les temps de réaction, la perception sensorielle et l'attention, utilisant des instruments comme le chronoscope pour mesurer les processus psychiques avec précision scientifique. Contrairement à une introspection subjective, sa méthode vise une objectivité comparable à celle de la chimie ou de la physique. &lt;/p&gt; &lt;p&gt; Ses œuvres ultérieures, comme Grundriss der Psychologie (1896) et la monumentale Völkerpsychologie (1900-1920, 10 volumes), étendent son analyse à la psychologie des peuples, couvrant langage, mythes, art et culture comme produits collectifs de l'esprit humain. Il distingue une psychologie expérimentale limitée aux processus élémentaires de l'"esprit inférieur" et une psychologie comparative pour les phénomènes culturels plus complexes. &lt;/p&gt; &lt;p&gt; Son influence est décisive : ses élèves, comme Edward Titchener (structuralisme), James McKeen Cattell ou G. Stanley Hall, diffusent ses idées aux États-Unis, fondant des laboratoires et associations psychologiques. Bien que critiqué plus tard pour le réductionnisme de l'introspection, il établit la psychologie comme science empirique, influençant la psychologie cognitive moderne et marquant la transition de la métaphysique philosophique vers l'expérimentation. &lt;/p&gt; 
 </t>
         </is>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F25" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="G24" s="9" t="s">
+      <c r="G25" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="H24" s="9" t="s">
+      <c r="H25" s="9" t="s">
         <v>209</v>
-      </c>
-      <c r="I24" s="7"/>
-      <c r="J24" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="N24" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="226.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="n">
-        <v>1833</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>215</v>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Wilhelm_Dilthey"  title=" Wikipedia"&gt;Wilhelm DILTHEY&lt;/a&gt; était un philosophe allemand connu pour sa distinction entre les sciences de la nature et les sciences humaines et pour sa thèse proposant de comprendre plutôt qu’expliquer &lt;a href="https://www.youtube.com/watch?v=dw_rVd4Fu5Y" title=" How Did Wilhelm Dilthey's Critique of Historical Reason Influence the Philosophy of History? par Open Answers"&gt;les actes humains. &lt;/a&gt; Cette orientation a marqué durablement les méthodologies des sciences humaines et sociales. Biographe de Schleiermacher, professeur à Berlin à partir de 1882, il publie en 1883 son &lt;em&gt;Introduction aux sciences de l’esprit&lt;/em&gt;. Sa formule est restée célèbre : « Nous expliquons la nature, nous comprenons la vie psychique. » &lt;/p&gt; &lt;p&gt; Pour lui, la science n’est pas uniquement une œuvre d’explication causaliste comme dans les sciences naturelles; elle repose sur la compréhension de l’esprit humain et de ses expressions historiques, sociales et culturelles. Il propose une ligne de démarcation entre les objets d’étude des sciences naturelles et ceux des sciences humaines, qui étudient la vie humaine et ses significations dans &lt;a href="https://www.persee.fr/doc/phlou_0035-3841_2014_num_112_4_8386_t1_0751_0000_3"  title=" La vie historique. Manuscrits relatifs à une suite de L’édification du monde historique dans les sciences de l’esprit.  par Open Persée"&gt;leur contexte historique. &lt;/a&gt; &lt;/p&gt; &lt;p&gt; Il est souvent vu comme un passeur entre le positivisme des sciences sociales et les approches interprétatives de la sociologie et de la  &lt;a href="https://www.youtube.com/watch?v=vWOt0ezdK4I" title=" Wilhelm Dilthey, l'importance de l'herméneutique par Open Leiden University"&gt;philosophie herméneutique &lt;/a&gt; qui dominent encore aujourd’hui. Ses idées ont nourri des débats sur les méthodes en sciences humaines, influence sur des penseurs ultérieurs et sur la reconnaissance des sciences humaines comme domaines autonomes de connaissance. Ses orientations ont été reprises et réinterprétées dans les courants phénoménologiques, herméneutiques et sociologiques, et ont contribué à la Querelle des méthodes en Allemagne au tournant du XXe siècle. &lt;/p&gt; </t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="G25" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="H25" s="9" t="s">
-        <v>219</v>
       </c>
       <c r="I25" s="7"/>
       <c r="J25" s="2" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>157</v>
+        <v>211</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="N25" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="145.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="226.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="n">
-        <v>1838</v>
+        <v>1833</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>225</v>
+        <v>215</v>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Wilhelm_Dilthey"  title=" Wikipedia"&gt;Wilhelm DILTHEY&lt;/a&gt; était un philosophe allemand connu pour sa distinction entre les sciences de la nature et les sciences humaines et pour sa thèse proposant de comprendre plutôt qu’expliquer &lt;a href="https://www.youtube.com/watch?v=dw_rVd4Fu5Y" title=" How Did Wilhelm Dilthey's Critique of Historical Reason Influence the Philosophy of History? par Open Answers"&gt;les actes humains. &lt;/a&gt; Cette orientation a marqué durablement les méthodologies des sciences humaines et sociales. Biographe de Schleiermacher, professeur à Berlin à partir de 1882, il publie en 1883 son &lt;em&gt;Introduction aux sciences de l’esprit&lt;/em&gt;. Sa formule est restée célèbre : « Nous expliquons la nature, nous comprenons la vie psychique. » &lt;/p&gt; &lt;p&gt; Pour lui, la science n’est pas uniquement une œuvre d’explication causaliste comme dans les sciences naturelles; elle repose sur la compréhension de l’esprit humain et de ses expressions historiques, sociales et culturelles. Il propose une ligne de démarcation entre les objets d’étude des sciences naturelles et ceux des sciences humaines, qui étudient la vie humaine et ses significations dans &lt;a href="https://www.persee.fr/doc/phlou_0035-3841_2014_num_112_4_8386_t1_0751_0000_3"  title=" La vie historique. Manuscrits relatifs à une suite de L’édification du monde historique dans les sciences de l’esprit.  par Open Persée"&gt;leur contexte historique. &lt;/a&gt; &lt;/p&gt; &lt;p&gt; Il est souvent vu comme un passeur entre le positivisme des sciences sociales et les approches interprétatives de la sociologie et de la  &lt;a href="https://www.youtube.com/watch?v=vWOt0ezdK4I" title=" Wilhelm Dilthey, l'importance de l'herméneutique par Open Leiden University"&gt;philosophie herméneutique &lt;/a&gt; qui dominent encore aujourd’hui. Ses idées ont nourri des débats sur les méthodes en sciences humaines, influence sur des penseurs ultérieurs et sur la reconnaissance des sciences humaines comme domaines autonomes de connaissance. Ses orientations ont été reprises et réinterprétées dans les courants phénoménologiques, herméneutiques et sociologiques, et ont contribué à la Querelle des méthodes en Allemagne au tournant du XXe siècle. &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F26" s="7" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="I26" s="7"/>
       <c r="J26" s="2" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>230</v>
+        <v>157</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="N26" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="145.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="n">
-        <v>1841</v>
+        <v>1838</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="I27" s="7"/>
       <c r="J27" s="2" t="s">
-        <v>118</v>
+        <v>229</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="N27" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="154.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="n">
-        <v>1842</v>
+        <v>1841</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="I28" s="7"/>
       <c r="J28" s="2" t="s">
-        <v>248</v>
+        <v>118</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="M28" s="0" t="s">
-        <v>186</v>
+        <v>240</v>
       </c>
       <c r="N28" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="284.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="154.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="n">
-        <v>1844</v>
+        <v>1842</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>253</v>
-      </c>
-      <c r="E29" s="18" t="s">
-        <v>254</v>
+        <v>243</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>244</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>255</v>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Le philosophe qui a défié Dieu et révolutionné la pensée" par Essence des Livres</t>
-        </is>
+        <v>245</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>246</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="I29" s="7"/>
       <c r="J29" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nihilisme ; Perspectivisme ; Irrationalisme ; Athéisme</t>
-        </is>
+        <v>248</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>249</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>259</v>
+        <v>250</v>
+      </c>
+      <c r="M29" s="0" t="s">
+        <v>186</v>
       </c>
       <c r="N29" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="O29" s="0" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="175.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="30" customFormat="false" ht="284.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="n">
-        <v>1848</v>
+        <v>1844</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>262</v>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Gottlob_Frege"  title=" Wikipedia"&gt;Gottlob FREGE&lt;/a&gt; était un philosophe allemand fondateur de la logique moderne et l'un des pères de la philosophie analytique. Il a développé des innovations révolutionnaires en &lt;a href="https://www.youtube.com/watch?v=sDlFaOn71n8" title=" Gottlob Frege - Du sens et de la référence par Jeffrey Kaplan"&gt;logique formelle&lt;/a&gt;, malgré une reconnaissance limitée de son vivant. Ses idées ont profondément influencé Russell, Wittgenstein et la philosophie du langage. &lt;/p&gt; &lt;p&gt; Il  invente la logique des prédicats modernes dans Begriffsschrift, introduisant une notation axiomatique complète pour &lt;a href="https://www.youtube.com/watch?v=OZlDzAxX2ik" title="L'énigme de Frege. par Philo Toutou"&gt;la logique propositionnelle &lt;/a&gt; et de premier ordre, avec quantification et distinction entre axiomes et règles d'inférence. Cela rompt avec la syllogistique aristotélicienne, fondant la logique contemporaine. Il traite les concepts comme des fonctions prenant des valeurs de vérité (Vrai ou Faux). &lt;/p&gt; &lt;p&gt; Défenseur du logisme, il vise à réduire l'arithmétique à la logique pure dans Grundlagen der Arithmetik (1884) et Grundgesetze der Arithmetik (1893-1903). Il critique le psychologisme, affirmant que les nombres sont des objets objectifs (extensions de concepts), non des idées mentales. Le paradoxe de Russell (1902) ruine son système, mais ses axiomes inspirent la théorie des ensembles. &lt;/p&gt; &lt;p&gt; Dans "Über Sinn und Bedeutung" (1892), Frege distingue le sens (Sinn, mode de présentation) de la référence (Bedeutung, objet désigné), expliquant pourquoi "l'étoile du matin" et "l'étoile du soir" ont le même référent (Vénus) mais des sens différents. Il introduit le principe de compositionnalité et le contexte, fondant la sémantique moderne. &lt;/p&gt; &lt;p&gt;  &lt;audio controls title="Le logicien Gottlob Frege n’est-il qu’un vulgaire plagiaire ? par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/21713-24.02.2021-ITEMA_22584463-2021C41495S0055-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
-        </is>
+        <v>253</v>
+      </c>
+      <c r="E30" s="18" t="s">
+        <v>254</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="G30" s="9" t="s">
-        <v>265</v>
+        <v>255</v>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Le philosophe qui a défié Dieu et révolutionné la pensée" par Essence des Livres</t>
+        </is>
       </c>
       <c r="H30" s="9" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="I30" s="7"/>
       <c r="J30" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>268</v>
+        <v>118</v>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nihilisme ; Perspectivisme ; Irrationalisme ; Athéisme</t>
+        </is>
       </c>
       <c r="L30" s="2" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="N30" s="0" t="s">
         <v>27</v>
       </c>
       <c r="O30" s="0" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="175.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="n">
         <v>1848</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>272</v>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Wilhelm_Windelband"  title=" Wikipedia"&gt;Wilhelm WINDELBAND&lt;/a&gt;  était un philosophe allemand  fondateur de l'école néokantienne de Bade (ou du Sud-Ouest), aux côtés de Heinrich Rickert, avec qui il forme un duo clé du  &lt;a href="https://www.youtube.com/watch?v=h2R8wj7Q9x8"  title="Néo-kantisme : définition, exemples. par le Savoir partagé"&gt;néokantisme tardif&lt;/a&gt;. Élève initialement influencé par la psychologie, il évolue vers un néokantisme anti-psychologiste, critiquant le relativisme historiciste et posant les bases d'une philosophie des valeurs. Professeur à Zurich, Fribourg-en-Brisgau, Strasbourg puis Heidelberg, il formule sa distinction la plus célèbre dans son discours de rectorat de Strasbourg, &lt;em&gt;Histoire et science de la nature&lt;/em&gt; (1894). &lt;/p&gt; &lt;p&gt; Il distingue &lt;a href="https://www.youtube.com/watch?v=Rr96FJSOcDU" title=" Wilhelm Windelband: Philosophy of Values and History par Philosopher Friends"&gt;les sciences &lt;/a&gt; nomothétiques (lois générales, comme la physique) des sciences idiographiques (individuel, historique), cette dichotomie méthodologique influençant Max Weber et la philosophie des sciences. Sa "philosophie des valeurs" transpose la critique kantienne vers la normativité : vérité, bien, beauté comme exigences objectives, sans recours au psychologisme ni au métaphysique spéculative. &lt;/p&gt; &lt;p&gt; Ses oeuvres principales sont : l’&lt;em&gt;Histoire de la philosophie moderne&lt;/em&gt; (1878-1880) et le &lt;em&gt;Manuel d’histoire de la philosophie&lt;/em&gt; (1892) : synthèses historiques rigoureuses, voyant l'histoire de la philosophie comme science autonome. "Präludien" en 1884, recueils d'essais : expose sa critique de la psychologie comme fondement du savoir et sa reformulation kantienne en termes normatifs. &lt;/p&gt; &lt;p&gt; Précurseur de la phénoménologie et des sciences humaines modernes, il impacte Rickert, Weber (types idéaux) et Jaspers, bien que moins systématique que les néokantiens de Marbourg. &lt;/p&gt; </t>
+        <v>262</v>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Gottlob_Frege"  title=" Wikipedia"&gt;Gottlob FREGE&lt;/a&gt; était un philosophe allemand fondateur de la logique moderne et l'un des pères de la philosophie analytique. Il a développé des innovations révolutionnaires en &lt;a href="https://www.youtube.com/watch?v=sDlFaOn71n8" title=" Gottlob Frege - Du sens et de la référence par Jeffrey Kaplan"&gt;logique formelle&lt;/a&gt;, malgré une reconnaissance limitée de son vivant. Ses idées ont profondément influencé Russell, Wittgenstein et la philosophie du langage. &lt;/p&gt; &lt;p&gt; Il  invente la logique des prédicats modernes dans Begriffsschrift, introduisant une notation axiomatique complète pour &lt;a href="https://www.youtube.com/watch?v=OZlDzAxX2ik" title="L'énigme de Frege. par Philo Toutou"&gt;la logique propositionnelle &lt;/a&gt; et de premier ordre, avec quantification et distinction entre axiomes et règles d'inférence. Cela rompt avec la syllogistique aristotélicienne, fondant la logique contemporaine. Il traite les concepts comme des fonctions prenant des valeurs de vérité (Vrai ou Faux). &lt;/p&gt; &lt;p&gt; Défenseur du logisme, il vise à réduire l'arithmétique à la logique pure dans Grundlagen der Arithmetik (1884) et Grundgesetze der Arithmetik (1893-1903). Il critique le psychologisme, affirmant que les nombres sont des objets objectifs (extensions de concepts), non des idées mentales. Le paradoxe de Russell (1902) ruine son système, mais ses axiomes inspirent la théorie des ensembles. &lt;/p&gt; &lt;p&gt; Dans "Über Sinn und Bedeutung" (1892), Frege distingue le sens (Sinn, mode de présentation) de la référence (Bedeutung, objet désigné), expliquant pourquoi "l'étoile du matin" et "l'étoile du soir" ont le même référent (Vénus) mais des sens différents. Il introduit le principe de compositionnalité et le contexte, fondant la sémantique moderne. &lt;/p&gt; &lt;p&gt;  &lt;audio controls title="Le logicien Gottlob Frege n’est-il qu’un vulgaire plagiaire ? par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/21713-24.02.2021-ITEMA_22584463-2021C41495S0055-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
         </is>
       </c>
       <c r="F31" s="7" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="I31" s="7"/>
       <c r="J31" s="2" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>249</v>
+        <v>268</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="N31" s="0" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="32" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="O31" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="n">
-        <v>1854</v>
+        <v>1848</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>280</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>281</v>
+        <v>272</v>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Wilhelm_Windelband"  title=" Wikipedia"&gt;Wilhelm WINDELBAND&lt;/a&gt;  était un philosophe allemand  fondateur de l'école néokantienne de Bade (ou du Sud-Ouest), aux côtés de Heinrich Rickert, avec qui il forme un duo clé du  &lt;a href="https://www.youtube.com/watch?v=h2R8wj7Q9x8"  title="Néo-kantisme : définition, exemples. par le Savoir partagé"&gt;néokantisme tardif&lt;/a&gt;. Élève initialement influencé par la psychologie, il évolue vers un néokantisme anti-psychologiste, critiquant le relativisme historiciste et posant les bases d'une philosophie des valeurs. Professeur à Zurich, Fribourg-en-Brisgau, Strasbourg puis Heidelberg, il formule sa distinction la plus célèbre dans son discours de rectorat de Strasbourg, &lt;em&gt;Histoire et science de la nature&lt;/em&gt; (1894). &lt;/p&gt; &lt;p&gt; Il distingue &lt;a href="https://www.youtube.com/watch?v=Rr96FJSOcDU" title=" Wilhelm Windelband: Philosophy of Values and History par Philosopher Friends"&gt;les sciences &lt;/a&gt; nomothétiques (lois générales, comme la physique) des sciences idiographiques (individuel, historique), cette dichotomie méthodologique influençant Max Weber et la philosophie des sciences. Sa "philosophie des valeurs" transpose la critique kantienne vers la normativité : vérité, bien, beauté comme exigences objectives, sans recours au psychologisme ni au métaphysique spéculative. &lt;/p&gt; &lt;p&gt; Ses oeuvres principales sont : l’&lt;em&gt;Histoire de la philosophie moderne&lt;/em&gt; (1878-1880) et le &lt;em&gt;Manuel d’histoire de la philosophie&lt;/em&gt; (1892) : synthèses historiques rigoureuses, voyant l'histoire de la philosophie comme science autonome. "Präludien" en 1884, recueils d'essais : expose sa critique de la psychologie comme fondement du savoir et sa reformulation kantienne en termes normatifs. &lt;/p&gt; &lt;p&gt; Précurseur de la phénoménologie et des sciences humaines modernes, il impacte Rickert, Weber (types idéaux) et Jaspers, bien que moins systématique que les néokantiens de Marbourg. &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F32" s="7" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="I32" s="7"/>
       <c r="J32" s="2" t="s">
@@ -3870,1122 +3893,1119 @@
         <v>249</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="N32" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="n">
-        <v>1856</v>
+        <v>1854</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>288</v>
-      </c>
-      <c r="E33" s="12" t="s">
-        <v>289</v>
+        <v>280</v>
+      </c>
+      <c r="E33" s="13" t="s">
+        <v>281</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="I33" s="7"/>
       <c r="J33" s="2" t="s">
         <v>248</v>
       </c>
       <c r="K33" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="N33" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="n">
+        <v>1856</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="H34" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="I34" s="7"/>
+      <c r="J34" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="K34" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="L33" s="2" t="s">
+      <c r="L34" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="M33" s="0" t="s">
+      <c r="M34" s="0" t="s">
         <v>186</v>
       </c>
-      <c r="N33" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="O33" s="0" t="n">
+      <c r="N34" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="O34" s="0" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="279" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="n">
+    <row r="35" customFormat="false" ht="279" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="n">
         <v>1858</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B35" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C35" s="7" t="s">
         <v>295</v>
       </c>
-      <c r="D34" s="11" t="s">
+      <c r="D35" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="E35" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Georg_Simmel" title=" Wikipedia"&gt;Georg SIMMEL&lt;/a&gt; était un philosophe du royaume de Prusse souvent considéré comme l’un des fondateurs de la sociologie de la modernité et de la   &lt;a href="https://www.youtube.com/watch?v=k2SZfvBp6H8"  title="Georg Simmel , sociologie urbaine . par PHILOVIBE"&gt;"sociologie formelle". &lt;/a&gt;  Il enseigne longtemps en marge de l’université, ce qui explique qu’il ait été moins institutionnalisé que Durkheim ou Weber, mais très influent sur eux et sur la sociologie ultérieure. &lt;/p&gt; &lt;p&gt; Il ne part pas de "la" société comme un grand tout, mais des formes d’interaction entre individus.  Il parle de sociologie formelle : les contenus (amour, travail, politique) varient, mais les formes (conflit, échange) se retrouvent partout et peuvent être étudiées en elles‑mêmes. Pour lui, la modernité se caractérise par une tension entre individu et société, entre culture subjective et culture objective.  La culture est produite par les individus mais devient ensuite une force autonome qui les dépasse, les contraint, et peut les écraser par sa complexité. &lt;/p&gt; &lt;p&gt; Il appartient au courant de la   &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_vie"  title="Philosophie de vie par Wikipedia"&gt;"philosophie de la vie" : &lt;/a&gt;  la vie est pour lui un flux créateur, mouvant, qui déborde toutes les formes fixes.  Les formes (institutions, normes, objets culturels) sont nécessaires pour donner sens au flux de la vie, mais elles se rigidifient et entrent en tension avec ce mouvement vital qui cherche toujours à se dépasser. Il  il insiste sur l’idée que la culture apparaît là où la vie rencontre des valeurs qui la transcendent (art, science, morale), mais ces valeurs finissent par se solidifier en systèmes objectifs qui peuvent aliéner l’individu. &lt;/p&gt;   &lt;audio controls title="Georg Simmel : Les grandes villes / Revue Questions internationales par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/12003-25.03.2013-ITEMA_20463123-2013C18006S0084-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
         </is>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="F35" s="7" t="s">
         <v>298</v>
       </c>
-      <c r="G34" s="9" t="s">
+      <c r="G35" s="9" t="s">
         <v>299</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="H35" s="9" t="s">
         <v>300</v>
       </c>
-      <c r="I34" s="9"/>
-      <c r="J34" s="2" t="s">
+      <c r="I35" s="9"/>
+      <c r="J35" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="K34" s="2" t="s">
+      <c r="K35" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="L34" s="2" t="s">
+      <c r="L35" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="M34" s="2" t="s">
+      <c r="M35" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="N34" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="245.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="n">
+      <c r="N35" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="245.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7" t="n">
         <v>1859</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B36" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C36" s="7" t="s">
         <v>303</v>
       </c>
-      <c r="D35" s="8" t="s">
+      <c r="D36" s="8" t="s">
         <v>304</v>
       </c>
-      <c r="E35" s="12" t="inlineStr">
+      <c r="E36" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt; &lt;a href="https://fr.wikipedia.org/wiki/Edmund_Husserl"  title=" Wikipedia"&gt; Edmund HUSSERL&lt;/a&gt; était un philosophe allemand d'origine juive connu pour être le fondateur de la  &lt;a href="https://www.youtube.com/watch?v=VaXxW0M9aIY"  title="Intro à la phénoménologie par Le Precepteur"&gt; phénoménologie&lt;/a&gt; qui est une méthode philosophique qui vise à décrire les structures de l'expérience telles qu'elles se présentent à la conscience, sans présuppositions théoriques ou métaphysiques. Il appelle cette approche "retour aux choses mêmes", ce qui signifie qu'il faut se concentrer sur les phénomènes tels qu'ils apparaissent à la conscience, plutôt que sur des interprétations ou des constructions théoriques. 
 Ses oeuvres les plus importantes : &lt;/p&gt; &lt;p&gt;"Idées directrices pour une phénoménologie pure et une philosophie phénoménologique" : il  y développe sa méthode de réduction phénoménologique et introduit le concept d'intentionnalité. &lt;/p&gt; &lt;p&gt;&lt;a href="https://www.persee.fr/doc/phlou_0035-3841_1954_num_52_33_4479"   title="Méditation cartésiennes par Persee"&gt; "Méditations cartésiennes"&lt;/a&gt; : Une série de conférences où il approfondit sa pensée sur l'ego transcendantal et l'intersubjectivité.&lt;/p&gt; &lt;p&gt;"Recherches logiques" (1900-1901) : Dans cet ouvrage, il critique le psychologisme (l'idée que les lois logiques sont des lois psychologiques) et pose les bases de sa phénoménologie.&lt;/p&gt; &lt;p&gt;"La crise des sciences européennes et la phénoménologie transcendantale" (1936) : Dans cet ouvrage posthume, il analyse la crise des sciences modernes et propose une refondation philosophique basée sur la phénoménologie.&lt;/p&gt; &lt;p&gt; Il a tenté de développer une méthode pour explorer la nature de la conscience humaine. Il a cherché à comprendre comment nous percevons le monde à travers nos sens, comment nous avons des pensées et des émotions, et comment nous nous rapportons à nous-mêmes et aux autres. &lt;/p&gt; &lt;p&gt; 
 La phénoménologie de Husserl a influencé de nombreux philosophes et écoles de pensée, notamment l'existentialisme (Sartre), la psychanalyse (Freud) et la philosophie de la perception. Ses travaux ont également inspiré des mouvements culturels tels que l'art abstrait et le modernisme.  &lt;/p&gt; &lt;audio controls title="Le phénomène Husserl par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/18755-09.03.2020-ITEMA_22302657-2.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
         </is>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="F36" s="7" t="s">
         <v>306</v>
       </c>
-      <c r="G35" s="9" t="s">
+      <c r="G36" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="H35" s="9" t="s">
+      <c r="H36" s="9" t="s">
         <v>308</v>
-      </c>
-      <c r="I35" s="7"/>
-      <c r="J35" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="M35" s="0" t="s">
-        <v>186</v>
-      </c>
-      <c r="N35" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="O35" s="0" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="251.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="n">
-        <v>1861</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>312</v>
-      </c>
-      <c r="E36" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Lou_Andreas-Salom%C3%A9" title=" Wikipedia"&gt;Lou ANDRÉAS-SALOMÉ&lt;/a&gt; était une écrivaine, philosophe, essayiste et psychanalyste allemande qui défendit une vision de la liberté incluant l'indépendance intellectuelle, émotionnelle et sexuelle. Elle rejette les conventions sociales et les rôles de genre traditionnels.  Ses principales oeuvres : &lt;/p&gt; &lt;p&gt;Friedrich Nietzsche à travers ses œuvres (1894) : Elle y analyse la philosophie de Nietzsche, en mettant l'accent sur ses idées sur la volonté de puissance, l'éternel retour et la mort de Dieu.  &lt;/p&gt; &lt;p&gt;Rainer Maria Rilke (1928) : Elle l'écrit après la mort de Rilke et elle y explore sa relation avec le poète et analyse son œuvre, en mettant l'accent sur sa quête spirituelle et artistique. &lt;/p&gt; &lt;p&gt;L'Érotisme (1910) : Elle explore la nature de l'érotisme et de la sexualité, en s'appuyant sur des réflexions psychologiques et philosophiques et défend une vision libérée et complexe de la sexualité. &lt;/p&gt; &lt;p&gt;Ma vie ( publié à titre posthume) : Dans son autobiographie, elle raconte &lt;a href="https://scienceetbiencommun.pressbooks.pub/femmessavantes3/chapter/lou-andreas-salome-femme-de-lettres-et-psychanalyste-1861-1937/" title="  Lou Andréas-Salomé, femme de lettres et psychanalyste par esbc"&gt;sa vie&lt;/a&gt;, ses relations et ses réflexions intellectuelles. &lt;/p&gt; &lt;p&gt; Bien qu'elle ne se définisse pas comme féministe, elle défend une vision de la femme comme être indépendant et complexe. Elle s'intéresse à la spiritualité et à la religion, en particulier dans ses écrits sur Nietzsche et Rilke. Elle explore des thèmes comme la quête de sens, la transcendance et la relation entre l'homme et le divin. &lt;/p&gt; &lt;p&gt;  Elle est l'une des &lt;a href="https://www.youtube.com/watch?v=SlLT7BXn_YI" title=" First Female Psychoanalyst: Lou Andreas Salomé par Orbit"&gt;premières femmes psychanalystes &lt;/a&gt; et ses écrits et ses réflexions ont contribué a son développement, en particulier dans les domaines de la sexualité et des relations humaines. &lt;/p&gt;  &lt;audio controls title="Lou Andreas-Salomé, la revendication d'un moi féminin libre par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/13915-16.08.2022-ITEMA_23103839-2021C3372E0235-NET_MFC_5D82F295-9FBD-4DEC-9B93-3E80E99A02A8-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  </t>
-        </is>
-      </c>
-      <c r="F36" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="G36" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>316</v>
       </c>
       <c r="I36" s="7"/>
       <c r="J36" s="2" t="s">
-        <v>317</v>
+        <v>229</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>318</v>
+        <v>230</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>320</v>
+        <v>186</v>
       </c>
       <c r="N36" s="0" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="224.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="O36" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="251.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="n">
-        <v>1863</v>
+        <v>1861</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>322</v>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Heinrich RICKERT</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Heinrich_Rickert" title=" Wikipedia"&gt;Heinrich RICKERT&lt;/a&gt; était un philosophe allemand  majeur du néokantisme, chef de file de l'école de Bade aux côtés de Wilhelm Windelband, axé sur &lt;a href="https://www.youtube.com/watch?v=-hQyRZfaCos"  title="Heinrich Rickert: Knowledge, Values, and Reality (#1349) par Philosopher Friends"&gt;une épistémologie &lt;/a&gt; distinguant les sciences nomologiques (naturelles) des sciences idiographiques (historiques et culturelles). &lt;/p&gt; &lt;p&gt; Ses oeuvres principales sont : "Der Gegenstand der Erkenntnis" paru en 1892, réédité jusqu'en 1928 : introduction à sa philosophie transcendantale, distinguant sujet et objet épistémologiques. "Die Grenzen der naturwissenschaftlichen Begriffsbildung" paru en 1902, plusieurs éditions : fondement de sa méthodologie, opposant généralisation scientifique et individualisation historique par des « concepts individuels », "Allgemeine Grundlegung der Philosophie" en 1921 et "Grundprobleme der Philosophie" en 1934 : systématisation de sa théorie de la connaissance et de l'ontologie. &lt;/p&gt; &lt;p&gt;&lt;a href="https://www.youtube.com/watch?v=nLzgyLsPWeI"  title="Heinrich Rickert et le concept logique de l'historique  par Nick Nielsen"&gt; Il  oppose &lt;/a&gt;  les sciences de la nature (recherche de lois générales) aux sciences culturelles (focalisées sur l'individuel et les valeurs), introduisant la notion de « relation aux valeurs » pour fonder l'objectivité historique. Il défend un idéalisme transcendantal kantien : la connaissance valide repose sur des principes a priori, avec une "transcendance" comme cause non empirique des expériences conscientes. Pour Rickert, l’historien ne juge pas les valeurs, mais il choisit ce qui mérite d’être raconté en rapportant les faits à des valeurs reconnues par une culture. Cette idée a profondément marqué le sociologue Max Weber. Professeur à Fribourg, puis à Heidelberg, il dirige à Fribourg l’habilitation du jeune Martin Heidegger. ​&lt;/p&gt; </t>
+        <v>311</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Lou_Andreas-Salom%C3%A9" title=" Wikipedia"&gt;Lou ANDRÉAS-SALOMÉ&lt;/a&gt; était une écrivaine, philosophe, essayiste et psychanalyste allemande qui défendit une vision de la liberté incluant l'indépendance intellectuelle, émotionnelle et sexuelle. Elle rejette les conventions sociales et les rôles de genre traditionnels.  Ses principales oeuvres : &lt;/p&gt; &lt;p&gt;Friedrich Nietzsche à travers ses œuvres (1894) : Elle y analyse la philosophie de Nietzsche, en mettant l'accent sur ses idées sur la volonté de puissance, l'éternel retour et la mort de Dieu.  &lt;/p&gt; &lt;p&gt;Rainer Maria Rilke (1928) : Elle l'écrit après la mort de Rilke et elle y explore sa relation avec le poète et analyse son œuvre, en mettant l'accent sur sa quête spirituelle et artistique. &lt;/p&gt; &lt;p&gt;L'Érotisme (1910) : Elle explore la nature de l'érotisme et de la sexualité, en s'appuyant sur des réflexions psychologiques et philosophiques et défend une vision libérée et complexe de la sexualité. &lt;/p&gt; &lt;p&gt;Ma vie ( publié à titre posthume) : Dans son autobiographie, elle raconte &lt;a href="https://scienceetbiencommun.pressbooks.pub/femmessavantes3/chapter/lou-andreas-salome-femme-de-lettres-et-psychanalyste-1861-1937/" title="  Lou Andréas-Salomé, femme de lettres et psychanalyste par esbc"&gt;sa vie&lt;/a&gt;, ses relations et ses réflexions intellectuelles. &lt;/p&gt; &lt;p&gt; Bien qu'elle ne se définisse pas comme féministe, elle défend une vision de la femme comme être indépendant et complexe. Elle s'intéresse à la spiritualité et à la religion, en particulier dans ses écrits sur Nietzsche et Rilke. Elle explore des thèmes comme la quête de sens, la transcendance et la relation entre l'homme et le divin. &lt;/p&gt; &lt;p&gt;  Elle est l'une des &lt;a href="https://www.youtube.com/watch?v=SlLT7BXn_YI" title=" First Female Psychoanalyst: Lou Andreas Salomé par Orbit"&gt;premières femmes psychanalystes &lt;/a&gt; et ses écrits et ses réflexions ont contribué a son développement, en particulier dans les domaines de la sexualité et des relations humaines. &lt;/p&gt;  &lt;audio controls title="Lou Andreas-Salomé, la revendication d'un moi féminin libre par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/13915-16.08.2022-ITEMA_23103839-2021C3372E0235-NET_MFC_5D82F295-9FBD-4DEC-9B93-3E80E99A02A8-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  </t>
         </is>
       </c>
       <c r="F37" s="7" t="s">
-        <v>325</v>
+        <v>314</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>326</v>
+        <v>315</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>327</v>
+        <v>316</v>
       </c>
       <c r="I37" s="7"/>
       <c r="J37" s="2" t="s">
-        <v>210</v>
+        <v>317</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>249</v>
+        <v>318</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>328</v>
+        <v>319</v>
+      </c>
+      <c r="M37" s="0" t="s">
+        <v>320</v>
       </c>
       <c r="N37" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="279" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="224.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="n">
-        <v>1867</v>
+        <v>1863</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="E38" s="14" t="s">
-        <v>332</v>
+        <v>322</v>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heinrich RICKERT</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Heinrich_Rickert" title=" Wikipedia"&gt;Heinrich RICKERT&lt;/a&gt; était un philosophe allemand  majeur du néokantisme, chef de file de l'école de Bade aux côtés de Wilhelm Windelband, axé sur &lt;a href="https://www.youtube.com/watch?v=-hQyRZfaCos"  title="Heinrich Rickert: Knowledge, Values, and Reality (#1349) par Philosopher Friends"&gt;une épistémologie &lt;/a&gt; distinguant les sciences nomologiques (naturelles) des sciences idiographiques (historiques et culturelles). &lt;/p&gt; &lt;p&gt; Ses oeuvres principales sont : "Der Gegenstand der Erkenntnis" paru en 1892, réédité jusqu'en 1928 : introduction à sa philosophie transcendantale, distinguant sujet et objet épistémologiques. "Die Grenzen der naturwissenschaftlichen Begriffsbildung" paru en 1902, plusieurs éditions : fondement de sa méthodologie, opposant généralisation scientifique et individualisation historique par des « concepts individuels », "Allgemeine Grundlegung der Philosophie" en 1921 et "Grundprobleme der Philosophie" en 1934 : systématisation de sa théorie de la connaissance et de l'ontologie. &lt;/p&gt; &lt;p&gt;&lt;a href="https://www.youtube.com/watch?v=nLzgyLsPWeI"  title="Heinrich Rickert et le concept logique de l'historique  par Nick Nielsen"&gt; Il  oppose &lt;/a&gt;  les sciences de la nature (recherche de lois générales) aux sciences culturelles (focalisées sur l'individuel et les valeurs), introduisant la notion de « relation aux valeurs » pour fonder l'objectivité historique. Il défend un idéalisme transcendantal kantien : la connaissance valide repose sur des principes a priori, avec une "transcendance" comme cause non empirique des expériences conscientes. Pour Rickert, l’historien ne juge pas les valeurs, mais il choisit ce qui mérite d’être raconté en rapportant les faits à des valeurs reconnues par une culture. Cette idée a profondément marqué le sociologue Max Weber. Professeur à Fribourg, puis à Heidelberg, il dirige à Fribourg l’habilitation du jeune Martin Heidegger. ​&lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F38" s="7" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="I38" s="7"/>
       <c r="J38" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="N38" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="279" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="n">
+        <v>1867</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="E39" s="14" t="s">
+        <v>332</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="H39" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="I39" s="7"/>
+      <c r="J39" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="K38" s="2" t="s">
+      <c r="K39" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="L38" s="19" t="s">
+      <c r="L39" s="19" t="s">
         <v>337</v>
       </c>
-      <c r="N38" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="267.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="n">
+      <c r="N39" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="267.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="n">
         <v>1871</v>
       </c>
-      <c r="B39" s="7" t="n">
+      <c r="B40" s="7" t="n">
         <v>1919</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="C40" s="7" t="s">
         <v>338</v>
       </c>
-      <c r="D39" s="8" t="s">
+      <c r="D40" s="8" t="s">
         <v>339</v>
       </c>
-      <c r="E39" s="14" t="s">
+      <c r="E40" s="14" t="s">
         <v>340</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="F40" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="G39" s="2" t="s">
+      <c r="G40" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="H39" s="2" t="s">
+      <c r="H40" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="J39" s="2" t="s">
+      <c r="J40" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="K39" s="2" t="s">
+      <c r="K40" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="L39" s="2" t="s">
+      <c r="L40" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="M39" s="0" t="s">
+      <c r="M40" s="0" t="s">
         <v>346</v>
       </c>
-      <c r="N39" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="O39" s="0" t="n">
+      <c r="N40" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="O40" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="XFC39" s="0"/>
-      <c r="XFD39" s="0"/>
-    </row>
-    <row r="40" customFormat="false" ht="284.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="n">
+      <c r="XFC40" s="0"/>
+      <c r="XFD40" s="0"/>
+    </row>
+    <row r="41" customFormat="false" ht="284.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="n">
         <v>1872</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B41" s="7" t="s">
         <v>347</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C41" s="7" t="s">
         <v>348</v>
       </c>
-      <c r="D40" s="8" t="s">
+      <c r="D41" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="E40" s="14" t="inlineStr">
+      <c r="E41" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Theodor_Lessing" title=" Wikipedia"&gt;Theodor LESSING&lt;/a&gt;  était un philosophe, essayiste et publiciste allemand &lt;a href="https://www.persee.fr/doc/rjuiv_0484-8616_1996_num_155_1_2554"  title="Lessing et le sionisme par persée"&gt;d’origine juive, &lt;/a&gt; connu comme un penseur critique de la modernité, du nationalisme et de l’antisémitisme. &lt;/p&gt; &lt;p&gt; Il s’inscrit surtout dans une philosophie de la culture et une philosophie sociale critique. Son travail ne cherche pas à construire un système abstrait, mais à analyser les maladies de la civilisation moderne, la violence des masses, la guerre, la ville industrielle et la destruction du vivant. Sa pensée est marquée par un humanisme pessimiste et engagé qui dénoncé le militarisme, la brutalisation de la société et les dérives autoritaires de l’Allemagne de Weimar, allant jusqu’à prévoir le danger nazi avant 1933. Il fut aussi l’un des premiers à réfléchir à la condition des minorités et à ce qu’il a appelé le &lt;a href="https://www.sifriatenou.com/2020/10/20/5449/"  title="lessing la haine de soi par sifriatenou"&gt;« judaïsme de haine de soi »,&lt;/a&gt; pour décrire les effets psychologiques de l’antisémitisme sur les Juifs eux-mêmes. &lt;/p&gt; &lt;p&gt; Il est également une figure de la critique écologique avant l’heure. Dès les années 1930, il s’inquiète de la déforestation, de la pollution urbaine et d’un possible dérèglement du climat, ce qui le rend étonnamment actuel. Il voit la modernité technique non comme un progrès neutre, mais comme une force capable de détruire les équilibres humains et naturels. &lt;/p&gt; &lt;p&gt; Sur le plan politique, il est un intellectuel indépendant, polémique et souvent isolé, qui s’oppose à l’autoritarisme autant qu’aux conformismes de son époque. Il a fini assassiné en exil   à Mariánské Lázně par des nationalistes sudètes, devenant l’une des premières victimes du nazisme hors d’Allemagne. &lt;/p&gt; 
 </t>
         </is>
       </c>
-      <c r="F40" s="7" t="s">
+      <c r="F41" s="7" t="s">
         <v>351</v>
       </c>
-      <c r="G40" s="9" t="s">
+      <c r="G41" s="9" t="s">
         <v>352</v>
       </c>
-      <c r="H40" s="9" t="s">
+      <c r="H41" s="9" t="s">
         <v>353</v>
       </c>
-      <c r="I40" s="7"/>
-      <c r="J40" s="2" t="s">
+      <c r="I41" s="7"/>
+      <c r="J41" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="K40" s="2" t="s">
+      <c r="K41" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="L40" s="19" t="s">
+      <c r="L41" s="19" t="s">
         <v>354</v>
       </c>
-      <c r="M40" s="0" t="s">
+      <c r="M41" s="0" t="s">
         <v>186</v>
       </c>
-      <c r="N40" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="253.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="n">
+      <c r="N41" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="253.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="n">
         <v>1874</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B42" s="7" t="s">
         <v>355</v>
       </c>
-      <c r="C41" s="7" t="s">
+      <c r="C42" s="7" t="s">
         <v>356</v>
       </c>
-      <c r="D41" s="8" t="s">
+      <c r="D42" s="8" t="s">
         <v>357</v>
       </c>
-      <c r="E41" s="12" t="inlineStr">
+      <c r="E42" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Max_Scheler" title=" Wikipedia"&gt;Max SCHELER&lt;/a&gt;  était un philosophe allemand, figure phare de la phénoménologie et de l’anthropologie philosophique, dont l’œuvre traverse des domaines variés comme l’éthique, l’axiologie et la sociologie de la connaissance. &lt;/p&gt; &lt;p&gt; Il élabore une &lt;a href="https://www.persee.fr/doc/phlou_0776-555x_1927_num_29_14_2467"  title="La philosophie de M. Scheler. Son analyse de la sympathie et de l'amour par Persée"&gt;hiérarchie des valeurs &lt;/a&gt; qui va des valeurs de l’agréable et du désagréable jusqu’aux valeurs spirituelles (beau/laid, juste/injuste, connaissance, et enfin le sacré et le profane). Cette hiérarchie sert de base à une éthique et à une phénoménologie de la sensation et des sentiments qui orientent l’action humaine. Il propose une approche phénoménologique qui insiste sur "l’attitude spirituelle" ou "l’œil vivant" vers le monde, en s’opposant à une réduction purement méthodologique et en valorisant l’intuition des valeurs telles qu’elles se donnent à la conscience. &lt;/p&gt; &lt;p&gt; Il fonde l’idée d’une anthropologie philosophique qui cherche à comprendre l’homme dans le vivant et ses rapports au monde, en intégrant des connaissances des sciences naturelles et des sciences humaines. &lt;a href="https://www.youtube.com/watch?v=pPuUoTPig7w" title="Le salut vient-il du travail ? - Valeur et dignité du travail selon Max SCHELER par Editions M-Editer"&gt;Cette orientation &lt;/a&gt; mène plus tard à une sociologie de la connaissance. &lt;/p&gt; &lt;p&gt;"Die Wissensformen und die Gesellschaft" paru en 1926 – synthèse de son projet de sociologie de la connaissance et jalon important de l’anthropologie philosophique et sociale. Cette œuvre est souvent citée comme fondatrice d’une approche sociologique qui rejoint les débats de Weimar.&lt;/p&gt; &lt;p&gt;"Stellung des Menschen im Kosmos" paru en 1928 – portrait philosophique de l’homme dans le cadre d’un ensemble plus large d’ouvrages préfigurant l’anthropologie philosophique et son intérêt pour le positionnement de l’homme dans l’ordre du vivant. &lt;/p&gt; &lt;p&gt; Son approche personnaliste et son engagement en faveur d’une philosophie sociale et éthique centrée sur la dignité humaine, &lt;a href="https://www.youtube.com/watch?v=HHAKQrNdMYk" title="
 Le ressentiment détruit ta vie… (Max Sheller, l'homme du ressentiment) par Timothée Delahaye"&gt;le resentiment &lt;/a&gt; et les valeurs morales continuent d’être discutés dans les études contemporaines, notamment dans les analyses qui situent Scheler dans le dialogue franco-allemand et dans les traditions de philosophie sociale et morale. &lt;/p&gt; </t>
         </is>
       </c>
-      <c r="F41" s="7" t="s">
+      <c r="F42" s="7" t="s">
         <v>359</v>
       </c>
-      <c r="G41" s="9" t="s">
+      <c r="G42" s="9" t="s">
         <v>360</v>
       </c>
-      <c r="H41" s="9" t="s">
+      <c r="H42" s="9" t="s">
         <v>361</v>
-      </c>
-      <c r="I41" s="7"/>
-      <c r="J41" s="2" t="s">
-        <v>362</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>363</v>
-      </c>
-      <c r="N41" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="217.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="n">
-        <v>1874</v>
-      </c>
-      <c r="B42" s="7" t="s">
-        <v>364</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>365</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>366</v>
-      </c>
-      <c r="E42" s="18" t="s">
-        <v>367</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>368</v>
-      </c>
-      <c r="G42" s="9" t="s">
-        <v>369</v>
-      </c>
-      <c r="H42" s="9" t="s">
-        <v>370</v>
       </c>
       <c r="I42" s="7"/>
       <c r="J42" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="N42" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="217.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="7" t="n">
+        <v>1874</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="E43" s="18" t="s">
+        <v>367</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="I43" s="7"/>
+      <c r="J43" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="K42" s="2" t="s">
+      <c r="K43" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="L42" s="19" t="s">
+      <c r="L43" s="19" t="s">
         <v>371</v>
       </c>
-      <c r="M42" s="0" t="s">
+      <c r="M43" s="0" t="s">
         <v>186</v>
       </c>
-      <c r="N42" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="227.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="n">
+      <c r="N43" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="227.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7" t="n">
         <v>1880</v>
       </c>
-      <c r="B43" s="7" t="s">
+      <c r="B44" s="7" t="s">
         <v>321</v>
       </c>
-      <c r="C43" s="7" t="s">
+      <c r="C44" s="7" t="s">
         <v>372</v>
       </c>
-      <c r="D43" s="8" t="s">
+      <c r="D44" s="8" t="s">
         <v>373</v>
       </c>
-      <c r="E43" s="9" t="inlineStr">
+      <c r="E44" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Oswald_Spengler"  title=" Wikipedia"&gt;Oswald SPENGLER&lt;/a&gt;  était un philosophe allemand célèbre pour sa vision cyclique de l'histoire des civilisations dans son œuvre majeure Le Déclin de l'Occident. Il développe une philosophie organique où les cultures sont comparées à des organismes vivants qui naissent, croissent, déclinent et meurent. &lt;/p&gt; &lt;p&gt; Il  rejette l'histoire linéaire ou universaliste au profit d'une "morphologie de l'histoire" : huit grandes cultures (égyptienne, chinoise, indienne, babylonienne, grecque, romaine, arabe, occidentale) évoluent indépendamment comme des entités biologiques. Chaque culture passe par des stades (printemps créatif, été apollinien, automne faustien pour l'Occident, hiver civilisationnel décadent). L'Occident, faustien et dynamique, entre dans une phase de déclin urbain, matérialiste et césariste depuis le XIXe siècle. &lt;/p&gt; &lt;p&gt; Ses oeuvres les plus importantes sont : Le Déclin de l'Occident paru entre 1918- et 1922 : analyse comparative des cultures, prédisant un avenir de "guerre d'anéantissement" et de dictatures pour l'Europe. Prussianisme et socialisme en 1919 : défense d'un socialisme prussien basé sur discipline et hiérarchie, opposé au marxisme. &lt;a href="http://www.exergue.com/h/2016-09/tt/spengler-technique.html" title="Oswald Spengler, L'Homme et la Technique par Exergue"&gt;"L'Homme et la technique" &lt;/a&gt; en 1931 : critique de la civilisation technicienne comme  &lt;a href="https://www.youtube.com/watch?v=RbISu_9rON0"  title=" L'âme de la culture occidentale - Les principaux symboles d'Oswald Spengler par ThinkingWest"&gt;symptôme de déclin.&lt;/a&gt; &lt;/p&gt; &lt;p&gt; Membre de la "Révolution conservatrice" de Weimar, il influence la pensée nationaliste mais critique le nazisme pour son racisme excessif, préférant des "Césars" comme Mussolini. Ses idées inspirent des débats sur le déclin occidental, de Heidegger à des auteurs contemporains, malgré les critiques d'historicisme relativiste &lt;/p&gt;  &lt;audio controls title="Oswald Spengler ou le destin de l’Occident par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/13915-01.11.2022-ITEMA_23183001-2010C3372E1812-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
 </t>
         </is>
       </c>
-      <c r="F43" s="7" t="s">
+      <c r="F44" s="7" t="s">
         <v>375</v>
       </c>
-      <c r="G43" s="9" t="s">
+      <c r="G44" s="9" t="s">
         <v>376</v>
       </c>
-      <c r="H43" s="9" t="s">
+      <c r="H44" s="9" t="s">
         <v>377</v>
-      </c>
-      <c r="I43" s="7"/>
-      <c r="J43" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="L43" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="N43" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="249.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="n">
-        <v>1880</v>
-      </c>
-      <c r="B44" s="7" t="s">
-        <v>380</v>
-      </c>
-      <c r="C44" s="7" t="s">
-        <v>381</v>
-      </c>
-      <c r="D44" s="8" t="s">
-        <v>382</v>
-      </c>
-      <c r="E44" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Hermann_von_Keyserling" title=" Wikipedia"&gt;Hermann Von KEYSERLING&lt;/a&gt;  était un philosophe  &lt;a href="https://www.persee.fr/doc/slaoc_1245-2491_1997_num_4_1_1809" style="color:#88A1E9" title=" Hermann von Keyserling et les interférences germano-slaves par Persée"&gt;germano-balte &lt;/a&gt; devenu philosophe voyageur, figure très en vue de la République de Weimar, connu pour son Journal de voyage d’un philosophe et pour son "École de la sagesse" à Darmstadt. &lt;/p&gt; &lt;p&gt; Il conçoit la philosophie non comme une science rigoureuse, mais comme sagesse vécue : "la vie elle-même sous la forme du savoir", contre les théories objectivantes du savoir technico-scientifique. Il s’inscrit dans la philosophie de la vie, mais de façon personnelle : importance de l’intuition, de la singularité des événements et de la transformation intérieure. Son projet est une nouvelle synthèse de l’âme et de l’esprit, la pénétration réciproque de sagesse et politique, et l’idée que dans la vie déterminée par l’esprit, c’est &lt;a href="https://www.youtube.com/watch?v=Y0DY8F72114" title="Eduard von Keyserling, DUMALA par Le Veilleur"&gt;le Sens &lt;/a&gt; qui crée les faits plutôt que l’inverse. &lt;/p&gt; &lt;p&gt; Il  utilise très tôt le terme Führerprinzip, en liant l’idée de "dirigeants nés" à un élitisme spiritualiste et social-darwinien, tout en refusant par la suite d’adhérer au national-socialisme, qu’il voit comme mouvement de masses manipulées.  Le régime nazi ferme son École de la sagesse au milieu des années 1930, lui interdit de publier et de voyager, tandis que sa réputation continue de grandir à l’étranger. &lt;/p&gt;&lt;p&gt; Ses oeuvres principales sont : "Reisetagebuch eines Philosophen"  paru en 1919 : récit de son tour du monde (1911-1912, Asie, Amérique, Europe du Sud) mêlant observations culturelles, méditations spirituelles et diagnostics sur les civilisations ; c’est son grand succès de librairie, largement traduit. -"Das Gefüge der Welt. Versuch einer kritischen Philosophie" (La Structure du monde, 1907) : tentative de "philosophie critique" personnelle, déjà marquée par l’idée que le savoir véritable est inséparable de la vie. "Schöpferische Erkenntnis" (Connaissance créatrice) et "Wiedergeburt" (Renaissance) : textes doctrinaux de l’"École de la sagesse", insistant sur la connaissance comme acte créateur, transformant la vie plutôt que la décrivant objectivement. &lt;/p&gt; </t>
-        </is>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>384</v>
-      </c>
-      <c r="G44" s="9" t="s">
-        <v>385</v>
-      </c>
-      <c r="H44" s="9" t="s">
-        <v>386</v>
       </c>
       <c r="I44" s="7"/>
       <c r="J44" s="2" t="s">
-        <v>108</v>
+        <v>166</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>387</v>
+        <v>378</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>388</v>
+        <v>379</v>
       </c>
       <c r="N44" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="297" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="249.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="n">
-        <v>1882</v>
-      </c>
-      <c r="B45" s="7" t="n">
-        <v>1936</v>
+        <v>1880</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>380</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>390</v>
-      </c>
-      <c r="E45" s="14" t="s">
-        <v>391</v>
+        <v>382</v>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Hermann_von_Keyserling" title=" Wikipedia"&gt;Hermann Von KEYSERLING&lt;/a&gt;  était un philosophe  &lt;a href="https://www.persee.fr/doc/slaoc_1245-2491_1997_num_4_1_1809" style="color:#88A1E9" title=" Hermann von Keyserling et les interférences germano-slaves par Persée"&gt;germano-balte &lt;/a&gt; devenu philosophe voyageur, figure très en vue de la République de Weimar, connu pour son Journal de voyage d’un philosophe et pour son "École de la sagesse" à Darmstadt. &lt;/p&gt; &lt;p&gt; Il conçoit la philosophie non comme une science rigoureuse, mais comme sagesse vécue : "la vie elle-même sous la forme du savoir", contre les théories objectivantes du savoir technico-scientifique. Il s’inscrit dans la philosophie de la vie, mais de façon personnelle : importance de l’intuition, de la singularité des événements et de la transformation intérieure. Son projet est une nouvelle synthèse de l’âme et de l’esprit, la pénétration réciproque de sagesse et politique, et l’idée que dans la vie déterminée par l’esprit, c’est &lt;a href="https://www.youtube.com/watch?v=Y0DY8F72114" title="Eduard von Keyserling, DUMALA par Le Veilleur"&gt;le Sens &lt;/a&gt; qui crée les faits plutôt que l’inverse. &lt;/p&gt; &lt;p&gt; Il  utilise très tôt le terme Führerprinzip, en liant l’idée de "dirigeants nés" à un élitisme spiritualiste et social-darwinien, tout en refusant par la suite d’adhérer au national-socialisme, qu’il voit comme mouvement de masses manipulées.  Le régime nazi ferme son École de la sagesse au milieu des années 1930, lui interdit de publier et de voyager, tandis que sa réputation continue de grandir à l’étranger. &lt;/p&gt;&lt;p&gt; Ses oeuvres principales sont : "Reisetagebuch eines Philosophen"  paru en 1919 : récit de son tour du monde (1911-1912, Asie, Amérique, Europe du Sud) mêlant observations culturelles, méditations spirituelles et diagnostics sur les civilisations ; c’est son grand succès de librairie, largement traduit. -"Das Gefüge der Welt. Versuch einer kritischen Philosophie" (La Structure du monde, 1907) : tentative de "philosophie critique" personnelle, déjà marquée par l’idée que le savoir véritable est inséparable de la vie. "Schöpferische Erkenntnis" (Connaissance créatrice) et "Wiedergeburt" (Renaissance) : textes doctrinaux de l’"École de la sagesse", insistant sur la connaissance comme acte créateur, transformant la vie plutôt que la décrivant objectivement. &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F45" s="7" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>393</v>
-      </c>
-      <c r="H45" s="12" t="s">
-        <v>394</v>
+        <v>385</v>
+      </c>
+      <c r="H45" s="9" t="s">
+        <v>386</v>
       </c>
       <c r="I45" s="7"/>
       <c r="J45" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="N45" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="297" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="n">
+        <v>1882</v>
+      </c>
+      <c r="B46" s="7" t="n">
+        <v>1936</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>391</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="G46" s="9" t="s">
+        <v>393</v>
+      </c>
+      <c r="H46" s="12" t="s">
+        <v>394</v>
+      </c>
+      <c r="I46" s="7"/>
+      <c r="J46" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="K45" s="2" t="s">
+      <c r="K46" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="L45" s="17" t="s">
+      <c r="L46" s="17" t="s">
         <v>397</v>
       </c>
-      <c r="N45" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="206.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="n">
+      <c r="N46" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="206.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="7" t="n">
         <v>1885</v>
       </c>
-      <c r="B46" s="7" t="s">
+      <c r="B47" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="C47" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="D46" s="8" t="s">
+      <c r="D47" s="8" t="s">
         <v>400</v>
       </c>
-      <c r="E46" s="13" t="inlineStr">
+      <c r="E47" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ernst_Bloch"  title=" Wikipedia"&gt;Ernst BLOCH&lt;/a&gt;  était un philosophe juif allemand  souvent rattaché au marxisme hétérodoxe et à la philosophie de l’espérance. Sa pensée se distingue par une défense de l’utopie comme force critique et émancipatrice, contre les lectures trop fermées ou déterministes de l’histoire. &lt;/p&gt; &lt;p&gt; Il part de l’idée que la réalité humaine n’est jamais complètement accomplie: il y a toujours du “pas encore” dans l’histoire, dans la société et dans la conscience. Il appelle cela le non-simultané ou le caractère inachevé du réel, ce qui permet de penser le futur comme ouvert plutôt que comme déjà écrit. &lt;/p&gt; &lt;p&gt; Son ouvrage majeur,  &lt;a href="https://www.youtube.com/watch?v=u-zXjE1duok"  title="Le principe de l’espérance par Culture Philo"&gt; Le Principe espérance, &lt;/a&gt; développe l’idée que l’espérance n’est pas une illusion passive, mais une énergie active qui pousse les hommes à transformer le monde. L’utopie, chez lui, n’est donc pas un rêve irréaliste: c’est une anticipation concrète de ce qui pourrait advenir. &lt;/p&gt; &lt;p&gt; Il accorde aussi une grande importance aux œuvres culturelles, à la religion, à l’art et même aux rêves éveillés, parce qu’ils contiennent des indices de possibles non réalisés. Il voit dans ces domaines des formes où s’exprime un dépassement de la situation présente, une ouverture vers un monde plus juste. &lt;/p&gt; &lt;p&gt; Sa philosophie est une pensée du possible et du futur. Elle combine critique du présent, héritage marxiste et réhabilitation de l’utopie pour montrer que l’histoire humaine peut encore être transformée. &lt;/p&gt;  &lt;audio controls title="A quoi bon espérer ? par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-27.06.2023-ITEMA_23423905-2023C48904S0178-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
 </t>
         </is>
       </c>
-      <c r="F46" s="7" t="s">
+      <c r="F47" s="7" t="s">
         <v>402</v>
       </c>
-      <c r="G46" s="9" t="s">
+      <c r="G47" s="9" t="s">
         <v>403</v>
       </c>
-      <c r="H46" s="9" t="s">
+      <c r="H47" s="9" t="s">
         <v>404</v>
-      </c>
-      <c r="I46" s="7"/>
-      <c r="J46" s="2" t="s">
-        <v>405</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="L46" s="17" t="s">
-        <v>407</v>
-      </c>
-      <c r="M46" s="0" t="s">
-        <v>186</v>
-      </c>
-      <c r="N46" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="n">
-        <v>1886</v>
-      </c>
-      <c r="B47" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="C47" s="7" t="s">
-        <v>409</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>410</v>
-      </c>
-      <c r="E47" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Korsch" title=" Wikipedia"&gt;Karl KORSCH&lt;/a&gt;  était un philosophe marxiste allemand,  théoricien du communisme de conseils et critique du léninisme orthodoxe. Issu d'un milieu bourgeois, il évolua du réformisme social au marxisme hétérodoxe, influençant les courants ultra-gauche via son rejet du matérialisme positiviste et son insistance sur la praxis révolutionnaire historique. Juriste de formation, il est en 1923 ministre de la Justice de Thuringe, puis député communiste au Reichstag.  Exclu du parti en 1926 pour "ultra-gauchisme", il émigra après 1933 vers les États-Unis, où il approfondit sa théorie marxiste. &lt;/p&gt; &lt;p&gt; Son œuvre majeure &lt;em&gt;Marxisme et philosophie&lt;/em&gt; paru en 1923 marque sa rupture avec le léninisme en critiquant sa dérive scientiste. Il   &lt;a href="https://www.zones-subversives.com/article-le-marxisme-critique-de-karl-korsch-116431466.html"  title="Le marxisme critique de Karl Korsch par Chroniques critiques"&gt;rejette le marxisme &lt;/a&gt; comme "science positive" figée ou philosophie matérialiste abstraite ; il le conçoit comme une théorie historique et concrète, liée à la lutte des classes et à la dialectique hégélienne réinterprétée comme expression de la révolution bourgeoise puis prolétarienne. &lt;/p&gt; &lt;p&gt; Il  théorise les conseils comme organes centraux de la transition socialiste, via la praxis dialectique et l'auto-activité des masses, contre la socialisation étatique. Ses écrits inspirent le KAPD et l'ultra-gauche, voyant les conseils comme alternative à la bureaucratisation stalinienne. Son influence perdure chez les communistes de conseils, soulignant la conscience ouvrière spontanée pour l'émancipation réelle. Aux États-Unis, il publie &lt;em&gt;Karl Marx&lt;/em&gt; (1938) et reste proche de Bertolt Brecht, qui le considérait comme son maître en marxisme. &lt;/p&gt; </t>
-        </is>
-      </c>
-      <c r="F47" s="7" t="s">
-        <v>412</v>
-      </c>
-      <c r="G47" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="H47" s="9" t="s">
-        <v>414</v>
       </c>
       <c r="I47" s="7"/>
       <c r="J47" s="2" t="s">
-        <v>344</v>
+        <v>405</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="L47" s="2" t="s">
-        <v>415</v>
+        <v>406</v>
+      </c>
+      <c r="L47" s="17" t="s">
+        <v>407</v>
+      </c>
+      <c r="M47" s="0" t="s">
+        <v>186</v>
       </c>
       <c r="N47" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="n">
         <v>1886</v>
       </c>
       <c r="B48" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="D48" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Korsch" title=" Wikipedia"&gt;Karl KORSCH&lt;/a&gt;  était un philosophe marxiste allemand,  théoricien du communisme de conseils et critique du léninisme orthodoxe. Issu d'un milieu bourgeois, il évolua du réformisme social au marxisme hétérodoxe, influençant les courants ultra-gauche via son rejet du matérialisme positiviste et son insistance sur la praxis révolutionnaire historique. Juriste de formation, il est en 1923 ministre de la Justice de Thuringe, puis député communiste au Reichstag.  Exclu du parti en 1926 pour "ultra-gauchisme", il émigra après 1933 vers les États-Unis, où il approfondit sa théorie marxiste. &lt;/p&gt; &lt;p&gt; Son œuvre majeure &lt;em&gt;Marxisme et philosophie&lt;/em&gt; paru en 1923 marque sa rupture avec le léninisme en critiquant sa dérive scientiste. Il   &lt;a href="https://www.zones-subversives.com/article-le-marxisme-critique-de-karl-korsch-116431466.html"  title="Le marxisme critique de Karl Korsch par Chroniques critiques"&gt;rejette le marxisme &lt;/a&gt; comme "science positive" figée ou philosophie matérialiste abstraite ; il le conçoit comme une théorie historique et concrète, liée à la lutte des classes et à la dialectique hégélienne réinterprétée comme expression de la révolution bourgeoise puis prolétarienne. &lt;/p&gt; &lt;p&gt; Il  théorise les conseils comme organes centraux de la transition socialiste, via la praxis dialectique et l'auto-activité des masses, contre la socialisation étatique. Ses écrits inspirent le KAPD et l'ultra-gauche, voyant les conseils comme alternative à la bureaucratisation stalinienne. Son influence perdure chez les communistes de conseils, soulignant la conscience ouvrière spontanée pour l'émancipation réelle. Aux États-Unis, il publie &lt;em&gt;Karl Marx&lt;/em&gt; (1938) et reste proche de Bertolt Brecht, qui le considérait comme son maître en marxisme. &lt;/p&gt; </t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="G48" s="9" t="s">
+        <v>413</v>
+      </c>
+      <c r="H48" s="9" t="s">
+        <v>414</v>
+      </c>
+      <c r="I48" s="7"/>
+      <c r="J48" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="N48" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="n">
+        <v>1886</v>
+      </c>
+      <c r="B49" s="7" t="s">
         <v>416</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="C49" s="7" t="s">
         <v>417</v>
       </c>
-      <c r="D48" s="8" t="s">
+      <c r="D49" s="8" t="s">
         <v>418</v>
       </c>
-      <c r="E48" s="9" t="inlineStr">
+      <c r="E49" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Franz_Rosenzweig" title=" Wikipedia"&gt;Franz ROSENZWEIG&lt;/a&gt; était un philosophe et théologien juif allemand et l’une des grandes voix du &lt;a href="https://journals.openedition.org/ceg/16724" title="Les visages du temps dans la pensée de Franz Rosenzweig  par Open Edition"&gt;renouveau de la pensée juive. &lt;/a&gt;  Il se forme d’abord dans l’orbite de l’idéalisme allemand, en particulier Hegel, mais va s’y opposer radicalement. Il critique l’idée de "totalité" qui engloberait et expliquerait tout ce qui est : pour lui, le réel est irréductiblement plural, composé d’éléments qui ne se laissent pas fondre dans un système unique. Il refuse la prétention de la philosophie à un "savoir absolu" qui surplomberait Dieu, le monde et l’homme. Sa démarche consiste à partir de l’expérience concrète, de la finitude et de la mortalité humaines, plutôt que de concepts abstraits de l’être. &lt;/p&gt; &lt;p&gt; Dans "L’Étoile de la rédemption", &lt;a href="https://www.youtube.com/watch?v=OSyPZERfePg"  title="Sur Franz Rosenzweig : Gérard Bensussan à Ombres Blanches, Toulouse  par LeBras videos et chocolat"&gt;il propose &lt;/a&gt; une grande architecture de pensée à partir de trois "éléments" fondamentaux : Dieu, le monde, l’homme. Ces trois réalités sont distinctes, irréductibles l’une à l’autre : on ne peut ni ramener Dieu au monde, ni réduire l’homme à un moment d’un tout cosmique. Elles entrent en relation à travers trois mouvements : création (Dieu–monde), révélation (Dieu–homme) et rédemption (homme–monde). &lt;/p&gt; &lt;p&gt; Un point central chez lui est la compréhension de la révélation comme événement adressé à un sujet concret dans le temps. Dieu est pensé comme "existant suprême et totalisateur" mais qui se révèle dans des actes, des paroles, une histoire avec un peuple et avec des individus. Le temps devient le lieu où se déploient création, révélation et rédemption : il insiste sur la mortalité de l’homme, mais aussi sur une forme de "vie éternelle" déjà à l’œuvre. &lt;/p&gt; 
    &lt;audio controls title="Franz Rosenzweig, l'anti-Hegel par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/12014-31.01.2017-ITEMA_21214189-2017C26359S0031-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
 </t>
         </is>
       </c>
-      <c r="F48" s="7" t="s">
+      <c r="F49" s="7" t="s">
         <v>420</v>
       </c>
-      <c r="G48" s="9" t="s">
+      <c r="G49" s="9" t="s">
         <v>421</v>
       </c>
-      <c r="H48" s="9" t="s">
+      <c r="H49" s="9" t="s">
         <v>422</v>
       </c>
-      <c r="I48" s="7"/>
-      <c r="J48" s="2" t="s">
+      <c r="I49" s="7"/>
+      <c r="J49" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="K48" s="2" t="s">
+      <c r="K49" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="L48" s="2" t="s">
+      <c r="L49" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="M48" s="0" t="s">
+      <c r="M49" s="0" t="s">
         <v>186</v>
       </c>
-      <c r="N48" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="n">
+      <c r="N49" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="7" t="n">
         <v>1888</v>
       </c>
-      <c r="B49" s="7" t="s">
+      <c r="B50" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="C49" s="7" t="s">
+      <c r="C50" s="7" t="s">
         <v>426</v>
       </c>
-      <c r="D49" s="8" t="s">
+      <c r="D50" s="8" t="s">
         <v>427</v>
       </c>
-      <c r="E49" s="9" t="inlineStr">
+      <c r="E50" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Carl_Schmitt" title=" Wikipedia"&gt;Carl SCHMITT&lt;/a&gt;  était un philosophe &amp; théologien politique allemand  controversé, connu pour ses critiques radicales du libéralisme parlementaire et sa proximité avec le nazisme. Il adhère au parti nazi en 1933, justifie en 1934 les assassinats de la Nuit des longs couteaux dans « Le Führer protège le droit » et tient des propos antisémites, avant d’être écarté par la SS en 1936. &lt;/p&gt; &lt;p&gt;Il rejette le libéralisme pour son neutralisme économique et juridique, prônant un  &lt;a href="https://www.liberation.fr/debats/2016/08/03/carl-schmitt-le-penseur-de-l-ennemi_1470100/"  title="Détournement de pensées (4/5) Carl Schmitt, le penseur de l’ennemi  par Libération"&gt;État fort &lt;/a&gt; capable de trancher dans l'état d'exception, où la norme juridique s'efface. Sa vision du politique comme conflit existentiel  &lt;a href="https://www.youtube.com/watch?v=vopSqS73tLI" title="Ami - Ennemi, le fondement du politique (Carl Schmitt)  par Ego Non"&gt;(ami/ennemi) &lt;/a&gt; influence la géopolitique et la critique de la mondialisation, voyant dans le nomos (ordre spatial) la base des relations internationales. Catholique puis critique du catholicisme politique, il admire Hobbes et le Léviathan comme modèle d'autorité absolue. &lt;/p&gt; &lt;p&gt; Ses oeuvres principales : "Théologie politique" paru en 1922 : définit le souverain comme "celui qui décide sur l'exception", liant décision politique et théologie, &lt;a href="https://www.youtube.com/watch?v=U8u4SUZNF9I" title="La politique, c'est la guerre (Carl Schmitt)and Mind  par Politikon"&gt;La Notion du politique" &lt;/a&gt; paru en 1932 : pose que le politique repose sur la distinction ami/ennemi, critiquant le parlementarisme comme dissolvant cette intensité et "Théorie de la Constitution" en 1928 et "Théorie du partisan" en 1963 : analyses du pouvoir constituant, de la dictature légitime et de la guerre irrégulière. &lt;/p&gt; &lt;p&gt; Admiré pour sa profondeur analytique par des intellectuels comme Chantal Mouffe ou Giorgio Agamben, mais rejeté comme idéologue nazi par d'autres, son œuvre reste étudiée pour comprendre les limites de la démocratie libérale. &lt;/p&gt;   &lt;audio controls title="Carl Schmitt : comment éradiquer nos ennemis ? par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2015/11/s48/NET_FC_320d8f8e-e840-4e7b-a1c5-c5b36f7e22c6.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
 </t>
         </is>
       </c>
-      <c r="F49" s="7" t="s">
+      <c r="F50" s="7" t="s">
         <v>429</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="G50" s="9" t="s">
         <v>430</v>
       </c>
-      <c r="H49" s="9" t="s">
+      <c r="H50" s="9" t="s">
         <v>431</v>
-      </c>
-      <c r="I49" s="7"/>
-      <c r="J49" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="K49" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="L49" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="N49" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7" t="n">
-        <v>1888</v>
-      </c>
-      <c r="B50" s="7" t="n">
-        <v>1973</v>
-      </c>
-      <c r="C50" s="7" t="s">
-        <v>433</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>434</v>
-      </c>
-      <c r="E50" s="12" t="s">
-        <v>435</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>436</v>
-      </c>
-      <c r="G50" s="9" t="s">
-        <v>437</v>
-      </c>
-      <c r="H50" s="12" t="s">
-        <v>438</v>
       </c>
       <c r="I50" s="7"/>
       <c r="J50" s="2" t="s">
-        <v>439</v>
+        <v>344</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>423</v>
+        <v>378</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="M50" s="0" t="s">
-        <v>186</v>
+        <v>432</v>
       </c>
       <c r="N50" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="n">
-        <v>1889</v>
-      </c>
-      <c r="B51" s="7" t="s">
-        <v>441</v>
+        <v>1888</v>
+      </c>
+      <c r="B51" s="7" t="n">
+        <v>1973</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>442</v>
+        <v>433</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>443</v>
-      </c>
-      <c r="E51" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Martin_Heidegger"  title=" Wikipedia"&gt;Martin HEIDEGGER&lt;/a&gt; (1889-1976) est un philosophe allemand, l’un des plus influents et des plus controversés du XXe siècle. Né à Messkirch, dans le pays de Bade, il se destine d’abord à la prêtrise, puis devient à Fribourg l’assistant de &lt;a href="https://fr.wikipedia.org/wiki/Edmund_Husserl" title=" Wikipedia"&gt;Husserl&lt;/a&gt;, dont il renouvelle &lt;a href="https://www.youtube.com/watch?v=t96HiEpxIB0&amp;ab_channel=MichelOnfray-Topic"   title="La phénoménologie par Michel Onfray "&gt;la phénoménologie&lt;/a&gt;. Professeur à Marbourg, il publie en 1927 son œuvre majeure, &lt;a href="https://www.youtube.com/watch?v=A7ke29MEYpY&amp;ab_channel=LePr%C3%A9cepteur"  title="Etre et Temps de Heidegger par le Precepteur "&gt;&lt;em&gt;Être et Temps&lt;/em&gt;&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Heidegger reproche à la philosophie occidentale, depuis Platon, d’avoir « oublié l’être » : elle a étudié les étants, les choses qui sont, sans se demander ce que veut dire « être ». Pour poser cette question, il part de l’existence humaine, qu’il nomme &lt;em&gt;Dasein&lt;/em&gt;, « être-là ». L’homme n’est pas un sujet face à des objets : il est d’emblée « au monde », pris dans des tâches et des outils qu’il utilise sans y penser, comme le marteau. Le plus souvent, il vit sur le mode impersonnel du « on ». L’angoisse le confronte à sa finitude : l’homme est un « être-pour-la-mort », et c’est en assumant sa mort qu’il peut exister de façon authentique. Dans ses œuvres plus tardives, Heidegger médite sur l’histoire de l’être, sur la poésie de Hölderlin et sur le langage, « maison de l’être ». Il voit dans la technique moderne non un simple ensemble d’outils, mais une manière de dévoiler le monde comme un stock de ressources à exploiter.&lt;/p&gt; &lt;p&gt;Recteur de l’université de Fribourg en 1933, membre du parti nazi jusqu’en 1945, il est interdit d’enseignement après la guerre ; ses &lt;em&gt;Cahiers noirs&lt;/em&gt;, publiés depuis 2014, révèlent un antisémitisme qui relance le débat. Son influence sur Sartre, Arendt, Levinas et Derrida est pourtant considérable.&lt;/p&gt;  &lt;audio controls title="L'antisémitisme dans la pensée de Heidegger par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2014/10/s40/RF_D01332FD-FB86-4C0A-BF38-A61BECB1EA38_GENE_2.MP3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
-        </is>
+        <v>434</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>435</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>445</v>
+        <v>436</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>446</v>
-      </c>
-      <c r="H51" s="9" t="s">
-        <v>447</v>
+        <v>437</v>
+      </c>
+      <c r="H51" s="12" t="s">
+        <v>438</v>
       </c>
       <c r="I51" s="7"/>
       <c r="J51" s="2" t="s">
-        <v>128</v>
+        <v>439</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>448</v>
+        <v>423</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>449</v>
+        <v>440</v>
+      </c>
+      <c r="M51" s="0" t="s">
+        <v>186</v>
       </c>
       <c r="N51" s="0" t="s">
         <v>27</v>
-      </c>
-      <c r="O51" s="0" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="n">
         <v>1889</v>
       </c>
-      <c r="B52" s="7" t="n">
-        <v>1964</v>
+      <c r="B52" s="7" t="s">
+        <v>441</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>450</v>
+        <v>442</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>451</v>
-      </c>
-      <c r="E52" s="20" t="s">
-        <v>452</v>
+        <v>443</v>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Martin_Heidegger"  title=" Wikipedia"&gt;Martin HEIDEGGER&lt;/a&gt; (1889-1976) est un philosophe allemand, l’un des plus influents et des plus controversés du XXe siècle. Né à Messkirch, dans le pays de Bade, il se destine d’abord à la prêtrise, puis devient à Fribourg l’assistant de &lt;a href="https://fr.wikipedia.org/wiki/Edmund_Husserl" title=" Wikipedia"&gt;Husserl&lt;/a&gt;, dont il renouvelle &lt;a href="https://www.youtube.com/watch?v=t96HiEpxIB0&amp;ab_channel=MichelOnfray-Topic"   title="La phénoménologie par Michel Onfray "&gt;la phénoménologie&lt;/a&gt;. Professeur à Marbourg, il publie en 1927 son œuvre majeure, &lt;a href="https://www.youtube.com/watch?v=A7ke29MEYpY&amp;ab_channel=LePr%C3%A9cepteur"  title="Etre et Temps de Heidegger par le Precepteur "&gt;&lt;em&gt;Être et Temps&lt;/em&gt;&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Heidegger reproche à la philosophie occidentale, depuis Platon, d’avoir « oublié l’être » : elle a étudié les étants, les choses qui sont, sans se demander ce que veut dire « être ». Pour poser cette question, il part de l’existence humaine, qu’il nomme &lt;em&gt;Dasein&lt;/em&gt;, « être-là ». L’homme n’est pas un sujet face à des objets : il est d’emblée « au monde », pris dans des tâches et des outils qu’il utilise sans y penser, comme le marteau. Le plus souvent, il vit sur le mode impersonnel du « on ». L’angoisse le confronte à sa finitude : l’homme est un « être-pour-la-mort », et c’est en assumant sa mort qu’il peut exister de façon authentique. Dans ses œuvres plus tardives, Heidegger médite sur l’histoire de l’être, sur la poésie de Hölderlin et sur le langage, « maison de l’être ». Il voit dans la technique moderne non un simple ensemble d’outils, mais une manière de dévoiler le monde comme un stock de ressources à exploiter.&lt;/p&gt; &lt;p&gt;Recteur de l’université de Fribourg en 1933, membre du parti nazi jusqu’en 1945, il est interdit d’enseignement après la guerre ; ses &lt;em&gt;Cahiers noirs&lt;/em&gt;, publiés depuis 2014, révèlent un antisémitisme qui relance le débat. Son influence sur Sartre, Arendt, Levinas et Derrida est pourtant considérable.&lt;/p&gt;  &lt;audio controls title="L'antisémitisme dans la pensée de Heidegger par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2014/10/s40/RF_D01332FD-FB86-4C0A-BF38-A61BECB1EA38_GENE_2.MP3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F52" s="7" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>454</v>
-      </c>
-      <c r="H52" s="12" t="s">
-        <v>455</v>
+        <v>446</v>
+      </c>
+      <c r="H52" s="9" t="s">
+        <v>447</v>
       </c>
       <c r="I52" s="7"/>
       <c r="J52" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="L52" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="N52" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="O52" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7" t="n">
+        <v>1889</v>
+      </c>
+      <c r="B53" s="7" t="n">
+        <v>1964</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="E53" s="20" t="s">
+        <v>452</v>
+      </c>
+      <c r="F53" s="7" t="s">
+        <v>453</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>454</v>
+      </c>
+      <c r="H53" s="12" t="s">
+        <v>455</v>
+      </c>
+      <c r="I53" s="7"/>
+      <c r="J53" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="K52" s="2" t="s">
+      <c r="K53" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="L52" s="10" t="s">
+      <c r="L53" s="10" t="s">
         <v>458</v>
       </c>
-      <c r="N52" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="244.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="n">
-        <v>1891</v>
-      </c>
-      <c r="B53" s="7" t="n">
-        <v>1942</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>459</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>460</v>
-      </c>
-      <c r="E53" s="14" t="s">
-        <v>461</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="J53" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="K53" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="L53" s="2" t="s">
-        <v>465</v>
-      </c>
-      <c r="M53" s="0" t="s">
-        <v>346</v>
-      </c>
       <c r="N53" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="O53" s="0" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="207" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="54" customFormat="false" ht="244.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="n">
         <v>1891</v>
       </c>
-      <c r="B54" s="7" t="s">
+      <c r="B54" s="7" t="n">
+        <v>1942</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>460</v>
+      </c>
+      <c r="E54" s="14" t="s">
+        <v>461</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="L54" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="M54" s="0" t="s">
+        <v>346</v>
+      </c>
+      <c r="N54" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="O54" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="207" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="7" t="n">
+        <v>1891</v>
+      </c>
+      <c r="B55" s="7" t="s">
         <v>466</v>
       </c>
-      <c r="C54" s="7" t="s">
+      <c r="C55" s="7" t="s">
         <v>467</v>
       </c>
-      <c r="D54" s="8" t="s">
+      <c r="D55" s="8" t="s">
         <v>468</v>
       </c>
-      <c r="E54" s="9" t="s">
+      <c r="E55" s="9" t="s">
         <v>469</v>
       </c>
-      <c r="F54" s="7" t="s">
+      <c r="F55" s="7" t="s">
         <v>470</v>
       </c>
-      <c r="G54" s="9" t="s">
+      <c r="G55" s="9" t="s">
         <v>471</v>
       </c>
-      <c r="H54" s="9" t="s">
+      <c r="H55" s="9" t="s">
         <v>472</v>
-      </c>
-      <c r="I54" s="7"/>
-      <c r="J54" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="K54" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Positivisme Logique ; Physicalisme ; Phénoménisme ; Réductionnisme</t>
-        </is>
-      </c>
-      <c r="L54" s="2" t="s">
-        <v>475</v>
-      </c>
-      <c r="N54" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="219.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7" t="n">
-        <v>1892</v>
-      </c>
-      <c r="B55" s="7" t="s">
-        <v>476</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>477</v>
-      </c>
-      <c r="D55" s="8" t="s">
-        <v>478</v>
-      </c>
-      <c r="E55" s="9" t="s">
-        <v>479</v>
-      </c>
-      <c r="F55" s="7" t="s">
-        <v>480</v>
-      </c>
-      <c r="G55" s="9" t="s">
-        <v>481</v>
-      </c>
-      <c r="H55" s="9" t="s">
-        <v>482</v>
       </c>
       <c r="I55" s="7"/>
       <c r="J55" s="2" t="s">
-        <v>483</v>
-      </c>
-      <c r="K55" s="2" t="s">
-        <v>484</v>
+        <v>473</v>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivisme Logique ; Physicalisme ; Phénoménisme ; Réductionnisme</t>
+        </is>
       </c>
       <c r="L55" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="M55" s="0" t="s">
-        <v>186</v>
+        <v>475</v>
       </c>
       <c r="N55" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="O55" s="0" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="144.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="56" customFormat="false" ht="219.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="n">
         <v>1892</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>425</v>
+        <v>476</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>486</v>
+        <v>477</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>487</v>
-      </c>
-      <c r="E56" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Helmuth_Plessner"  title=" Wikipedia"&gt;Helmuth PLESSNER&lt;/a&gt; était un philosophe allemand, fondateur clé de &lt;a href="https://publictionnaire.huma-num.fr/notice/plessner-helmuth/"   title="L’apport de l’anthropologie  par Publitionnaire"&gt;l'anthropologie philosophique &lt;/a&gt;  européenne aux côtés de figures comme Max Scheler et Arnold Gehlen. Influencé par le néokantisme, la phénoménologie et la biologie, il développa une vision de l'humain comme être "naturellement artificiel", marqué par une "positionnalité excentrique" qui le distingue des animaux. &lt;/p&gt; &lt;p&gt;  L'homme vit à distance de son corps et de son milieu, possédant simultanément un corps et étant un corps vivant. Cela génère trois lois anthropologiques : la loi de l'"excentricité", celle de la "médiation"  et celle de l'"utopie naturelle". &lt;/p&gt; &lt;p&gt; Il dépasse le dualisme nature/esprit en fondant une herméneutique biologique : la vie s'exprime via les frontières organiques, et l'intentionnalité humaine émerge de cette interaction environnementale, non d'un ego transcendantal. &lt;/p&gt; &lt;p&gt;  Dans "Rire et pleurer", il analyse ces expressions comme réponses excentriques au pathique, révélant la distance ironique de l'humain à soi. Quant à &lt;em&gt;Les Limites de la communauté&lt;/em&gt;, paru en 1924, il rejette le radicalisme communautaire au profit d'une sociologie de la "distance naturelle", préfigurant Habermas. Son œuvre principale, &lt;em&gt;Les Degrés de l’organique et l’homme&lt;/em&gt; (1928), décrit la vie à partir de la manière dont chaque être se rapporte à sa limite : la plante est ouverte à son milieu, l’animal est centré sur lui-même, l’homme seul peut se voir de l’extérieur. D’origine juive, Plessner doit quitter l’Allemagne en 1933 pour les Pays-Bas. Dans &lt;em&gt;La Nation retardée&lt;/em&gt;, il analyse les causes du nazisme. Revenu en 1951, il enseigne la sociologie à Göttingen. &lt;/p&gt; </t>
-        </is>
+        <v>478</v>
+      </c>
+      <c r="E56" s="9" t="s">
+        <v>479</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>489</v>
+        <v>480</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
       <c r="I56" s="7"/>
       <c r="J56" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="M56" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="N56" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="O56" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="144.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="7" t="n">
+        <v>1892</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>425</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D57" s="8" t="s">
+        <v>487</v>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Helmuth_Plessner"  title=" Wikipedia"&gt;Helmuth PLESSNER&lt;/a&gt; était un philosophe allemand, fondateur clé de &lt;a href="https://publictionnaire.huma-num.fr/notice/plessner-helmuth/"   title="L’apport de l’anthropologie  par Publitionnaire"&gt;l'anthropologie philosophique &lt;/a&gt;  européenne aux côtés de figures comme Max Scheler et Arnold Gehlen. Influencé par le néokantisme, la phénoménologie et la biologie, il développa une vision de l'humain comme être "naturellement artificiel", marqué par une "positionnalité excentrique" qui le distingue des animaux. &lt;/p&gt; &lt;p&gt;  L'homme vit à distance de son corps et de son milieu, possédant simultanément un corps et étant un corps vivant. Cela génère trois lois anthropologiques : la loi de l'"excentricité", celle de la "médiation"  et celle de l'"utopie naturelle". &lt;/p&gt; &lt;p&gt; Il dépasse le dualisme nature/esprit en fondant une herméneutique biologique : la vie s'exprime via les frontières organiques, et l'intentionnalité humaine émerge de cette interaction environnementale, non d'un ego transcendantal. &lt;/p&gt; &lt;p&gt;  Dans "Rire et pleurer", il analyse ces expressions comme réponses excentriques au pathique, révélant la distance ironique de l'humain à soi. Quant à &lt;em&gt;Les Limites de la communauté&lt;/em&gt;, paru en 1924, il rejette le radicalisme communautaire au profit d'une sociologie de la "distance naturelle", préfigurant Habermas. Son œuvre principale, &lt;em&gt;Les Degrés de l’organique et l’homme&lt;/em&gt; (1928), décrit la vie à partir de la manière dont chaque être se rapporte à sa limite : la plante est ouverte à son milieu, l’animal est centré sur lui-même, l’homme seul peut se voir de l’extérieur. D’origine juive, Plessner doit quitter l’Allemagne en 1933 pour les Pays-Bas. Dans &lt;em&gt;La Nation retardée&lt;/em&gt;, il analyse les causes du nazisme. Revenu en 1951, il enseigne la sociologie à Göttingen. &lt;/p&gt; </t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>490</v>
+      </c>
+      <c r="H57" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="I57" s="7"/>
+      <c r="J57" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="K56" s="2" t="s">
+      <c r="K57" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="L56" s="2" t="s">
+      <c r="L57" s="2" t="s">
         <v>492</v>
       </c>
-      <c r="N56" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="7" t="n">
+      <c r="N57" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="7" t="n">
         <v>1893</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="B58" s="7" t="s">
         <v>493</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="C58" s="7" t="s">
         <v>494</v>
       </c>
-      <c r="D57" s="8" t="s">
+      <c r="D58" s="8" t="s">
         <v>495</v>
       </c>
-      <c r="E57" s="13" t="inlineStr">
+      <c r="E58" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Mannheim" title=" Wikipedia"&gt;Karl MANNHEIM&lt;/a&gt;  était un philosophe allemand d'origine hongroise classé dans la sociologie de la connaissance et dans la sociologie compréhensive, à la frontière de la philosophie et des sciences sociales. Il ne sépare pas vraiment les deux domaines, car il cherche à montrer que la pensée dépend toujours d’un contexte social et historique. &lt;/p&gt; &lt;p&gt; Sa contribution la plus célèbre est  &lt;a href="https://www.youtube.com/watch?v=bBVJF4k_4-s"  title="transsiional sociologist par Socio exploration"&gt;Idéologie et utopie.&lt;/a&gt;  Dans ce livre, il explique que nos idées ne sont pas produites dans le vide: elles sont liées à notre position dans la société, à notre époque et à nos groupes d’appartenance. &lt;/p&gt; &lt;p&gt; Il  distingue notamment plusieurs formes d’idéologie et d’utopie. L’idéologie tend à justifier l’ordre existant, tandis que l’utopie ouvre la pensée vers une transformation du monde social. &lt;/p&gt; &lt;p&gt; Il défend aussi une forme de relationnisme: il ne dit pas que toute vérité est fausse, mais que les points de vue sont toujours partiels et situés. Cela lui permet de critiquer le relativisme absolu tout en reconnaissant que la connaissance humaine est historiquement conditionnée. Il  est un penseur des rapports entre   &lt;a href="https://www.youtube.com/watch?v=6R-Fre-UwgQ"  title="Sociological theory of culture  par Mannheuim"&gt;pensée, société et histoire.&lt;/a&gt;  On peut donc le ranger parmi les grands théoriciens de l’idéologie, de l’utopie et de la sociologie de la connaissance.   &lt;/p&gt; Né à Budapest en 1893, membre du cercle de Georg Lukács, il enseigne à Heidelberg puis à Francfort, avant de devoir fuir le nazisme en 1933 pour la London School of Economics. Dans un essai célèbre, il fait de la « génération » une notion sociologique : ceux qui ont vécu les mêmes événements à un âge semblable partagent une manière de voir le monde.
 </t>
         </is>
       </c>
-      <c r="F57" s="7" t="s">
+      <c r="F58" s="7" t="s">
         <v>497</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="G58" s="9" t="s">
         <v>498</v>
       </c>
-      <c r="H57" s="9" t="s">
+      <c r="H58" s="9" t="s">
         <v>499</v>
-      </c>
-      <c r="I57" s="7"/>
-      <c r="J57" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="K57" s="2" t="s">
-        <v>500</v>
-      </c>
-      <c r="L57" s="17" t="s">
-        <v>501</v>
-      </c>
-      <c r="M57" s="0" t="s">
-        <v>186</v>
-      </c>
-      <c r="N57" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7" t="n">
-        <v>1895</v>
-      </c>
-      <c r="B58" s="7" t="s">
-        <v>502</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>503</v>
-      </c>
-      <c r="D58" s="8" t="s">
-        <v>504</v>
-      </c>
-      <c r="E58" s="9" t="s">
-        <v>505</v>
-      </c>
-      <c r="F58" s="7" t="s">
-        <v>506</v>
-      </c>
-      <c r="G58" s="9" t="s">
-        <v>507</v>
-      </c>
-      <c r="H58" s="9" t="s">
-        <v>508</v>
       </c>
       <c r="I58" s="7"/>
       <c r="J58" s="2" t="s">
-        <v>147</v>
+        <v>44</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>509</v>
-      </c>
-      <c r="L58" s="2" t="s">
-        <v>510</v>
+        <v>500</v>
+      </c>
+      <c r="L58" s="17" t="s">
+        <v>501</v>
       </c>
       <c r="M58" s="0" t="s">
         <v>186</v>
@@ -4994,40 +5014,40 @@
         <v>27</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="215.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="n">
-        <v>1897</v>
+        <v>1895</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>511</v>
+        <v>502</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>512</v>
+        <v>503</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>513</v>
-      </c>
-      <c r="E59" s="12" t="s">
-        <v>514</v>
+        <v>504</v>
+      </c>
+      <c r="E59" s="9" t="s">
+        <v>505</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>516</v>
+        <v>507</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>517</v>
+        <v>508</v>
       </c>
       <c r="I59" s="7"/>
       <c r="J59" s="2" t="s">
-        <v>518</v>
+        <v>147</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>519</v>
+        <v>509</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>520</v>
+        <v>510</v>
       </c>
       <c r="M59" s="0" t="s">
         <v>186</v>
@@ -5036,171 +5056,171 @@
         <v>27</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="316.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="215.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="n">
+        <v>1897</v>
+      </c>
+      <c r="B60" s="7" t="s">
+        <v>511</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>512</v>
+      </c>
+      <c r="D60" s="8" t="s">
+        <v>513</v>
+      </c>
+      <c r="E60" s="12" t="s">
+        <v>514</v>
+      </c>
+      <c r="F60" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>516</v>
+      </c>
+      <c r="H60" s="9" t="s">
+        <v>517</v>
+      </c>
+      <c r="I60" s="7"/>
+      <c r="J60" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="L60" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="M60" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="N60" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="316.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="7" t="n">
         <v>1899</v>
       </c>
-      <c r="B60" s="7" t="n">
+      <c r="B61" s="7" t="n">
         <v>1973</v>
       </c>
-      <c r="C60" s="7" t="s">
+      <c r="C61" s="7" t="s">
         <v>521</v>
       </c>
-      <c r="D60" s="8" t="inlineStr">
+      <c r="D61" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Leo STRAUSS</t>
         </is>
       </c>
-      <c r="E60" s="14" t="inlineStr">
+      <c r="E61" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Leo_Strauss" title=" Wikipedia"&gt;Leo STRAUSS&lt;/a&gt; était un philosophe politique germano-américain, connu pour sa critique profonde de la modernité et pour sa relecture des grands textes de la philosophie politique classique. Sa pensée a eu une influence durable, notamment aux États‑Unis, où elle a marqué des générations d’étudiants en théorie politique. &lt;/p&gt; &lt;p&gt; Au cœur de sa philosophie se trouve l’idée que la modernité a rompu avec le droit naturel classique, c’est‑à‑dire avec la recherche de ce qui est juste par nature et non simplement selon l’histoire ou les sciences sociales. Il voit dans le positivisme, le relativisme et l’historicisme modernes une source de décadence intellectuelle, car ils empêchent de poser les questions normatives fondamentales : qu’est‑ce qu’une vie bonne, qu’est‑ce qu’un régime politique juste. Pour lui, la  &lt;a href="https://www.persee.fr/doc/rfsp_0035-2950_1985_num_35_4_394205" title="philosophie et zscience politique par persée"&gt;philosophie politique authentique &lt;/a&gt; doit réactiver ces questions et affronter directement les notions de meilleur régime et d’ordre politique juste, plutôt que de se contenter de descriptions neutres. &lt;/p&gt; &lt;p&gt; Cette critique le conduit à renouer avec les auteurs de l’Antiquité, en particulier Platon, Aristote et les philosophes médiévaux juifs et arabes, qu’il lit souvent contre les interprétations modernes. Il insiste sur la dimension éducative de la philosophie : il parle de « liberal education » comme d’une libération de la vulgarité, entendue comme manque d’expérience des belles choses. La fréquentation des grands textes est, pour lui, une école de modestie et d’audace intellectuelle, parce qu’elle oblige à mesurer nos catégories modernes à celles d’auteurs qui pensaient autrement le politique et le juste. &lt;/p&gt; &lt;p&gt; Célèbre pour sa thèse sur l’« écriture ésotérique » : selon lui, nombre de philosophes du passé ont écrit de manière volontairement oblique pour se protéger de la censure ou de la persécution, réservant un sens plus profond aux lecteurs attentifs. Cela l’amène à distinguer entre le message « exotérique » (apparent, destiné au grand public) et le message « ésotérique » (plus exigeant, adressé à une minorité philosophique). Cette hypothèse sur la lecture des classiques s’articule à sa conception du   &lt;a href="https://www.youtube.com/watch?v=9Vhsveytymk" title="nihilisme et politique leo strauss par bildung et culture"&gt;mode de vie philosophique, &lt;/a&gt; toujours exposé au risque de la tyrannie et de l’incompréhension. Ainsi, sa philosophie politique est à la fois une critique de la modernité et une tentative de redécouvrir la place de la philosophie au cœur du politique contemporain. &lt;/p&gt; 
  &lt;audio controls title="la pensée de leon strauss par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/13397-05.04.2008-ITEMA_20118283-2008C3397E0019-ITE_00016207_RSCE-21.mp3" type="audio/mpeg" align="center"&gt;&lt;/audio&gt;  
 </t>
         </is>
       </c>
-      <c r="F60" s="7" t="s">
+      <c r="F61" s="7" t="s">
         <v>524</v>
       </c>
-      <c r="G60" s="9" t="s">
+      <c r="G61" s="9" t="s">
         <v>525</v>
       </c>
-      <c r="H60" s="12" t="s">
+      <c r="H61" s="12" t="s">
         <v>526</v>
-      </c>
-      <c r="I60" s="7"/>
-      <c r="J60" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="K60" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="L60" s="2" t="s">
-        <v>528</v>
-      </c>
-      <c r="M60" s="0" t="s">
-        <v>186</v>
-      </c>
-      <c r="N60" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="231.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="7" t="n">
-        <v>1900</v>
-      </c>
-      <c r="B61" s="7" t="s">
-        <v>529</v>
-      </c>
-      <c r="C61" s="7" t="s">
-        <v>530</v>
-      </c>
-      <c r="D61" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="E61" s="13" t="s">
-        <v>532</v>
-      </c>
-      <c r="F61" s="7" t="s">
-        <v>533</v>
-      </c>
-      <c r="G61" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Gadamer on Language &amp; Understanding (1970)" par Philosophy Overdose</t>
-        </is>
-      </c>
-      <c r="H61" s="9" t="s">
-        <v>535</v>
       </c>
       <c r="I61" s="7"/>
       <c r="J61" s="2" t="s">
-        <v>210</v>
+        <v>344</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="L61" s="17" t="s">
-        <v>536</v>
+        <v>527</v>
+      </c>
+      <c r="L61" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="M61" s="0" t="s">
+        <v>186</v>
       </c>
       <c r="N61" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="231.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="n">
-        <v>1903</v>
+        <v>1900</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>539</v>
-      </c>
-      <c r="E62" s="9" t="s">
-        <v>540</v>
+        <v>531</v>
+      </c>
+      <c r="E62" s="13" t="s">
+        <v>532</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>541</v>
-      </c>
-      <c r="G62" s="9" t="s">
-        <v>542</v>
+        <v>533</v>
+      </c>
+      <c r="G62" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Gadamer on Language &amp; Understanding (1970)" par Philosophy Overdose</t>
+        </is>
       </c>
       <c r="H62" s="9" t="s">
-        <v>543</v>
+        <v>535</v>
       </c>
       <c r="I62" s="7"/>
       <c r="J62" s="2" t="s">
-        <v>544</v>
+        <v>210</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>509</v>
-      </c>
-      <c r="L62" s="2" t="s">
-        <v>545</v>
-      </c>
-      <c r="M62" s="0" t="s">
-        <v>186</v>
+        <v>157</v>
+      </c>
+      <c r="L62" s="17" t="s">
+        <v>536</v>
       </c>
       <c r="N62" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="176.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="n">
         <v>1903</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>546</v>
+        <v>537</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>547</v>
+        <v>538</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>548</v>
-      </c>
-      <c r="E63" s="12" t="s">
-        <v>549</v>
+        <v>539</v>
+      </c>
+      <c r="E63" s="9" t="s">
+        <v>540</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>550</v>
+        <v>541</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>551</v>
+        <v>542</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>552</v>
+        <v>543</v>
       </c>
       <c r="I63" s="7"/>
       <c r="J63" s="2" t="s">
-        <v>362</v>
+        <v>544</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>553</v>
+        <v>509</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>554</v>
+        <v>545</v>
       </c>
       <c r="M63" s="0" t="s">
         <v>186</v>
@@ -5209,40 +5229,43 @@
         <v>27</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="195.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="176.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="n">
-        <v>1904</v>
+        <v>1903</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>441</v>
+        <v>546</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>556</v>
-      </c>
-      <c r="E64" s="13" t="s">
-        <v>557</v>
+        <v>548</v>
+      </c>
+      <c r="E64" s="12" t="s">
+        <v>549</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>558</v>
+        <v>550</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>559</v>
+        <v>551</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>560</v>
+        <v>552</v>
       </c>
       <c r="I64" s="7"/>
       <c r="J64" s="2" t="s">
-        <v>44</v>
+        <v>362</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="L64" s="17" t="s">
-        <v>561</v>
+        <v>553</v>
+      </c>
+      <c r="L64" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="M64" s="0" t="s">
+        <v>186</v>
       </c>
       <c r="N64" s="0" t="s">
         <v>27</v>
@@ -5250,238 +5273,216 @@
     </row>
     <row r="65" customFormat="false" ht="195.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="n">
-        <v>1922</v>
-      </c>
-      <c r="B65" s="7" t="n">
-        <v>2017</v>
+        <v>1904</v>
+      </c>
+      <c r="B65" s="7" t="s">
+        <v>441</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>562</v>
+        <v>555</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>563</v>
-      </c>
-      <c r="E65" s="21" t="s">
-        <v>564</v>
+        <v>556</v>
+      </c>
+      <c r="E65" s="13" t="s">
+        <v>557</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>565</v>
-      </c>
-      <c r="G65" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Karl-Otto APEL par Daniel Ronnedal</t>
-        </is>
-      </c>
-      <c r="H65" s="12" t="s">
-        <v>567</v>
+        <v>558</v>
+      </c>
+      <c r="G65" s="9" t="s">
+        <v>559</v>
+      </c>
+      <c r="H65" s="9" t="s">
+        <v>560</v>
       </c>
       <c r="I65" s="7"/>
       <c r="J65" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="L65" s="17" t="s">
+        <v>561</v>
+      </c>
+      <c r="N65" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="195.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="7" t="n">
+        <v>1922</v>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>562</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>563</v>
+      </c>
+      <c r="E66" s="21" t="s">
+        <v>564</v>
+      </c>
+      <c r="F66" s="7" t="s">
+        <v>565</v>
+      </c>
+      <c r="G66" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Karl-Otto APEL par Daniel Ronnedal</t>
+        </is>
+      </c>
+      <c r="H66" s="12" t="s">
+        <v>567</v>
+      </c>
+      <c r="I66" s="7"/>
+      <c r="J66" s="2" t="s">
         <v>568</v>
       </c>
-      <c r="K65" s="2" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Théorie Critique ; Déontologisme</t>
         </is>
       </c>
-      <c r="L65" s="17" t="s">
+      <c r="L66" s="17" t="s">
         <v>569</v>
       </c>
-      <c r="N65" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="202.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="1" t="n">
+      <c r="N66" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="202.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="n">
         <v>1929</v>
       </c>
-      <c r="B66" s="1" t="n">
+      <c r="B67" s="1" t="n">
         <v>2026</v>
       </c>
-      <c r="C66" s="1" t="s">
+      <c r="C67" s="1" t="s">
         <v>570</v>
       </c>
-      <c r="D66" s="22" t="s">
+      <c r="D67" s="22" t="s">
         <v>571</v>
       </c>
-      <c r="E66" s="19" t="inlineStr">
+      <c r="E67" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/J%C3%BCrgen_Habermas"  title=" Wikipedia"&gt;Jürgen HABERMAS&lt;/a&gt; est un philosophe allemand connu pour avoir écrit  "Théorie de l'agir communicationnel" où il développe la théorie de l'agir communicationnel, qui met l'accent sur le rôle de la communication et du langage dans la construction de la société.  &lt;/p&gt; &lt;p&gt; Dans son livre  &lt;a href="https://www.persee.fr/doc/polix_0295-2319_1989_num_2_5_2021" title="Extrait de l'espace public par Persée.fr"&gt;"L'espace public"&lt;/a&gt;, ( le premier à avoir aborder le sujet fut KANT) il considère que c'est un lieu crucial de débat et de délibération, c'est l'agir communicationnel où les citoyens peuvent  &lt;a href="https://www.youtube.com/watch?v=PnY0Jg8NH1g"   title="t l'espace public par Mélannie Moreau"&gt;s'exprimer &lt;/a&gt; et discuter de manière ouverte et équitable des questions politiques et sociales qui les concernent. Ils ont une capacité innée à communiquer et à agir ensemble de manière coopérative leurs permettant de réguler les relations entre les individus et de créer des normes et des valeurs partagées. &lt;/p&gt; &lt;p&gt;  Il considère que l'expansion des systèmes bureaucratiques et économiques ont réduit les possibilités  &lt;a href="https://www.youtube.com/watch?v=R1K46oK3xTU&amp;ab_channel=Then%26Now"  title="La transformation structurelle de la sphère publique par Then &amp; Now"&gt;d'interaction sociale &lt;/a&gt; et ont aliéné les individus de leurs propres intérêts et valeurs et il pense que la participation active des citoyens à la vie politique est essentielle pour garantir une société juste et équitable. &lt;/p&gt; &lt;p&gt;  Il  théorise la démocratie délibérative, où la légitimité naît du débat rationnel plutôt que du marché ou de la tradition. Ses  &lt;a href="https://www.youtube.com/watch?v=OzAWFDkaCcE"   title="Il s’est trompé depuis 40 ans par Tocsin et 2 autres"&gt;interventions sur l'Europe&lt;/a&gt;, le droit et la religion ("post-sécularisme") influencent la philosophie politique globale, reliant émancipation individuelle et solidarité collective.   &lt;/p&gt;  &lt;audio controls title="Habernas, le dernier philosophe ? par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2015/09/s38/NET_FC_c7667f83-aa22-41cb-ba4e-d7567cc16be1.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
-      <c r="F66" s="23" t="s">
+      <c r="F67" s="23" t="s">
         <v>573</v>
       </c>
-      <c r="G66" s="10" t="s">
+      <c r="G67" s="10" t="s">
         <v>574</v>
       </c>
-      <c r="H66" s="10" t="s">
+      <c r="H67" s="10" t="s">
         <v>575</v>
       </c>
-      <c r="I66" s="10"/>
-      <c r="J66" s="2" t="s">
+      <c r="I67" s="10"/>
+      <c r="J67" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="K66" s="2" t="inlineStr">
+      <c r="K67" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Théorie Critique ; Déontologisme</t>
         </is>
       </c>
-      <c r="L66" s="2" t="s">
+      <c r="L67" s="2" t="s">
         <v>576</v>
       </c>
-      <c r="N66" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="O66" s="0" t="n">
+      <c r="N67" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="O67" s="0" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="183.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="7" t="n">
+    <row r="68" customFormat="false" ht="183.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="7" t="n">
         <v>1941</v>
       </c>
-      <c r="B67" s="7" t="n">
+      <c r="B68" s="7" t="n">
         <v>1993</v>
       </c>
-      <c r="C67" s="7" t="s">
+      <c r="C68" s="7" t="s">
         <v>577</v>
       </c>
-      <c r="D67" s="8" t="s">
+      <c r="D68" s="8" t="s">
         <v>578</v>
       </c>
-      <c r="E67" s="14" t="s">
+      <c r="E68" s="14" t="s">
         <v>579</v>
       </c>
-      <c r="F67" s="7" t="s">
+      <c r="F68" s="7" t="s">
         <v>580</v>
       </c>
-      <c r="G67" s="9" t="s">
+      <c r="G68" s="9" t="s">
         <v>581</v>
       </c>
-      <c r="H67" s="9" t="s">
+      <c r="H68" s="9" t="s">
         <v>582</v>
       </c>
-      <c r="I67" s="9"/>
-      <c r="J67" s="2" t="s">
+      <c r="I68" s="9"/>
+      <c r="J68" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="K67" s="2" t="s">
+      <c r="K68" s="2" t="s">
         <v>583</v>
       </c>
-      <c r="L67" s="2" t="s">
+      <c r="L68" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="N67" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="267.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0">
+      <c r="N68" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="267.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="0">
         <v>1883</v>
       </c>
-      <c r="B68" s="0" t="inlineStr">
+      <c r="B69" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">1969</t>
         </is>
       </c>
-      <c r="C68" s="0" t="inlineStr">
+      <c r="C69" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">1883 – 1969</t>
         </is>
       </c>
-      <c r="D68" s="0" t="inlineStr">
+      <c r="D69" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Karl JASPERS</t>
         </is>
       </c>
-      <c r="E68" s="0" t="inlineStr">
+      <c r="E69" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Jaspers" title=" Wikipedia"&gt;Karl JASPERS&lt;/a&gt; est un psychiatre et philosophe allemand, l’un des fondateurs de la philosophie de l’existence. Né à Oldenbourg, il étudie le droit puis la médecine et travaille à la clinique psychiatrique de Heidelberg. Son &lt;em&gt;Psychopathologie générale&lt;/em&gt; (1913) renouvelle la psychiatrie en distinguant ce que l’on peut « expliquer » par des causes et ce que l’on doit « comprendre » de l’intérieur, dans l’expérience du malade. Il se tourne ensuite vers la philosophie, qu’il enseigne à Heidelberg.&lt;/p&gt; &lt;p&gt;Dans sa &lt;em&gt;Philosophie&lt;/em&gt; (1932), il distingue l’existence de tout ce que la science peut connaître : ce que je suis vraiment ne se laisse pas réduire à un objet. C’est dans les « situations limites », la mort, la souffrance, la lutte, la culpabilité, que l’homme découvre qu’il ne peut rien maîtriser et s’ouvre à la « transcendance ». La communication authentique avec autrui, une « lutte aimante », est le lieu où chacun devient lui-même. Il forge aussi la notion d’« âge axial » pour désigner le moment, autour du VIe siècle avant notre ère, où naissent presque en même temps les grandes sagesses de la Chine, de l’Inde, de la Perse, d’Israël et de la Grèce.&lt;/p&gt; &lt;p&gt;Marié à une femme juive, Gertrud, il est privé d’enseignement par les nazis en 1937 et vit sous la menace de la déportation. Après la guerre, il publie &lt;em&gt;La Culpabilité allemande&lt;/em&gt; (1946), où il distingue culpabilité criminelle, politique, morale et métaphysique. Maître et ami d’&lt;a href="https://fr.wikipedia.org/wiki/Hannah_Arendt" title=" Wikipedia"&gt;Hannah Arendt&lt;/a&gt;, il s’installe à Bâle en 1948 et y meurt en 1969.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F68" s="0"/>
-      <c r="G68" s="0"/>
-      <c r="H68" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/jaspers-mini.webp</t>
-        </is>
-      </c>
-      <c r="I68" s="0"/>
-      <c r="J68" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">metaphysique ; politique</t>
-        </is>
-      </c>
-      <c r="K68" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Existentialisme</t>
-        </is>
-      </c>
-      <c r="L68" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">psychiatre et philosophe allemand, penseur de l’existence, des situations limites et de la culpabilité.</t>
-        </is>
-      </c>
-      <c r="N68" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O68">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0">
-        <v>1850</v>
-      </c>
-      <c r="B69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1932</t>
-        </is>
-      </c>
-      <c r="C69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1850 – 1932</t>
-        </is>
-      </c>
-      <c r="D69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Eduard BERNSTEIN</t>
-        </is>
-      </c>
-      <c r="E69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Eduard_Bernstein" title=" Wikipedia"&gt;Eduard BERNSTEIN&lt;/a&gt; est un théoricien et homme politique allemand, le père du « révisionnisme » et l’un des fondateurs de la &lt;a href="https://fr.wikipedia.org/wiki/Social-d%C3%A9mocratie" title=" Wikipedia"&gt;social-démocratie&lt;/a&gt; moderne. Né à Berlin en 1850 dans une famille juive modeste, fils d’un mécanicien de locomotive, il est employé de banque quand il adhère en 1872 au parti social-démocrate. Les lois antisocialistes de Bismarck le contraignent à l’exil : en Suisse, où il dirige le journal du parti, puis à Londres, où il devient l’ami et le collaborateur de Friedrich Engels, qui fait de lui l’un de ses exécuteurs testamentaires.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Les Présupposés du socialisme&lt;/em&gt; (1899), il soumet le marxisme à l’épreuve des faits. Le capitalisme ne s’effondre pas, les classes moyennes ne disparaissent pas, la misère ouvrière ne s’aggrave pas : la théorie de la catastrophe finale est démentie. Le socialisme ne viendra pas d’une révolution, mais de réformes progressives, conquises par les syndicats, les coopératives et le suffrage universel. Il est l’héritier du libéralisme, et doit s’appuyer sur une éthique d’inspiration kantienne plutôt que sur une prétendue nécessité de l’histoire. « Ce qu’on appelle d’ordinaire le but final du socialisme n’est rien pour moi, le mouvement est tout. »&lt;/p&gt; &lt;p&gt;Ce « révisionnisme » déclenche une violente controverse. Karl Kautsky le combat au nom de l’orthodoxie, et &lt;a href="https://fr.wikipedia.org/wiki/Rosa_Luxemburg" title=" Wikipedia"&gt;Rosa Luxemburg&lt;/a&gt; lui répond par &lt;em&gt;Réforme sociale ou révolution ?&lt;/em&gt; (1899). Officiellement condamné par le parti, Bernstein inspire pourtant sa pratique réelle. Député au Reichstag, il vote en 1915 contre les crédits de guerre. Il meurt à Berlin en décembre 1932, peu avant l’arrivée de Hitler au pouvoir. En 1959, le programme de Bad Godesberg, par lequel le SPD renonce au marxisme, consacre ses idées.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F69" s="0"/>
       <c r="G69" s="0"/>
       <c r="H69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/bernstein-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/jaspers-mini.webp</t>
         </is>
       </c>
       <c r="I69" s="0"/>
       <c r="J69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">politique</t>
+          <t xml:space="preserve">metaphysique ; politique</t>
         </is>
       </c>
       <c r="K69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social-démocratie ; Marxisme</t>
+          <t xml:space="preserve">Existentialisme</t>
         </is>
       </c>
       <c r="L69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">théoricien socialiste allemand, père du révisionnisme et de la social-démocratie réformiste.</t>
-        </is>
-      </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">juive</t>
+          <t xml:space="preserve">psychiatre et philosophe allemand, penseur de l’existence, des situations limites et de la culpabilité.</t>
         </is>
       </c>
       <c r="N69" s="0" t="inlineStr">
@@ -5489,52 +5490,60 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
-      <c r="O69"/>
-      <c r="XFC69" s="0"/>
-      <c r="XFD69" s="0"/>
+      <c r="O69">
+        <v>3</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="0">
-        <v>1801</v>
+        <v>1850</v>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1893</t>
+          <t xml:space="preserve">1932</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1801 – 1893</t>
+          <t xml:space="preserve">1850 – 1932</t>
         </is>
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Karl Ludwig MICHELET</t>
+          <t xml:space="preserve">Eduard BERNSTEIN</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Ludwig_Michelet" title=" Wikipedia"&gt;Karl Ludwig MICHELET&lt;/a&gt; est un philosophe allemand, l’un des disciples les plus fidèles de &lt;a href="https://fr.wikipedia.org/wiki/Georg_Wilhelm_Friedrich_Hegel" title=" Wikipedia"&gt;Hegel&lt;/a&gt;. Né à Berlin en 1801 dans une famille de marchands huguenots, d’origine française, il suit les cours de Hegel et enseigne à l’université de Berlin pendant des décennies. Après la mort du maître en 1831, il fait partie du groupe d’élèves qui publient ses œuvres complètes et prépare l’édition de ses &lt;em&gt;Leçons sur l’histoire de la philosophie&lt;/em&gt;.&lt;/p&gt; &lt;p&gt;Spécialiste d’Aristote, il écrit en français un &lt;em&gt;Examen critique du livre d’Aristote intitulé Métaphysique&lt;/em&gt;, couronné en 1836 par l’Académie des sciences morales et politiques en même temps que l’essai de Félix Ravaisson. Quand l’école de Hegel se divise sur la religion et la politique, il reprend la distinction proposée par son élève David Friedrich Strauss entre une « droite », fidèle au christianisme, une « gauche », celle des &lt;a href="https://fr.wikipedia.org/wiki/Jeunes_h%C3%A9g%C3%A9liens" title=" Wikipedia"&gt;Jeunes hégéliens&lt;/a&gt;, et un « centre », auquel il se rattache. Pour lui, Dieu n’est pas une personne séparée du monde : il devient personnel dans l’esprit humain, et l’immortalité n’est pas celle de l’individu, mais celle de l’esprit qui se développe dans l’histoire.&lt;/p&gt; &lt;p&gt;En 1843, il fonde avec ses élèves la Société philosophique de Berlin, qui maintient la tradition hégélienne pendant tout le siècle. Il y défend Hegel contre la critique que lui adresse Schelling, revenu à Berlin en 1841, et publie une histoire de la philosophie allemande de Kant à Hegel, puis une philosophie du droit. Fidèle jusqu’au bout, il intitule l’un de ses derniers livres &lt;em&gt;Hegel, le philosophe universel irréfuté&lt;/em&gt; (1870). Il meurt à Berlin en 1893, à quatre-vingt-onze ans.&lt;/p&gt;</t>
-        </is>
-      </c>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Eduard_Bernstein" title=" Wikipedia"&gt;Eduard BERNSTEIN&lt;/a&gt; est un théoricien et homme politique allemand, le père du « révisionnisme » et l’un des fondateurs de la &lt;a href="https://fr.wikipedia.org/wiki/Social-d%C3%A9mocratie" title=" Wikipedia"&gt;social-démocratie&lt;/a&gt; moderne. Né à Berlin en 1850 dans une famille juive modeste, fils d’un mécanicien de locomotive, il est employé de banque quand il adhère en 1872 au parti social-démocrate. Les lois antisocialistes de Bismarck le contraignent à l’exil : en Suisse, où il dirige le journal du parti, puis à Londres, où il devient l’ami et le collaborateur de Friedrich Engels, qui fait de lui l’un de ses exécuteurs testamentaires.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Les Présupposés du socialisme&lt;/em&gt; (1899), il soumet le marxisme à l’épreuve des faits. Le capitalisme ne s’effondre pas, les classes moyennes ne disparaissent pas, la misère ouvrière ne s’aggrave pas : la théorie de la catastrophe finale est démentie. Le socialisme ne viendra pas d’une révolution, mais de réformes progressives, conquises par les syndicats, les coopératives et le suffrage universel. Il est l’héritier du libéralisme, et doit s’appuyer sur une éthique d’inspiration kantienne plutôt que sur une prétendue nécessité de l’histoire. « Ce qu’on appelle d’ordinaire le but final du socialisme n’est rien pour moi, le mouvement est tout. »&lt;/p&gt; &lt;p&gt;Ce « révisionnisme » déclenche une violente controverse. Karl Kautsky le combat au nom de l’orthodoxie, et &lt;a href="https://fr.wikipedia.org/wiki/Rosa_Luxemburg" title=" Wikipedia"&gt;Rosa Luxemburg&lt;/a&gt; lui répond par &lt;em&gt;Réforme sociale ou révolution ?&lt;/em&gt; (1899). Officiellement condamné par le parti, Bernstein inspire pourtant sa pratique réelle. Député au Reichstag, il vote en 1915 contre les crédits de guerre. Il meurt à Berlin en décembre 1932, peu avant l’arrivée de Hitler au pouvoir. En 1959, le programme de Bad Godesberg, par lequel le SPD renonce au marxisme, consacre ses idées.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F70" s="0"/>
+      <c r="G70" s="0"/>
       <c r="H70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/klmichelet-mini.webp</t>
-        </is>
-      </c>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/bernstein-mini.webp</t>
+        </is>
+      </c>
+      <c r="I70" s="0"/>
       <c r="J70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">metaphysique ; ethique</t>
+          <t xml:space="preserve">politique</t>
         </is>
       </c>
       <c r="K70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Idéalisme allemand</t>
+          <t xml:space="preserve">Social-démocratie ; Marxisme</t>
         </is>
       </c>
       <c r="L70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe allemand, disciple et éditeur de Hegel, chef du « centre » hégélien.</t>
+          <t xml:space="preserve">théoricien socialiste allemand, père du révisionnisme et de la social-démocratie réformiste.</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
         </is>
       </c>
       <c r="N70" s="0" t="inlineStr">
@@ -5543,6 +5552,8 @@
         </is>
       </c>
       <c r="O70"/>
+      <c r="XFC70" s="0"/>
+      <c r="XFD70" s="0"/>
     </row>
     <row r="71" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="0">
@@ -5604,39 +5615,39 @@
     <hyperlink ref="E7" r:id="rId1" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Friedrich_Schleiermacher&quot;   title=&quot; Wikipedia&quot;&gt;Friedrich SCHLEIERMACHER&lt;/a&gt;  était un philosophe prussien,  souvent considéré comme le &quot;père de la théologie libérale moderne&quot;. &lt;a href=&quot;https://www.persee.fr/doc/rhpr_0035-2403_2011_num_91_1_1522&quot;  title=&quot;son apport théorique et pratique par persée&quot;&gt;Sa philosophie &lt;/a&gt; intègre des éléments du romantisme, de l'idéalisme allemand et du piétisme, en centrant l'humain sur une conscience intuitive de l'infini. Il édita Platon, prêcha et influença le protestantisme européen sans séparer foi et culture. &lt;/p&gt; &lt;p&gt;  Il pose le sentiment religieux comme une conscience immédiate de la dépendance absolue envers l'infini (Dieu), distincte du savoir ou de la morale kantienne. L'ego est une individualisation de la  &lt;a href=&quot;https://www.youtube.com/watch?v=gvpaUR1XceM&quot;  style=&quot;color:#88A1E9&quot;  title=&quot;Schleiermacher: The Man Behind Protestant Liberalism par Stephen D Morrison&quot;&gt;raison universelle, &lt;/a&gt; un microcosme où univers et individu s'unissent via la conscience de soi. Il articule individualité et communauté via la communication, honorant la finitude humaine et l'invention de soi contre l'absolutisme idéaliste. &lt;/p&gt; &lt;p&gt; Ses œuvres majeures sont &quot;Discours sur la religion&quot; paru en 1799 et &quot;La foi chrétienne&quot;  paru vers 1821, où il réconcilie rationalité et piété. Il a profondément marqué la théologie protestante moderne en introduisant une approche centrée sur le sentiment religieux et l'expérience personnelle, plutôt que sur les dogmes rigides ou la raison pure. Son idée de &quot;dépendance absolue&quot; envers Dieu et la relativisation des doctrines comme expressions humaines de la piété ont pavé la voie au &lt;a href=&quot;https://www.youtube.com/watch?v=1FveOtAB86s&quot;  title=&quot;L'argument éthique de Schleiermacher en faveur de l'universalisme par Sola Media&quot;&gt;libéralisme théologique. &lt;/a&gt;&lt;/p&gt; &lt;p&gt;  Fondateur de l'herméneutique moderne, art général d'interprétation reliant traduction, littérature et exégèse biblique, il lance l'herméneutique critique de l'Écriture et une théologie pratique pertinente pour la modernité, influençant Ritschl et l'individualisme religieux.&lt;/p&gt; "/>
     <hyperlink ref="E11" r:id="rId2" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Friedrich_Schlegel&quot;   title=&quot; Wikipedia&quot;&gt;Friedrich SCHLEGEL&lt;/a&gt;  était un philosophe,  poète, critique littéraire et théoricien allemand clé du romantisme initial.  Figure centrale du Cercle d'Iéna avec son frère August Wilhelm, Novalis et Schleiermacher, il a théorisé une esthétique romantique centrée sur l'ironie, la fragmentation et &lt;a href=&quot;https://www.persee.fr/doc/litt_0047-4800_2000_num_120_4_1695&quot;  title=&quot;Friedrich Schlegel, entre histoire de la poésie et critique de la philosophie par Persée&quot;&gt; la fusion des genres artistiques.&lt;/a&gt; &lt;/p&gt; &lt;p&gt; Il développe une philosophie non fondationaliste, holistique et historique, opposée au système rigide de Fichte : il propose un &quot;Wechselerweis&quot; où principes et preuves s'entremêlent sans base absolue. L'ironie romantique y est centrale : une conscience infinie de la subjectivité et des limites du savoir, mêlant humour et infinitude. Il valorise l'amour comme union sensuelle-spirituelle et la philologie comme clé de l'histoire des peuples, influençant la grammaire comparative. &lt;/p&gt; &lt;p&gt; Ses oeuvres majeures : -  &lt;a href=&quot;https://www.youtube.com/watch?v=Q8QBiix0hIQ&quot;  title=&quot; &quot;Lucinde&quot; By Friedrich Schlegel par Noterich&quot;&gt; &quot;Lucinde&quot; &lt;/a&gt; paru en 1799 est un  roman scandaleux prônant la liberté individuelle et l'érotisme comme allégorie cosmique. Ensuite : - Athenaeum-Fragmente en 1798, c'est un aphorisme fondateur du romantisme, définissant la poésie comme &quot;art progressif du roman universel&quot;. -  &quot;Philosophie de la vie&quot; et &quot;Philosophie de l'histoire&quot;  en1829, c'est une réflexion tardives sur religion, politique et histoire, influencées par sa catholicisme. &lt;/p&gt; &lt;p&gt; Pionnier du romantisme subjectif, il passe d'un idéalisme athée à un conservatisme catholique, critiquant le parlementarisme et l'idéalisme moderne dans &quot;Signatur des Zeitalters&quot;. Il inspire Hegel (rival), la philologie et la pensée conservatrice allemande, tout en posant les bases d'une esthétique fragmentaire encore vivante. &lt;/p&gt; &#10;&#10;&#10;"/>
     <hyperlink ref="E12" r:id="rId3" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Friedrich_Wilhelm_Joseph_von_Schelling&quot;  title=&quot; Wikipedia&quot;&gt;Friedrich Wilhelm Joseph von SCHELLING&lt;/a&gt; était un philosophe allemand de &lt;a href=&quot;https://www.persee.fr/doc/rscir_0035-2217_1990_num_64_1_3136&quot; title=&quot;L'idéalisme allemand figure accomplie de la modernité  par Persée&quot;&gt;l’idéalisme allemand&lt;/a&gt; contemporain et ami-ennemi de Hegel et Hölderlin. Il est surtout connu pour sa tentative de  &lt;a href=&quot;https://www.youtube.com/watch?v=j5aQ-2kA1Fw&amp;t=1s&quot; style=&quot;color:#88A1E9&quot; title=&quot; F. W. SCHELLING (1775-1854) : Clara, l'amour et le monde des esprits – Une vie, une œuvre par Rien ne veut rien dire&quot;&gt;penser ensemble&lt;/a&gt; la nature, l’esprit et l’absolu, dans une œuvre en plusieurs “phases” qui a profondément marqué la philosophie, le romantisme allemand et la pensée de la liberté. &lt;/p&gt; &lt;p&gt; Sa pensée est souvent décrite comme une “odyssée intellectuelle”, composée de plusieurs grands moments : une  &lt;a href=&quot;https://www.youtube.com/watch?v=YBA9kdr2wV8&quot;  title=&quot; The Forgotten Genius Who Saw Spirit in Nature - Friedrich Schelling par Spiritual Quest&quot;&gt;philosophie de la nature&lt;/a&gt; (Naturphilosophie), une “philosophie de l’identité”, puis une philosophie de la liberté, de la mythologie et de la révélation. Dans ses premiers écrits, influencés par Kant et Fichte, il met au centre le Moi comme principe de la philosophie, puis cherche à dépasser l’opposition sujet/objet en affirmant une unité plus profonde, l’Absolu, dont nature et esprit sont deux faces. Il veut montrer que la nature n’est pas seulement un ensemble de choses inertes, mais une productivité vivante, un “organisme” où agissent des forces opposées qui se composent dans un devenir permanent. La philosophie de l’identité soutient qu’au niveau de l’Absolu, sujet et objet, esprit et nature, idéal et réel sont identiques, ce qui inspirera aussi sa réflexion sur l’art comme lieu privilégié où cette identité se manifeste. &lt;/p&gt; &lt;p&gt; Dans sa période dite “positive”, il s’éloigne des systèmes purement rationnels et accorde un rôle central à la liberté, au temps, à l’histoire, au mal et à la révélation, cherchant à penser la réalité concrète plutôt qu’un système achevé. Il distingue une “philosophie négative” (pure construction rationnelle de l’absolu) et une “philosophie positive” qui part de l’existence, des faits de la révélation et de l’histoire pour comprendre Dieu, le monde et la liberté. &lt;/p&gt; "/>
-    <hyperlink ref="E16" r:id="rId4" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Ludwig_Feuerbach&quot;  title=&quot; Wikipedia&quot;&gt;Ludwig FEUERBACH&lt;/a&gt; était un philosophe bavarois qui a commencé sa carrière en défendant les idées hégéliennes, mais il s’est rapidement éloigné de l’idéalisme de Hegel, qu’il jugeait trop proche de la théologie chrétienne. Son ouvrage majeur, &lt;a href=&quot;https://www.youtube.com/watch?v=ni-uusn_4u4&quot;  title=&quot;Ludwig Feuerbach: Préface à la seconde édition de &quot;l'Essence du Christianisme&quot; par Le Gros Rouge qui Tache&quot;&gt;&quot; L’Essence du christianisme&quot;&lt;/a&gt; paru en 1841, constitue une critique radicale de la religion, où il affirme que Dieu n’est qu’une projection des qualités humaines, une aliénation par laquelle l’homme se dépossède de ses propres forces et valeurs. Cette idée a eu une influence majeure sur les penseurs de gauche, notamment Karl Marx, qui a repris et développé la notion  &lt;a href=&quot;https://www.youtube.com/watch?v=hCdmjaVFrts&quot; title=&quot;Feuerbach, dépasser l'aliénation religieuse vers le vrai humanisme par François Jourde&quot;&gt;d’aliénation chez Feuerbach&lt;/a&gt;. &lt;/p&gt; &lt;p&gt; Il développe une philosophie humaniste et sensualiste, plaçant l’homme et ses sentiments au centre de la réalité.​ Selon lui, la suppression de Dieu ne doit pas conduire à l’effondrement de la morale, mais au contraire à une responsabilité accrue de l’homme envers ses semblables.​ Il insiste sur l’importance de l’amour collectif et de l’altruisme comme fondements d’une société humaine authentique.​ &lt;/p&gt; &lt;p&gt; Il a profondément marqué la pensée du XIXe siècle, notamment par sa critique de la religion et son influence sur le matérialisme et le socialisme. Il a inspiré Marx, Engels et d’autres penseurs du mouvement ouvrier, tout en restant un philosophe indépendant, peu engagé dans la politique directe.​ Il est un penseur clé de  &lt;a href=&quot;https://books.openedition.org/pufc/40697?lang=fr&quot; title=&quot;Ludwig Feuerbach : la nature et la nature humaine comme fondement d’une praxis sociale et politique par Open Edition&quot;&gt;la transition&lt;/a&gt; entre l’idéalisme hégélien et le matérialisme moderne, dont la critique de la religion et la philosophie humaniste continuent d’inspirer la réflexion philosophique et sociale.  &lt;/p&gt; "/>
-    <hyperlink ref="E17" r:id="rId5" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Max_Stirner&quot;  title=&quot; Wikipedia&quot;&gt;Max STIRNER&lt;/a&gt;, de son vrai nom Johann Kaspar Schmidt était un philosophe bavarois, figure clé des Jeunes Hégéliens et précurseur de &lt;a href=&quot;https://www.youtube.com/watch?v=FG42gogWdCM&quot; title=&quot;L'anarchisme individualiste par Politikon&quot;&gt;l'anarchisme individualiste&lt;/a&gt; et de l'égoïsme philosophique. &lt;/p&gt; &lt;p&gt; Dans &quot;&quot;L'Unique et sa propriété&quot;, il rejette toutes les abstractions – Dieu, État, humanité, moralité, révolution – comme des &quot;spectres&quot; ou &quot;fixations&quot; qui aliènent l'individu au profit d'idées supérieures. Il prône l'&quot;égoïsme conscient&quot; : l'Unigue (le Moi unique) s'approprie ce qui lui est propre par la force de sa volonté, sans devoir ni norme externe.  &lt;a href=&quot;https://journals.openedition.org/rg/8578&quot; title=&quot;La philosophie politique de Max Stirner par OpenEdition&quot;&gt;Ce texte&lt;/a&gt; marque la fin de l'hégélianisme et annonce nihilisme, existentialisme et postmodernisme. &lt;/p&gt; &lt;p&gt; Il dissout le sujet en un &quot;Moi&quot; fluide, sans essence fixe ni mission universelle, opposé à l'idéalisme hégélien ou feuerbachien. Toute société repose sur des illusions collectives ; l'individu doit les détruire pour affirmer sa puissance propre, formant des unions temporaires par intérêt mutuel. Il critique le christianisme, le socialisme et le libéralisme comme autant de tyrannies déguisées.&lt;/p&gt; &lt;p&gt; Son radicalisme inspire l'anarchisme individualiste (bien qu'il le refuse), des illegalistes, existentialistes comme Nietzsche, et même des penseurs postmodernes ou libertariens. Marx lui consacre un long pamphlet dans L'Idéologie allemande, voyant en lui un danger pour le collectivisme. Redécouvert au XXe siècle, il reste un penseur &quot;inassimilable&quot; défiant toute allégeance. &lt;/p&gt; "/>
-    <hyperlink ref="E20" r:id="rId6" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Rudolf_Hermann_Lotze&quot;  title=&quot; Wikipedia&quot;&gt;Rudolf Hermann LOTZE&lt;/a&gt;  était un philosophe allemand, fils d'un médecin militaire, il étudie la médecine et la philosophie à l'université de Leipzig ou il enseigne ensuite, puis est nommé professeur de philosophie à Göttingen en 1844, succédant à Herbart, avant de rejoindre Berlin en 1880, où il décède l'année suivante. Sa carrière académique est marquée par une vaste érudition, alliant sciences naturelles et réflexion philosophique. Il est aussi poète et traducteur, ayant rendu Antigone de Sophocle en latin. &lt;/p&gt; &lt;p&gt; Il rejette à la fois le matérialisme et la philosophie romantique de la nature, critiquant la notion de &quot;force vitale&quot; popularisée par Schelling. Influencé par Leibniz, Hegel et Kant, il défend un &lt;a href=&quot;https://www.youtube.com/watch?v=H3FEXnD8Zb4&quot;  title=&quot;Hermann Lotze Microcosmus par The Spirit of hegel&quot;&gt;mécanisme explicatif &lt;/a&gt;  pour les phénomènes physiques, applicable à la biologie sans recourir à des causes surnaturelles. La téléologie n'est pour lui qu'un principe régulateur subjectif, compatible avec le mécanisme : l'ordre du monde exprime un dessein spirituel, mais la science doit s'en tenir aux lois causales. Dans ses travaux précoces comme De futurae biologiae principiis philosophicis (1838), il pose les bases d'une biologie philosophique rigoureuse. &lt;/p&gt; &lt;p&gt; Ses œuvres majeures, telles &lt;a href=&quot;https://journals.openedition.org/rgi/323&quot;  title=&quot;Hermann Lotze Microcosmus par openedition&quot;&gt;Mikrokosmos (1856-1864), &lt;/a&gt;  explorent l'être humain comme microcosme du monde, distinguant faits, lois et valeurs, unies dans la réalité mais séparées par notre pensée. Logik (1874) et Metaphysik (1879) forment un système philosophique quasi exhaustif, intégrant logique, ontologie et psychologie. Il y insiste sur les limites du langage et de la pensée, tout en proscrivant les déductions a priori spéculatives au profit d'une approche empirique et scientifique. Il fonde ainsi une psychologie scientifique, préfigurant des disciplines modernes. &lt;/p&gt; &lt;p&gt; Il  marque la transition entre l'idéalisme absolu post-hégélien et le néo-kantisme, évitant l'absolutisme idéaliste comme le réalisme atomistique. Il valorise les sciences naturelles tout en préservant une dimension éthique et téléologique : l'existence (Sein) doit être interprétée par son sens (Soll), via un langage des valeurs plutôt que des impératifs moraux stricts. Anti-naturaliste après la &quot;controverse du matérialisme&quot; de 1854, il intègre émotions et jugements de valeur à la connaissance humaine. &lt;/p&gt; &lt;p&gt; Son influence est immense jusqu'à la Première Guerre mondiale, impactant néo-kantiens, phénoménologues, positivistes logiques et même la psychologie anglo-saxonne via William James. En Allemagne, il ferme l'ère spéculative pour ouvrir une philosophie plus sobre et scientifique. Aux États-Unis, ses idées sur la causalité et la pensée relationnelle imprègnent le pragmatisme naissant. Il reste une figure pivot, liant science et métaphysique dans une vision unifiée de l'univers comme plan rationnel et spirituel. &lt;/p&gt; &#10;&#10;&#10;"/>
-    <hyperlink ref="E21" r:id="rId7" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl_Marx&quot;  title=&quot; Wikipedia&quot;&gt;Karl MARX&lt;/a&gt; était un philosophe, économiste et révolutionnaire allemand né à Trèves, est le fondateur  &lt;a href=&quot;https://www.youtube.com/watch?v=W_ZwUjnl4W4&quot;  title=&quot;La philosophie de Karl Marx par Parole de philosophe&quot;&gt;du marxisme &lt;/a&gt; avec Friedrich Engels. Issu d'une famille juive convertie au protestantisme, il étudie le droit et la philosophie à Bonn, Berlin et Iéna, où il est influencé par Hegel et les jeunes hégéliens comme David Strauss, dont il critique les idées religieuses dans sa jeunesse. Exilé en France puis en Angleterre après les révolutions de 1848, il vit dans la précarité à Londres, soutenu par Engels, et milite au sein de l'Internationale ouvrière. Son portrait de 1875 le montre barbu, pensif, incarnation du penseur engagé.   &lt;/p&gt; &lt;p&gt;    Sa philosophie repose sur le matérialisme historique et dialectique, voyant l'histoire comme une succession de modes de production (esclavagiste, féodal, capitaliste) mue par  &lt;a href=&quot;https://www.youtube.com/watch?v=1pYmqDnvTh8&quot;  title=&quot;Les classes sociales par DigiSchool Lycee &quot;&gt;la lutte des classes &lt;/a&gt; entre exploiteurs et exploités. Dans  &lt;a href=&quot;https://www.youtube.com/watch?v=jb-5oSF2dpU&amp;ab_channel=TanguyLacroix&quot;  title=&quot;Le Manifeste du Parti Communiste par Tanguy Lacroix &quot;&gt;&quot;Le Manifeste communiste  &lt;/a&gt; (1848), coécrit avec Engels, il appelle le prolétariat à abolir la propriété privée des moyens de production pour instaurer une société sans classes. Le Capital (1867-1883) analyse le capitalisme comme un système d'exploitation via la plus-value extraite du travail   &lt;a href=&quot;https://www.youtube.com/watch?v=rEAxxsX_um0&amp;t=4s&amp;ab_channel=LePr%C3%A9cepteur&quot;  title=&quot;L'Aliénation par le Précepteur &quot;&gt;salarié aliéné, &lt;/a&gt;  prédisant sa chute par ses contradictions internes. &lt;/p&gt; &lt;p&gt;  Il rejette la religion comme « opium du peuple », outil d'aliénation masquant l'exploitation réelle, et prône la praxis révolutionnaire : transformer le monde par l'action collective des travailleurs. Critiquant le libéralisme et le socialisme utopique, il envisage une dictature du prolétariat transitoire menant au communisme, où l'État dépérit et les besoins sont satisfaits selon les capacités. Ses idées opposent radicalement celles de Donoso Cortés, qui y voyait un aboutissement satanique du libéralisme. &lt;/p&gt;   &lt;p&gt; Sa contribution la plus importante à la théorie politique est sa conception du  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Mat%C3%A9rialisme_dialectique&quot;  title=&quot;Le Marxisme Dialectique par Wikipedia &quot;&gt;&quot;matérialisme dialectique&quot;&lt;/a&gt;, qui est l'idée que le changement historique est motivé par des conflits entre des classes sociales opposées et que ces conflits sont finalement résolus par la révolution. &lt;/p&gt; &lt;p&gt; Il a également écrit abondamment sur l'économie, en particulier sur la théorie de la valeur-travail, qui postule que la valeur d'un bien ou d'un service est basée sur la quantité de travail nécessaire pour le produire. &lt;/p&gt; &lt;p&gt;     Son influence sur le XXe siècle est immense : révolutions bolchevique, chinoise, mouvements ouvriers mondiaux, et disciplines comme la sociologie ou l'économie. Malgré les échecs des régimes « marxistes », sa critique du capitalisme reste débattue aujourd'hui. &lt;/p&gt;    &lt;audio controls title=&quot;Pour l'avenir par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10467-26.09.2020-ITEMA_22438423-2020C40092E0005-1779455909.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
-    <hyperlink ref="E22" r:id="rId8" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Friedrich_Engels&quot;   title=&quot; Wikipedia&quot;&gt;Friedrich ENGELS&lt;/a&gt;  était un  philosophe, théoricien socialiste allemand et le plus  &lt;a href=&quot;https://www.youtube.com/watch?v=K3GsK_RbVwI&quot; title=&quot;Friedrich Engels : Dans l'ombre de Marx, Arte 2024 par Crevoisier Philippe&quot;&gt;proche collaborateur&lt;/a&gt; de Karl Marx dans la fondation du marxisme et du communisme moderne. Son œuvre philosophique et politique a profondément marqué l'histoire intellectuelle et politique du XIXe siècle. Il travailla dans l'entreprise de son père, ce qui lui permet d'étudier directement les conditions de vie de la classe ouvrière britannique. C'est à cette époque qu'il rédige &quot;La Situation de la classe laborieuse en Angleterre&quot;, une analyse des conditions sociales des ouvriers. &lt;/p&gt; &lt;p&gt; En 1844, il rencontre Marx à Paris ; cette rencontre scelle leur collaboration intellectuelle et politique. Ensemble, ils écrivent plusieurs textes majeurs, notamment &quot;L’Idéologie allemande&quot; paru en 1845, &lt;a href=&quot;https://www.youtube.com/watch?v=xiJx1g91LYk&quot;  title=&quot;Marx, Engels - Manifeste du parti communiste  par Politikon&quot;&gt;&quot;Le Manifeste du Parti communiste&quot;&lt;/a&gt; en 1848, et fondent la Ligue des communistes. Après la mort de Marx, il prend en charge la publication des volumes II et III du &quot;Capital&quot;. Il fut un théoricien encyclopédique, passionné par la philosophie, les sciences, la littérature et l’histoire et il a anticipé certains développements scientifiques avec son ouvrage &quot;La dialectique de la nature&quot;, où il applique la méthode marxiste à l’étude des lois de la nature. &lt;/p&gt; &lt;p&gt; Il a conceptualisé le matérialisme historique avec Marx, affirmant que ce sont les conditions matérielles – et non les idées ou la conscience – qui déterminent le cours de l’histoire. Il l'a aidé financièrement et a mis sa capacité d'organisation au service du mouvement révolutionnaire européen. Sa pensée sur le matérialisme dialectique et la transformation sociale demeure une référence centrale dans les sciences humaines et politiques.Il est également reconnu pour ses analyses sur l’origine de la famille, de la propriété privée et de l’État.  &lt;/p&gt; &lt;audio controls title=&quot; Friedrich Engels, penser le marxisme à deux par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10081-24.10.2024-ITEMA_23903110-2024C29629S0298-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
-    <hyperlink ref="E23" r:id="rId9" display="&lt;p&gt;&lt;a href=&quot;https://en.wikipedia.org/wiki/Gustav_Teichm%C3%BCller&quot;  title=&quot; Wikipedia&quot;&gt;Gustav TEICHMÜLLER&lt;/a&gt; était un philosophe allemand, professeur à Bâle puis à Dorpat (aujourd’hui Tartu, en Estonie), considéré comme le fondateur du personnalisme russe et l’une des figures majeures de l’idéalisme tardif du XIXe siècle. Né à Braunschweig, formé à Berlin et Tübingen, il enseigne d’abord en Allemagne, puis en Suisse, avant d’occuper la chaire de philosophie de Tartu de 1871 jusqu’à sa mort en 1888, où il forme toute une génération de philosophes, dont Jēkabs Osis. &lt;/p&gt; &lt;p&gt; Il élabore, surtout à partir des années 1880, une « nouvelle philosophie » qu’il qualifie lui-même de personnalisme, à la fois contre l’idéalisme absolu (de type hégélien) et contre le matérialisme ou le positivisme de son temps. Son objectif central est de « sauver la personne » : il veut retrouver la réalité concrète des individus conscients, perdue selon lui dans les systèmes qui réduisent le monde à des représentations, à un Esprit unique ou à de la matière inerte. Pour lui, la réalité ultime est constituée de substances psychiques individuelles (des monades, des âmes), chacune étant un centre actif de conscience, de sentiment et de volonté. &lt;/p&gt; &lt;p&gt; Dans son ouvrage principal, Die wirkliche und die scheinbare Welt (Le monde réel et le monde apparent, 1882), il distingue le monde tel qu’il est en soi (un système de personnes/monades) et le monde tel qu’il nous apparaît à travers nos représentations. Il développe une forme de perspectivisme : chaque sujet connaît le monde depuis son point de vue propre, ce qui rend toute connaissance à la fois partielle et dépendante de la structure de la personne connaissante. Cette idée influence notamment Friedrich Nietzsche, qui reprend et transforme le motif perspectiviste dans sa propre critique de la vérité et de la métaphysique traditionnelle. &lt;/p&gt; &lt;p&gt; Il est aussi l’un des premiers à pratiquer systématiquement l’histoire des concepts (Begriffsgeschichte), en étudiant la genèse et les transformations des notions philosophiques majeures (être, substance, personne, etc.). Ce travail prépare, à long terme, des projets comme le Historisches Wörterbuch der Philosophie. Par son enseignement à Tartu et ses écrits, il fonde le personnalisme russe et marque durablement la philosophie lettone et estonienne, en faisant de la personne le centre d’une métaphysique qui cherche à concilier rigueur conceptuelle et respect de la réalité concrète des individus. &lt;/p&gt;&#10;"/>
-    <hyperlink ref="H23" r:id="rId10" display="https://www.laphilo.fr/pho/gteichmuller-mini.webp"/>
-    <hyperlink ref="I23" r:id="rId11" display="https://www.laphilo.fr/photo/gteichmuller.webp"/>
-    <hyperlink ref="E31" r:id="rId12" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Wilhelm_Windelband&quot;  title=&quot; Wikipedia&quot;&gt;Wilhelm WINDELBAND&lt;/a&gt;  était un philosophe allemand  fondateur de l'école néokantienne de Bade (ou du Sud-Ouest), aux côtés de Heinrich Rickert, avec qui il forme un duo clé du  &lt;a href=&quot;https://www.youtube.com/watch?v=h2R8wj7Q9x8&quot;  title=&quot;Néo-kantisme : définition, exemples. par le Savoir partagé&quot;&gt;néokantisme tardif &lt;/a&gt;. Élève initialement influencé par la psychologie, il évolue vers un néokantisme anti-psychologiste, critiquant le relativisme historiciste et posant les bases d'une philosophie des valeurs. &lt;/p&gt; &lt;p&gt; Il distingue &lt;a href=&quot;https://www.youtube.com/watch?v=Rr96FJSOcDU&quot; title=&quot; Wilhelm Windelband: Philosophy of Values and History par Philosopher Friends&quot;&gt;les sciences &lt;/a&gt; nomothétiques (lois générales, comme la physique) des sciences idiographiques (individuel, historique), cette dichotomie méthodologique influençant Max Weber et la philosophie des sciences. Sa &quot;philosophie des valeurs&quot; transpose la critique kantienne vers la normativité : vérité, bien, beauté comme exigences objectives, sans recours au psychologisme ni au métaphysique spéculative. &lt;/p&gt; &lt;p&gt; Ses oeuvres principales sont : - &quot;Histoire de la philosophie du Nouveau Temps' paru en 1880 et &quot;Histoire du problème philosophique de la liberté&quot; en 189 : synthèses historiques rigoureuses, voyant l'histoire de la philosophie comme science autonome. - &quot;Präludien&quot; en 1884, recueils d'essais : expose sa critique de la psychologie comme fondement du savoir et sa reformulation kantienne en termes normatifs. &lt;/p&gt; &lt;p&gt; Précurseur de la phénoménologie et des sciences humaines modernes, il impacte Rickert, Weber (types idéaux) et Jaspers, bien que moins systématique que les néokantiens de Marbourg. &lt;/p&gt; "/>
-    <hyperlink ref="E33" r:id="rId13" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Sigmund_Freud&quot;  title=&quot; Wikipedia&quot;&gt; Sigmund FREUD&lt;/a&gt; est un neurologue et philosophe Allemand connu pour son travail sur la Psychanalyse et son point de vue sur  &lt;a  href=&quot;https://www.youtube.com/watch?v=uYd0Xi3ACQ8&amp;t=17s&amp;ab_channel=LePr%C3%A9cepteur&quot;  title=&quot;L'origine de la religion par Le Précepteur&quot;&gt;la Religion&lt;/a&gt;. &lt;/p&gt; &lt;p&gt;  Et si ce n’était pas la raison et la volonté, mais l’inconscient et ses pulsions violentes et destructrices, qui étaient la grande force de l’esprit et de l’histoire ? Voilà l’hypothèse scandaleuse qui est au cœur de l’œuvre de Freud. &lt;/p&gt; &lt;p&gt; Si l’idée d’une vie psychique inconsciente avait déjà été envisagée par d’autres, de Leibniz à Schopenhauer et Nietzsche, Freud est le premier à en faire l’objet d’une méthode d’investigation et de soin : la psychanalyse. &lt;a  href=&quot;/document/le_reve_et_son_interpretation.pdf&quot;  title=&quot;Le rêve et son interprétation en version numérique&quot;&gt;&quot;Le rêve et son interprétation&quot;&lt;/a&gt;, publié en 1900, fait de l’analyse des rêves la « voie royale » pour aborder l’inconscient.&lt;/p&gt; &lt;p&gt;  Il est amené à repenser son modèle pour en accentuer la dimension conflictuelle entre ce qu’il nomme désormais &lt;a  href=&quot;https://www.youtube.com/watch?v=QO7HTLC0r6I&amp;ab_channel=Coursitout&quot; title=&quot;Le ça, le moi et le surmoi par Coursitout&quot;&gt;le « Ça », le « Moi » et le « Surmoi »&lt;/a&gt;. &lt;/p&gt; &lt;p&gt; Le Ça, correspondant à l’inconscient, est la partie obscure et inaccessible de notre personnalité. Le Moi, socle de la personnalité, est l’instance intermédiaire qui doit concilier les exigences contradictoires du Ça et du Surmoi. Le Surmoi, lui, est le juge intérieur qui naît de l’intériorisation des interdits sociaux. &lt;/p&gt; &lt;p&gt; Si  &lt;a  href=&quot;https://www.youtube.com/watch?v=b_v6YfaC5gU&amp;t=17s&amp;ab_channel=LePr%C3%A9cepteur&quot;  title=&quot;L'inconscient par Le Précepteur&quot;&gt;l’inconscient&lt;/a&gt; est ce chaos au cœur de l’individu, il devient le cœur du processus de civilisation. &lt;/p&gt; &lt;p&gt; En 1933, les œuvres de Freud sont brûlées par les Nazis mais le travail de Freud n’en reste pas moins incontournable dans l’histoire de la psychologie moderne. Sa postérité est immense. &lt;/p&gt;  &lt;audio controls title=&quot;L'Ombilic des rêves par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/19288-29.07.2018-ITEMA_21741416-2.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; &#10;&#10;"/>
-    <hyperlink ref="E35" r:id="rId14" display="&lt;p&gt; &lt;a href=&quot;https://fr.wikipedia.org/wiki/Edmund_Husserl&quot;  title=&quot; Wikipedia&quot;&gt; Edmund HUSSERL&lt;/a&gt; était un philosophe allemand d'origine juive connu pour être le fondateur de la  &lt;a href=&quot;https://www.youtube.com/watch?v=VaXxW0M9aIY&quot;  title=&quot;Intro à la phénoménologie par Le Precepteur&quot;&gt; phénoménologie&lt;/a&gt; qui est une méthode philosophique qui vise à décrire les structures de l'expérience telles qu'elles se présentent à la conscience, sans présuppositions théoriques ou métaphysiques. Il appelle cette approche &quot;retour aux choses mêmes&quot;, ce qui signifie qu'il faut se concentrer sur les phénomènes tels qu'ils apparaissent à la conscience, plutôt que sur des interprétations ou des constructions théoriques. &#10;Ses oeuvres les plus importantes : &lt;/p&gt; &lt;p&gt; -  &quot;Idées directrices pour une phénoménologie pure et une philosophie phénoménologique&quot; : il  y développe sa méthode de réduction phénoménologique et introduit le concept d'intentionnalité. &lt;/p&gt; &lt;p&gt; - &lt;a href=&quot;https://www.persee.fr/doc/phlou_0035-3841_1954_num_52_33_4479&quot;   title=&quot;Méditation cartésiennes par Persee&quot;&gt; &quot;Méditations cartésiennes&quot;&lt;/a&gt; : Une série de conférences où il approfondit sa pensée sur l'ego transcendantal et l'intersubjectivité.&lt;/p&gt; &lt;p&gt; - &quot;Recherches logiques&quot; (1900-1901) : Dans cet ouvrage, il critique le psychologisme (l'idée que les lois logiques sont des lois psychologiques) et pose les bases de sa phénoménologie.&lt;/p&gt; &lt;p&gt; - &quot;La crise des sciences européennes et la phénoménologie transcendantale&quot; (1936) : Dans cet ouvrage posthume, il analyse la crise des sciences modernes et propose une refondation philosophique basée sur la phénoménologie.&lt;/p&gt; &lt;p&gt; Il a tenté de développer une méthode pour explorer la nature de la conscience humaine. Il a cherché à comprendre comment nous percevons le monde à travers nos sens, comment nous avons des pensées et des émotions, et comment nous nous rapportons à nous-mêmes et aux autres. &lt;/p&gt; &lt;p&gt; &#10;La phénoménologie de Husserl a influencé de nombreux philosophes et écoles de pensée, notamment l'existentialisme (Sartre) , la psychanalyse (Freud) et la philosophie de la perception. Ses travaux ont également inspiré des mouvements culturels tels que l'art abstrait et le modernisme.  &lt;/p&gt; &lt;audio controls title=&quot;Le phénomène Husserl par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/18755-09.03.2020-ITEMA_22302657-2.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
-    <hyperlink ref="E36" r:id="rId15" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Lou_Andreas-Salom%C3%A9&quot; title=&quot; Wikipedia&quot;&gt;Lou ANDRÉAS-SALOMÉ&lt;/a&gt; était une écrivaine, philosophe, essayiste et psychanalyste allemande qui défendit une vision de la liberté incluant l'indépendance intellectuelle, émotionnelle et sexuelle. Elle rejette les conventions sociales et les rôles de genre traditionnels.  Ses principales oeuvres : &lt;/p&gt; &#10;&lt;p&gt; - Friedrich Nietzsche à travers ses œuvres (1894) : Elle y analyse la philosophie de Nietzsche, en mettant l'accent sur ses idées sur la volonté de puissance, l'éternel retour et la mort de Dieu.  &lt;/p&gt; &#10;&lt;p&gt; -  Rainer Maria Rilke (1928) : Elle l'écrit après la mort de Rilke et elle y explore sa relation avec le poète et analyse son œuvre, en mettant l'accent sur sa quête spirituelle et artistique. &lt;/p&gt; &#10;&lt;p&gt; - L'Érotisme (1910) : Elle explore la nature de l'érotisme et de la sexualité, en s'appuyant sur des réflexions psychologiques et philosophiques et défend une vision libérée et complexe de la sexualité. &lt;/p&gt; &#10;&lt;p&gt; -  Ma vie ( publié à titre posthume) : Dans son autobiographie, elle raconte &lt;a href=&quot;https://scienceetbiencommun.pressbooks.pub/femmessavantes3/chapter/lou-andreas-salome-femme-de-lettres-et-psychanalyste-1861-1937/&quot; title=&quot;  Lou Andréas-Salomé, femme de lettres et psychanalyste par esbc&quot;&gt;sa vie &lt;/a&gt;, ses relations et ses réflexions intellectuelles. &lt;/p&gt;  &lt;p&gt; Bien qu'elle ne se définisse pas comme féministe, elle défend une vision de la femme comme être indépendant et complexe. Elle s'intéresse à la spiritualité et à la religion, en particulier dans ses écrits sur Nietzsche et Rilke. Elle explore des thèmes comme la quête de sens, la transcendance et la relation entre l'homme et le divin. &lt;/p&gt; &lt;p&gt;  Elle est l'une des &lt;a href=&quot;https://www.youtube.com/watch?v=SlLT7BXn_YI&quot; title=&quot; First Female Psychoanalyst: Lou Andreas Salomé par Orbit&quot;&gt;premières femmes psychanalystes &lt;/a&gt; et ses écrits et ses réflexions ont contribué a son développement, en particulier dans les domaines de la sexualité et des relations humaines. &lt;/p&gt;  &lt;audio controls title=&quot;Lou Andreas-Salomé, la revendication d'un moi féminin libre par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13915-16.08.2022-ITEMA_23103839-2021C3372E0235-NET_MFC_5D82F295-9FBD-4DEC-9B93-3E80E99A02A8-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;  "/>
-    <hyperlink ref="E38" r:id="rId16" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hans_Driesch&quot; title=&quot; Wikipedia&quot;&gt;Hans DRIESCH&lt;/a&gt;  était un zoologiste, biologiste et philosophe allemand, fils unique d'un négociant prospère de Hambourg, il grandit dans un environnement propice à développer une vocation précoce de zoologiste : sa mère élevait des oiseaux exotiques et toutes sortes d'animaux, remplissant la maison de cages et de vivariums. Il devient en 1912 professeur de philosophie à Heidelberg, enseignera ensuite à Cologne en 1919, puis à Leipzig en 1921. En 1922-1923, il donne des cours en Chine aux universités de Nankin et Pékin, en 1926-1927 aux États-Unis à l'université du Wisconsin, et en 1928 à l'université de Buenos Aires. Le régime nazi le met d'office à la retraite en 1933, mais il continue à travailler jusqu'à sa mort survenue en pleine guerre. &lt;/p&gt; &lt;p&gt; En 1891, il réalise une expérience fondamentale : il dissocie deux blastomères d'oursin et montre que chacun se développe en une larve complète, bien que plus petite que la moyenne. Cette découverte contredit la théorie de Wilhelm Roux (1888) sur le développement en mosaïque, qui affirmait que chaque cellule initiale avait un rôle précis et formait seulement une partie de l'embryon. En 1892, il procède à une autre expérience capitale en comprimant les œufs d'oursin au stade de division en quatre cellules, déplaçant les noyaux anarchiquement dans le cytoplasme : les larves obtenues sont parfaitement normales, prouvant que tous les noyaux sont équivalents et renferment tous les gènes. Il a ainsi défendu l'épigenèse contre le préformisme et fait faire à l'embryologie un grand bond en avant. &lt;/p&gt; &lt;p&gt; Il  est le dernier grand &lt;a href=&quot;https://fr.wikipedia.org/wiki/Vitalisme&quot;  title=&quot;vitalisme par wikipedia&quot;&gt;porte-parole du vitalisme,&lt;/a&gt;  la théorie selon laquelle la vie ne peut être expliquée comme un phénomène purement physique ou chimique. Vers 1895, il devient un vitaliste convaincu. Il introduit le concept aristotélicien d'entéléchie pour désigner une force vitale qui régule le développement organique vers un but. Cette entéléchie est une force vitale logée dans l'œuf, tendant toujours vers le même but, expliquant pourquoi une cellule séparée peut donner une larve entière. &lt;/p&gt; &lt;p&gt; Il  apparaît comme une  &lt;a href=&quot;https://www.persee.fr/doc/phlou_0776-555x_1930_num_32_28_2598_t1_0464_0000_3&quot;  title=&quot;l’homme et le monde par persée&quot;&gt;figure originale &lt;/a&gt; tant parmi les scientifiques que parmi les philosophes, ayant introduit la biologie comme nouveau continent au sein de la réflexion philosophique. Sa philosophie de l'organique est étroitement liée à ses recherches biologiques. Toutefois, les théories vitalistes qu'il défendait sont aujourd'hui complètement abandonnées. On doit lui reconnaître le mérite d'avoir stimulé le progrès de l'embryologie expérimentale et d'avoir ouvert à la biologie de vastes perspectives. &lt;/p&gt; &#10;&#10;&#10;"/>
-    <hyperlink ref="H39" r:id="rId17" display="https://www.laphilo.fr/pho/rluxemburg-mini.webp"/>
-    <hyperlink ref="E40" r:id="rId18" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Theodor_Lessing&quot; title=&quot; Wikipedia&quot;&gt;Theodor LESSING&lt;/a&gt;  était un philosophe, essayiste et publiciste allemand &lt;a href=&quot;https://www.persee.fr/doc/rjuiv_0484-8616_1996_num_155_1_2554&quot;  title=&quot;Lessing et le sionisme par persée&quot;&gt;d’origine juive, &lt;/a&gt; connu comme un penseur critique de la modernité, du nationalisme et de l’antisémitisme. &lt;/p&gt; &lt;p&gt; Il s’inscrit surtout dans une philosophie de la culture et une philosophie sociale critique. Son travail ne cherche pas à construire un système abstrait, mais à analyser les maladies de la civilisation moderne, la violence des masses, la guerre, la ville industrielle et la destruction du vivant. Sa pensée est marquée par un humanisme pessimiste et engagé qui dénoncé le militarisme, la brutalisation de la société et les dérives autoritaires de l’Allemagne de Weimar, allant jusqu’à prévoir le danger nazi avant 1933. Il fut aussi l’un des premiers à réfléchir à la condition des minorités et à ce qu’il a appelé le &lt;a href=&quot;https://www.sifriatenou.com/2020/10/20/5449/&quot;  title=&quot;lessing la haine de soi par sifriatenou&quot;&gt;« judaïsme de haine de soi »,&lt;/a&gt; pour décrire les effets psychologiques de l’antisémitisme sur les Juifs eux-mêmes. &lt;/p&gt; &lt;p&gt; Il est également une figure de la critique écologique avant l’heure. Dès les années 1930, il s’inquiète de la déforestation, de la pollution urbaine et d’un possible dérèglement du climat, ce qui le rend étonnamment actuel. Il voit la modernité technique non comme un progrès neutre, mais comme une force capable de détruire les équilibres humains et naturels. &lt;/p&gt; &lt;p&gt; Sur le plan politique, il est un intellectuel indépendant, polémique et souvent isolé, qui s’oppose à l’autoritarisme autant qu’aux conformismes de son époque. Il a &lt;a href=&quot;https://www.youtube.com/watch?v=pdcxbRYcn&quot;  title=&quot;lessing par jacques Aron et Editions harmattan&quot;&gt;fini assassiné en exil &lt;/a&gt;  à Mariánské Lázně par des nationalistes sudètes, devenant l’une des premières victimes du nazisme hors d’Allemagne. &lt;/p&gt; &#10;"/>
-    <hyperlink ref="E41" r:id="rId19" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Max_Scheler&quot; title=&quot; Wikipedia&quot;&gt;Max SCHELER&lt;/a&gt;  était un philosophe allemand, figure phare de la phénoménologie et de l’anthropologie philosophique, dont l’œuvre traverse des domaines variés comme l’éthique, l’axiologie et la sociologie de la connaissance. &lt;/p&gt; &lt;p&gt; Il élabore une &lt;a href=&quot;https://www.persee.fr/doc/phlou_0776-555x_1927_num_29_14_2467&quot;  title=&quot;La philosophie de M. Scheler. Son analyse de la sympathie et de l'amour par Persée&quot;&gt;hiérarchie des valeurs &lt;/a&gt; qui va des valeurs de l’agréable et du désagréable jusqu’aux valeurs spirituelles (beau/laid, juste/injuste, connaissance, et enfin le sacré et le profane). Cette hiérarchie sert de base à une éthique et à une phénoménologie de la sensation et des sentiments qui orientent l’action humaine. Il propose une approche phénoménologique qui insiste sur &quot;l’attitude spirituelle&quot; ou &quot;l’œil vivant&quot; vers le monde, en s’opposant à une réduction purement méthodologique et en valorisant l’intuition des valeurs telles qu’elles se donnent à la conscience. &lt;/p&gt; &lt;p&gt; Il fonde l’idée d’une anthropologie philosophique qui cherche à comprendre l’homme dans le vivant et ses rapports au monde, en intégrant des connaissances des sciences naturelles et des sciences humaines. &lt;a href=&quot;https://www.youtube.com/watch?v=pPuUoTPig7w&quot; title=&quot;Le salut vient-il du travail ? - Valeur et dignité du travail selon Max SCHELER par Editions M-Editer&quot;&gt;Cette orientation &lt;/a&gt; mène plus tard à une sociologie de la connaissance. Voici ses oeuvres majeures : &lt;/p&gt; &lt;p&gt; - &quot;Die Wissensformen und die Gesellschaft&quot; paru en 1926 – synthèse de son projet de sociologie de la connaissance et jalon important de l’anthropologie philosophique et sociale. Cette œuvre est souvent citée comme fondatrice d’une approche sociologique qui rejoint les débats de Weimar.&lt;/p&gt; &lt;p&gt; - &quot;Stellung des Menschen im Kosmos&quot; paru en 1928 – portrait philosophique de l’homme dans le cadre d’un ensemble plus large d’ouvrages préfigurant l’anthropologie philosophique et son intérêt pour le positionnement de l’homme dans l’ordre du vivant. &lt;/p&gt; &lt;p&gt; Son approche personnaliste et son engagement en faveur d’une philosophie sociale et éthique centrée sur la dignité humaine, &lt;a href=&quot;https://www.youtube.com/watch?v=HHAKQrNdMYk&quot; title=&quot;&#10;Le ressentiment détruit ta vie… (Max Sheller, l'homme du ressentiment) par Timothée Delahaye&quot;&gt;le resentiment &lt;/a&gt; et les valeurs morales continuent d’être discutés dans les études contemporaines, notamment dans les analyses qui situent Scheler dans le dialogue franco-allemand et dans les traditions de philosophie sociale et morale. &lt;/p&gt; "/>
-    <hyperlink ref="E44" r:id="rId20" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hermann_von_Keyserling&quot; title=&quot; Wikipedia&quot;&gt;Hermann Von KEYSERLING&lt;/a&gt;  était un philosophe  &lt;a href=&quot;https://www.persee.fr/doc/slaoc_1245-2491_1997_num_4_1_1809&quot; style=&quot;color:#88A1E9&quot; title=&quot; Hermann von Keyserling et les interférences germano-slaves par Persée&quot;&gt;germano-balte &lt;/a&gt; devenu philosophe voyageur, figure très en vue de la République de Weimar, connu pour son Journal de voyage d’un philosophe et pour son &quot;École de la sagesse&quot; à Darmstadt. &lt;/p&gt; &lt;p&gt; Il conçoit la philosophie non comme une science rigoureuse, mais comme sagesse vécue : &quot;la vie elle-même sous la forme du savoir&quot;, contre les théories objectivantes du savoir technico-scientifique. Il s’inscrit dans la philosophie de la vie, mais de façon personnelle : importance de l’intuition, de la singularité des événements et de la transformation intérieure. Son projet est une nouvelle synthèse de l’âme et de l’esprit, la pénétration réciproque de sagesse et politique, et l’idée que dans la vie déterminée par l’esprit, c’est &lt;a href=&quot;https://www.youtube.com/watch?v=Y0DY8F72114&quot; title=&quot;Eduard von Keyserling, DUMALA par Le Veilleur&quot;&gt;le Sens &lt;/a&gt; qui crée les faits plutôt que l’inverse. &lt;/p&gt; &lt;p&gt; Il  utilise très tôt le terme Führerprinzip, en liant l’idée de &quot;dirigeants nés&quot; à un élitisme spiritualiste et social-darwinien, tout en refusant par la suite d’adhérer au national-socialisme, qu’il voit comme mouvement de masses manipulées.  Le régime nazi ferme son École de la sagesse au milieu des années 1930, lui interdit de publier et de voyager, tandis que sa réputation continue de grandir à l’étranger. &lt;/p&gt;&lt;p&gt; Ses oeuvres principales sont : - &quot;Reisetagebuch eines Philosophen&quot;  paru en 1919 : récit de son tour du monde (1911-1912, Asie, Amérique, Europe du Sud) mêlant observations culturelles, méditations spirituelles et diagnostics sur les civilisations ; c’est son grand succès de librairie, largement traduit. -&quot;Das Gefüge der Welt. Versuch einer kritischen Philosophie&quot; (La Structure du monde, 1907) : tentative de &quot;philosophie critique&quot; personnelle, déjà marquée par l’idée que le savoir véritable est inséparable de la vie. - &quot;Schöpferische Erkenntnis&quot; (Connaissance créatrice) et &quot;Wiedergeburt&quot; (Renaissance) : textes doctrinaux de l’&quot;École de la sagesse&quot;, insistant sur la connaissance comme acte créateur, transformant la vie plutôt que la décrivant objectivement. &lt;/p&gt; "/>
-    <hyperlink ref="E45" r:id="rId21" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Moritz_Schlick&quot;  title=&quot; Wikipedia&quot;&gt;Moritz SCHLICK&lt;/a&gt; était un philosophe allemand, physicien de formation, et l’une des figures centrales de l’empirisme logique. Il est surtout connu comme le fondateur et le dirigeant intellectuel du Cercle de Vienne, groupe qui se réunissait autour de la philosophie des sciences dans les années 1920 et 1930. Il occupa à Vienne une chaire autrefois associée à Ernst Mach et à Ludwig Boltzmann. &lt;/p&gt; &lt;p&gt; Sa première grande œuvre est la Théorie générale de la connaissance (Allgemeine Erkenntnislehre, 1918). Dans cet ouvrage, il défend encore une forme de réalisme scientifique : le monde extérieur existe indépendamment de nous et peut être connu grâce aux sciences. Il s’oppose ainsi à l’idéalisme et à l’idée kantienne selon laquelle nous ne connaîtrions jamais les choses en elles-mêmes. Pour lui, connaître consiste notamment à coordonner des signes et des concepts avec les objets et les processus étudiés par les sciences. &lt;/p&gt; &lt;p&gt;  À partir des années 1920, son orientation évolue sous l’influence de Wittgenstein et du développement de la logique moderne. Il affirme alors que la philosophie ne doit pas construire une nouvelle vision métaphysique du monde, mais clarifier le sens des propositions. Une &lt;a href=&quot;https://encyclo-philo.fr/schlick-a&quot;  title=&quot;l’encyclopedie philosophique : schick par encyclophilo&quot;&gt;proposition authentiquement scientifique &lt;/a&gt; doit pouvoir être reliée à une méthode possible de vérification empirique ; les énoncés de logique et de mathématiques sont, quant à eux, analytiques ou tautologiques. Cette orientation est souvent résumée par la formule : « le sens d’une proposition est sa méthode de vérification ». &lt;/p&gt; &lt;p&gt; Il faut cependant éviter de le réduire à un vérificationnisme simpliste. Il admet qu’une proposition puisse être vérifiable en principe, même si la vérification ne peut pas être réalisée immédiatement ou matériellement. La vérification ne signifie donc pas forcément une observation actuelle, mais la possibilité de décrire une procédure permettant de déterminer si l’énoncé est vrai ou faux. Sur le plan éthique, Il ne pense pas que les jugements de valeur soient des connaissances scientifiques ; il leur accorde néanmoins une importance dans la vie humaine et dans l’analyse des motivations. &lt;/p&gt; &lt;p&gt; On peut le classer comme un philosophe des sciences, un empiriste logique, &lt;a href=&quot;https://www.youtube.com/watch?v=ESWQzsf1Fr4&quot;  title=&quot;la fin du positivisme logique par philo analytique&quot;&gt;un positiviste logique &lt;/a&gt; et un représentant de la philosophie analytique naissante. Il est plus central et plus systématique que Hans Hahn dans l’organisation du Cercle de Vienne, tandis que Hahn était avant tout mathématicien et philosophe des fondements des mathématiques. Sa pensée se situe à la rencontre du réalisme scientifique, de l’empirisme, de l’analyse logique du langage et de l’anti-métaphysique ; son projet fondamental était de faire de la philosophie une activité de clarification au service de la connaissance scientifique. &lt;/p&gt; &#10;"/>
-    <hyperlink ref="H45" r:id="rId22" display="https://www.laphilo.fr/pho/mschlick-mini.webp"/>
-    <hyperlink ref="E47" r:id="rId23" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl_Korsch&quot; title=&quot; Wikipedia&quot;&gt;Karl KORDCH&lt;/a&gt;  était un philosophe marxiste allemand,  théoricien du communisme de conseils et critique du léninisme orthodoxe. Issu d'un milieu bourgeois, il évolua du réformisme social au marxisme hétérodoxe, influençant les courants ultra-gauche via son rejet du matérialisme positiviste et son insistance sur la praxis révolutionnaire historique.  Exclu du parti en 1926 pour &quot;ultra-gauchisme&quot;, il émigra après 1933 vers les USA, où il approfondit sa théorie marxiste. &lt;/p&gt; &lt;p&gt; Son œuvre majeure &quot;Marxisme et philosophie&quot; paru en 1923 marque sa rupture avec le léninisme en critiquant sa dérive scientiste. Il   &lt;a href=&quot;https://www.zones-subversives.com/article-le-marxisme-critique-de-karl-korsch-116431466.html&quot;  title=&quot;Le marxisme critique de Karl Korsch par Chroniques critiques&quot;&gt;rejette le marxisme &lt;/a&gt; comme &quot;science positive&quot; figée ou philosophie matérialiste abstraite ; il le conçoit comme une théorie historique et concrète, liée à la lutte des classes et à la dialectique hégélienne réinterprétée comme expression de la révolution bourgeoise puis prolétarienne. &lt;/p&gt; &lt;p&gt; Il  théorise les conseils comme organes centraux de la transition socialiste, via la praxis dialectique et l'auto-activité des masses, contre la socialisation étatique. Ses écrits inspirent le KAPD et l'ultra-gauche, voyant les conseils comme alternative à la bureaucratisation stalinienne. Son influence perdure chez les communistes de conseils, soulignant la conscience ouvrière spontanée pour l'émancipation réelle. &lt;/p&gt; "/>
-    <hyperlink ref="E50" r:id="rId24" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Eugen_Rosenstock-Huessy&quot; title=&quot; Wikipedia&quot;&gt;Eugen ROSENSTOCK-HUESSY&lt;/a&gt; était un penseur germano‑américain dont l'œuvre mêle philosophie sociale, histoire des idées et une théorie du langage centrée sur la parole comme acte créateur et structurant de la vie collective. Né en Allemagne, il forma des liens intellectuels avec des figures comme Franz Rosenzweig et Martin Buber, fut professeur (notamment aux États‑Unis après son exil) et créa une œuvre originale qui vise à comprendre comment les communautés se constituent et se transforment dans le temps par des échanges de parole. &lt;/p&gt; &lt;p&gt; Au  &lt;a href=&quot;https://www.en-attendant-nadeau.fr/2019/11/19/homme-quadridimensionnel-rosenstock//&quot;  title=&quot;l’homme quadridimensionnel par ean&quot;&gt;cœur de sa pensée &lt;/a&gt;  se trouve la notion de &quot;speech thinking&quot; (pensée de la parole) : il soutient que la parole n’est pas qu’un moyen descriptif, mais un acte répondant et créatif qui institue des relations sociales, forge des temporalités collectives et permet la transmission et la renouvellement des institutions humaines. Il affirme que, par le langage, les groupes deviennent « maîtres du temps » en fondant de nouveaux commencements, en rappelant le passé et en orientant l’action future — d’où son intérêt pour la densité historique de la vie sociale et le rôle des rituels, des serments et des discours publics. &lt;/p&gt; &lt;p&gt; Sur la religion et la théologie, il s’inscrit dans un courant post‑nietzschéen de renouveau religieux qui comprend Rosenzweig et Buber; il considère les énoncés religieux comme des actes de parole non‑métaphysiques qui dévoilent des dimensions de l’expérience humaine et communautaire inaccessibles aux seules sciences naturelles. Cette orientation le conduit à une pensée intégrative où philosophie, théologie et histoire participent à une réflexion pratique sur la transformation sociale et la responsabilité collective. &lt;/p&gt; &lt;p&gt; Ses livres et conférences couvrent une grande variété de thèmes — histoire des peuples, rhétorique sociale, philosophie de la loi et de l’éducation — et sa méthode combine analyses historiques, typologies du langage et propositions pour renouveler la vie civique; son influence se voit aujourd’hui dans des études sur la communication, la sociologie historique et la philosophie de la culture. &lt;/p&gt; "/>
-    <hyperlink ref="H50" r:id="rId25" display="https://www.laphilo.fr/pho/erhuessy-mini.webp"/>
-    <hyperlink ref="E52" r:id="rId26" display="&lt;p&gt; &lt;a href=&quot;https://fr.wikipedia.org/wiki/Oskar_Becker&quot;  title=&quot; Wikipedia&quot;&gt;Oskar BECKER&lt;/a&gt; était un philosophe, logicien, mathématicien et historien des mathématiques allemand, connu comme l’un des élèves les plus importants d’Edmund Husserl et comme un interlocuteur clé de Martin Heidegger. Sa pensée se situe à la croisée de la phénoménologie, de la philosophie des mathématiques, de la logique modale et de l’existentialisme. &lt;/p&gt; &lt;p&gt; Il utilise la phénoménologie husserlienne pour analyser les fondements de la géométrie, de l’arithmétique et de la logique, en cherchant à décrire les expériences vécues (compter, mesurer, démontrer) comme actes de conscience. Il tente ainsi de fonder une  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Ph%C3%A9nom%C3%A9nologie&quot;  title=&quot;phénoménologie par wikipedia&quot;&gt; sémantique phénoménologique &lt;/a&gt; de la logique intuitionniste, et ses idées sont reprises par Arend Heyting dans sa formalisation de cette logique. À la fin de sa vie, il insiste sur une distinction entre une intuition du domaine formel et platonicien (mathématiques pures) et un domaine existentiel concret, en utilisant parfois un vocabulaire proche de la « divination ». &lt;/p&gt; &lt;p&gt;Il est aussi un pionnier de la logique modale (logique de la nécessité et de la possibilité). On lui doit notamment ce qu’on appelle le postulat de Becker : l’idée que le statut modal est nécessaire, par exemple que la possibilité de PPP implique la nécessité de la possibilité de PPP, ainsi que certaines lois d’itération de la nécessité. Ces résultats ont joué un rôle important dans le développement de la logique modale au XXᵉ siècle. &lt;/p&gt; &lt;p&gt; Il entretient un dialogue étroit avec Heidegger : il reprend certains thèmes existentialistes (finitude, historicité, être-pour-la-mort) et les applique à des domaines comme les mathématiques, ce qui est très controversé (par exemple, discuter du comptage arithmétique comme « être-pour-la-mort »). Il développe également une « paraontologie » : une doctrine de l’essence et de la permanence des choses, distincte de l’ontologie heideggérienne centrée sur l’existence du Dasein. Pour lui, l’être humain n’existe pas seulement comme existence, mais aussi comme « paraexistence », incluant des dimensions inconscientes et surconscientes. &lt;/p&gt; &#10;&#10;"/>
-    <hyperlink ref="H52" r:id="rId27" display="https://www.laphilo.fr/pho/obecker-mini.webp"/>
-    <hyperlink ref="E53" r:id="rId28" display="https://fr.wikipedia.org/wiki/Edith_Stein"/>
-    <hyperlink ref="H53" r:id="rId29" display="https://www.laphilo.fr/pho/estein-mini.webp"/>
-    <hyperlink ref="E59" r:id="rId30" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Gershom_Scholem&quot; title=&quot; Wikipedia&quot;&gt;Gershom SCHOLEM&lt;/a&gt; était un philosophe juif germano-israélien,  fondateur de l'étude académique moderne de la Kabbale et grand expert de  &lt;a href=&quot;https://www.nonfiction.fr/article-12478-gershom-scholem-de-berlin-a-la-palestine.htm&quot; title=&quot;Gershom Scholem : de Berlin à la Palestine  par nonfiction&quot;&gt;la mystique juive. &lt;/a&gt; Né à Berlin dans une famille assimilée, il s'est tourné vers le sionisme jeune et a immigré en Palestine en 1923, devenant professeur à l'Université hébraïque de Jérusalem. &lt;/p&gt; &lt;p&gt; Il a étudié les mathématiques, la philosophie et les langues sémitiques à Berlin, Iéna et Munich, où il a soutenu une thèse sur le &quot;Sefer ha-Bahir&quot;, un texte kabbalistique ancien. Ami proche de Walter Benjamin et correspondant de Leo Strauss, il a fui l'Europe nazie et s'est consacré à la recherche sur les manuscrits juifs pillés. &lt;/p&gt; &lt;p&gt; Il voyait  &lt;a href=&quot;https://www.youtube.com/watch?v=5HvDF8-XTjc&quot;  title=&quot;Dieu son nom et la Cabale selon Gershom Scholem  par Xavier Charles DJEBALI&quot;&gt;la Kabbale &lt;/a&gt; non comme une superstition marginale, mais au cœur de l'essence spirituelle du judaïsme, explorée via des méthodes scientifiques et historiques. Il insistait sur le rôle du messianisme et de la tradition comme forces de renouvellement, où la révélation divine est infiniment interprétable et liée à l'expérience historique du peuple juif. Pour lui, le sionisme allait au-delà de la politique : c'était un renouveau profond du judaïsme, unissant ancien et nouveau contre l'assimilation. &lt;/p&gt; &lt;p&gt; Son oeuvre majeure &quot;Les Grandes tendances de la mystique juive&quot; paru en 1941, basé sur des conférences, dédié à Benjamin, explore l'évolution de la mystique juive. Sa pensée met l'accent sur l'identité juive forgée par l'histoire, où la tradition intègre la nouveauté pour survivre aux crises. &lt;/p&gt; &lt;audio controls title=&quot;Des livres pour notre temps et les mondes à venir. 1/2 Gershom Scholem : penser dans les marges de la marge par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13094-10.11.2019-ITEMA_22199082-0.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
-    <hyperlink ref="E60" r:id="rId31" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Leo_Strauss&quot; title=&quot; Wikipedia&quot;&gt;Leo SRAUSS&lt;/a&gt; était un philosophe politique germano-américain, connu pour sa critique profonde de la modernité et pour sa relecture des grands textes de la philosophie politique classique. Sa pensée a eu une influence durable, notamment aux États‑Unis, où elle a marqué des générations d’étudiants en théorie politique. &lt;/p&gt; &lt;p&gt; Au cœur de sa philosophie se trouve l’idée que la modernité a rompu avec le droit naturel classique, c’est‑à‑dire avec la recherche de ce qui est juste par nature et non simplement selon l’histoire ou les sciences sociales. Il voit dans le positivisme, le relativisme et l’historicisme modernes une source de décadence intellectuelle, car ils empêchent de poser les questions normatives fondamentales : qu’est‑ce qu’une vie bonne, qu’est‑ce qu’un régime politique juste. Pour lui, la  &lt;a href=&quot;https://www.persee.fr/doc/rfsp_0035-2950_1985_num_35_4_394205&quot; title=&quot;philosophie et zscience politique par persée&quot;&gt;philosophie politique authentique &lt;/a&gt; doit réactiver ces questions et affronter directement les notions de meilleur régime et d’ordre politique juste, plutôt que de se contenter de descriptions neutres. &lt;/p&gt; &lt;p&gt; Cette critique le conduit à renouer avec les auteurs de l’Antiquité, en particulier Platon, Aristote et les philosophes médiévaux juifs et arabes, qu’il lit souvent contre les interprétations modernes. Il insiste sur la dimension éducative de la philosophie : il parle de « liberal education » comme d’une libération de la vulgarité, entendue comme manque d’expérience des belles choses. La fréquentation des grands textes est, pour lui, une école de modestie et d’audace intellectuelle, parce qu’elle oblige à mesurer nos catégories modernes à celles d’auteurs qui pensaient autrement le politique et le juste. &lt;/p&gt; &lt;p&gt; Célèbre pour sa thèse sur l’« écriture ésotérique » : selon lui, nombre de philosophes du passé ont écrit de manière volontairement oblique pour se protéger de la censure ou de la persécution, réservant un sens plus profond aux lecteurs attentifs. Cela l’amène à distinguer entre le message « exotérique » (apparent, destiné au grand public) et le message « ésotérique » (plus exigeant, adressé à une minorité philosophique). Cette hypothèse sur la lecture des classiques s’articule à sa conception du   &lt;a href=&quot;https://www.youtube.com/watch?v=9Vhsveytymk&quot; title=&quot;nihilisme et politique leo strauss par bildung et culture&quot;&gt;mode de vie philosophique, &lt;/a&gt; toujours exposé au risque de la tyrannie et de l’incompréhension. Ainsi, sa philosophie politique est à la fois une critique de la modernité et une tentative de redécouvrir la place de la philosophie au cœur du politique contemporain. &lt;/p&gt; &#10; &lt;audio controls title=&quot;la pensée de leon strauss par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13397-05.04.2008-ITEMA_20118283-2008C3397E0019-ITE_00016207_RSCE-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;  &#10;"/>
-    <hyperlink ref="H60" r:id="rId32" display="https://www.laphilo.fr/pho/lstrauss-mini.webp"/>
-    <hyperlink ref="E63" r:id="rId33" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hans_Jonas&quot; title=&quot; Wikipedia&quot;&gt;Hans JONAS&lt;/a&gt;  était un philosophe germano-américain connu pour ses travaux sur l'éthique de la technologie et &lt;a href=&quot;https://www.youtube.com/watch?v=NPIJHZO7hQo&quot; title=&quot; Le PRINCIPE RESPONSABILITÉ en 6 minutes ! (HANS JONAS) par Culture Philo&quot;&gt;la responsabilité&lt;/a&gt; envers les générations futures. Ses premières recherches portent sur le gnosticisme, vu comme une réponse à l'aliénation existentielle dans un monde hostile. Dans les années 1960, il développe une philosophie de la vie organique (The Phenomenon of Life), critiquant le dualisme cartésien et valorisant la nature vivante contre la technoscience destructrice. Son œuvre maîtresse &lt;a href=&quot;https://www.youtube.com/watch?v=LsIWCR9_N64&quot; style=&quot;color:#88A1E9&quot; title=&quot; Philo, Hans jonas, Le principe responsabilité, Bac philo par SOS Bac Français&quot;&gt; &quot;Le Principe responsabilité&quot;&lt;/a&gt; paru en1979, formule un impératif éthique pour l'ère technologique : &quot;Agis de façon que les effets de ton action soient compatibles avec la permanence d'une vie authentiquement humaine sur Terre&quot;. &lt;/p&gt; &lt;p&gt; Il  anticipe les crises écologiques et bioéthiques, proposant une &quot;heuristique de la peur&quot; pour guider l'action humaine face aux risques imprévisibles de la puissance technique. Influencé par sa tradition juive et Heidegger, il réconcilie existentialisme, phénoménologie et morale prophétique, impactant l'éthique environnementale contemporaine. &lt;/p&gt; &lt;p&gt; Il observe un &quot;déchaînement prométhéen&quot; : l'humanité acquiert un pouvoir inédit sur la nature via la science et la technique, capable de menacer sa propre survie et celle des générations futures. Contrairement aux éthiques classiques (kantienne ou utilitariste), limitées au présent ou aux intentions, sa réflexion intègre les conséquences à long terme, imprévisibles et collectives, sur la vie humaine et la planète. Face aux risques inconnus (nucléaire, génétique, environnementaux), il prône une &quot;heuristique de la peur&quot; : anticiper le pire scénario (in dubio pro malo) pour guider l'action, sans paralyser le progrès mais en le subordonnant à la préservation de la vie. Le savoir devient un devoir moral prioritaire, élargissant l'éthique à la nature et aux générations absentes.&lt;/p&gt;  &lt;/p&gt; &lt;p&gt;  &lt;audio controls title=&quot; Hans Jonas. Pour une éthique de la société technologique par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/22267-14.06.2021-ITEMA_22702122-2014C12410E0357.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
-    <hyperlink ref="E65" r:id="rId34" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl-Otto_Apel&quot; title=&quot; Wikipedia&quot;&gt;Karl-Otto APEL&lt;/a&gt; était un philosophe allemand majeur de l’après-guerre, surtout connu pour avoir développé, avec Jürgen Habermas, l’éthique du discours et pour sa « pragmatique transcendantale », une tentative de refonder la philosophie à partir des présupposés normatifs de l’argumentation. &lt;/p&gt; &lt;p&gt; Il est souvent crédité d’avoir opéré la « linguistification » de la philosophie transcendantale kantienne : au lieu de partir de la conscience ou du sujet (comme chez Kant ou Husserl), il part du fait que toute connaissance et toute action s’inscrivent dans un langage commun et une communauté de communication. Pour lui, les conditions de possibilité de la connaissance ne sont pas d’abord dans la structure de la conscience, mais dans les règles implicites de l’usage du langage et de l’argumentation. &lt;/p&gt; &lt;p&gt;  &lt;a href=&quot;https://www.youtube.com/watch?v=R9jQv_akxFE&quot; &gt;Sa notion centrale &lt;/a&gt; est celle d’a priori de la communauté de communication : le simple fait d’argumenter présuppose déjà un cadre normatif inévitable (recherche de vérité, reconnaissance mutuelle des interlocuteurs, exigence de cohérence, etc.). Quiconque tente de nier ces présupposés tombe dans une auto-contradiction performative : en les contestant par la parole, il les utilise déjà. Il en tire l’idée d’une fondation ultime de la rationalité et de l’éthique à partir de la structure même de l’argumentation. &lt;/p&gt; &lt;p&gt; À partir de cette base, il développe une éthique du discours : seules sont moralement justifiées les normes qui pourraient être acceptées par tous les concernés dans un discours pratique idéal, où chacun est reconnu comme partenaire égal de l’argumentation. Cette éthique vise à fournir un fondement universel à la morale, sans retomber dans un absolutisme dogmatique ni dans un relativisme pur : l’universalité vient des conditions mêmes de l’argumentation rationnelle. Elle influence profondément Habermas, même si il insiste davantage sur la dimension de fondation ultime et sur l’obligation morale inconditionnelle qui en découle. &lt;/p&gt; &#10;"/>
-    <hyperlink ref="H65" r:id="rId35" display="https://www.laphilo.fr/pho/koapel-mini.webp"/>
-    <hyperlink ref="E67" r:id="rId36" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Reiner_Sch%C3%BCrmann&quot;  title=&quot; Wikipedia&quot;&gt;Reiner SCHÜRMANN&lt;/a&gt; est un philosophe allemand d’expression française, né à Amsterdam et mort à New York, où il a enseigné à la New School for Social Research à partir de 1975. Très marqué par la phénoménologie et la pensée de Heidegger, il se distingue par une réflexion exigeante sur la métaphysique, l’histoire de la philosophie et l’agir humain, développée dans trois grands ouvrages : Maître Eckhart et la joie errante (1972), Le principe d’anarchie (1982) et Des hégémonies brisées (posthume, 1996). &lt;/p&gt;&lt;p&gt; Dans Maître Eckhart et la joie errante, Schürmann reprend la pensée du mystique allemand du XIVᵉ siècle pour explorer la possibilité d’une vie spirituelle détachée de toute identité fixe ou de tout fondement stable. Il met en avant ce qu’il appelle une « joie errante » : une forme de liberté intérieure où le sujet ne se réclame plus d’une essence, d’un Dieu garanti ou d’une identité nationale, mais accepte de vivre dans une errance originaire et sans fondement. &lt;/p&gt; &lt;p&gt; Dans Le principe d’anarchie (souvent considéré comme son chef‑d’œuvre), Schürmann interprète Heidegger comme une pensée qui conduit à la ruine de tout principe premier (« archè ») sur lequel la tradition occidentale aurait voulu fonder la connaissance, la morale et la politique. Il en tire une théorie de l’« anarchie » non pas comme désordre, mais comme conscience lucide de l’absence de fondement ultime : l’agir humain doit alors se penser comme une praxis ouverte, responsable et créative, sans recours à une règle suprême. &lt;/p&gt; &lt;p&gt; Dans Des hégémonies brisées, Schürmann entreprend une vaste reconstruction de l’histoire de la philosophie occidentale comme succession d’« hégémonies » (modèles de vérité, de métaphysique, de politique) qui s’imposent, puis se défont. Il montre comment la modernité et la déconstruction heideggérienne ont dissous les grands systèmes de pensée, ouvrant à ce qu’il nomme une « philosophie tragique » où l’être se donne comme événement contingent, marqué par une distance, une fracture intérieure, plutôt que par une harmonie ou une cohérence totale. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="E17" r:id="rId4" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Ludwig_Feuerbach&quot;  title=&quot; Wikipedia&quot;&gt;Ludwig FEUERBACH&lt;/a&gt; était un philosophe bavarois qui a commencé sa carrière en défendant les idées hégéliennes, mais il s’est rapidement éloigné de l’idéalisme de Hegel, qu’il jugeait trop proche de la théologie chrétienne. Son ouvrage majeur, &lt;a href=&quot;https://www.youtube.com/watch?v=ni-uusn_4u4&quot;  title=&quot;Ludwig Feuerbach: Préface à la seconde édition de &quot;l'Essence du Christianisme&quot; par Le Gros Rouge qui Tache&quot;&gt;&quot; L’Essence du christianisme&quot;&lt;/a&gt; paru en 1841, constitue une critique radicale de la religion, où il affirme que Dieu n’est qu’une projection des qualités humaines, une aliénation par laquelle l’homme se dépossède de ses propres forces et valeurs. Cette idée a eu une influence majeure sur les penseurs de gauche, notamment Karl Marx, qui a repris et développé la notion  &lt;a href=&quot;https://www.youtube.com/watch?v=hCdmjaVFrts&quot; title=&quot;Feuerbach, dépasser l'aliénation religieuse vers le vrai humanisme par François Jourde&quot;&gt;d’aliénation chez Feuerbach&lt;/a&gt;. &lt;/p&gt; &lt;p&gt; Il développe une philosophie humaniste et sensualiste, plaçant l’homme et ses sentiments au centre de la réalité.​ Selon lui, la suppression de Dieu ne doit pas conduire à l’effondrement de la morale, mais au contraire à une responsabilité accrue de l’homme envers ses semblables.​ Il insiste sur l’importance de l’amour collectif et de l’altruisme comme fondements d’une société humaine authentique.​ &lt;/p&gt; &lt;p&gt; Il a profondément marqué la pensée du XIXe siècle, notamment par sa critique de la religion et son influence sur le matérialisme et le socialisme. Il a inspiré Marx, Engels et d’autres penseurs du mouvement ouvrier, tout en restant un philosophe indépendant, peu engagé dans la politique directe.​ Il est un penseur clé de  &lt;a href=&quot;https://books.openedition.org/pufc/40697?lang=fr&quot; title=&quot;Ludwig Feuerbach : la nature et la nature humaine comme fondement d’une praxis sociale et politique par Open Edition&quot;&gt;la transition&lt;/a&gt; entre l’idéalisme hégélien et le matérialisme moderne, dont la critique de la religion et la philosophie humaniste continuent d’inspirer la réflexion philosophique et sociale.  &lt;/p&gt; "/>
+    <hyperlink ref="E18" r:id="rId5" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Max_Stirner&quot;  title=&quot; Wikipedia&quot;&gt;Max STIRNER&lt;/a&gt;, de son vrai nom Johann Kaspar Schmidt était un philosophe bavarois, figure clé des Jeunes Hégéliens et précurseur de &lt;a href=&quot;https://www.youtube.com/watch?v=FG42gogWdCM&quot; title=&quot;L'anarchisme individualiste par Politikon&quot;&gt;l'anarchisme individualiste&lt;/a&gt; et de l'égoïsme philosophique. &lt;/p&gt; &lt;p&gt; Dans &quot;&quot;L'Unique et sa propriété&quot;, il rejette toutes les abstractions – Dieu, État, humanité, moralité, révolution – comme des &quot;spectres&quot; ou &quot;fixations&quot; qui aliènent l'individu au profit d'idées supérieures. Il prône l'&quot;égoïsme conscient&quot; : l'Unigue (le Moi unique) s'approprie ce qui lui est propre par la force de sa volonté, sans devoir ni norme externe.  &lt;a href=&quot;https://journals.openedition.org/rg/8578&quot; title=&quot;La philosophie politique de Max Stirner par OpenEdition&quot;&gt;Ce texte&lt;/a&gt; marque la fin de l'hégélianisme et annonce nihilisme, existentialisme et postmodernisme. &lt;/p&gt; &lt;p&gt; Il dissout le sujet en un &quot;Moi&quot; fluide, sans essence fixe ni mission universelle, opposé à l'idéalisme hégélien ou feuerbachien. Toute société repose sur des illusions collectives ; l'individu doit les détruire pour affirmer sa puissance propre, formant des unions temporaires par intérêt mutuel. Il critique le christianisme, le socialisme et le libéralisme comme autant de tyrannies déguisées.&lt;/p&gt; &lt;p&gt; Son radicalisme inspire l'anarchisme individualiste (bien qu'il le refuse), des illegalistes, existentialistes comme Nietzsche, et même des penseurs postmodernes ou libertariens. Marx lui consacre un long pamphlet dans L'Idéologie allemande, voyant en lui un danger pour le collectivisme. Redécouvert au XXe siècle, il reste un penseur &quot;inassimilable&quot; défiant toute allégeance. &lt;/p&gt; "/>
+    <hyperlink ref="E21" r:id="rId6" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Rudolf_Hermann_Lotze&quot;  title=&quot; Wikipedia&quot;&gt;Rudolf Hermann LOTZE&lt;/a&gt;  était un philosophe allemand, fils d'un médecin militaire, il étudie la médecine et la philosophie à l'université de Leipzig ou il enseigne ensuite, puis est nommé professeur de philosophie à Göttingen en 1844, succédant à Herbart, avant de rejoindre Berlin en 1880, où il décède l'année suivante. Sa carrière académique est marquée par une vaste érudition, alliant sciences naturelles et réflexion philosophique. Il est aussi poète et traducteur, ayant rendu Antigone de Sophocle en latin. &lt;/p&gt; &lt;p&gt; Il rejette à la fois le matérialisme et la philosophie romantique de la nature, critiquant la notion de &quot;force vitale&quot; popularisée par Schelling. Influencé par Leibniz, Hegel et Kant, il défend un &lt;a href=&quot;https://www.youtube.com/watch?v=H3FEXnD8Zb4&quot;  title=&quot;Hermann Lotze Microcosmus par The Spirit of hegel&quot;&gt;mécanisme explicatif &lt;/a&gt;  pour les phénomènes physiques, applicable à la biologie sans recourir à des causes surnaturelles. La téléologie n'est pour lui qu'un principe régulateur subjectif, compatible avec le mécanisme : l'ordre du monde exprime un dessein spirituel, mais la science doit s'en tenir aux lois causales. Dans ses travaux précoces comme De futurae biologiae principiis philosophicis (1838), il pose les bases d'une biologie philosophique rigoureuse. &lt;/p&gt; &lt;p&gt; Ses œuvres majeures, telles &lt;a href=&quot;https://journals.openedition.org/rgi/323&quot;  title=&quot;Hermann Lotze Microcosmus par openedition&quot;&gt;Mikrokosmos (1856-1864), &lt;/a&gt;  explorent l'être humain comme microcosme du monde, distinguant faits, lois et valeurs, unies dans la réalité mais séparées par notre pensée. Logik (1874) et Metaphysik (1879) forment un système philosophique quasi exhaustif, intégrant logique, ontologie et psychologie. Il y insiste sur les limites du langage et de la pensée, tout en proscrivant les déductions a priori spéculatives au profit d'une approche empirique et scientifique. Il fonde ainsi une psychologie scientifique, préfigurant des disciplines modernes. &lt;/p&gt; &lt;p&gt; Il  marque la transition entre l'idéalisme absolu post-hégélien et le néo-kantisme, évitant l'absolutisme idéaliste comme le réalisme atomistique. Il valorise les sciences naturelles tout en préservant une dimension éthique et téléologique : l'existence (Sein) doit être interprétée par son sens (Soll), via un langage des valeurs plutôt que des impératifs moraux stricts. Anti-naturaliste après la &quot;controverse du matérialisme&quot; de 1854, il intègre émotions et jugements de valeur à la connaissance humaine. &lt;/p&gt; &lt;p&gt; Son influence est immense jusqu'à la Première Guerre mondiale, impactant néo-kantiens, phénoménologues, positivistes logiques et même la psychologie anglo-saxonne via William James. En Allemagne, il ferme l'ère spéculative pour ouvrir une philosophie plus sobre et scientifique. Aux États-Unis, ses idées sur la causalité et la pensée relationnelle imprègnent le pragmatisme naissant. Il reste une figure pivot, liant science et métaphysique dans une vision unifiée de l'univers comme plan rationnel et spirituel. &lt;/p&gt; &#10;&#10;&#10;"/>
+    <hyperlink ref="E22" r:id="rId7" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl_Marx&quot;  title=&quot; Wikipedia&quot;&gt;Karl MARX&lt;/a&gt; était un philosophe, économiste et révolutionnaire allemand né à Trèves, est le fondateur  &lt;a href=&quot;https://www.youtube.com/watch?v=W_ZwUjnl4W4&quot;  title=&quot;La philosophie de Karl Marx par Parole de philosophe&quot;&gt;du marxisme &lt;/a&gt; avec Friedrich Engels. Issu d'une famille juive convertie au protestantisme, il étudie le droit et la philosophie à Bonn, Berlin et Iéna, où il est influencé par Hegel et les jeunes hégéliens comme David Strauss, dont il critique les idées religieuses dans sa jeunesse. Exilé en France puis en Angleterre après les révolutions de 1848, il vit dans la précarité à Londres, soutenu par Engels, et milite au sein de l'Internationale ouvrière. Son portrait de 1875 le montre barbu, pensif, incarnation du penseur engagé.   &lt;/p&gt; &lt;p&gt;    Sa philosophie repose sur le matérialisme historique et dialectique, voyant l'histoire comme une succession de modes de production (esclavagiste, féodal, capitaliste) mue par  &lt;a href=&quot;https://www.youtube.com/watch?v=1pYmqDnvTh8&quot;  title=&quot;Les classes sociales par DigiSchool Lycee &quot;&gt;la lutte des classes &lt;/a&gt; entre exploiteurs et exploités. Dans  &lt;a href=&quot;https://www.youtube.com/watch?v=jb-5oSF2dpU&amp;ab_channel=TanguyLacroix&quot;  title=&quot;Le Manifeste du Parti Communiste par Tanguy Lacroix &quot;&gt;&quot;Le Manifeste communiste  &lt;/a&gt; (1848), coécrit avec Engels, il appelle le prolétariat à abolir la propriété privée des moyens de production pour instaurer une société sans classes. Le Capital (1867-1883) analyse le capitalisme comme un système d'exploitation via la plus-value extraite du travail   &lt;a href=&quot;https://www.youtube.com/watch?v=rEAxxsX_um0&amp;t=4s&amp;ab_channel=LePr%C3%A9cepteur&quot;  title=&quot;L'Aliénation par le Précepteur &quot;&gt;salarié aliéné, &lt;/a&gt;  prédisant sa chute par ses contradictions internes. &lt;/p&gt; &lt;p&gt;  Il rejette la religion comme « opium du peuple », outil d'aliénation masquant l'exploitation réelle, et prône la praxis révolutionnaire : transformer le monde par l'action collective des travailleurs. Critiquant le libéralisme et le socialisme utopique, il envisage une dictature du prolétariat transitoire menant au communisme, où l'État dépérit et les besoins sont satisfaits selon les capacités. Ses idées opposent radicalement celles de Donoso Cortés, qui y voyait un aboutissement satanique du libéralisme. &lt;/p&gt;   &lt;p&gt; Sa contribution la plus importante à la théorie politique est sa conception du  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Mat%C3%A9rialisme_dialectique&quot;  title=&quot;Le Marxisme Dialectique par Wikipedia &quot;&gt;&quot;matérialisme dialectique&quot;&lt;/a&gt;, qui est l'idée que le changement historique est motivé par des conflits entre des classes sociales opposées et que ces conflits sont finalement résolus par la révolution. &lt;/p&gt; &lt;p&gt; Il a également écrit abondamment sur l'économie, en particulier sur la théorie de la valeur-travail, qui postule que la valeur d'un bien ou d'un service est basée sur la quantité de travail nécessaire pour le produire. &lt;/p&gt; &lt;p&gt;     Son influence sur le XXe siècle est immense : révolutions bolchevique, chinoise, mouvements ouvriers mondiaux, et disciplines comme la sociologie ou l'économie. Malgré les échecs des régimes « marxistes », sa critique du capitalisme reste débattue aujourd'hui. &lt;/p&gt;    &lt;audio controls title=&quot;Pour l'avenir par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10467-26.09.2020-ITEMA_22438423-2020C40092E0005-1779455909.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
+    <hyperlink ref="E23" r:id="rId8" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Friedrich_Engels&quot;   title=&quot; Wikipedia&quot;&gt;Friedrich ENGELS&lt;/a&gt;  était un  philosophe, théoricien socialiste allemand et le plus  &lt;a href=&quot;https://www.youtube.com/watch?v=K3GsK_RbVwI&quot; title=&quot;Friedrich Engels : Dans l'ombre de Marx, Arte 2024 par Crevoisier Philippe&quot;&gt;proche collaborateur&lt;/a&gt; de Karl Marx dans la fondation du marxisme et du communisme moderne. Son œuvre philosophique et politique a profondément marqué l'histoire intellectuelle et politique du XIXe siècle. Il travailla dans l'entreprise de son père, ce qui lui permet d'étudier directement les conditions de vie de la classe ouvrière britannique. C'est à cette époque qu'il rédige &quot;La Situation de la classe laborieuse en Angleterre&quot;, une analyse des conditions sociales des ouvriers. &lt;/p&gt; &lt;p&gt; En 1844, il rencontre Marx à Paris ; cette rencontre scelle leur collaboration intellectuelle et politique. Ensemble, ils écrivent plusieurs textes majeurs, notamment &quot;L’Idéologie allemande&quot; paru en 1845, &lt;a href=&quot;https://www.youtube.com/watch?v=xiJx1g91LYk&quot;  title=&quot;Marx, Engels - Manifeste du parti communiste  par Politikon&quot;&gt;&quot;Le Manifeste du Parti communiste&quot;&lt;/a&gt; en 1848, et fondent la Ligue des communistes. Après la mort de Marx, il prend en charge la publication des volumes II et III du &quot;Capital&quot;. Il fut un théoricien encyclopédique, passionné par la philosophie, les sciences, la littérature et l’histoire et il a anticipé certains développements scientifiques avec son ouvrage &quot;La dialectique de la nature&quot;, où il applique la méthode marxiste à l’étude des lois de la nature. &lt;/p&gt; &lt;p&gt; Il a conceptualisé le matérialisme historique avec Marx, affirmant que ce sont les conditions matérielles – et non les idées ou la conscience – qui déterminent le cours de l’histoire. Il l'a aidé financièrement et a mis sa capacité d'organisation au service du mouvement révolutionnaire européen. Sa pensée sur le matérialisme dialectique et la transformation sociale demeure une référence centrale dans les sciences humaines et politiques.Il est également reconnu pour ses analyses sur l’origine de la famille, de la propriété privée et de l’État.  &lt;/p&gt; &lt;audio controls title=&quot; Friedrich Engels, penser le marxisme à deux par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10081-24.10.2024-ITEMA_23903110-2024C29629S0298-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
+    <hyperlink ref="E24" r:id="rId9" display="&lt;p&gt;&lt;a href=&quot;https://en.wikipedia.org/wiki/Gustav_Teichm%C3%BCller&quot;  title=&quot; Wikipedia&quot;&gt;Gustav TEICHMÜLLER&lt;/a&gt; était un philosophe allemand, professeur à Bâle puis à Dorpat (aujourd’hui Tartu, en Estonie), considéré comme le fondateur du personnalisme russe et l’une des figures majeures de l’idéalisme tardif du XIXe siècle. Né à Braunschweig, formé à Berlin et Tübingen, il enseigne d’abord en Allemagne, puis en Suisse, avant d’occuper la chaire de philosophie de Tartu de 1871 jusqu’à sa mort en 1888, où il forme toute une génération de philosophes, dont Jēkabs Osis. &lt;/p&gt; &lt;p&gt; Il élabore, surtout à partir des années 1880, une « nouvelle philosophie » qu’il qualifie lui-même de personnalisme, à la fois contre l’idéalisme absolu (de type hégélien) et contre le matérialisme ou le positivisme de son temps. Son objectif central est de « sauver la personne » : il veut retrouver la réalité concrète des individus conscients, perdue selon lui dans les systèmes qui réduisent le monde à des représentations, à un Esprit unique ou à de la matière inerte. Pour lui, la réalité ultime est constituée de substances psychiques individuelles (des monades, des âmes), chacune étant un centre actif de conscience, de sentiment et de volonté. &lt;/p&gt; &lt;p&gt; Dans son ouvrage principal, Die wirkliche und die scheinbare Welt (Le monde réel et le monde apparent, 1882), il distingue le monde tel qu’il est en soi (un système de personnes/monades) et le monde tel qu’il nous apparaît à travers nos représentations. Il développe une forme de perspectivisme : chaque sujet connaît le monde depuis son point de vue propre, ce qui rend toute connaissance à la fois partielle et dépendante de la structure de la personne connaissante. Cette idée influence notamment Friedrich Nietzsche, qui reprend et transforme le motif perspectiviste dans sa propre critique de la vérité et de la métaphysique traditionnelle. &lt;/p&gt; &lt;p&gt; Il est aussi l’un des premiers à pratiquer systématiquement l’histoire des concepts (Begriffsgeschichte), en étudiant la genèse et les transformations des notions philosophiques majeures (être, substance, personne, etc.). Ce travail prépare, à long terme, des projets comme le Historisches Wörterbuch der Philosophie. Par son enseignement à Tartu et ses écrits, il fonde le personnalisme russe et marque durablement la philosophie lettone et estonienne, en faisant de la personne le centre d’une métaphysique qui cherche à concilier rigueur conceptuelle et respect de la réalité concrète des individus. &lt;/p&gt;&#10;"/>
+    <hyperlink ref="H24" r:id="rId10" display="https://www.laphilo.fr/pho/gteichmuller-mini.webp"/>
+    <hyperlink ref="I24" r:id="rId11" display="https://www.laphilo.fr/photo/gteichmuller.webp"/>
+    <hyperlink ref="E32" r:id="rId12" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Wilhelm_Windelband&quot;  title=&quot; Wikipedia&quot;&gt;Wilhelm WINDELBAND&lt;/a&gt;  était un philosophe allemand  fondateur de l'école néokantienne de Bade (ou du Sud-Ouest), aux côtés de Heinrich Rickert, avec qui il forme un duo clé du  &lt;a href=&quot;https://www.youtube.com/watch?v=h2R8wj7Q9x8&quot;  title=&quot;Néo-kantisme : définition, exemples. par le Savoir partagé&quot;&gt;néokantisme tardif &lt;/a&gt;. Élève initialement influencé par la psychologie, il évolue vers un néokantisme anti-psychologiste, critiquant le relativisme historiciste et posant les bases d'une philosophie des valeurs. &lt;/p&gt; &lt;p&gt; Il distingue &lt;a href=&quot;https://www.youtube.com/watch?v=Rr96FJSOcDU&quot; title=&quot; Wilhelm Windelband: Philosophy of Values and History par Philosopher Friends&quot;&gt;les sciences &lt;/a&gt; nomothétiques (lois générales, comme la physique) des sciences idiographiques (individuel, historique), cette dichotomie méthodologique influençant Max Weber et la philosophie des sciences. Sa &quot;philosophie des valeurs&quot; transpose la critique kantienne vers la normativité : vérité, bien, beauté comme exigences objectives, sans recours au psychologisme ni au métaphysique spéculative. &lt;/p&gt; &lt;p&gt; Ses oeuvres principales sont : - &quot;Histoire de la philosophie du Nouveau Temps' paru en 1880 et &quot;Histoire du problème philosophique de la liberté&quot; en 189 : synthèses historiques rigoureuses, voyant l'histoire de la philosophie comme science autonome. - &quot;Präludien&quot; en 1884, recueils d'essais : expose sa critique de la psychologie comme fondement du savoir et sa reformulation kantienne en termes normatifs. &lt;/p&gt; &lt;p&gt; Précurseur de la phénoménologie et des sciences humaines modernes, il impacte Rickert, Weber (types idéaux) et Jaspers, bien que moins systématique que les néokantiens de Marbourg. &lt;/p&gt; "/>
+    <hyperlink ref="E34" r:id="rId13" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Sigmund_Freud&quot;  title=&quot; Wikipedia&quot;&gt; Sigmund FREUD&lt;/a&gt; est un neurologue et philosophe Allemand connu pour son travail sur la Psychanalyse et son point de vue sur  &lt;a  href=&quot;https://www.youtube.com/watch?v=uYd0Xi3ACQ8&amp;t=17s&amp;ab_channel=LePr%C3%A9cepteur&quot;  title=&quot;L'origine de la religion par Le Précepteur&quot;&gt;la Religion&lt;/a&gt;. &lt;/p&gt; &lt;p&gt;  Et si ce n’était pas la raison et la volonté, mais l’inconscient et ses pulsions violentes et destructrices, qui étaient la grande force de l’esprit et de l’histoire ? Voilà l’hypothèse scandaleuse qui est au cœur de l’œuvre de Freud. &lt;/p&gt; &lt;p&gt; Si l’idée d’une vie psychique inconsciente avait déjà été envisagée par d’autres, de Leibniz à Schopenhauer et Nietzsche, Freud est le premier à en faire l’objet d’une méthode d’investigation et de soin : la psychanalyse. &lt;a  href=&quot;/document/le_reve_et_son_interpretation.pdf&quot;  title=&quot;Le rêve et son interprétation en version numérique&quot;&gt;&quot;Le rêve et son interprétation&quot;&lt;/a&gt;, publié en 1900, fait de l’analyse des rêves la « voie royale » pour aborder l’inconscient.&lt;/p&gt; &lt;p&gt;  Il est amené à repenser son modèle pour en accentuer la dimension conflictuelle entre ce qu’il nomme désormais &lt;a  href=&quot;https://www.youtube.com/watch?v=QO7HTLC0r6I&amp;ab_channel=Coursitout&quot; title=&quot;Le ça, le moi et le surmoi par Coursitout&quot;&gt;le « Ça », le « Moi » et le « Surmoi »&lt;/a&gt;. &lt;/p&gt; &lt;p&gt; Le Ça, correspondant à l’inconscient, est la partie obscure et inaccessible de notre personnalité. Le Moi, socle de la personnalité, est l’instance intermédiaire qui doit concilier les exigences contradictoires du Ça et du Surmoi. Le Surmoi, lui, est le juge intérieur qui naît de l’intériorisation des interdits sociaux. &lt;/p&gt; &lt;p&gt; Si  &lt;a  href=&quot;https://www.youtube.com/watch?v=b_v6YfaC5gU&amp;t=17s&amp;ab_channel=LePr%C3%A9cepteur&quot;  title=&quot;L'inconscient par Le Précepteur&quot;&gt;l’inconscient&lt;/a&gt; est ce chaos au cœur de l’individu, il devient le cœur du processus de civilisation. &lt;/p&gt; &lt;p&gt; En 1933, les œuvres de Freud sont brûlées par les Nazis mais le travail de Freud n’en reste pas moins incontournable dans l’histoire de la psychologie moderne. Sa postérité est immense. &lt;/p&gt;  &lt;audio controls title=&quot;L'Ombilic des rêves par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/19288-29.07.2018-ITEMA_21741416-2.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; &#10;&#10;"/>
+    <hyperlink ref="E36" r:id="rId14" display="&lt;p&gt; &lt;a href=&quot;https://fr.wikipedia.org/wiki/Edmund_Husserl&quot;  title=&quot; Wikipedia&quot;&gt; Edmund HUSSERL&lt;/a&gt; était un philosophe allemand d'origine juive connu pour être le fondateur de la  &lt;a href=&quot;https://www.youtube.com/watch?v=VaXxW0M9aIY&quot;  title=&quot;Intro à la phénoménologie par Le Precepteur&quot;&gt; phénoménologie&lt;/a&gt; qui est une méthode philosophique qui vise à décrire les structures de l'expérience telles qu'elles se présentent à la conscience, sans présuppositions théoriques ou métaphysiques. Il appelle cette approche &quot;retour aux choses mêmes&quot;, ce qui signifie qu'il faut se concentrer sur les phénomènes tels qu'ils apparaissent à la conscience, plutôt que sur des interprétations ou des constructions théoriques. &#10;Ses oeuvres les plus importantes : &lt;/p&gt; &lt;p&gt; -  &quot;Idées directrices pour une phénoménologie pure et une philosophie phénoménologique&quot; : il  y développe sa méthode de réduction phénoménologique et introduit le concept d'intentionnalité. &lt;/p&gt; &lt;p&gt; - &lt;a href=&quot;https://www.persee.fr/doc/phlou_0035-3841_1954_num_52_33_4479&quot;   title=&quot;Méditation cartésiennes par Persee&quot;&gt; &quot;Méditations cartésiennes&quot;&lt;/a&gt; : Une série de conférences où il approfondit sa pensée sur l'ego transcendantal et l'intersubjectivité.&lt;/p&gt; &lt;p&gt; - &quot;Recherches logiques&quot; (1900-1901) : Dans cet ouvrage, il critique le psychologisme (l'idée que les lois logiques sont des lois psychologiques) et pose les bases de sa phénoménologie.&lt;/p&gt; &lt;p&gt; - &quot;La crise des sciences européennes et la phénoménologie transcendantale&quot; (1936) : Dans cet ouvrage posthume, il analyse la crise des sciences modernes et propose une refondation philosophique basée sur la phénoménologie.&lt;/p&gt; &lt;p&gt; Il a tenté de développer une méthode pour explorer la nature de la conscience humaine. Il a cherché à comprendre comment nous percevons le monde à travers nos sens, comment nous avons des pensées et des émotions, et comment nous nous rapportons à nous-mêmes et aux autres. &lt;/p&gt; &lt;p&gt; &#10;La phénoménologie de Husserl a influencé de nombreux philosophes et écoles de pensée, notamment l'existentialisme (Sartre) , la psychanalyse (Freud) et la philosophie de la perception. Ses travaux ont également inspiré des mouvements culturels tels que l'art abstrait et le modernisme.  &lt;/p&gt; &lt;audio controls title=&quot;Le phénomène Husserl par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/18755-09.03.2020-ITEMA_22302657-2.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
+    <hyperlink ref="E37" r:id="rId15" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Lou_Andreas-Salom%C3%A9&quot; title=&quot; Wikipedia&quot;&gt;Lou ANDRÉAS-SALOMÉ&lt;/a&gt; était une écrivaine, philosophe, essayiste et psychanalyste allemande qui défendit une vision de la liberté incluant l'indépendance intellectuelle, émotionnelle et sexuelle. Elle rejette les conventions sociales et les rôles de genre traditionnels.  Ses principales oeuvres : &lt;/p&gt; &#10;&lt;p&gt; - Friedrich Nietzsche à travers ses œuvres (1894) : Elle y analyse la philosophie de Nietzsche, en mettant l'accent sur ses idées sur la volonté de puissance, l'éternel retour et la mort de Dieu.  &lt;/p&gt; &#10;&lt;p&gt; -  Rainer Maria Rilke (1928) : Elle l'écrit après la mort de Rilke et elle y explore sa relation avec le poète et analyse son œuvre, en mettant l'accent sur sa quête spirituelle et artistique. &lt;/p&gt; &#10;&lt;p&gt; - L'Érotisme (1910) : Elle explore la nature de l'érotisme et de la sexualité, en s'appuyant sur des réflexions psychologiques et philosophiques et défend une vision libérée et complexe de la sexualité. &lt;/p&gt; &#10;&lt;p&gt; -  Ma vie ( publié à titre posthume) : Dans son autobiographie, elle raconte &lt;a href=&quot;https://scienceetbiencommun.pressbooks.pub/femmessavantes3/chapter/lou-andreas-salome-femme-de-lettres-et-psychanalyste-1861-1937/&quot; title=&quot;  Lou Andréas-Salomé, femme de lettres et psychanalyste par esbc&quot;&gt;sa vie &lt;/a&gt;, ses relations et ses réflexions intellectuelles. &lt;/p&gt;  &lt;p&gt; Bien qu'elle ne se définisse pas comme féministe, elle défend une vision de la femme comme être indépendant et complexe. Elle s'intéresse à la spiritualité et à la religion, en particulier dans ses écrits sur Nietzsche et Rilke. Elle explore des thèmes comme la quête de sens, la transcendance et la relation entre l'homme et le divin. &lt;/p&gt; &lt;p&gt;  Elle est l'une des &lt;a href=&quot;https://www.youtube.com/watch?v=SlLT7BXn_YI&quot; title=&quot; First Female Psychoanalyst: Lou Andreas Salomé par Orbit&quot;&gt;premières femmes psychanalystes &lt;/a&gt; et ses écrits et ses réflexions ont contribué a son développement, en particulier dans les domaines de la sexualité et des relations humaines. &lt;/p&gt;  &lt;audio controls title=&quot;Lou Andreas-Salomé, la revendication d'un moi féminin libre par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13915-16.08.2022-ITEMA_23103839-2021C3372E0235-NET_MFC_5D82F295-9FBD-4DEC-9B93-3E80E99A02A8-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;  "/>
+    <hyperlink ref="E39" r:id="rId16" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hans_Driesch&quot; title=&quot; Wikipedia&quot;&gt;Hans DRIESCH&lt;/a&gt;  était un zoologiste, biologiste et philosophe allemand, fils unique d'un négociant prospère de Hambourg, il grandit dans un environnement propice à développer une vocation précoce de zoologiste : sa mère élevait des oiseaux exotiques et toutes sortes d'animaux, remplissant la maison de cages et de vivariums. Il devient en 1912 professeur de philosophie à Heidelberg, enseignera ensuite à Cologne en 1919, puis à Leipzig en 1921. En 1922-1923, il donne des cours en Chine aux universités de Nankin et Pékin, en 1926-1927 aux États-Unis à l'université du Wisconsin, et en 1928 à l'université de Buenos Aires. Le régime nazi le met d'office à la retraite en 1933, mais il continue à travailler jusqu'à sa mort survenue en pleine guerre. &lt;/p&gt; &lt;p&gt; En 1891, il réalise une expérience fondamentale : il dissocie deux blastomères d'oursin et montre que chacun se développe en une larve complète, bien que plus petite que la moyenne. Cette découverte contredit la théorie de Wilhelm Roux (1888) sur le développement en mosaïque, qui affirmait que chaque cellule initiale avait un rôle précis et formait seulement une partie de l'embryon. En 1892, il procède à une autre expérience capitale en comprimant les œufs d'oursin au stade de division en quatre cellules, déplaçant les noyaux anarchiquement dans le cytoplasme : les larves obtenues sont parfaitement normales, prouvant que tous les noyaux sont équivalents et renferment tous les gènes. Il a ainsi défendu l'épigenèse contre le préformisme et fait faire à l'embryologie un grand bond en avant. &lt;/p&gt; &lt;p&gt; Il  est le dernier grand &lt;a href=&quot;https://fr.wikipedia.org/wiki/Vitalisme&quot;  title=&quot;vitalisme par wikipedia&quot;&gt;porte-parole du vitalisme,&lt;/a&gt;  la théorie selon laquelle la vie ne peut être expliquée comme un phénomène purement physique ou chimique. Vers 1895, il devient un vitaliste convaincu. Il introduit le concept aristotélicien d'entéléchie pour désigner une force vitale qui régule le développement organique vers un but. Cette entéléchie est une force vitale logée dans l'œuf, tendant toujours vers le même but, expliquant pourquoi une cellule séparée peut donner une larve entière. &lt;/p&gt; &lt;p&gt; Il  apparaît comme une  &lt;a href=&quot;https://www.persee.fr/doc/phlou_0776-555x_1930_num_32_28_2598_t1_0464_0000_3&quot;  title=&quot;l’homme et le monde par persée&quot;&gt;figure originale &lt;/a&gt; tant parmi les scientifiques que parmi les philosophes, ayant introduit la biologie comme nouveau continent au sein de la réflexion philosophique. Sa philosophie de l'organique est étroitement liée à ses recherches biologiques. Toutefois, les théories vitalistes qu'il défendait sont aujourd'hui complètement abandonnées. On doit lui reconnaître le mérite d'avoir stimulé le progrès de l'embryologie expérimentale et d'avoir ouvert à la biologie de vastes perspectives. &lt;/p&gt; &#10;&#10;&#10;"/>
+    <hyperlink ref="H40" r:id="rId17" display="https://www.laphilo.fr/pho/rluxemburg-mini.webp"/>
+    <hyperlink ref="E41" r:id="rId18" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Theodor_Lessing&quot; title=&quot; Wikipedia&quot;&gt;Theodor LESSING&lt;/a&gt;  était un philosophe, essayiste et publiciste allemand &lt;a href=&quot;https://www.persee.fr/doc/rjuiv_0484-8616_1996_num_155_1_2554&quot;  title=&quot;Lessing et le sionisme par persée&quot;&gt;d’origine juive, &lt;/a&gt; connu comme un penseur critique de la modernité, du nationalisme et de l’antisémitisme. &lt;/p&gt; &lt;p&gt; Il s’inscrit surtout dans une philosophie de la culture et une philosophie sociale critique. Son travail ne cherche pas à construire un système abstrait, mais à analyser les maladies de la civilisation moderne, la violence des masses, la guerre, la ville industrielle et la destruction du vivant. Sa pensée est marquée par un humanisme pessimiste et engagé qui dénoncé le militarisme, la brutalisation de la société et les dérives autoritaires de l’Allemagne de Weimar, allant jusqu’à prévoir le danger nazi avant 1933. Il fut aussi l’un des premiers à réfléchir à la condition des minorités et à ce qu’il a appelé le &lt;a href=&quot;https://www.sifriatenou.com/2020/10/20/5449/&quot;  title=&quot;lessing la haine de soi par sifriatenou&quot;&gt;« judaïsme de haine de soi »,&lt;/a&gt; pour décrire les effets psychologiques de l’antisémitisme sur les Juifs eux-mêmes. &lt;/p&gt; &lt;p&gt; Il est également une figure de la critique écologique avant l’heure. Dès les années 1930, il s’inquiète de la déforestation, de la pollution urbaine et d’un possible dérèglement du climat, ce qui le rend étonnamment actuel. Il voit la modernité technique non comme un progrès neutre, mais comme une force capable de détruire les équilibres humains et naturels. &lt;/p&gt; &lt;p&gt; Sur le plan politique, il est un intellectuel indépendant, polémique et souvent isolé, qui s’oppose à l’autoritarisme autant qu’aux conformismes de son époque. Il a &lt;a href=&quot;https://www.youtube.com/watch?v=pdcxbRYcn&quot;  title=&quot;lessing par jacques Aron et Editions harmattan&quot;&gt;fini assassiné en exil &lt;/a&gt;  à Mariánské Lázně par des nationalistes sudètes, devenant l’une des premières victimes du nazisme hors d’Allemagne. &lt;/p&gt; &#10;"/>
+    <hyperlink ref="E42" r:id="rId19" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Max_Scheler&quot; title=&quot; Wikipedia&quot;&gt;Max SCHELER&lt;/a&gt;  était un philosophe allemand, figure phare de la phénoménologie et de l’anthropologie philosophique, dont l’œuvre traverse des domaines variés comme l’éthique, l’axiologie et la sociologie de la connaissance. &lt;/p&gt; &lt;p&gt; Il élabore une &lt;a href=&quot;https://www.persee.fr/doc/phlou_0776-555x_1927_num_29_14_2467&quot;  title=&quot;La philosophie de M. Scheler. Son analyse de la sympathie et de l'amour par Persée&quot;&gt;hiérarchie des valeurs &lt;/a&gt; qui va des valeurs de l’agréable et du désagréable jusqu’aux valeurs spirituelles (beau/laid, juste/injuste, connaissance, et enfin le sacré et le profane). Cette hiérarchie sert de base à une éthique et à une phénoménologie de la sensation et des sentiments qui orientent l’action humaine. Il propose une approche phénoménologique qui insiste sur &quot;l’attitude spirituelle&quot; ou &quot;l’œil vivant&quot; vers le monde, en s’opposant à une réduction purement méthodologique et en valorisant l’intuition des valeurs telles qu’elles se donnent à la conscience. &lt;/p&gt; &lt;p&gt; Il fonde l’idée d’une anthropologie philosophique qui cherche à comprendre l’homme dans le vivant et ses rapports au monde, en intégrant des connaissances des sciences naturelles et des sciences humaines. &lt;a href=&quot;https://www.youtube.com/watch?v=pPuUoTPig7w&quot; title=&quot;Le salut vient-il du travail ? - Valeur et dignité du travail selon Max SCHELER par Editions M-Editer&quot;&gt;Cette orientation &lt;/a&gt; mène plus tard à une sociologie de la connaissance. Voici ses oeuvres majeures : &lt;/p&gt; &lt;p&gt; - &quot;Die Wissensformen und die Gesellschaft&quot; paru en 1926 – synthèse de son projet de sociologie de la connaissance et jalon important de l’anthropologie philosophique et sociale. Cette œuvre est souvent citée comme fondatrice d’une approche sociologique qui rejoint les débats de Weimar.&lt;/p&gt; &lt;p&gt; - &quot;Stellung des Menschen im Kosmos&quot; paru en 1928 – portrait philosophique de l’homme dans le cadre d’un ensemble plus large d’ouvrages préfigurant l’anthropologie philosophique et son intérêt pour le positionnement de l’homme dans l’ordre du vivant. &lt;/p&gt; &lt;p&gt; Son approche personnaliste et son engagement en faveur d’une philosophie sociale et éthique centrée sur la dignité humaine, &lt;a href=&quot;https://www.youtube.com/watch?v=HHAKQrNdMYk&quot; title=&quot;&#10;Le ressentiment détruit ta vie… (Max Sheller, l'homme du ressentiment) par Timothée Delahaye&quot;&gt;le resentiment &lt;/a&gt; et les valeurs morales continuent d’être discutés dans les études contemporaines, notamment dans les analyses qui situent Scheler dans le dialogue franco-allemand et dans les traditions de philosophie sociale et morale. &lt;/p&gt; "/>
+    <hyperlink ref="E45" r:id="rId20" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hermann_von_Keyserling&quot; title=&quot; Wikipedia&quot;&gt;Hermann Von KEYSERLING&lt;/a&gt;  était un philosophe  &lt;a href=&quot;https://www.persee.fr/doc/slaoc_1245-2491_1997_num_4_1_1809&quot; style=&quot;color:#88A1E9&quot; title=&quot; Hermann von Keyserling et les interférences germano-slaves par Persée&quot;&gt;germano-balte &lt;/a&gt; devenu philosophe voyageur, figure très en vue de la République de Weimar, connu pour son Journal de voyage d’un philosophe et pour son &quot;École de la sagesse&quot; à Darmstadt. &lt;/p&gt; &lt;p&gt; Il conçoit la philosophie non comme une science rigoureuse, mais comme sagesse vécue : &quot;la vie elle-même sous la forme du savoir&quot;, contre les théories objectivantes du savoir technico-scientifique. Il s’inscrit dans la philosophie de la vie, mais de façon personnelle : importance de l’intuition, de la singularité des événements et de la transformation intérieure. Son projet est une nouvelle synthèse de l’âme et de l’esprit, la pénétration réciproque de sagesse et politique, et l’idée que dans la vie déterminée par l’esprit, c’est &lt;a href=&quot;https://www.youtube.com/watch?v=Y0DY8F72114&quot; title=&quot;Eduard von Keyserling, DUMALA par Le Veilleur&quot;&gt;le Sens &lt;/a&gt; qui crée les faits plutôt que l’inverse. &lt;/p&gt; &lt;p&gt; Il  utilise très tôt le terme Führerprinzip, en liant l’idée de &quot;dirigeants nés&quot; à un élitisme spiritualiste et social-darwinien, tout en refusant par la suite d’adhérer au national-socialisme, qu’il voit comme mouvement de masses manipulées.  Le régime nazi ferme son École de la sagesse au milieu des années 1930, lui interdit de publier et de voyager, tandis que sa réputation continue de grandir à l’étranger. &lt;/p&gt;&lt;p&gt; Ses oeuvres principales sont : - &quot;Reisetagebuch eines Philosophen&quot;  paru en 1919 : récit de son tour du monde (1911-1912, Asie, Amérique, Europe du Sud) mêlant observations culturelles, méditations spirituelles et diagnostics sur les civilisations ; c’est son grand succès de librairie, largement traduit. -&quot;Das Gefüge der Welt. Versuch einer kritischen Philosophie&quot; (La Structure du monde, 1907) : tentative de &quot;philosophie critique&quot; personnelle, déjà marquée par l’idée que le savoir véritable est inséparable de la vie. - &quot;Schöpferische Erkenntnis&quot; (Connaissance créatrice) et &quot;Wiedergeburt&quot; (Renaissance) : textes doctrinaux de l’&quot;École de la sagesse&quot;, insistant sur la connaissance comme acte créateur, transformant la vie plutôt que la décrivant objectivement. &lt;/p&gt; "/>
+    <hyperlink ref="E46" r:id="rId21" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Moritz_Schlick&quot;  title=&quot; Wikipedia&quot;&gt;Moritz SCHLICK&lt;/a&gt; était un philosophe allemand, physicien de formation, et l’une des figures centrales de l’empirisme logique. Il est surtout connu comme le fondateur et le dirigeant intellectuel du Cercle de Vienne, groupe qui se réunissait autour de la philosophie des sciences dans les années 1920 et 1930. Il occupa à Vienne une chaire autrefois associée à Ernst Mach et à Ludwig Boltzmann. &lt;/p&gt; &lt;p&gt; Sa première grande œuvre est la Théorie générale de la connaissance (Allgemeine Erkenntnislehre, 1918). Dans cet ouvrage, il défend encore une forme de réalisme scientifique : le monde extérieur existe indépendamment de nous et peut être connu grâce aux sciences. Il s’oppose ainsi à l’idéalisme et à l’idée kantienne selon laquelle nous ne connaîtrions jamais les choses en elles-mêmes. Pour lui, connaître consiste notamment à coordonner des signes et des concepts avec les objets et les processus étudiés par les sciences. &lt;/p&gt; &lt;p&gt;  À partir des années 1920, son orientation évolue sous l’influence de Wittgenstein et du développement de la logique moderne. Il affirme alors que la philosophie ne doit pas construire une nouvelle vision métaphysique du monde, mais clarifier le sens des propositions. Une &lt;a href=&quot;https://encyclo-philo.fr/schlick-a&quot;  title=&quot;l’encyclopedie philosophique : schick par encyclophilo&quot;&gt;proposition authentiquement scientifique &lt;/a&gt; doit pouvoir être reliée à une méthode possible de vérification empirique ; les énoncés de logique et de mathématiques sont, quant à eux, analytiques ou tautologiques. Cette orientation est souvent résumée par la formule : « le sens d’une proposition est sa méthode de vérification ». &lt;/p&gt; &lt;p&gt; Il faut cependant éviter de le réduire à un vérificationnisme simpliste. Il admet qu’une proposition puisse être vérifiable en principe, même si la vérification ne peut pas être réalisée immédiatement ou matériellement. La vérification ne signifie donc pas forcément une observation actuelle, mais la possibilité de décrire une procédure permettant de déterminer si l’énoncé est vrai ou faux. Sur le plan éthique, Il ne pense pas que les jugements de valeur soient des connaissances scientifiques ; il leur accorde néanmoins une importance dans la vie humaine et dans l’analyse des motivations. &lt;/p&gt; &lt;p&gt; On peut le classer comme un philosophe des sciences, un empiriste logique, &lt;a href=&quot;https://www.youtube.com/watch?v=ESWQzsf1Fr4&quot;  title=&quot;la fin du positivisme logique par philo analytique&quot;&gt;un positiviste logique &lt;/a&gt; et un représentant de la philosophie analytique naissante. Il est plus central et plus systématique que Hans Hahn dans l’organisation du Cercle de Vienne, tandis que Hahn était avant tout mathématicien et philosophe des fondements des mathématiques. Sa pensée se situe à la rencontre du réalisme scientifique, de l’empirisme, de l’analyse logique du langage et de l’anti-métaphysique ; son projet fondamental était de faire de la philosophie une activité de clarification au service de la connaissance scientifique. &lt;/p&gt; &#10;"/>
+    <hyperlink ref="H46" r:id="rId22" display="https://www.laphilo.fr/pho/mschlick-mini.webp"/>
+    <hyperlink ref="E48" r:id="rId23" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl_Korsch&quot; title=&quot; Wikipedia&quot;&gt;Karl KORDCH&lt;/a&gt;  était un philosophe marxiste allemand,  théoricien du communisme de conseils et critique du léninisme orthodoxe. Issu d'un milieu bourgeois, il évolua du réformisme social au marxisme hétérodoxe, influençant les courants ultra-gauche via son rejet du matérialisme positiviste et son insistance sur la praxis révolutionnaire historique.  Exclu du parti en 1926 pour &quot;ultra-gauchisme&quot;, il émigra après 1933 vers les USA, où il approfondit sa théorie marxiste. &lt;/p&gt; &lt;p&gt; Son œuvre majeure &quot;Marxisme et philosophie&quot; paru en 1923 marque sa rupture avec le léninisme en critiquant sa dérive scientiste. Il   &lt;a href=&quot;https://www.zones-subversives.com/article-le-marxisme-critique-de-karl-korsch-116431466.html&quot;  title=&quot;Le marxisme critique de Karl Korsch par Chroniques critiques&quot;&gt;rejette le marxisme &lt;/a&gt; comme &quot;science positive&quot; figée ou philosophie matérialiste abstraite ; il le conçoit comme une théorie historique et concrète, liée à la lutte des classes et à la dialectique hégélienne réinterprétée comme expression de la révolution bourgeoise puis prolétarienne. &lt;/p&gt; &lt;p&gt; Il  théorise les conseils comme organes centraux de la transition socialiste, via la praxis dialectique et l'auto-activité des masses, contre la socialisation étatique. Ses écrits inspirent le KAPD et l'ultra-gauche, voyant les conseils comme alternative à la bureaucratisation stalinienne. Son influence perdure chez les communistes de conseils, soulignant la conscience ouvrière spontanée pour l'émancipation réelle. &lt;/p&gt; "/>
+    <hyperlink ref="E51" r:id="rId24" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Eugen_Rosenstock-Huessy&quot; title=&quot; Wikipedia&quot;&gt;Eugen ROSENSTOCK-HUESSY&lt;/a&gt; était un penseur germano‑américain dont l'œuvre mêle philosophie sociale, histoire des idées et une théorie du langage centrée sur la parole comme acte créateur et structurant de la vie collective. Né en Allemagne, il forma des liens intellectuels avec des figures comme Franz Rosenzweig et Martin Buber, fut professeur (notamment aux États‑Unis après son exil) et créa une œuvre originale qui vise à comprendre comment les communautés se constituent et se transforment dans le temps par des échanges de parole. &lt;/p&gt; &lt;p&gt; Au  &lt;a href=&quot;https://www.en-attendant-nadeau.fr/2019/11/19/homme-quadridimensionnel-rosenstock//&quot;  title=&quot;l’homme quadridimensionnel par ean&quot;&gt;cœur de sa pensée &lt;/a&gt;  se trouve la notion de &quot;speech thinking&quot; (pensée de la parole) : il soutient que la parole n’est pas qu’un moyen descriptif, mais un acte répondant et créatif qui institue des relations sociales, forge des temporalités collectives et permet la transmission et la renouvellement des institutions humaines. Il affirme que, par le langage, les groupes deviennent « maîtres du temps » en fondant de nouveaux commencements, en rappelant le passé et en orientant l’action future — d’où son intérêt pour la densité historique de la vie sociale et le rôle des rituels, des serments et des discours publics. &lt;/p&gt; &lt;p&gt; Sur la religion et la théologie, il s’inscrit dans un courant post‑nietzschéen de renouveau religieux qui comprend Rosenzweig et Buber; il considère les énoncés religieux comme des actes de parole non‑métaphysiques qui dévoilent des dimensions de l’expérience humaine et communautaire inaccessibles aux seules sciences naturelles. Cette orientation le conduit à une pensée intégrative où philosophie, théologie et histoire participent à une réflexion pratique sur la transformation sociale et la responsabilité collective. &lt;/p&gt; &lt;p&gt; Ses livres et conférences couvrent une grande variété de thèmes — histoire des peuples, rhétorique sociale, philosophie de la loi et de l’éducation — et sa méthode combine analyses historiques, typologies du langage et propositions pour renouveler la vie civique; son influence se voit aujourd’hui dans des études sur la communication, la sociologie historique et la philosophie de la culture. &lt;/p&gt; "/>
+    <hyperlink ref="H51" r:id="rId25" display="https://www.laphilo.fr/pho/erhuessy-mini.webp"/>
+    <hyperlink ref="E53" r:id="rId26" display="&lt;p&gt; &lt;a href=&quot;https://fr.wikipedia.org/wiki/Oskar_Becker&quot;  title=&quot; Wikipedia&quot;&gt;Oskar BECKER&lt;/a&gt; était un philosophe, logicien, mathématicien et historien des mathématiques allemand, connu comme l’un des élèves les plus importants d’Edmund Husserl et comme un interlocuteur clé de Martin Heidegger. Sa pensée se situe à la croisée de la phénoménologie, de la philosophie des mathématiques, de la logique modale et de l’existentialisme. &lt;/p&gt; &lt;p&gt; Il utilise la phénoménologie husserlienne pour analyser les fondements de la géométrie, de l’arithmétique et de la logique, en cherchant à décrire les expériences vécues (compter, mesurer, démontrer) comme actes de conscience. Il tente ainsi de fonder une  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Ph%C3%A9nom%C3%A9nologie&quot;  title=&quot;phénoménologie par wikipedia&quot;&gt; sémantique phénoménologique &lt;/a&gt; de la logique intuitionniste, et ses idées sont reprises par Arend Heyting dans sa formalisation de cette logique. À la fin de sa vie, il insiste sur une distinction entre une intuition du domaine formel et platonicien (mathématiques pures) et un domaine existentiel concret, en utilisant parfois un vocabulaire proche de la « divination ». &lt;/p&gt; &lt;p&gt;Il est aussi un pionnier de la logique modale (logique de la nécessité et de la possibilité). On lui doit notamment ce qu’on appelle le postulat de Becker : l’idée que le statut modal est nécessaire, par exemple que la possibilité de PPP implique la nécessité de la possibilité de PPP, ainsi que certaines lois d’itération de la nécessité. Ces résultats ont joué un rôle important dans le développement de la logique modale au XXᵉ siècle. &lt;/p&gt; &lt;p&gt; Il entretient un dialogue étroit avec Heidegger : il reprend certains thèmes existentialistes (finitude, historicité, être-pour-la-mort) et les applique à des domaines comme les mathématiques, ce qui est très controversé (par exemple, discuter du comptage arithmétique comme « être-pour-la-mort »). Il développe également une « paraontologie » : une doctrine de l’essence et de la permanence des choses, distincte de l’ontologie heideggérienne centrée sur l’existence du Dasein. Pour lui, l’être humain n’existe pas seulement comme existence, mais aussi comme « paraexistence », incluant des dimensions inconscientes et surconscientes. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="H53" r:id="rId27" display="https://www.laphilo.fr/pho/obecker-mini.webp"/>
+    <hyperlink ref="E54" r:id="rId28" display="https://fr.wikipedia.org/wiki/Edith_Stein"/>
+    <hyperlink ref="H54" r:id="rId29" display="https://www.laphilo.fr/pho/estein-mini.webp"/>
+    <hyperlink ref="E60" r:id="rId30" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Gershom_Scholem&quot; title=&quot; Wikipedia&quot;&gt;Gershom SCHOLEM&lt;/a&gt; était un philosophe juif germano-israélien,  fondateur de l'étude académique moderne de la Kabbale et grand expert de  &lt;a href=&quot;https://www.nonfiction.fr/article-12478-gershom-scholem-de-berlin-a-la-palestine.htm&quot; title=&quot;Gershom Scholem : de Berlin à la Palestine  par nonfiction&quot;&gt;la mystique juive. &lt;/a&gt; Né à Berlin dans une famille assimilée, il s'est tourné vers le sionisme jeune et a immigré en Palestine en 1923, devenant professeur à l'Université hébraïque de Jérusalem. &lt;/p&gt; &lt;p&gt; Il a étudié les mathématiques, la philosophie et les langues sémitiques à Berlin, Iéna et Munich, où il a soutenu une thèse sur le &quot;Sefer ha-Bahir&quot;, un texte kabbalistique ancien. Ami proche de Walter Benjamin et correspondant de Leo Strauss, il a fui l'Europe nazie et s'est consacré à la recherche sur les manuscrits juifs pillés. &lt;/p&gt; &lt;p&gt; Il voyait  &lt;a href=&quot;https://www.youtube.com/watch?v=5HvDF8-XTjc&quot;  title=&quot;Dieu son nom et la Cabale selon Gershom Scholem  par Xavier Charles DJEBALI&quot;&gt;la Kabbale &lt;/a&gt; non comme une superstition marginale, mais au cœur de l'essence spirituelle du judaïsme, explorée via des méthodes scientifiques et historiques. Il insistait sur le rôle du messianisme et de la tradition comme forces de renouvellement, où la révélation divine est infiniment interprétable et liée à l'expérience historique du peuple juif. Pour lui, le sionisme allait au-delà de la politique : c'était un renouveau profond du judaïsme, unissant ancien et nouveau contre l'assimilation. &lt;/p&gt; &lt;p&gt; Son oeuvre majeure &quot;Les Grandes tendances de la mystique juive&quot; paru en 1941, basé sur des conférences, dédié à Benjamin, explore l'évolution de la mystique juive. Sa pensée met l'accent sur l'identité juive forgée par l'histoire, où la tradition intègre la nouveauté pour survivre aux crises. &lt;/p&gt; &lt;audio controls title=&quot;Des livres pour notre temps et les mondes à venir. 1/2 Gershom Scholem : penser dans les marges de la marge par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13094-10.11.2019-ITEMA_22199082-0.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
+    <hyperlink ref="E61" r:id="rId31" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Leo_Strauss&quot; title=&quot; Wikipedia&quot;&gt;Leo SRAUSS&lt;/a&gt; était un philosophe politique germano-américain, connu pour sa critique profonde de la modernité et pour sa relecture des grands textes de la philosophie politique classique. Sa pensée a eu une influence durable, notamment aux États‑Unis, où elle a marqué des générations d’étudiants en théorie politique. &lt;/p&gt; &lt;p&gt; Au cœur de sa philosophie se trouve l’idée que la modernité a rompu avec le droit naturel classique, c’est‑à‑dire avec la recherche de ce qui est juste par nature et non simplement selon l’histoire ou les sciences sociales. Il voit dans le positivisme, le relativisme et l’historicisme modernes une source de décadence intellectuelle, car ils empêchent de poser les questions normatives fondamentales : qu’est‑ce qu’une vie bonne, qu’est‑ce qu’un régime politique juste. Pour lui, la  &lt;a href=&quot;https://www.persee.fr/doc/rfsp_0035-2950_1985_num_35_4_394205&quot; title=&quot;philosophie et zscience politique par persée&quot;&gt;philosophie politique authentique &lt;/a&gt; doit réactiver ces questions et affronter directement les notions de meilleur régime et d’ordre politique juste, plutôt que de se contenter de descriptions neutres. &lt;/p&gt; &lt;p&gt; Cette critique le conduit à renouer avec les auteurs de l’Antiquité, en particulier Platon, Aristote et les philosophes médiévaux juifs et arabes, qu’il lit souvent contre les interprétations modernes. Il insiste sur la dimension éducative de la philosophie : il parle de « liberal education » comme d’une libération de la vulgarité, entendue comme manque d’expérience des belles choses. La fréquentation des grands textes est, pour lui, une école de modestie et d’audace intellectuelle, parce qu’elle oblige à mesurer nos catégories modernes à celles d’auteurs qui pensaient autrement le politique et le juste. &lt;/p&gt; &lt;p&gt; Célèbre pour sa thèse sur l’« écriture ésotérique » : selon lui, nombre de philosophes du passé ont écrit de manière volontairement oblique pour se protéger de la censure ou de la persécution, réservant un sens plus profond aux lecteurs attentifs. Cela l’amène à distinguer entre le message « exotérique » (apparent, destiné au grand public) et le message « ésotérique » (plus exigeant, adressé à une minorité philosophique). Cette hypothèse sur la lecture des classiques s’articule à sa conception du   &lt;a href=&quot;https://www.youtube.com/watch?v=9Vhsveytymk&quot; title=&quot;nihilisme et politique leo strauss par bildung et culture&quot;&gt;mode de vie philosophique, &lt;/a&gt; toujours exposé au risque de la tyrannie et de l’incompréhension. Ainsi, sa philosophie politique est à la fois une critique de la modernité et une tentative de redécouvrir la place de la philosophie au cœur du politique contemporain. &lt;/p&gt; &#10; &lt;audio controls title=&quot;la pensée de leon strauss par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13397-05.04.2008-ITEMA_20118283-2008C3397E0019-ITE_00016207_RSCE-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;  &#10;"/>
+    <hyperlink ref="H61" r:id="rId32" display="https://www.laphilo.fr/pho/lstrauss-mini.webp"/>
+    <hyperlink ref="E64" r:id="rId33" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hans_Jonas&quot; title=&quot; Wikipedia&quot;&gt;Hans JONAS&lt;/a&gt;  était un philosophe germano-américain connu pour ses travaux sur l'éthique de la technologie et &lt;a href=&quot;https://www.youtube.com/watch?v=NPIJHZO7hQo&quot; title=&quot; Le PRINCIPE RESPONSABILITÉ en 6 minutes ! (HANS JONAS) par Culture Philo&quot;&gt;la responsabilité&lt;/a&gt; envers les générations futures. Ses premières recherches portent sur le gnosticisme, vu comme une réponse à l'aliénation existentielle dans un monde hostile. Dans les années 1960, il développe une philosophie de la vie organique (The Phenomenon of Life), critiquant le dualisme cartésien et valorisant la nature vivante contre la technoscience destructrice. Son œuvre maîtresse &lt;a href=&quot;https://www.youtube.com/watch?v=LsIWCR9_N64&quot; style=&quot;color:#88A1E9&quot; title=&quot; Philo, Hans jonas, Le principe responsabilité, Bac philo par SOS Bac Français&quot;&gt; &quot;Le Principe responsabilité&quot;&lt;/a&gt; paru en1979, formule un impératif éthique pour l'ère technologique : &quot;Agis de façon que les effets de ton action soient compatibles avec la permanence d'une vie authentiquement humaine sur Terre&quot;. &lt;/p&gt; &lt;p&gt; Il  anticipe les crises écologiques et bioéthiques, proposant une &quot;heuristique de la peur&quot; pour guider l'action humaine face aux risques imprévisibles de la puissance technique. Influencé par sa tradition juive et Heidegger, il réconcilie existentialisme, phénoménologie et morale prophétique, impactant l'éthique environnementale contemporaine. &lt;/p&gt; &lt;p&gt; Il observe un &quot;déchaînement prométhéen&quot; : l'humanité acquiert un pouvoir inédit sur la nature via la science et la technique, capable de menacer sa propre survie et celle des générations futures. Contrairement aux éthiques classiques (kantienne ou utilitariste), limitées au présent ou aux intentions, sa réflexion intègre les conséquences à long terme, imprévisibles et collectives, sur la vie humaine et la planète. Face aux risques inconnus (nucléaire, génétique, environnementaux), il prône une &quot;heuristique de la peur&quot; : anticiper le pire scénario (in dubio pro malo) pour guider l'action, sans paralyser le progrès mais en le subordonnant à la préservation de la vie. Le savoir devient un devoir moral prioritaire, élargissant l'éthique à la nature et aux générations absentes.&lt;/p&gt;  &lt;/p&gt; &lt;p&gt;  &lt;audio controls title=&quot; Hans Jonas. Pour une éthique de la société technologique par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/22267-14.06.2021-ITEMA_22702122-2014C12410E0357.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
+    <hyperlink ref="E66" r:id="rId34" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl-Otto_Apel&quot; title=&quot; Wikipedia&quot;&gt;Karl-Otto APEL&lt;/a&gt; était un philosophe allemand majeur de l’après-guerre, surtout connu pour avoir développé, avec Jürgen Habermas, l’éthique du discours et pour sa « pragmatique transcendantale », une tentative de refonder la philosophie à partir des présupposés normatifs de l’argumentation. &lt;/p&gt; &lt;p&gt; Il est souvent crédité d’avoir opéré la « linguistification » de la philosophie transcendantale kantienne : au lieu de partir de la conscience ou du sujet (comme chez Kant ou Husserl), il part du fait que toute connaissance et toute action s’inscrivent dans un langage commun et une communauté de communication. Pour lui, les conditions de possibilité de la connaissance ne sont pas d’abord dans la structure de la conscience, mais dans les règles implicites de l’usage du langage et de l’argumentation. &lt;/p&gt; &lt;p&gt;  &lt;a href=&quot;https://www.youtube.com/watch?v=R9jQv_akxFE&quot; &gt;Sa notion centrale &lt;/a&gt; est celle d’a priori de la communauté de communication : le simple fait d’argumenter présuppose déjà un cadre normatif inévitable (recherche de vérité, reconnaissance mutuelle des interlocuteurs, exigence de cohérence, etc.). Quiconque tente de nier ces présupposés tombe dans une auto-contradiction performative : en les contestant par la parole, il les utilise déjà. Il en tire l’idée d’une fondation ultime de la rationalité et de l’éthique à partir de la structure même de l’argumentation. &lt;/p&gt; &lt;p&gt; À partir de cette base, il développe une éthique du discours : seules sont moralement justifiées les normes qui pourraient être acceptées par tous les concernés dans un discours pratique idéal, où chacun est reconnu comme partenaire égal de l’argumentation. Cette éthique vise à fournir un fondement universel à la morale, sans retomber dans un absolutisme dogmatique ni dans un relativisme pur : l’universalité vient des conditions mêmes de l’argumentation rationnelle. Elle influence profondément Habermas, même si il insiste davantage sur la dimension de fondation ultime et sur l’obligation morale inconditionnelle qui en découle. &lt;/p&gt; &#10;"/>
+    <hyperlink ref="H66" r:id="rId35" display="https://www.laphilo.fr/pho/koapel-mini.webp"/>
+    <hyperlink ref="E68" r:id="rId36" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Reiner_Sch%C3%BCrmann&quot;  title=&quot; Wikipedia&quot;&gt;Reiner SCHÜRMANN&lt;/a&gt; est un philosophe allemand d’expression française, né à Amsterdam et mort à New York, où il a enseigné à la New School for Social Research à partir de 1975. Très marqué par la phénoménologie et la pensée de Heidegger, il se distingue par une réflexion exigeante sur la métaphysique, l’histoire de la philosophie et l’agir humain, développée dans trois grands ouvrages : Maître Eckhart et la joie errante (1972), Le principe d’anarchie (1982) et Des hégémonies brisées (posthume, 1996). &lt;/p&gt;&lt;p&gt; Dans Maître Eckhart et la joie errante, Schürmann reprend la pensée du mystique allemand du XIVᵉ siècle pour explorer la possibilité d’une vie spirituelle détachée de toute identité fixe ou de tout fondement stable. Il met en avant ce qu’il appelle une « joie errante » : une forme de liberté intérieure où le sujet ne se réclame plus d’une essence, d’un Dieu garanti ou d’une identité nationale, mais accepte de vivre dans une errance originaire et sans fondement. &lt;/p&gt; &lt;p&gt; Dans Le principe d’anarchie (souvent considéré comme son chef‑d’œuvre), Schürmann interprète Heidegger comme une pensée qui conduit à la ruine de tout principe premier (« archè ») sur lequel la tradition occidentale aurait voulu fonder la connaissance, la morale et la politique. Il en tire une théorie de l’« anarchie » non pas comme désordre, mais comme conscience lucide de l’absence de fondement ultime : l’agir humain doit alors se penser comme une praxis ouverte, responsable et créative, sans recours à une règle suprême. &lt;/p&gt; &lt;p&gt; Dans Des hégémonies brisées, Schürmann entreprend une vaste reconstruction de l’histoire de la philosophie occidentale comme succession d’« hégémonies » (modèles de vérité, de métaphysique, de politique) qui s’imposent, puis se défont. Il montre comment la modernité et la déconstruction heideggérienne ont dissous les grands systèmes de pensée, ouvrant à ce qu’il nomme une « philosophie tragique » où l’être se donne comme événement contingent, marqué par une distance, une fracture intérieure, plutôt que par une harmonie ou une cohérence totale. &lt;/p&gt; &#10;&#10;"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Fiches — 13 fiches modifiées : Karl JASPERS, Roy Wood SELLARS, Susan WOLF, Patrick CHAMOISEAU, John D. NORTON, Pierre TEILHARD DE CHARDIN et 7 autre(s) ; 9 images
Publié depuis l'éditeur des fiches.
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -4499,555 +4499,577 @@
         <v>27</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="206.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="n">
+    <row r="47" customFormat="false" ht="267.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="0">
+        <v>1883</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1969</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1883 – 1969</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Karl JASPERS</t>
+        </is>
+      </c>
+      <c r="E47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Jaspers" title=" Wikipedia"&gt;Karl JASPERS&lt;/a&gt; est un psychiatre et philosophe allemand, l’un des fondateurs de la philosophie de l’existence. Né à Oldenbourg, il étudie le droit puis la médecine et travaille à la clinique psychiatrique de Heidelberg. Son &lt;em&gt;Psychopathologie générale&lt;/em&gt; (1913) renouvelle la psychiatrie en distinguant ce que l’on peut « expliquer » par des causes et ce que l’on doit « comprendre » de l’intérieur, dans l’expérience du malade. Il se tourne ensuite&lt;a href="https://www.persee.fr/doc/rhpr_0035-2403_1957_num_37_3_3504" title="Philosophie et Religion chez Karl Jaspers par persée"&gt; vers la philosophie&lt;/a&gt;, qu’il enseigne à Heidelberg.&lt;/p&gt; &lt;p&gt;Dans sa &lt;em&gt;Philosophie&lt;/em&gt; (1932), il &lt;a href="https://www.youtube.com/watch?v=BfXnx_rj4nI" title="Karl Jaspers - Introduction à la philosophie (Résumé de livre) par COGNITO FR"&gt;distingue l’existence&lt;/a&gt; de tout ce que la science peut connaître : ce que je suis vraiment ne se laisse pas réduire à un objet. C’est dans les "situations limites", la mort, la souffrance, la lutte, la culpabilité, que l’homme découvre qu’il ne peut rien maîtriser et s’ouvre à la « transcendance ». La communication authentique avec autrui, une « lutte aimante », est le lieu où chacun devient lui-même. Il forge aussi la notion d’« âge axial » pour désigner le moment, autour du VIe siècle avant notre ère, où naissent presque en même temps les grandes sagesses de la Chine, de l’Inde, de la Perse, d’Israël et de la Grèce.&lt;/p&gt; &lt;p&gt;Marié à une femme juive, Gertrud, il est privé d’enseignement par les nazis en 1937 et vit sous la menace de la déportation. Après la guerre, il publie &lt;em&gt;La Culpabilité allemande&lt;/em&gt; (1946), où il distingue culpabilité criminelle, politique, morale et métaphysique. Maître et ami d’&lt;a href="https://fr.wikipedia.org/wiki/Hannah_Arendt" title=" Wikipedia"&gt;Hannah Arendt&lt;/a&gt;, il s’installe à Bâle en 1948 et y meurt en 1969.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">_X502cqdYWk</t>
+        </is>
+      </c>
+      <c r="G47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"KARL JASPERS : le philosophe allemand de l'existence et de la liberté | Histoire pour Dormir" par Voyages Endormis</t>
+        </is>
+      </c>
+      <c r="H47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/jaspers-mini.webp</t>
+        </is>
+      </c>
+      <c r="I47" s="0"/>
+      <c r="J47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique ; politique</t>
+        </is>
+      </c>
+      <c r="K47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Existentialisme</t>
+        </is>
+      </c>
+      <c r="L47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">psychiatre et philosophe allemand, penseur de l’existence, des situations limites et de la culpabilité.</t>
+        </is>
+      </c>
+      <c r="N47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O47">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="206.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="7" t="n">
         <v>1885</v>
       </c>
-      <c r="B47" s="7" t="s">
+      <c r="B48" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="C47" s="7" t="s">
+      <c r="C48" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="D47" s="8" t="s">
+      <c r="D48" s="8" t="s">
         <v>400</v>
       </c>
-      <c r="E47" s="13" t="inlineStr">
+      <c r="E48" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ernst_Bloch"  title=" Wikipedia"&gt;Ernst BLOCH&lt;/a&gt;  était un philosophe juif allemand  souvent rattaché au marxisme hétérodoxe et à la philosophie de l’espérance. Sa pensée se distingue par une défense de l’utopie comme force critique et émancipatrice, contre les lectures trop fermées ou déterministes de l’histoire. &lt;/p&gt; &lt;p&gt; Il part de l’idée que la réalité humaine n’est jamais complètement accomplie: il y a toujours du “pas encore” dans l’histoire, dans la société et dans la conscience. Il appelle cela le non-simultané ou le caractère inachevé du réel, ce qui permet de penser le futur comme ouvert plutôt que comme déjà écrit. &lt;/p&gt; &lt;p&gt; Son ouvrage majeur,  &lt;a href="https://www.youtube.com/watch?v=u-zXjE1duok"  title="Le principe de l’espérance par Culture Philo"&gt; Le Principe espérance, &lt;/a&gt; développe l’idée que l’espérance n’est pas une illusion passive, mais une énergie active qui pousse les hommes à transformer le monde. L’utopie, chez lui, n’est donc pas un rêve irréaliste: c’est une anticipation concrète de ce qui pourrait advenir. &lt;/p&gt; &lt;p&gt; Il accorde aussi une grande importance aux œuvres culturelles, à la religion, à l’art et même aux rêves éveillés, parce qu’ils contiennent des indices de possibles non réalisés. Il voit dans ces domaines des formes où s’exprime un dépassement de la situation présente, une ouverture vers un monde plus juste. &lt;/p&gt; &lt;p&gt; Sa philosophie est une pensée du possible et du futur. Elle combine critique du présent, héritage marxiste et réhabilitation de l’utopie pour montrer que l’histoire humaine peut encore être transformée. &lt;/p&gt;  &lt;audio controls title="A quoi bon espérer ? par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-27.06.2023-ITEMA_23423905-2023C48904S0178-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
 </t>
         </is>
       </c>
-      <c r="F47" s="7" t="s">
+      <c r="F48" s="7" t="s">
         <v>402</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G48" s="9" t="s">
         <v>403</v>
       </c>
-      <c r="H47" s="9" t="s">
+      <c r="H48" s="9" t="s">
         <v>404</v>
-      </c>
-      <c r="I47" s="7"/>
-      <c r="J47" s="2" t="s">
-        <v>405</v>
-      </c>
-      <c r="K47" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="L47" s="17" t="s">
-        <v>407</v>
-      </c>
-      <c r="M47" s="0" t="s">
-        <v>186</v>
-      </c>
-      <c r="N47" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="n">
-        <v>1886</v>
-      </c>
-      <c r="B48" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="C48" s="7" t="s">
-        <v>409</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>410</v>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Korsch" title=" Wikipedia"&gt;Karl KORSCH&lt;/a&gt;  était un philosophe marxiste allemand,  théoricien du communisme de conseils et critique du léninisme orthodoxe. Issu d'un milieu bourgeois, il évolua du réformisme social au marxisme hétérodoxe, influençant les courants ultra-gauche via son rejet du matérialisme positiviste et son insistance sur la praxis révolutionnaire historique. Juriste de formation, il est en 1923 ministre de la Justice de Thuringe, puis député communiste au Reichstag.  Exclu du parti en 1926 pour "ultra-gauchisme", il émigra après 1933 vers les États-Unis, où il approfondit sa théorie marxiste. &lt;/p&gt; &lt;p&gt; Son œuvre majeure &lt;em&gt;Marxisme et philosophie&lt;/em&gt; paru en 1923 marque sa rupture avec le léninisme en critiquant sa dérive scientiste. Il   &lt;a href="https://www.zones-subversives.com/article-le-marxisme-critique-de-karl-korsch-116431466.html"  title="Le marxisme critique de Karl Korsch par Chroniques critiques"&gt;rejette le marxisme &lt;/a&gt; comme "science positive" figée ou philosophie matérialiste abstraite ; il le conçoit comme une théorie historique et concrète, liée à la lutte des classes et à la dialectique hégélienne réinterprétée comme expression de la révolution bourgeoise puis prolétarienne. &lt;/p&gt; &lt;p&gt; Il  théorise les conseils comme organes centraux de la transition socialiste, via la praxis dialectique et l'auto-activité des masses, contre la socialisation étatique. Ses écrits inspirent le KAPD et l'ultra-gauche, voyant les conseils comme alternative à la bureaucratisation stalinienne. Son influence perdure chez les communistes de conseils, soulignant la conscience ouvrière spontanée pour l'émancipation réelle. Aux États-Unis, il publie &lt;em&gt;Karl Marx&lt;/em&gt; (1938) et reste proche de Bertolt Brecht, qui le considérait comme son maître en marxisme. &lt;/p&gt; </t>
-        </is>
-      </c>
-      <c r="F48" s="7" t="s">
-        <v>412</v>
-      </c>
-      <c r="G48" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="H48" s="9" t="s">
-        <v>414</v>
       </c>
       <c r="I48" s="7"/>
       <c r="J48" s="2" t="s">
-        <v>344</v>
+        <v>405</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="L48" s="2" t="s">
-        <v>415</v>
+        <v>406</v>
+      </c>
+      <c r="L48" s="17" t="s">
+        <v>407</v>
+      </c>
+      <c r="M48" s="0" t="s">
+        <v>186</v>
       </c>
       <c r="N48" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="n">
         <v>1886</v>
       </c>
       <c r="B49" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="E49" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Korsch" title=" Wikipedia"&gt;Karl KORSCH&lt;/a&gt;  était un philosophe marxiste allemand,  théoricien du communisme de conseils et critique du léninisme orthodoxe. Issu d'un milieu bourgeois, il évolua du réformisme social au marxisme hétérodoxe, influençant les courants ultra-gauche via son rejet du matérialisme positiviste et son insistance sur la praxis révolutionnaire historique. Juriste de formation, il est en 1923 ministre de la Justice de Thuringe, puis député communiste au Reichstag.  Exclu du parti en 1926 pour "ultra-gauchisme", il émigra après 1933 vers les États-Unis, où il approfondit sa théorie marxiste. &lt;/p&gt; &lt;p&gt; Son œuvre majeure &lt;em&gt;Marxisme et philosophie&lt;/em&gt; paru en 1923 marque sa rupture avec le léninisme en critiquant sa dérive scientiste. Il   &lt;a href="https://www.zones-subversives.com/article-le-marxisme-critique-de-karl-korsch-116431466.html"  title="Le marxisme critique de Karl Korsch par Chroniques critiques"&gt;rejette le marxisme &lt;/a&gt; comme "science positive" figée ou philosophie matérialiste abstraite ; il le conçoit comme une théorie historique et concrète, liée à la lutte des classes et à la dialectique hégélienne réinterprétée comme expression de la révolution bourgeoise puis prolétarienne. &lt;/p&gt; &lt;p&gt; Il  théorise les conseils comme organes centraux de la transition socialiste, via la praxis dialectique et l'auto-activité des masses, contre la socialisation étatique. Ses écrits inspirent le KAPD et l'ultra-gauche, voyant les conseils comme alternative à la bureaucratisation stalinienne. Son influence perdure chez les communistes de conseils, soulignant la conscience ouvrière spontanée pour l'émancipation réelle. Aux États-Unis, il publie &lt;em&gt;Karl Marx&lt;/em&gt; (1938) et reste proche de Bertolt Brecht, qui le considérait comme son maître en marxisme. &lt;/p&gt; </t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>413</v>
+      </c>
+      <c r="H49" s="9" t="s">
+        <v>414</v>
+      </c>
+      <c r="I49" s="7"/>
+      <c r="J49" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="L49" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="N49" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="7" t="n">
+        <v>1886</v>
+      </c>
+      <c r="B50" s="7" t="s">
         <v>416</v>
       </c>
-      <c r="C49" s="7" t="s">
+      <c r="C50" s="7" t="s">
         <v>417</v>
       </c>
-      <c r="D49" s="8" t="s">
+      <c r="D50" s="8" t="s">
         <v>418</v>
       </c>
-      <c r="E49" s="9" t="inlineStr">
+      <c r="E50" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Franz_Rosenzweig" title=" Wikipedia"&gt;Franz ROSENZWEIG&lt;/a&gt; était un philosophe et théologien juif allemand et l’une des grandes voix du &lt;a href="https://journals.openedition.org/ceg/16724" title="Les visages du temps dans la pensée de Franz Rosenzweig  par Open Edition"&gt;renouveau de la pensée juive. &lt;/a&gt;  Il se forme d’abord dans l’orbite de l’idéalisme allemand, en particulier Hegel, mais va s’y opposer radicalement. Il critique l’idée de "totalité" qui engloberait et expliquerait tout ce qui est : pour lui, le réel est irréductiblement plural, composé d’éléments qui ne se laissent pas fondre dans un système unique. Il refuse la prétention de la philosophie à un "savoir absolu" qui surplomberait Dieu, le monde et l’homme. Sa démarche consiste à partir de l’expérience concrète, de la finitude et de la mortalité humaines, plutôt que de concepts abstraits de l’être. &lt;/p&gt; &lt;p&gt; Dans "L’Étoile de la rédemption", &lt;a href="https://www.youtube.com/watch?v=OSyPZERfePg"  title="Sur Franz Rosenzweig : Gérard Bensussan à Ombres Blanches, Toulouse  par LeBras videos et chocolat"&gt;il propose &lt;/a&gt; une grande architecture de pensée à partir de trois "éléments" fondamentaux : Dieu, le monde, l’homme. Ces trois réalités sont distinctes, irréductibles l’une à l’autre : on ne peut ni ramener Dieu au monde, ni réduire l’homme à un moment d’un tout cosmique. Elles entrent en relation à travers trois mouvements : création (Dieu–monde), révélation (Dieu–homme) et rédemption (homme–monde). &lt;/p&gt; &lt;p&gt; Un point central chez lui est la compréhension de la révélation comme événement adressé à un sujet concret dans le temps. Dieu est pensé comme "existant suprême et totalisateur" mais qui se révèle dans des actes, des paroles, une histoire avec un peuple et avec des individus. Le temps devient le lieu où se déploient création, révélation et rédemption : il insiste sur la mortalité de l’homme, mais aussi sur une forme de "vie éternelle" déjà à l’œuvre. &lt;/p&gt; 
    &lt;audio controls title="Franz Rosenzweig, l'anti-Hegel par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/12014-31.01.2017-ITEMA_21214189-2017C26359S0031-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
 </t>
         </is>
       </c>
-      <c r="F49" s="7" t="s">
+      <c r="F50" s="7" t="s">
         <v>420</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="G50" s="9" t="s">
         <v>421</v>
       </c>
-      <c r="H49" s="9" t="s">
+      <c r="H50" s="9" t="s">
         <v>422</v>
       </c>
-      <c r="I49" s="7"/>
-      <c r="J49" s="2" t="s">
+      <c r="I50" s="7"/>
+      <c r="J50" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="K49" s="2" t="s">
+      <c r="K50" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="L49" s="2" t="s">
+      <c r="L50" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="M49" s="0" t="s">
+      <c r="M50" s="0" t="s">
         <v>186</v>
       </c>
-      <c r="N49" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7" t="n">
+      <c r="N50" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="7" t="n">
         <v>1888</v>
       </c>
-      <c r="B50" s="7" t="s">
+      <c r="B51" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="C50" s="7" t="s">
+      <c r="C51" s="7" t="s">
         <v>426</v>
       </c>
-      <c r="D50" s="8" t="s">
+      <c r="D51" s="8" t="s">
         <v>427</v>
       </c>
-      <c r="E50" s="9" t="inlineStr">
+      <c r="E51" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Carl_Schmitt" title=" Wikipedia"&gt;Carl SCHMITT&lt;/a&gt;  était un philosophe &amp; théologien politique allemand  controversé, connu pour ses critiques radicales du libéralisme parlementaire et sa proximité avec le nazisme. Il adhère au parti nazi en 1933, justifie en 1934 les assassinats de la Nuit des longs couteaux dans « Le Führer protège le droit » et tient des propos antisémites, avant d’être écarté par la SS en 1936. &lt;/p&gt; &lt;p&gt;Il rejette le libéralisme pour son neutralisme économique et juridique, prônant un  &lt;a href="https://www.liberation.fr/debats/2016/08/03/carl-schmitt-le-penseur-de-l-ennemi_1470100/"  title="Détournement de pensées (4/5) Carl Schmitt, le penseur de l’ennemi  par Libération"&gt;État fort &lt;/a&gt; capable de trancher dans l'état d'exception, où la norme juridique s'efface. Sa vision du politique comme conflit existentiel  &lt;a href="https://www.youtube.com/watch?v=vopSqS73tLI" title="Ami - Ennemi, le fondement du politique (Carl Schmitt)  par Ego Non"&gt;(ami/ennemi) &lt;/a&gt; influence la géopolitique et la critique de la mondialisation, voyant dans le nomos (ordre spatial) la base des relations internationales. Catholique puis critique du catholicisme politique, il admire Hobbes et le Léviathan comme modèle d'autorité absolue. &lt;/p&gt; &lt;p&gt; Ses oeuvres principales : "Théologie politique" paru en 1922 : définit le souverain comme "celui qui décide sur l'exception", liant décision politique et théologie, &lt;a href="https://www.youtube.com/watch?v=U8u4SUZNF9I" title="La politique, c'est la guerre (Carl Schmitt)and Mind  par Politikon"&gt;La Notion du politique" &lt;/a&gt; paru en 1932 : pose que le politique repose sur la distinction ami/ennemi, critiquant le parlementarisme comme dissolvant cette intensité et "Théorie de la Constitution" en 1928 et "Théorie du partisan" en 1963 : analyses du pouvoir constituant, de la dictature légitime et de la guerre irrégulière. &lt;/p&gt; &lt;p&gt; Admiré pour sa profondeur analytique par des intellectuels comme Chantal Mouffe ou Giorgio Agamben, mais rejeté comme idéologue nazi par d'autres, son œuvre reste étudiée pour comprendre les limites de la démocratie libérale. &lt;/p&gt;   &lt;audio controls title="Carl Schmitt : comment éradiquer nos ennemis ? par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2015/11/s48/NET_FC_320d8f8e-e840-4e7b-a1c5-c5b36f7e22c6.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
 </t>
         </is>
       </c>
-      <c r="F50" s="7" t="s">
+      <c r="F51" s="7" t="s">
         <v>429</v>
       </c>
-      <c r="G50" s="9" t="s">
+      <c r="G51" s="9" t="s">
         <v>430</v>
       </c>
-      <c r="H50" s="9" t="s">
+      <c r="H51" s="9" t="s">
         <v>431</v>
-      </c>
-      <c r="I50" s="7"/>
-      <c r="J50" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="K50" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="L50" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="N50" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="n">
-        <v>1888</v>
-      </c>
-      <c r="B51" s="7" t="n">
-        <v>1973</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>433</v>
-      </c>
-      <c r="D51" s="8" t="s">
-        <v>434</v>
-      </c>
-      <c r="E51" s="12" t="s">
-        <v>435</v>
-      </c>
-      <c r="F51" s="7" t="s">
-        <v>436</v>
-      </c>
-      <c r="G51" s="9" t="s">
-        <v>437</v>
-      </c>
-      <c r="H51" s="12" t="s">
-        <v>438</v>
       </c>
       <c r="I51" s="7"/>
       <c r="J51" s="2" t="s">
-        <v>439</v>
+        <v>344</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>423</v>
+        <v>378</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="M51" s="0" t="s">
-        <v>186</v>
+        <v>432</v>
       </c>
       <c r="N51" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="n">
-        <v>1889</v>
-      </c>
-      <c r="B52" s="7" t="s">
-        <v>441</v>
+        <v>1888</v>
+      </c>
+      <c r="B52" s="7" t="n">
+        <v>1973</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>442</v>
+        <v>433</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>443</v>
-      </c>
-      <c r="E52" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Martin_Heidegger"  title=" Wikipedia"&gt;Martin HEIDEGGER&lt;/a&gt; (1889-1976) est un philosophe allemand, l’un des plus influents et des plus controversés du XXe siècle. Né à Messkirch, dans le pays de Bade, il se destine d’abord à la prêtrise, puis devient à Fribourg l’assistant de &lt;a href="https://fr.wikipedia.org/wiki/Edmund_Husserl" title=" Wikipedia"&gt;Husserl&lt;/a&gt;, dont il renouvelle &lt;a href="https://www.youtube.com/watch?v=t96HiEpxIB0&amp;ab_channel=MichelOnfray-Topic"   title="La phénoménologie par Michel Onfray "&gt;la phénoménologie&lt;/a&gt;. Professeur à Marbourg, il publie en 1927 son œuvre majeure, &lt;a href="https://www.youtube.com/watch?v=A7ke29MEYpY&amp;ab_channel=LePr%C3%A9cepteur"  title="Etre et Temps de Heidegger par le Precepteur "&gt;&lt;em&gt;Être et Temps&lt;/em&gt;&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Heidegger reproche à la philosophie occidentale, depuis Platon, d’avoir « oublié l’être » : elle a étudié les étants, les choses qui sont, sans se demander ce que veut dire « être ». Pour poser cette question, il part de l’existence humaine, qu’il nomme &lt;em&gt;Dasein&lt;/em&gt;, « être-là ». L’homme n’est pas un sujet face à des objets : il est d’emblée « au monde », pris dans des tâches et des outils qu’il utilise sans y penser, comme le marteau. Le plus souvent, il vit sur le mode impersonnel du « on ». L’angoisse le confronte à sa finitude : l’homme est un « être-pour-la-mort », et c’est en assumant sa mort qu’il peut exister de façon authentique. Dans ses œuvres plus tardives, Heidegger médite sur l’histoire de l’être, sur la poésie de Hölderlin et sur le langage, « maison de l’être ». Il voit dans la technique moderne non un simple ensemble d’outils, mais une manière de dévoiler le monde comme un stock de ressources à exploiter.&lt;/p&gt; &lt;p&gt;Recteur de l’université de Fribourg en 1933, membre du parti nazi jusqu’en 1945, il est interdit d’enseignement après la guerre ; ses &lt;em&gt;Cahiers noirs&lt;/em&gt;, publiés depuis 2014, révèlent un antisémitisme qui relance le débat. Son influence sur Sartre, Arendt, Levinas et Derrida est pourtant considérable.&lt;/p&gt;  &lt;audio controls title="L'antisémitisme dans la pensée de Heidegger par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2014/10/s40/RF_D01332FD-FB86-4C0A-BF38-A61BECB1EA38_GENE_2.MP3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
-        </is>
+        <v>434</v>
+      </c>
+      <c r="E52" s="12" t="s">
+        <v>435</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>445</v>
+        <v>436</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>446</v>
-      </c>
-      <c r="H52" s="9" t="s">
-        <v>447</v>
+        <v>437</v>
+      </c>
+      <c r="H52" s="12" t="s">
+        <v>438</v>
       </c>
       <c r="I52" s="7"/>
       <c r="J52" s="2" t="s">
-        <v>128</v>
+        <v>439</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>448</v>
+        <v>423</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>449</v>
+        <v>440</v>
+      </c>
+      <c r="M52" s="0" t="s">
+        <v>186</v>
       </c>
       <c r="N52" s="0" t="s">
         <v>27</v>
-      </c>
-      <c r="O52" s="0" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="n">
         <v>1889</v>
       </c>
-      <c r="B53" s="7" t="n">
-        <v>1964</v>
+      <c r="B53" s="7" t="s">
+        <v>441</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>450</v>
+        <v>442</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>451</v>
-      </c>
-      <c r="E53" s="20" t="s">
-        <v>452</v>
+        <v>443</v>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Martin_Heidegger"  title=" Wikipedia"&gt;Martin HEIDEGGER&lt;/a&gt; (1889-1976) est un philosophe allemand, l’un des plus influents et des plus controversés du XXe siècle. Né à Messkirch, dans le pays de Bade, il se destine d’abord à la prêtrise, puis devient à Fribourg l’assistant de &lt;a href="https://fr.wikipedia.org/wiki/Edmund_Husserl" title=" Wikipedia"&gt;Husserl&lt;/a&gt;, dont il renouvelle &lt;a href="https://www.youtube.com/watch?v=t96HiEpxIB0&amp;ab_channel=MichelOnfray-Topic"   title="La phénoménologie par Michel Onfray "&gt;la phénoménologie&lt;/a&gt;. Professeur à Marbourg, il publie en 1927 son œuvre majeure, &lt;a href="https://www.youtube.com/watch?v=A7ke29MEYpY&amp;ab_channel=LePr%C3%A9cepteur"  title="Etre et Temps de Heidegger par le Precepteur "&gt;&lt;em&gt;Être et Temps&lt;/em&gt;&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Heidegger reproche à la philosophie occidentale, depuis Platon, d’avoir « oublié l’être » : elle a étudié les étants, les choses qui sont, sans se demander ce que veut dire « être ». Pour poser cette question, il part de l’existence humaine, qu’il nomme &lt;em&gt;Dasein&lt;/em&gt;, « être-là ». L’homme n’est pas un sujet face à des objets : il est d’emblée « au monde », pris dans des tâches et des outils qu’il utilise sans y penser, comme le marteau. Le plus souvent, il vit sur le mode impersonnel du « on ». L’angoisse le confronte à sa finitude : l’homme est un « être-pour-la-mort », et c’est en assumant sa mort qu’il peut exister de façon authentique. Dans ses œuvres plus tardives, Heidegger médite sur l’histoire de l’être, sur la poésie de Hölderlin et sur le langage, « maison de l’être ». Il voit dans la technique moderne non un simple ensemble d’outils, mais une manière de dévoiler le monde comme un stock de ressources à exploiter.&lt;/p&gt; &lt;p&gt;Recteur de l’université de Fribourg en 1933, membre du parti nazi jusqu’en 1945, il est interdit d’enseignement après la guerre ; ses &lt;em&gt;Cahiers noirs&lt;/em&gt;, publiés depuis 2014, révèlent un antisémitisme qui relance le débat. Son influence sur Sartre, Arendt, Levinas et Derrida est pourtant considérable.&lt;/p&gt;  &lt;audio controls title="L'antisémitisme dans la pensée de Heidegger par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2014/10/s40/RF_D01332FD-FB86-4C0A-BF38-A61BECB1EA38_GENE_2.MP3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F53" s="7" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>454</v>
-      </c>
-      <c r="H53" s="12" t="s">
-        <v>455</v>
+        <v>446</v>
+      </c>
+      <c r="H53" s="9" t="s">
+        <v>447</v>
       </c>
       <c r="I53" s="7"/>
       <c r="J53" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="N53" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="O53" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="213" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7" t="n">
+        <v>1889</v>
+      </c>
+      <c r="B54" s="7" t="n">
+        <v>1964</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="E54" s="20" t="s">
+        <v>452</v>
+      </c>
+      <c r="F54" s="7" t="s">
+        <v>453</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>454</v>
+      </c>
+      <c r="H54" s="12" t="s">
+        <v>455</v>
+      </c>
+      <c r="I54" s="7"/>
+      <c r="J54" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="K53" s="2" t="s">
+      <c r="K54" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="L53" s="10" t="s">
+      <c r="L54" s="10" t="s">
         <v>458</v>
       </c>
-      <c r="N53" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="244.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7" t="n">
-        <v>1891</v>
-      </c>
-      <c r="B54" s="7" t="n">
-        <v>1942</v>
-      </c>
-      <c r="C54" s="7" t="s">
-        <v>459</v>
-      </c>
-      <c r="D54" s="8" t="s">
-        <v>460</v>
-      </c>
-      <c r="E54" s="14" t="s">
-        <v>461</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="J54" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="K54" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="L54" s="2" t="s">
-        <v>465</v>
-      </c>
-      <c r="M54" s="0" t="s">
-        <v>346</v>
-      </c>
       <c r="N54" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="O54" s="0" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="207" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="55" customFormat="false" ht="244.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="n">
         <v>1891</v>
       </c>
-      <c r="B55" s="7" t="s">
+      <c r="B55" s="7" t="n">
+        <v>1942</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>460</v>
+      </c>
+      <c r="E55" s="14" t="s">
+        <v>461</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="M55" s="0" t="s">
+        <v>346</v>
+      </c>
+      <c r="N55" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="O55" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="207" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="7" t="n">
+        <v>1891</v>
+      </c>
+      <c r="B56" s="7" t="s">
         <v>466</v>
       </c>
-      <c r="C55" s="7" t="s">
+      <c r="C56" s="7" t="s">
         <v>467</v>
       </c>
-      <c r="D55" s="8" t="s">
+      <c r="D56" s="8" t="s">
         <v>468</v>
       </c>
-      <c r="E55" s="9" t="s">
+      <c r="E56" s="9" t="s">
         <v>469</v>
       </c>
-      <c r="F55" s="7" t="s">
+      <c r="F56" s="7" t="s">
         <v>470</v>
       </c>
-      <c r="G55" s="9" t="s">
+      <c r="G56" s="9" t="s">
         <v>471</v>
       </c>
-      <c r="H55" s="9" t="s">
+      <c r="H56" s="9" t="s">
         <v>472</v>
-      </c>
-      <c r="I55" s="7"/>
-      <c r="J55" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="K55" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Positivisme Logique ; Physicalisme ; Phénoménisme ; Réductionnisme</t>
-        </is>
-      </c>
-      <c r="L55" s="2" t="s">
-        <v>475</v>
-      </c>
-      <c r="N55" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="219.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7" t="n">
-        <v>1892</v>
-      </c>
-      <c r="B56" s="7" t="s">
-        <v>476</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>477</v>
-      </c>
-      <c r="D56" s="8" t="s">
-        <v>478</v>
-      </c>
-      <c r="E56" s="9" t="s">
-        <v>479</v>
-      </c>
-      <c r="F56" s="7" t="s">
-        <v>480</v>
-      </c>
-      <c r="G56" s="9" t="s">
-        <v>481</v>
-      </c>
-      <c r="H56" s="9" t="s">
-        <v>482</v>
       </c>
       <c r="I56" s="7"/>
       <c r="J56" s="2" t="s">
-        <v>483</v>
-      </c>
-      <c r="K56" s="2" t="s">
-        <v>484</v>
+        <v>473</v>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivisme Logique ; Physicalisme ; Phénoménisme ; Réductionnisme</t>
+        </is>
       </c>
       <c r="L56" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="M56" s="0" t="s">
-        <v>186</v>
+        <v>475</v>
       </c>
       <c r="N56" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="O56" s="0" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="144.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="57" customFormat="false" ht="219.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="n">
         <v>1892</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>425</v>
+        <v>476</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>486</v>
+        <v>477</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>487</v>
-      </c>
-      <c r="E57" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Helmuth_Plessner"  title=" Wikipedia"&gt;Helmuth PLESSNER&lt;/a&gt; était un philosophe allemand, fondateur clé de &lt;a href="https://publictionnaire.huma-num.fr/notice/plessner-helmuth/"   title="L’apport de l’anthropologie  par Publitionnaire"&gt;l'anthropologie philosophique &lt;/a&gt;  européenne aux côtés de figures comme Max Scheler et Arnold Gehlen. Influencé par le néokantisme, la phénoménologie et la biologie, il développa une vision de l'humain comme être "naturellement artificiel", marqué par une "positionnalité excentrique" qui le distingue des animaux. &lt;/p&gt; &lt;p&gt;  L'homme vit à distance de son corps et de son milieu, possédant simultanément un corps et étant un corps vivant. Cela génère trois lois anthropologiques : la loi de l'"excentricité", celle de la "médiation"  et celle de l'"utopie naturelle". &lt;/p&gt; &lt;p&gt; Il dépasse le dualisme nature/esprit en fondant une herméneutique biologique : la vie s'exprime via les frontières organiques, et l'intentionnalité humaine émerge de cette interaction environnementale, non d'un ego transcendantal. &lt;/p&gt; &lt;p&gt;  Dans "Rire et pleurer", il analyse ces expressions comme réponses excentriques au pathique, révélant la distance ironique de l'humain à soi. Quant à &lt;em&gt;Les Limites de la communauté&lt;/em&gt;, paru en 1924, il rejette le radicalisme communautaire au profit d'une sociologie de la "distance naturelle", préfigurant Habermas. Son œuvre principale, &lt;em&gt;Les Degrés de l’organique et l’homme&lt;/em&gt; (1928), décrit la vie à partir de la manière dont chaque être se rapporte à sa limite : la plante est ouverte à son milieu, l’animal est centré sur lui-même, l’homme seul peut se voir de l’extérieur. D’origine juive, Plessner doit quitter l’Allemagne en 1933 pour les Pays-Bas. Dans &lt;em&gt;La Nation retardée&lt;/em&gt;, il analyse les causes du nazisme. Revenu en 1951, il enseigne la sociologie à Göttingen. &lt;/p&gt; </t>
-        </is>
+        <v>478</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>479</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>489</v>
+        <v>480</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
       <c r="H57" s="9" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
       <c r="I57" s="7"/>
       <c r="J57" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="L57" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="M57" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="N57" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="O57" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="144.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="7" t="n">
+        <v>1892</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>425</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>487</v>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Helmuth_Plessner"  title=" Wikipedia"&gt;Helmuth PLESSNER&lt;/a&gt; était un philosophe allemand, fondateur clé de &lt;a href="https://publictionnaire.huma-num.fr/notice/plessner-helmuth/"   title="L’apport de l’anthropologie  par Publitionnaire"&gt;l'anthropologie philosophique &lt;/a&gt;  européenne aux côtés de figures comme Max Scheler et Arnold Gehlen. Influencé par le néokantisme, la phénoménologie et la biologie, il développa une vision de l'humain comme être "naturellement artificiel", marqué par une "positionnalité excentrique" qui le distingue des animaux. &lt;/p&gt; &lt;p&gt;  L'homme vit à distance de son corps et de son milieu, possédant simultanément un corps et étant un corps vivant. Cela génère trois lois anthropologiques : la loi de l'"excentricité", celle de la "médiation"  et celle de l'"utopie naturelle". &lt;/p&gt; &lt;p&gt; Il dépasse le dualisme nature/esprit en fondant une herméneutique biologique : la vie s'exprime via les frontières organiques, et l'intentionnalité humaine émerge de cette interaction environnementale, non d'un ego transcendantal. &lt;/p&gt; &lt;p&gt;  Dans "Rire et pleurer", il analyse ces expressions comme réponses excentriques au pathique, révélant la distance ironique de l'humain à soi. Quant à &lt;em&gt;Les Limites de la communauté&lt;/em&gt;, paru en 1924, il rejette le radicalisme communautaire au profit d'une sociologie de la "distance naturelle", préfigurant Habermas. Son œuvre principale, &lt;em&gt;Les Degrés de l’organique et l’homme&lt;/em&gt; (1928), décrit la vie à partir de la manière dont chaque être se rapporte à sa limite : la plante est ouverte à son milieu, l’animal est centré sur lui-même, l’homme seul peut se voir de l’extérieur. D’origine juive, Plessner doit quitter l’Allemagne en 1933 pour les Pays-Bas. Dans &lt;em&gt;La Nation retardée&lt;/em&gt;, il analyse les causes du nazisme. Revenu en 1951, il enseigne la sociologie à Göttingen. &lt;/p&gt; </t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="G58" s="9" t="s">
+        <v>490</v>
+      </c>
+      <c r="H58" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="I58" s="7"/>
+      <c r="J58" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="K57" s="2" t="s">
+      <c r="K58" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="L57" s="2" t="s">
+      <c r="L58" s="2" t="s">
         <v>492</v>
       </c>
-      <c r="N57" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7" t="n">
+      <c r="N58" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="7" t="n">
         <v>1893</v>
       </c>
-      <c r="B58" s="7" t="s">
+      <c r="B59" s="7" t="s">
         <v>493</v>
       </c>
-      <c r="C58" s="7" t="s">
+      <c r="C59" s="7" t="s">
         <v>494</v>
       </c>
-      <c r="D58" s="8" t="s">
+      <c r="D59" s="8" t="s">
         <v>495</v>
       </c>
-      <c r="E58" s="13" t="inlineStr">
+      <c r="E59" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Mannheim" title=" Wikipedia"&gt;Karl MANNHEIM&lt;/a&gt;  était un philosophe allemand d'origine hongroise classé dans la sociologie de la connaissance et dans la sociologie compréhensive, à la frontière de la philosophie et des sciences sociales. Il ne sépare pas vraiment les deux domaines, car il cherche à montrer que la pensée dépend toujours d’un contexte social et historique. &lt;/p&gt; &lt;p&gt; Sa contribution la plus célèbre est  &lt;a href="https://www.youtube.com/watch?v=bBVJF4k_4-s"  title="transsiional sociologist par Socio exploration"&gt;Idéologie et utopie.&lt;/a&gt;  Dans ce livre, il explique que nos idées ne sont pas produites dans le vide: elles sont liées à notre position dans la société, à notre époque et à nos groupes d’appartenance. &lt;/p&gt; &lt;p&gt; Il  distingue notamment plusieurs formes d’idéologie et d’utopie. L’idéologie tend à justifier l’ordre existant, tandis que l’utopie ouvre la pensée vers une transformation du monde social. &lt;/p&gt; &lt;p&gt; Il défend aussi une forme de relationnisme: il ne dit pas que toute vérité est fausse, mais que les points de vue sont toujours partiels et situés. Cela lui permet de critiquer le relativisme absolu tout en reconnaissant que la connaissance humaine est historiquement conditionnée. Il  est un penseur des rapports entre   &lt;a href="https://www.youtube.com/watch?v=6R-Fre-UwgQ"  title="Sociological theory of culture  par Mannheuim"&gt;pensée, société et histoire.&lt;/a&gt;  On peut donc le ranger parmi les grands théoriciens de l’idéologie, de l’utopie et de la sociologie de la connaissance.   &lt;/p&gt; Né à Budapest en 1893, membre du cercle de Georg Lukács, il enseigne à Heidelberg puis à Francfort, avant de devoir fuir le nazisme en 1933 pour la London School of Economics. Dans un essai célèbre, il fait de la « génération » une notion sociologique : ceux qui ont vécu les mêmes événements à un âge semblable partagent une manière de voir le monde.
 </t>
         </is>
       </c>
-      <c r="F58" s="7" t="s">
+      <c r="F59" s="7" t="s">
         <v>497</v>
       </c>
-      <c r="G58" s="9" t="s">
+      <c r="G59" s="9" t="s">
         <v>498</v>
       </c>
-      <c r="H58" s="9" t="s">
+      <c r="H59" s="9" t="s">
         <v>499</v>
-      </c>
-      <c r="I58" s="7"/>
-      <c r="J58" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="K58" s="2" t="s">
-        <v>500</v>
-      </c>
-      <c r="L58" s="17" t="s">
-        <v>501</v>
-      </c>
-      <c r="M58" s="0" t="s">
-        <v>186</v>
-      </c>
-      <c r="N58" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="7" t="n">
-        <v>1895</v>
-      </c>
-      <c r="B59" s="7" t="s">
-        <v>502</v>
-      </c>
-      <c r="C59" s="7" t="s">
-        <v>503</v>
-      </c>
-      <c r="D59" s="8" t="s">
-        <v>504</v>
-      </c>
-      <c r="E59" s="9" t="s">
-        <v>505</v>
-      </c>
-      <c r="F59" s="7" t="s">
-        <v>506</v>
-      </c>
-      <c r="G59" s="9" t="s">
-        <v>507</v>
-      </c>
-      <c r="H59" s="9" t="s">
-        <v>508</v>
       </c>
       <c r="I59" s="7"/>
       <c r="J59" s="2" t="s">
-        <v>147</v>
+        <v>44</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>509</v>
-      </c>
-      <c r="L59" s="2" t="s">
-        <v>510</v>
+        <v>500</v>
+      </c>
+      <c r="L59" s="17" t="s">
+        <v>501</v>
       </c>
       <c r="M59" s="0" t="s">
         <v>186</v>
@@ -5056,40 +5078,40 @@
         <v>27</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="215.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="n">
-        <v>1897</v>
+        <v>1895</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>511</v>
+        <v>502</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>512</v>
+        <v>503</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>513</v>
-      </c>
-      <c r="E60" s="12" t="s">
-        <v>514</v>
+        <v>504</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>505</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>516</v>
+        <v>507</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>517</v>
+        <v>508</v>
       </c>
       <c r="I60" s="7"/>
       <c r="J60" s="2" t="s">
-        <v>518</v>
+        <v>147</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>519</v>
+        <v>509</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>520</v>
+        <v>510</v>
       </c>
       <c r="M60" s="0" t="s">
         <v>186</v>
@@ -5098,171 +5120,171 @@
         <v>27</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="316.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="215.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="n">
+        <v>1897</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>511</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>512</v>
+      </c>
+      <c r="D61" s="8" t="s">
+        <v>513</v>
+      </c>
+      <c r="E61" s="12" t="s">
+        <v>514</v>
+      </c>
+      <c r="F61" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>516</v>
+      </c>
+      <c r="H61" s="9" t="s">
+        <v>517</v>
+      </c>
+      <c r="I61" s="7"/>
+      <c r="J61" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="L61" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="M61" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="N61" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="316.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="7" t="n">
         <v>1899</v>
       </c>
-      <c r="B61" s="7" t="n">
+      <c r="B62" s="7" t="n">
         <v>1973</v>
       </c>
-      <c r="C61" s="7" t="s">
+      <c r="C62" s="7" t="s">
         <v>521</v>
       </c>
-      <c r="D61" s="8" t="inlineStr">
+      <c r="D62" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Leo STRAUSS</t>
         </is>
       </c>
-      <c r="E61" s="14" t="inlineStr">
+      <c r="E62" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Leo_Strauss" title=" Wikipedia"&gt;Leo STRAUSS&lt;/a&gt; était un philosophe politique germano-américain, connu pour sa critique profonde de la modernité et pour sa relecture des grands textes de la philosophie politique classique. Sa pensée a eu une influence durable, notamment aux États‑Unis, où elle a marqué des générations d’étudiants en théorie politique. &lt;/p&gt; &lt;p&gt; Au cœur de sa philosophie se trouve l’idée que la modernité a rompu avec le droit naturel classique, c’est‑à‑dire avec la recherche de ce qui est juste par nature et non simplement selon l’histoire ou les sciences sociales. Il voit dans le positivisme, le relativisme et l’historicisme modernes une source de décadence intellectuelle, car ils empêchent de poser les questions normatives fondamentales : qu’est‑ce qu’une vie bonne, qu’est‑ce qu’un régime politique juste. Pour lui, la  &lt;a href="https://www.persee.fr/doc/rfsp_0035-2950_1985_num_35_4_394205" title="philosophie et zscience politique par persée"&gt;philosophie politique authentique &lt;/a&gt; doit réactiver ces questions et affronter directement les notions de meilleur régime et d’ordre politique juste, plutôt que de se contenter de descriptions neutres. &lt;/p&gt; &lt;p&gt; Cette critique le conduit à renouer avec les auteurs de l’Antiquité, en particulier Platon, Aristote et les philosophes médiévaux juifs et arabes, qu’il lit souvent contre les interprétations modernes. Il insiste sur la dimension éducative de la philosophie : il parle de « liberal education » comme d’une libération de la vulgarité, entendue comme manque d’expérience des belles choses. La fréquentation des grands textes est, pour lui, une école de modestie et d’audace intellectuelle, parce qu’elle oblige à mesurer nos catégories modernes à celles d’auteurs qui pensaient autrement le politique et le juste. &lt;/p&gt; &lt;p&gt; Célèbre pour sa thèse sur l’« écriture ésotérique » : selon lui, nombre de philosophes du passé ont écrit de manière volontairement oblique pour se protéger de la censure ou de la persécution, réservant un sens plus profond aux lecteurs attentifs. Cela l’amène à distinguer entre le message « exotérique » (apparent, destiné au grand public) et le message « ésotérique » (plus exigeant, adressé à une minorité philosophique). Cette hypothèse sur la lecture des classiques s’articule à sa conception du   &lt;a href="https://www.youtube.com/watch?v=9Vhsveytymk" title="nihilisme et politique leo strauss par bildung et culture"&gt;mode de vie philosophique, &lt;/a&gt; toujours exposé au risque de la tyrannie et de l’incompréhension. Ainsi, sa philosophie politique est à la fois une critique de la modernité et une tentative de redécouvrir la place de la philosophie au cœur du politique contemporain. &lt;/p&gt; 
  &lt;audio controls title="la pensée de leon strauss par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/13397-05.04.2008-ITEMA_20118283-2008C3397E0019-ITE_00016207_RSCE-21.mp3" type="audio/mpeg" align="center"&gt;&lt;/audio&gt;  
 </t>
         </is>
       </c>
-      <c r="F61" s="7" t="s">
+      <c r="F62" s="7" t="s">
         <v>524</v>
       </c>
-      <c r="G61" s="9" t="s">
+      <c r="G62" s="9" t="s">
         <v>525</v>
       </c>
-      <c r="H61" s="12" t="s">
+      <c r="H62" s="12" t="s">
         <v>526</v>
-      </c>
-      <c r="I61" s="7"/>
-      <c r="J61" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="K61" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="L61" s="2" t="s">
-        <v>528</v>
-      </c>
-      <c r="M61" s="0" t="s">
-        <v>186</v>
-      </c>
-      <c r="N61" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="231.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="7" t="n">
-        <v>1900</v>
-      </c>
-      <c r="B62" s="7" t="s">
-        <v>529</v>
-      </c>
-      <c r="C62" s="7" t="s">
-        <v>530</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="E62" s="13" t="s">
-        <v>532</v>
-      </c>
-      <c r="F62" s="7" t="s">
-        <v>533</v>
-      </c>
-      <c r="G62" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Gadamer on Language &amp; Understanding (1970)" par Philosophy Overdose</t>
-        </is>
-      </c>
-      <c r="H62" s="9" t="s">
-        <v>535</v>
       </c>
       <c r="I62" s="7"/>
       <c r="J62" s="2" t="s">
-        <v>210</v>
+        <v>344</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="L62" s="17" t="s">
-        <v>536</v>
+        <v>527</v>
+      </c>
+      <c r="L62" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="M62" s="0" t="s">
+        <v>186</v>
       </c>
       <c r="N62" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="231.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="n">
-        <v>1903</v>
+        <v>1900</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>539</v>
-      </c>
-      <c r="E63" s="9" t="s">
-        <v>540</v>
+        <v>531</v>
+      </c>
+      <c r="E63" s="13" t="s">
+        <v>532</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>541</v>
-      </c>
-      <c r="G63" s="9" t="s">
-        <v>542</v>
+        <v>533</v>
+      </c>
+      <c r="G63" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Gadamer on Language &amp; Understanding (1970)" par Philosophy Overdose</t>
+        </is>
       </c>
       <c r="H63" s="9" t="s">
-        <v>543</v>
+        <v>535</v>
       </c>
       <c r="I63" s="7"/>
       <c r="J63" s="2" t="s">
-        <v>544</v>
+        <v>210</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>509</v>
-      </c>
-      <c r="L63" s="2" t="s">
-        <v>545</v>
-      </c>
-      <c r="M63" s="0" t="s">
-        <v>186</v>
+        <v>157</v>
+      </c>
+      <c r="L63" s="17" t="s">
+        <v>536</v>
       </c>
       <c r="N63" s="0" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="176.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="n">
         <v>1903</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>546</v>
+        <v>537</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>547</v>
+        <v>538</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>548</v>
-      </c>
-      <c r="E64" s="12" t="s">
-        <v>549</v>
+        <v>539</v>
+      </c>
+      <c r="E64" s="9" t="s">
+        <v>540</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>550</v>
+        <v>541</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>551</v>
+        <v>542</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>552</v>
+        <v>543</v>
       </c>
       <c r="I64" s="7"/>
       <c r="J64" s="2" t="s">
-        <v>362</v>
+        <v>544</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>553</v>
+        <v>509</v>
       </c>
       <c r="L64" s="2" t="s">
-        <v>554</v>
+        <v>545</v>
       </c>
       <c r="M64" s="0" t="s">
         <v>186</v>
@@ -5271,40 +5293,43 @@
         <v>27</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="195.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="176.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="n">
-        <v>1904</v>
+        <v>1903</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>441</v>
+        <v>546</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>556</v>
-      </c>
-      <c r="E65" s="13" t="s">
-        <v>557</v>
+        <v>548</v>
+      </c>
+      <c r="E65" s="12" t="s">
+        <v>549</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>558</v>
+        <v>550</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>559</v>
+        <v>551</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>560</v>
+        <v>552</v>
       </c>
       <c r="I65" s="7"/>
       <c r="J65" s="2" t="s">
-        <v>44</v>
+        <v>362</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="L65" s="17" t="s">
-        <v>561</v>
+        <v>553</v>
+      </c>
+      <c r="L65" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="M65" s="0" t="s">
+        <v>186</v>
       </c>
       <c r="N65" s="0" t="s">
         <v>27</v>
@@ -5312,186 +5337,169 @@
     </row>
     <row r="66" customFormat="false" ht="195.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="n">
-        <v>1922</v>
-      </c>
-      <c r="B66" s="7" t="n">
-        <v>2017</v>
+        <v>1904</v>
+      </c>
+      <c r="B66" s="7" t="s">
+        <v>441</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>562</v>
+        <v>555</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>563</v>
-      </c>
-      <c r="E66" s="21" t="s">
-        <v>564</v>
+        <v>556</v>
+      </c>
+      <c r="E66" s="13" t="s">
+        <v>557</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>565</v>
-      </c>
-      <c r="G66" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Karl-Otto APEL par Daniel Ronnedal</t>
-        </is>
-      </c>
-      <c r="H66" s="12" t="s">
-        <v>567</v>
+        <v>558</v>
+      </c>
+      <c r="G66" s="9" t="s">
+        <v>559</v>
+      </c>
+      <c r="H66" s="9" t="s">
+        <v>560</v>
       </c>
       <c r="I66" s="7"/>
       <c r="J66" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="L66" s="17" t="s">
+        <v>561</v>
+      </c>
+      <c r="N66" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="195.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="7" t="n">
+        <v>1922</v>
+      </c>
+      <c r="B67" s="7" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>562</v>
+      </c>
+      <c r="D67" s="8" t="s">
+        <v>563</v>
+      </c>
+      <c r="E67" s="21" t="s">
+        <v>564</v>
+      </c>
+      <c r="F67" s="7" t="s">
+        <v>565</v>
+      </c>
+      <c r="G67" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Karl-Otto APEL par Daniel Ronnedal</t>
+        </is>
+      </c>
+      <c r="H67" s="12" t="s">
+        <v>567</v>
+      </c>
+      <c r="I67" s="7"/>
+      <c r="J67" s="2" t="s">
         <v>568</v>
       </c>
-      <c r="K66" s="2" t="inlineStr">
+      <c r="K67" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Théorie Critique ; Déontologisme</t>
         </is>
       </c>
-      <c r="L66" s="17" t="s">
+      <c r="L67" s="17" t="s">
         <v>569</v>
       </c>
-      <c r="N66" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="202.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="1" t="n">
+      <c r="N67" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="202.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="n">
         <v>1929</v>
       </c>
-      <c r="B67" s="1" t="n">
+      <c r="B68" s="1" t="n">
         <v>2026</v>
       </c>
-      <c r="C67" s="1" t="s">
+      <c r="C68" s="1" t="s">
         <v>570</v>
       </c>
-      <c r="D67" s="22" t="s">
+      <c r="D68" s="22" t="s">
         <v>571</v>
       </c>
-      <c r="E67" s="19" t="inlineStr">
+      <c r="E68" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/J%C3%BCrgen_Habermas"  title=" Wikipedia"&gt;Jürgen HABERMAS&lt;/a&gt; est un philosophe allemand connu pour avoir écrit  "Théorie de l'agir communicationnel" où il développe la théorie de l'agir communicationnel, qui met l'accent sur le rôle de la communication et du langage dans la construction de la société.  &lt;/p&gt; &lt;p&gt; Dans son livre  &lt;a href="https://www.persee.fr/doc/polix_0295-2319_1989_num_2_5_2021" title="Extrait de l'espace public par Persée.fr"&gt;"L'espace public"&lt;/a&gt;, ( le premier à avoir aborder le sujet fut KANT) il considère que c'est un lieu crucial de débat et de délibération, c'est l'agir communicationnel où les citoyens peuvent  &lt;a href="https://www.youtube.com/watch?v=PnY0Jg8NH1g"   title="t l'espace public par Mélannie Moreau"&gt;s'exprimer &lt;/a&gt; et discuter de manière ouverte et équitable des questions politiques et sociales qui les concernent. Ils ont une capacité innée à communiquer et à agir ensemble de manière coopérative leurs permettant de réguler les relations entre les individus et de créer des normes et des valeurs partagées. &lt;/p&gt; &lt;p&gt;  Il considère que l'expansion des systèmes bureaucratiques et économiques ont réduit les possibilités  &lt;a href="https://www.youtube.com/watch?v=R1K46oK3xTU&amp;ab_channel=Then%26Now"  title="La transformation structurelle de la sphère publique par Then &amp; Now"&gt;d'interaction sociale &lt;/a&gt; et ont aliéné les individus de leurs propres intérêts et valeurs et il pense que la participation active des citoyens à la vie politique est essentielle pour garantir une société juste et équitable. &lt;/p&gt; &lt;p&gt;  Il  théorise la démocratie délibérative, où la légitimité naît du débat rationnel plutôt que du marché ou de la tradition. Ses  &lt;a href="https://www.youtube.com/watch?v=OzAWFDkaCcE"   title="Il s’est trompé depuis 40 ans par Tocsin et 2 autres"&gt;interventions sur l'Europe&lt;/a&gt;, le droit et la religion ("post-sécularisme") influencent la philosophie politique globale, reliant émancipation individuelle et solidarité collective.   &lt;/p&gt;  &lt;audio controls title="Habernas, le dernier philosophe ? par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2015/09/s38/NET_FC_c7667f83-aa22-41cb-ba4e-d7567cc16be1.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
-      <c r="F67" s="23" t="s">
+      <c r="F68" s="23" t="s">
         <v>573</v>
       </c>
-      <c r="G67" s="10" t="s">
+      <c r="G68" s="10" t="s">
         <v>574</v>
       </c>
-      <c r="H67" s="10" t="s">
+      <c r="H68" s="10" t="s">
         <v>575</v>
       </c>
-      <c r="I67" s="10"/>
-      <c r="J67" s="2" t="s">
+      <c r="I68" s="10"/>
+      <c r="J68" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="K67" s="2" t="inlineStr">
+      <c r="K68" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Théorie Critique ; Déontologisme</t>
         </is>
       </c>
-      <c r="L67" s="2" t="s">
+      <c r="L68" s="2" t="s">
         <v>576</v>
       </c>
-      <c r="N67" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="O67" s="0" t="n">
+      <c r="N68" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="O68" s="0" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="183.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="7" t="n">
+    <row r="69" customFormat="false" ht="183.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="7" t="n">
         <v>1941</v>
       </c>
-      <c r="B68" s="7" t="n">
+      <c r="B69" s="7" t="n">
         <v>1993</v>
       </c>
-      <c r="C68" s="7" t="s">
+      <c r="C69" s="7" t="s">
         <v>577</v>
       </c>
-      <c r="D68" s="8" t="s">
+      <c r="D69" s="8" t="s">
         <v>578</v>
       </c>
-      <c r="E68" s="14" t="s">
+      <c r="E69" s="14" t="s">
         <v>579</v>
       </c>
-      <c r="F68" s="7" t="s">
+      <c r="F69" s="7" t="s">
         <v>580</v>
       </c>
-      <c r="G68" s="9" t="s">
+      <c r="G69" s="9" t="s">
         <v>581</v>
       </c>
-      <c r="H68" s="9" t="s">
+      <c r="H69" s="9" t="s">
         <v>582</v>
       </c>
-      <c r="I68" s="9"/>
-      <c r="J68" s="2" t="s">
+      <c r="I69" s="9"/>
+      <c r="J69" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="K68" s="2" t="s">
+      <c r="K69" s="2" t="s">
         <v>583</v>
       </c>
-      <c r="L68" s="2" t="s">
+      <c r="L69" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="N68" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="267.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0">
-        <v>1883</v>
-      </c>
-      <c r="B69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1969</t>
-        </is>
-      </c>
-      <c r="C69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1883 – 1969</t>
-        </is>
-      </c>
-      <c r="D69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Karl JASPERS</t>
-        </is>
-      </c>
-      <c r="E69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Karl_Jaspers" title=" Wikipedia"&gt;Karl JASPERS&lt;/a&gt; est un psychiatre et philosophe allemand, l’un des fondateurs de la philosophie de l’existence. Né à Oldenbourg, il étudie le droit puis la médecine et travaille à la clinique psychiatrique de Heidelberg. Son &lt;em&gt;Psychopathologie générale&lt;/em&gt; (1913) renouvelle la psychiatrie en distinguant ce que l’on peut « expliquer » par des causes et ce que l’on doit « comprendre » de l’intérieur, dans l’expérience du malade. Il se tourne ensuite vers la philosophie, qu’il enseigne à Heidelberg.&lt;/p&gt; &lt;p&gt;Dans sa &lt;em&gt;Philosophie&lt;/em&gt; (1932), il distingue l’existence de tout ce que la science peut connaître : ce que je suis vraiment ne se laisse pas réduire à un objet. C’est dans les « situations limites », la mort, la souffrance, la lutte, la culpabilité, que l’homme découvre qu’il ne peut rien maîtriser et s’ouvre à la « transcendance ». La communication authentique avec autrui, une « lutte aimante », est le lieu où chacun devient lui-même. Il forge aussi la notion d’« âge axial » pour désigner le moment, autour du VIe siècle avant notre ère, où naissent presque en même temps les grandes sagesses de la Chine, de l’Inde, de la Perse, d’Israël et de la Grèce.&lt;/p&gt; &lt;p&gt;Marié à une femme juive, Gertrud, il est privé d’enseignement par les nazis en 1937 et vit sous la menace de la déportation. Après la guerre, il publie &lt;em&gt;La Culpabilité allemande&lt;/em&gt; (1946), où il distingue culpabilité criminelle, politique, morale et métaphysique. Maître et ami d’&lt;a href="https://fr.wikipedia.org/wiki/Hannah_Arendt" title=" Wikipedia"&gt;Hannah Arendt&lt;/a&gt;, il s’installe à Bâle en 1948 et y meurt en 1969.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F69" s="0"/>
-      <c r="G69" s="0"/>
-      <c r="H69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/jaspers-mini.webp</t>
-        </is>
-      </c>
-      <c r="I69" s="0"/>
-      <c r="J69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">metaphysique ; politique</t>
-        </is>
-      </c>
-      <c r="K69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Existentialisme</t>
-        </is>
-      </c>
-      <c r="L69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">psychiatre et philosophe allemand, penseur de l’existence, des situations limites et de la culpabilité.</t>
-        </is>
-      </c>
-      <c r="N69" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O69">
-        <v>3</v>
+      <c r="N69" s="0" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5634,20 +5642,20 @@
     <hyperlink ref="E45" r:id="rId20" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hermann_von_Keyserling&quot; title=&quot; Wikipedia&quot;&gt;Hermann Von KEYSERLING&lt;/a&gt;  était un philosophe  &lt;a href=&quot;https://www.persee.fr/doc/slaoc_1245-2491_1997_num_4_1_1809&quot; style=&quot;color:#88A1E9&quot; title=&quot; Hermann von Keyserling et les interférences germano-slaves par Persée&quot;&gt;germano-balte &lt;/a&gt; devenu philosophe voyageur, figure très en vue de la République de Weimar, connu pour son Journal de voyage d’un philosophe et pour son &quot;École de la sagesse&quot; à Darmstadt. &lt;/p&gt; &lt;p&gt; Il conçoit la philosophie non comme une science rigoureuse, mais comme sagesse vécue : &quot;la vie elle-même sous la forme du savoir&quot;, contre les théories objectivantes du savoir technico-scientifique. Il s’inscrit dans la philosophie de la vie, mais de façon personnelle : importance de l’intuition, de la singularité des événements et de la transformation intérieure. Son projet est une nouvelle synthèse de l’âme et de l’esprit, la pénétration réciproque de sagesse et politique, et l’idée que dans la vie déterminée par l’esprit, c’est &lt;a href=&quot;https://www.youtube.com/watch?v=Y0DY8F72114&quot; title=&quot;Eduard von Keyserling, DUMALA par Le Veilleur&quot;&gt;le Sens &lt;/a&gt; qui crée les faits plutôt que l’inverse. &lt;/p&gt; &lt;p&gt; Il  utilise très tôt le terme Führerprinzip, en liant l’idée de &quot;dirigeants nés&quot; à un élitisme spiritualiste et social-darwinien, tout en refusant par la suite d’adhérer au national-socialisme, qu’il voit comme mouvement de masses manipulées.  Le régime nazi ferme son École de la sagesse au milieu des années 1930, lui interdit de publier et de voyager, tandis que sa réputation continue de grandir à l’étranger. &lt;/p&gt;&lt;p&gt; Ses oeuvres principales sont : - &quot;Reisetagebuch eines Philosophen&quot;  paru en 1919 : récit de son tour du monde (1911-1912, Asie, Amérique, Europe du Sud) mêlant observations culturelles, méditations spirituelles et diagnostics sur les civilisations ; c’est son grand succès de librairie, largement traduit. -&quot;Das Gefüge der Welt. Versuch einer kritischen Philosophie&quot; (La Structure du monde, 1907) : tentative de &quot;philosophie critique&quot; personnelle, déjà marquée par l’idée que le savoir véritable est inséparable de la vie. - &quot;Schöpferische Erkenntnis&quot; (Connaissance créatrice) et &quot;Wiedergeburt&quot; (Renaissance) : textes doctrinaux de l’&quot;École de la sagesse&quot;, insistant sur la connaissance comme acte créateur, transformant la vie plutôt que la décrivant objectivement. &lt;/p&gt; "/>
     <hyperlink ref="E46" r:id="rId21" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Moritz_Schlick&quot;  title=&quot; Wikipedia&quot;&gt;Moritz SCHLICK&lt;/a&gt; était un philosophe allemand, physicien de formation, et l’une des figures centrales de l’empirisme logique. Il est surtout connu comme le fondateur et le dirigeant intellectuel du Cercle de Vienne, groupe qui se réunissait autour de la philosophie des sciences dans les années 1920 et 1930. Il occupa à Vienne une chaire autrefois associée à Ernst Mach et à Ludwig Boltzmann. &lt;/p&gt; &lt;p&gt; Sa première grande œuvre est la Théorie générale de la connaissance (Allgemeine Erkenntnislehre, 1918). Dans cet ouvrage, il défend encore une forme de réalisme scientifique : le monde extérieur existe indépendamment de nous et peut être connu grâce aux sciences. Il s’oppose ainsi à l’idéalisme et à l’idée kantienne selon laquelle nous ne connaîtrions jamais les choses en elles-mêmes. Pour lui, connaître consiste notamment à coordonner des signes et des concepts avec les objets et les processus étudiés par les sciences. &lt;/p&gt; &lt;p&gt;  À partir des années 1920, son orientation évolue sous l’influence de Wittgenstein et du développement de la logique moderne. Il affirme alors que la philosophie ne doit pas construire une nouvelle vision métaphysique du monde, mais clarifier le sens des propositions. Une &lt;a href=&quot;https://encyclo-philo.fr/schlick-a&quot;  title=&quot;l’encyclopedie philosophique : schick par encyclophilo&quot;&gt;proposition authentiquement scientifique &lt;/a&gt; doit pouvoir être reliée à une méthode possible de vérification empirique ; les énoncés de logique et de mathématiques sont, quant à eux, analytiques ou tautologiques. Cette orientation est souvent résumée par la formule : « le sens d’une proposition est sa méthode de vérification ». &lt;/p&gt; &lt;p&gt; Il faut cependant éviter de le réduire à un vérificationnisme simpliste. Il admet qu’une proposition puisse être vérifiable en principe, même si la vérification ne peut pas être réalisée immédiatement ou matériellement. La vérification ne signifie donc pas forcément une observation actuelle, mais la possibilité de décrire une procédure permettant de déterminer si l’énoncé est vrai ou faux. Sur le plan éthique, Il ne pense pas que les jugements de valeur soient des connaissances scientifiques ; il leur accorde néanmoins une importance dans la vie humaine et dans l’analyse des motivations. &lt;/p&gt; &lt;p&gt; On peut le classer comme un philosophe des sciences, un empiriste logique, &lt;a href=&quot;https://www.youtube.com/watch?v=ESWQzsf1Fr4&quot;  title=&quot;la fin du positivisme logique par philo analytique&quot;&gt;un positiviste logique &lt;/a&gt; et un représentant de la philosophie analytique naissante. Il est plus central et plus systématique que Hans Hahn dans l’organisation du Cercle de Vienne, tandis que Hahn était avant tout mathématicien et philosophe des fondements des mathématiques. Sa pensée se situe à la rencontre du réalisme scientifique, de l’empirisme, de l’analyse logique du langage et de l’anti-métaphysique ; son projet fondamental était de faire de la philosophie une activité de clarification au service de la connaissance scientifique. &lt;/p&gt; &#10;"/>
     <hyperlink ref="H46" r:id="rId22" display="https://www.laphilo.fr/pho/mschlick-mini.webp"/>
-    <hyperlink ref="E48" r:id="rId23" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl_Korsch&quot; title=&quot; Wikipedia&quot;&gt;Karl KORDCH&lt;/a&gt;  était un philosophe marxiste allemand,  théoricien du communisme de conseils et critique du léninisme orthodoxe. Issu d'un milieu bourgeois, il évolua du réformisme social au marxisme hétérodoxe, influençant les courants ultra-gauche via son rejet du matérialisme positiviste et son insistance sur la praxis révolutionnaire historique.  Exclu du parti en 1926 pour &quot;ultra-gauchisme&quot;, il émigra après 1933 vers les USA, où il approfondit sa théorie marxiste. &lt;/p&gt; &lt;p&gt; Son œuvre majeure &quot;Marxisme et philosophie&quot; paru en 1923 marque sa rupture avec le léninisme en critiquant sa dérive scientiste. Il   &lt;a href=&quot;https://www.zones-subversives.com/article-le-marxisme-critique-de-karl-korsch-116431466.html&quot;  title=&quot;Le marxisme critique de Karl Korsch par Chroniques critiques&quot;&gt;rejette le marxisme &lt;/a&gt; comme &quot;science positive&quot; figée ou philosophie matérialiste abstraite ; il le conçoit comme une théorie historique et concrète, liée à la lutte des classes et à la dialectique hégélienne réinterprétée comme expression de la révolution bourgeoise puis prolétarienne. &lt;/p&gt; &lt;p&gt; Il  théorise les conseils comme organes centraux de la transition socialiste, via la praxis dialectique et l'auto-activité des masses, contre la socialisation étatique. Ses écrits inspirent le KAPD et l'ultra-gauche, voyant les conseils comme alternative à la bureaucratisation stalinienne. Son influence perdure chez les communistes de conseils, soulignant la conscience ouvrière spontanée pour l'émancipation réelle. &lt;/p&gt; "/>
-    <hyperlink ref="E51" r:id="rId24" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Eugen_Rosenstock-Huessy&quot; title=&quot; Wikipedia&quot;&gt;Eugen ROSENSTOCK-HUESSY&lt;/a&gt; était un penseur germano‑américain dont l'œuvre mêle philosophie sociale, histoire des idées et une théorie du langage centrée sur la parole comme acte créateur et structurant de la vie collective. Né en Allemagne, il forma des liens intellectuels avec des figures comme Franz Rosenzweig et Martin Buber, fut professeur (notamment aux États‑Unis après son exil) et créa une œuvre originale qui vise à comprendre comment les communautés se constituent et se transforment dans le temps par des échanges de parole. &lt;/p&gt; &lt;p&gt; Au  &lt;a href=&quot;https://www.en-attendant-nadeau.fr/2019/11/19/homme-quadridimensionnel-rosenstock//&quot;  title=&quot;l’homme quadridimensionnel par ean&quot;&gt;cœur de sa pensée &lt;/a&gt;  se trouve la notion de &quot;speech thinking&quot; (pensée de la parole) : il soutient que la parole n’est pas qu’un moyen descriptif, mais un acte répondant et créatif qui institue des relations sociales, forge des temporalités collectives et permet la transmission et la renouvellement des institutions humaines. Il affirme que, par le langage, les groupes deviennent « maîtres du temps » en fondant de nouveaux commencements, en rappelant le passé et en orientant l’action future — d’où son intérêt pour la densité historique de la vie sociale et le rôle des rituels, des serments et des discours publics. &lt;/p&gt; &lt;p&gt; Sur la religion et la théologie, il s’inscrit dans un courant post‑nietzschéen de renouveau religieux qui comprend Rosenzweig et Buber; il considère les énoncés religieux comme des actes de parole non‑métaphysiques qui dévoilent des dimensions de l’expérience humaine et communautaire inaccessibles aux seules sciences naturelles. Cette orientation le conduit à une pensée intégrative où philosophie, théologie et histoire participent à une réflexion pratique sur la transformation sociale et la responsabilité collective. &lt;/p&gt; &lt;p&gt; Ses livres et conférences couvrent une grande variété de thèmes — histoire des peuples, rhétorique sociale, philosophie de la loi et de l’éducation — et sa méthode combine analyses historiques, typologies du langage et propositions pour renouveler la vie civique; son influence se voit aujourd’hui dans des études sur la communication, la sociologie historique et la philosophie de la culture. &lt;/p&gt; "/>
-    <hyperlink ref="H51" r:id="rId25" display="https://www.laphilo.fr/pho/erhuessy-mini.webp"/>
-    <hyperlink ref="E53" r:id="rId26" display="&lt;p&gt; &lt;a href=&quot;https://fr.wikipedia.org/wiki/Oskar_Becker&quot;  title=&quot; Wikipedia&quot;&gt;Oskar BECKER&lt;/a&gt; était un philosophe, logicien, mathématicien et historien des mathématiques allemand, connu comme l’un des élèves les plus importants d’Edmund Husserl et comme un interlocuteur clé de Martin Heidegger. Sa pensée se situe à la croisée de la phénoménologie, de la philosophie des mathématiques, de la logique modale et de l’existentialisme. &lt;/p&gt; &lt;p&gt; Il utilise la phénoménologie husserlienne pour analyser les fondements de la géométrie, de l’arithmétique et de la logique, en cherchant à décrire les expériences vécues (compter, mesurer, démontrer) comme actes de conscience. Il tente ainsi de fonder une  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Ph%C3%A9nom%C3%A9nologie&quot;  title=&quot;phénoménologie par wikipedia&quot;&gt; sémantique phénoménologique &lt;/a&gt; de la logique intuitionniste, et ses idées sont reprises par Arend Heyting dans sa formalisation de cette logique. À la fin de sa vie, il insiste sur une distinction entre une intuition du domaine formel et platonicien (mathématiques pures) et un domaine existentiel concret, en utilisant parfois un vocabulaire proche de la « divination ». &lt;/p&gt; &lt;p&gt;Il est aussi un pionnier de la logique modale (logique de la nécessité et de la possibilité). On lui doit notamment ce qu’on appelle le postulat de Becker : l’idée que le statut modal est nécessaire, par exemple que la possibilité de PPP implique la nécessité de la possibilité de PPP, ainsi que certaines lois d’itération de la nécessité. Ces résultats ont joué un rôle important dans le développement de la logique modale au XXᵉ siècle. &lt;/p&gt; &lt;p&gt; Il entretient un dialogue étroit avec Heidegger : il reprend certains thèmes existentialistes (finitude, historicité, être-pour-la-mort) et les applique à des domaines comme les mathématiques, ce qui est très controversé (par exemple, discuter du comptage arithmétique comme « être-pour-la-mort »). Il développe également une « paraontologie » : une doctrine de l’essence et de la permanence des choses, distincte de l’ontologie heideggérienne centrée sur l’existence du Dasein. Pour lui, l’être humain n’existe pas seulement comme existence, mais aussi comme « paraexistence », incluant des dimensions inconscientes et surconscientes. &lt;/p&gt; &#10;&#10;"/>
-    <hyperlink ref="H53" r:id="rId27" display="https://www.laphilo.fr/pho/obecker-mini.webp"/>
-    <hyperlink ref="E54" r:id="rId28" display="https://fr.wikipedia.org/wiki/Edith_Stein"/>
-    <hyperlink ref="H54" r:id="rId29" display="https://www.laphilo.fr/pho/estein-mini.webp"/>
-    <hyperlink ref="E60" r:id="rId30" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Gershom_Scholem&quot; title=&quot; Wikipedia&quot;&gt;Gershom SCHOLEM&lt;/a&gt; était un philosophe juif germano-israélien,  fondateur de l'étude académique moderne de la Kabbale et grand expert de  &lt;a href=&quot;https://www.nonfiction.fr/article-12478-gershom-scholem-de-berlin-a-la-palestine.htm&quot; title=&quot;Gershom Scholem : de Berlin à la Palestine  par nonfiction&quot;&gt;la mystique juive. &lt;/a&gt; Né à Berlin dans une famille assimilée, il s'est tourné vers le sionisme jeune et a immigré en Palestine en 1923, devenant professeur à l'Université hébraïque de Jérusalem. &lt;/p&gt; &lt;p&gt; Il a étudié les mathématiques, la philosophie et les langues sémitiques à Berlin, Iéna et Munich, où il a soutenu une thèse sur le &quot;Sefer ha-Bahir&quot;, un texte kabbalistique ancien. Ami proche de Walter Benjamin et correspondant de Leo Strauss, il a fui l'Europe nazie et s'est consacré à la recherche sur les manuscrits juifs pillés. &lt;/p&gt; &lt;p&gt; Il voyait  &lt;a href=&quot;https://www.youtube.com/watch?v=5HvDF8-XTjc&quot;  title=&quot;Dieu son nom et la Cabale selon Gershom Scholem  par Xavier Charles DJEBALI&quot;&gt;la Kabbale &lt;/a&gt; non comme une superstition marginale, mais au cœur de l'essence spirituelle du judaïsme, explorée via des méthodes scientifiques et historiques. Il insistait sur le rôle du messianisme et de la tradition comme forces de renouvellement, où la révélation divine est infiniment interprétable et liée à l'expérience historique du peuple juif. Pour lui, le sionisme allait au-delà de la politique : c'était un renouveau profond du judaïsme, unissant ancien et nouveau contre l'assimilation. &lt;/p&gt; &lt;p&gt; Son oeuvre majeure &quot;Les Grandes tendances de la mystique juive&quot; paru en 1941, basé sur des conférences, dédié à Benjamin, explore l'évolution de la mystique juive. Sa pensée met l'accent sur l'identité juive forgée par l'histoire, où la tradition intègre la nouveauté pour survivre aux crises. &lt;/p&gt; &lt;audio controls title=&quot;Des livres pour notre temps et les mondes à venir. 1/2 Gershom Scholem : penser dans les marges de la marge par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13094-10.11.2019-ITEMA_22199082-0.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
-    <hyperlink ref="E61" r:id="rId31" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Leo_Strauss&quot; title=&quot; Wikipedia&quot;&gt;Leo SRAUSS&lt;/a&gt; était un philosophe politique germano-américain, connu pour sa critique profonde de la modernité et pour sa relecture des grands textes de la philosophie politique classique. Sa pensée a eu une influence durable, notamment aux États‑Unis, où elle a marqué des générations d’étudiants en théorie politique. &lt;/p&gt; &lt;p&gt; Au cœur de sa philosophie se trouve l’idée que la modernité a rompu avec le droit naturel classique, c’est‑à‑dire avec la recherche de ce qui est juste par nature et non simplement selon l’histoire ou les sciences sociales. Il voit dans le positivisme, le relativisme et l’historicisme modernes une source de décadence intellectuelle, car ils empêchent de poser les questions normatives fondamentales : qu’est‑ce qu’une vie bonne, qu’est‑ce qu’un régime politique juste. Pour lui, la  &lt;a href=&quot;https://www.persee.fr/doc/rfsp_0035-2950_1985_num_35_4_394205&quot; title=&quot;philosophie et zscience politique par persée&quot;&gt;philosophie politique authentique &lt;/a&gt; doit réactiver ces questions et affronter directement les notions de meilleur régime et d’ordre politique juste, plutôt que de se contenter de descriptions neutres. &lt;/p&gt; &lt;p&gt; Cette critique le conduit à renouer avec les auteurs de l’Antiquité, en particulier Platon, Aristote et les philosophes médiévaux juifs et arabes, qu’il lit souvent contre les interprétations modernes. Il insiste sur la dimension éducative de la philosophie : il parle de « liberal education » comme d’une libération de la vulgarité, entendue comme manque d’expérience des belles choses. La fréquentation des grands textes est, pour lui, une école de modestie et d’audace intellectuelle, parce qu’elle oblige à mesurer nos catégories modernes à celles d’auteurs qui pensaient autrement le politique et le juste. &lt;/p&gt; &lt;p&gt; Célèbre pour sa thèse sur l’« écriture ésotérique » : selon lui, nombre de philosophes du passé ont écrit de manière volontairement oblique pour se protéger de la censure ou de la persécution, réservant un sens plus profond aux lecteurs attentifs. Cela l’amène à distinguer entre le message « exotérique » (apparent, destiné au grand public) et le message « ésotérique » (plus exigeant, adressé à une minorité philosophique). Cette hypothèse sur la lecture des classiques s’articule à sa conception du   &lt;a href=&quot;https://www.youtube.com/watch?v=9Vhsveytymk&quot; title=&quot;nihilisme et politique leo strauss par bildung et culture&quot;&gt;mode de vie philosophique, &lt;/a&gt; toujours exposé au risque de la tyrannie et de l’incompréhension. Ainsi, sa philosophie politique est à la fois une critique de la modernité et une tentative de redécouvrir la place de la philosophie au cœur du politique contemporain. &lt;/p&gt; &#10; &lt;audio controls title=&quot;la pensée de leon strauss par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13397-05.04.2008-ITEMA_20118283-2008C3397E0019-ITE_00016207_RSCE-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;  &#10;"/>
-    <hyperlink ref="H61" r:id="rId32" display="https://www.laphilo.fr/pho/lstrauss-mini.webp"/>
-    <hyperlink ref="E64" r:id="rId33" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hans_Jonas&quot; title=&quot; Wikipedia&quot;&gt;Hans JONAS&lt;/a&gt;  était un philosophe germano-américain connu pour ses travaux sur l'éthique de la technologie et &lt;a href=&quot;https://www.youtube.com/watch?v=NPIJHZO7hQo&quot; title=&quot; Le PRINCIPE RESPONSABILITÉ en 6 minutes ! (HANS JONAS) par Culture Philo&quot;&gt;la responsabilité&lt;/a&gt; envers les générations futures. Ses premières recherches portent sur le gnosticisme, vu comme une réponse à l'aliénation existentielle dans un monde hostile. Dans les années 1960, il développe une philosophie de la vie organique (The Phenomenon of Life), critiquant le dualisme cartésien et valorisant la nature vivante contre la technoscience destructrice. Son œuvre maîtresse &lt;a href=&quot;https://www.youtube.com/watch?v=LsIWCR9_N64&quot; style=&quot;color:#88A1E9&quot; title=&quot; Philo, Hans jonas, Le principe responsabilité, Bac philo par SOS Bac Français&quot;&gt; &quot;Le Principe responsabilité&quot;&lt;/a&gt; paru en1979, formule un impératif éthique pour l'ère technologique : &quot;Agis de façon que les effets de ton action soient compatibles avec la permanence d'une vie authentiquement humaine sur Terre&quot;. &lt;/p&gt; &lt;p&gt; Il  anticipe les crises écologiques et bioéthiques, proposant une &quot;heuristique de la peur&quot; pour guider l'action humaine face aux risques imprévisibles de la puissance technique. Influencé par sa tradition juive et Heidegger, il réconcilie existentialisme, phénoménologie et morale prophétique, impactant l'éthique environnementale contemporaine. &lt;/p&gt; &lt;p&gt; Il observe un &quot;déchaînement prométhéen&quot; : l'humanité acquiert un pouvoir inédit sur la nature via la science et la technique, capable de menacer sa propre survie et celle des générations futures. Contrairement aux éthiques classiques (kantienne ou utilitariste), limitées au présent ou aux intentions, sa réflexion intègre les conséquences à long terme, imprévisibles et collectives, sur la vie humaine et la planète. Face aux risques inconnus (nucléaire, génétique, environnementaux), il prône une &quot;heuristique de la peur&quot; : anticiper le pire scénario (in dubio pro malo) pour guider l'action, sans paralyser le progrès mais en le subordonnant à la préservation de la vie. Le savoir devient un devoir moral prioritaire, élargissant l'éthique à la nature et aux générations absentes.&lt;/p&gt;  &lt;/p&gt; &lt;p&gt;  &lt;audio controls title=&quot; Hans Jonas. Pour une éthique de la société technologique par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/22267-14.06.2021-ITEMA_22702122-2014C12410E0357.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
-    <hyperlink ref="E66" r:id="rId34" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl-Otto_Apel&quot; title=&quot; Wikipedia&quot;&gt;Karl-Otto APEL&lt;/a&gt; était un philosophe allemand majeur de l’après-guerre, surtout connu pour avoir développé, avec Jürgen Habermas, l’éthique du discours et pour sa « pragmatique transcendantale », une tentative de refonder la philosophie à partir des présupposés normatifs de l’argumentation. &lt;/p&gt; &lt;p&gt; Il est souvent crédité d’avoir opéré la « linguistification » de la philosophie transcendantale kantienne : au lieu de partir de la conscience ou du sujet (comme chez Kant ou Husserl), il part du fait que toute connaissance et toute action s’inscrivent dans un langage commun et une communauté de communication. Pour lui, les conditions de possibilité de la connaissance ne sont pas d’abord dans la structure de la conscience, mais dans les règles implicites de l’usage du langage et de l’argumentation. &lt;/p&gt; &lt;p&gt;  &lt;a href=&quot;https://www.youtube.com/watch?v=R9jQv_akxFE&quot; &gt;Sa notion centrale &lt;/a&gt; est celle d’a priori de la communauté de communication : le simple fait d’argumenter présuppose déjà un cadre normatif inévitable (recherche de vérité, reconnaissance mutuelle des interlocuteurs, exigence de cohérence, etc.). Quiconque tente de nier ces présupposés tombe dans une auto-contradiction performative : en les contestant par la parole, il les utilise déjà. Il en tire l’idée d’une fondation ultime de la rationalité et de l’éthique à partir de la structure même de l’argumentation. &lt;/p&gt; &lt;p&gt; À partir de cette base, il développe une éthique du discours : seules sont moralement justifiées les normes qui pourraient être acceptées par tous les concernés dans un discours pratique idéal, où chacun est reconnu comme partenaire égal de l’argumentation. Cette éthique vise à fournir un fondement universel à la morale, sans retomber dans un absolutisme dogmatique ni dans un relativisme pur : l’universalité vient des conditions mêmes de l’argumentation rationnelle. Elle influence profondément Habermas, même si il insiste davantage sur la dimension de fondation ultime et sur l’obligation morale inconditionnelle qui en découle. &lt;/p&gt; &#10;"/>
-    <hyperlink ref="H66" r:id="rId35" display="https://www.laphilo.fr/pho/koapel-mini.webp"/>
-    <hyperlink ref="E68" r:id="rId36" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Reiner_Sch%C3%BCrmann&quot;  title=&quot; Wikipedia&quot;&gt;Reiner SCHÜRMANN&lt;/a&gt; est un philosophe allemand d’expression française, né à Amsterdam et mort à New York, où il a enseigné à la New School for Social Research à partir de 1975. Très marqué par la phénoménologie et la pensée de Heidegger, il se distingue par une réflexion exigeante sur la métaphysique, l’histoire de la philosophie et l’agir humain, développée dans trois grands ouvrages : Maître Eckhart et la joie errante (1972), Le principe d’anarchie (1982) et Des hégémonies brisées (posthume, 1996). &lt;/p&gt;&lt;p&gt; Dans Maître Eckhart et la joie errante, Schürmann reprend la pensée du mystique allemand du XIVᵉ siècle pour explorer la possibilité d’une vie spirituelle détachée de toute identité fixe ou de tout fondement stable. Il met en avant ce qu’il appelle une « joie errante » : une forme de liberté intérieure où le sujet ne se réclame plus d’une essence, d’un Dieu garanti ou d’une identité nationale, mais accepte de vivre dans une errance originaire et sans fondement. &lt;/p&gt; &lt;p&gt; Dans Le principe d’anarchie (souvent considéré comme son chef‑d’œuvre), Schürmann interprète Heidegger comme une pensée qui conduit à la ruine de tout principe premier (« archè ») sur lequel la tradition occidentale aurait voulu fonder la connaissance, la morale et la politique. Il en tire une théorie de l’« anarchie » non pas comme désordre, mais comme conscience lucide de l’absence de fondement ultime : l’agir humain doit alors se penser comme une praxis ouverte, responsable et créative, sans recours à une règle suprême. &lt;/p&gt; &lt;p&gt; Dans Des hégémonies brisées, Schürmann entreprend une vaste reconstruction de l’histoire de la philosophie occidentale comme succession d’« hégémonies » (modèles de vérité, de métaphysique, de politique) qui s’imposent, puis se défont. Il montre comment la modernité et la déconstruction heideggérienne ont dissous les grands systèmes de pensée, ouvrant à ce qu’il nomme une « philosophie tragique » où l’être se donne comme événement contingent, marqué par une distance, une fracture intérieure, plutôt que par une harmonie ou une cohérence totale. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="E49" r:id="rId23" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl_Korsch&quot; title=&quot; Wikipedia&quot;&gt;Karl KORDCH&lt;/a&gt;  était un philosophe marxiste allemand,  théoricien du communisme de conseils et critique du léninisme orthodoxe. Issu d'un milieu bourgeois, il évolua du réformisme social au marxisme hétérodoxe, influençant les courants ultra-gauche via son rejet du matérialisme positiviste et son insistance sur la praxis révolutionnaire historique.  Exclu du parti en 1926 pour &quot;ultra-gauchisme&quot;, il émigra après 1933 vers les USA, où il approfondit sa théorie marxiste. &lt;/p&gt; &lt;p&gt; Son œuvre majeure &quot;Marxisme et philosophie&quot; paru en 1923 marque sa rupture avec le léninisme en critiquant sa dérive scientiste. Il   &lt;a href=&quot;https://www.zones-subversives.com/article-le-marxisme-critique-de-karl-korsch-116431466.html&quot;  title=&quot;Le marxisme critique de Karl Korsch par Chroniques critiques&quot;&gt;rejette le marxisme &lt;/a&gt; comme &quot;science positive&quot; figée ou philosophie matérialiste abstraite ; il le conçoit comme une théorie historique et concrète, liée à la lutte des classes et à la dialectique hégélienne réinterprétée comme expression de la révolution bourgeoise puis prolétarienne. &lt;/p&gt; &lt;p&gt; Il  théorise les conseils comme organes centraux de la transition socialiste, via la praxis dialectique et l'auto-activité des masses, contre la socialisation étatique. Ses écrits inspirent le KAPD et l'ultra-gauche, voyant les conseils comme alternative à la bureaucratisation stalinienne. Son influence perdure chez les communistes de conseils, soulignant la conscience ouvrière spontanée pour l'émancipation réelle. &lt;/p&gt; "/>
+    <hyperlink ref="E52" r:id="rId24" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Eugen_Rosenstock-Huessy&quot; title=&quot; Wikipedia&quot;&gt;Eugen ROSENSTOCK-HUESSY&lt;/a&gt; était un penseur germano‑américain dont l'œuvre mêle philosophie sociale, histoire des idées et une théorie du langage centrée sur la parole comme acte créateur et structurant de la vie collective. Né en Allemagne, il forma des liens intellectuels avec des figures comme Franz Rosenzweig et Martin Buber, fut professeur (notamment aux États‑Unis après son exil) et créa une œuvre originale qui vise à comprendre comment les communautés se constituent et se transforment dans le temps par des échanges de parole. &lt;/p&gt; &lt;p&gt; Au  &lt;a href=&quot;https://www.en-attendant-nadeau.fr/2019/11/19/homme-quadridimensionnel-rosenstock//&quot;  title=&quot;l’homme quadridimensionnel par ean&quot;&gt;cœur de sa pensée &lt;/a&gt;  se trouve la notion de &quot;speech thinking&quot; (pensée de la parole) : il soutient que la parole n’est pas qu’un moyen descriptif, mais un acte répondant et créatif qui institue des relations sociales, forge des temporalités collectives et permet la transmission et la renouvellement des institutions humaines. Il affirme que, par le langage, les groupes deviennent « maîtres du temps » en fondant de nouveaux commencements, en rappelant le passé et en orientant l’action future — d’où son intérêt pour la densité historique de la vie sociale et le rôle des rituels, des serments et des discours publics. &lt;/p&gt; &lt;p&gt; Sur la religion et la théologie, il s’inscrit dans un courant post‑nietzschéen de renouveau religieux qui comprend Rosenzweig et Buber; il considère les énoncés religieux comme des actes de parole non‑métaphysiques qui dévoilent des dimensions de l’expérience humaine et communautaire inaccessibles aux seules sciences naturelles. Cette orientation le conduit à une pensée intégrative où philosophie, théologie et histoire participent à une réflexion pratique sur la transformation sociale et la responsabilité collective. &lt;/p&gt; &lt;p&gt; Ses livres et conférences couvrent une grande variété de thèmes — histoire des peuples, rhétorique sociale, philosophie de la loi et de l’éducation — et sa méthode combine analyses historiques, typologies du langage et propositions pour renouveler la vie civique; son influence se voit aujourd’hui dans des études sur la communication, la sociologie historique et la philosophie de la culture. &lt;/p&gt; "/>
+    <hyperlink ref="H52" r:id="rId25" display="https://www.laphilo.fr/pho/erhuessy-mini.webp"/>
+    <hyperlink ref="E54" r:id="rId26" display="&lt;p&gt; &lt;a href=&quot;https://fr.wikipedia.org/wiki/Oskar_Becker&quot;  title=&quot; Wikipedia&quot;&gt;Oskar BECKER&lt;/a&gt; était un philosophe, logicien, mathématicien et historien des mathématiques allemand, connu comme l’un des élèves les plus importants d’Edmund Husserl et comme un interlocuteur clé de Martin Heidegger. Sa pensée se situe à la croisée de la phénoménologie, de la philosophie des mathématiques, de la logique modale et de l’existentialisme. &lt;/p&gt; &lt;p&gt; Il utilise la phénoménologie husserlienne pour analyser les fondements de la géométrie, de l’arithmétique et de la logique, en cherchant à décrire les expériences vécues (compter, mesurer, démontrer) comme actes de conscience. Il tente ainsi de fonder une  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Ph%C3%A9nom%C3%A9nologie&quot;  title=&quot;phénoménologie par wikipedia&quot;&gt; sémantique phénoménologique &lt;/a&gt; de la logique intuitionniste, et ses idées sont reprises par Arend Heyting dans sa formalisation de cette logique. À la fin de sa vie, il insiste sur une distinction entre une intuition du domaine formel et platonicien (mathématiques pures) et un domaine existentiel concret, en utilisant parfois un vocabulaire proche de la « divination ». &lt;/p&gt; &lt;p&gt;Il est aussi un pionnier de la logique modale (logique de la nécessité et de la possibilité). On lui doit notamment ce qu’on appelle le postulat de Becker : l’idée que le statut modal est nécessaire, par exemple que la possibilité de PPP implique la nécessité de la possibilité de PPP, ainsi que certaines lois d’itération de la nécessité. Ces résultats ont joué un rôle important dans le développement de la logique modale au XXᵉ siècle. &lt;/p&gt; &lt;p&gt; Il entretient un dialogue étroit avec Heidegger : il reprend certains thèmes existentialistes (finitude, historicité, être-pour-la-mort) et les applique à des domaines comme les mathématiques, ce qui est très controversé (par exemple, discuter du comptage arithmétique comme « être-pour-la-mort »). Il développe également une « paraontologie » : une doctrine de l’essence et de la permanence des choses, distincte de l’ontologie heideggérienne centrée sur l’existence du Dasein. Pour lui, l’être humain n’existe pas seulement comme existence, mais aussi comme « paraexistence », incluant des dimensions inconscientes et surconscientes. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="H54" r:id="rId27" display="https://www.laphilo.fr/pho/obecker-mini.webp"/>
+    <hyperlink ref="E55" r:id="rId28" display="https://fr.wikipedia.org/wiki/Edith_Stein"/>
+    <hyperlink ref="H55" r:id="rId29" display="https://www.laphilo.fr/pho/estein-mini.webp"/>
+    <hyperlink ref="E61" r:id="rId30" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Gershom_Scholem&quot; title=&quot; Wikipedia&quot;&gt;Gershom SCHOLEM&lt;/a&gt; était un philosophe juif germano-israélien,  fondateur de l'étude académique moderne de la Kabbale et grand expert de  &lt;a href=&quot;https://www.nonfiction.fr/article-12478-gershom-scholem-de-berlin-a-la-palestine.htm&quot; title=&quot;Gershom Scholem : de Berlin à la Palestine  par nonfiction&quot;&gt;la mystique juive. &lt;/a&gt; Né à Berlin dans une famille assimilée, il s'est tourné vers le sionisme jeune et a immigré en Palestine en 1923, devenant professeur à l'Université hébraïque de Jérusalem. &lt;/p&gt; &lt;p&gt; Il a étudié les mathématiques, la philosophie et les langues sémitiques à Berlin, Iéna et Munich, où il a soutenu une thèse sur le &quot;Sefer ha-Bahir&quot;, un texte kabbalistique ancien. Ami proche de Walter Benjamin et correspondant de Leo Strauss, il a fui l'Europe nazie et s'est consacré à la recherche sur les manuscrits juifs pillés. &lt;/p&gt; &lt;p&gt; Il voyait  &lt;a href=&quot;https://www.youtube.com/watch?v=5HvDF8-XTjc&quot;  title=&quot;Dieu son nom et la Cabale selon Gershom Scholem  par Xavier Charles DJEBALI&quot;&gt;la Kabbale &lt;/a&gt; non comme une superstition marginale, mais au cœur de l'essence spirituelle du judaïsme, explorée via des méthodes scientifiques et historiques. Il insistait sur le rôle du messianisme et de la tradition comme forces de renouvellement, où la révélation divine est infiniment interprétable et liée à l'expérience historique du peuple juif. Pour lui, le sionisme allait au-delà de la politique : c'était un renouveau profond du judaïsme, unissant ancien et nouveau contre l'assimilation. &lt;/p&gt; &lt;p&gt; Son oeuvre majeure &quot;Les Grandes tendances de la mystique juive&quot; paru en 1941, basé sur des conférences, dédié à Benjamin, explore l'évolution de la mystique juive. Sa pensée met l'accent sur l'identité juive forgée par l'histoire, où la tradition intègre la nouveauté pour survivre aux crises. &lt;/p&gt; &lt;audio controls title=&quot;Des livres pour notre temps et les mondes à venir. 1/2 Gershom Scholem : penser dans les marges de la marge par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13094-10.11.2019-ITEMA_22199082-0.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
+    <hyperlink ref="E62" r:id="rId31" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Leo_Strauss&quot; title=&quot; Wikipedia&quot;&gt;Leo SRAUSS&lt;/a&gt; était un philosophe politique germano-américain, connu pour sa critique profonde de la modernité et pour sa relecture des grands textes de la philosophie politique classique. Sa pensée a eu une influence durable, notamment aux États‑Unis, où elle a marqué des générations d’étudiants en théorie politique. &lt;/p&gt; &lt;p&gt; Au cœur de sa philosophie se trouve l’idée que la modernité a rompu avec le droit naturel classique, c’est‑à‑dire avec la recherche de ce qui est juste par nature et non simplement selon l’histoire ou les sciences sociales. Il voit dans le positivisme, le relativisme et l’historicisme modernes une source de décadence intellectuelle, car ils empêchent de poser les questions normatives fondamentales : qu’est‑ce qu’une vie bonne, qu’est‑ce qu’un régime politique juste. Pour lui, la  &lt;a href=&quot;https://www.persee.fr/doc/rfsp_0035-2950_1985_num_35_4_394205&quot; title=&quot;philosophie et zscience politique par persée&quot;&gt;philosophie politique authentique &lt;/a&gt; doit réactiver ces questions et affronter directement les notions de meilleur régime et d’ordre politique juste, plutôt que de se contenter de descriptions neutres. &lt;/p&gt; &lt;p&gt; Cette critique le conduit à renouer avec les auteurs de l’Antiquité, en particulier Platon, Aristote et les philosophes médiévaux juifs et arabes, qu’il lit souvent contre les interprétations modernes. Il insiste sur la dimension éducative de la philosophie : il parle de « liberal education » comme d’une libération de la vulgarité, entendue comme manque d’expérience des belles choses. La fréquentation des grands textes est, pour lui, une école de modestie et d’audace intellectuelle, parce qu’elle oblige à mesurer nos catégories modernes à celles d’auteurs qui pensaient autrement le politique et le juste. &lt;/p&gt; &lt;p&gt; Célèbre pour sa thèse sur l’« écriture ésotérique » : selon lui, nombre de philosophes du passé ont écrit de manière volontairement oblique pour se protéger de la censure ou de la persécution, réservant un sens plus profond aux lecteurs attentifs. Cela l’amène à distinguer entre le message « exotérique » (apparent, destiné au grand public) et le message « ésotérique » (plus exigeant, adressé à une minorité philosophique). Cette hypothèse sur la lecture des classiques s’articule à sa conception du   &lt;a href=&quot;https://www.youtube.com/watch?v=9Vhsveytymk&quot; title=&quot;nihilisme et politique leo strauss par bildung et culture&quot;&gt;mode de vie philosophique, &lt;/a&gt; toujours exposé au risque de la tyrannie et de l’incompréhension. Ainsi, sa philosophie politique est à la fois une critique de la modernité et une tentative de redécouvrir la place de la philosophie au cœur du politique contemporain. &lt;/p&gt; &#10; &lt;audio controls title=&quot;la pensée de leon strauss par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/13397-05.04.2008-ITEMA_20118283-2008C3397E0019-ITE_00016207_RSCE-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;  &#10;"/>
+    <hyperlink ref="H62" r:id="rId32" display="https://www.laphilo.fr/pho/lstrauss-mini.webp"/>
+    <hyperlink ref="E65" r:id="rId33" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Hans_Jonas&quot; title=&quot; Wikipedia&quot;&gt;Hans JONAS&lt;/a&gt;  était un philosophe germano-américain connu pour ses travaux sur l'éthique de la technologie et &lt;a href=&quot;https://www.youtube.com/watch?v=NPIJHZO7hQo&quot; title=&quot; Le PRINCIPE RESPONSABILITÉ en 6 minutes ! (HANS JONAS) par Culture Philo&quot;&gt;la responsabilité&lt;/a&gt; envers les générations futures. Ses premières recherches portent sur le gnosticisme, vu comme une réponse à l'aliénation existentielle dans un monde hostile. Dans les années 1960, il développe une philosophie de la vie organique (The Phenomenon of Life), critiquant le dualisme cartésien et valorisant la nature vivante contre la technoscience destructrice. Son œuvre maîtresse &lt;a href=&quot;https://www.youtube.com/watch?v=LsIWCR9_N64&quot; style=&quot;color:#88A1E9&quot; title=&quot; Philo, Hans jonas, Le principe responsabilité, Bac philo par SOS Bac Français&quot;&gt; &quot;Le Principe responsabilité&quot;&lt;/a&gt; paru en1979, formule un impératif éthique pour l'ère technologique : &quot;Agis de façon que les effets de ton action soient compatibles avec la permanence d'une vie authentiquement humaine sur Terre&quot;. &lt;/p&gt; &lt;p&gt; Il  anticipe les crises écologiques et bioéthiques, proposant une &quot;heuristique de la peur&quot; pour guider l'action humaine face aux risques imprévisibles de la puissance technique. Influencé par sa tradition juive et Heidegger, il réconcilie existentialisme, phénoménologie et morale prophétique, impactant l'éthique environnementale contemporaine. &lt;/p&gt; &lt;p&gt; Il observe un &quot;déchaînement prométhéen&quot; : l'humanité acquiert un pouvoir inédit sur la nature via la science et la technique, capable de menacer sa propre survie et celle des générations futures. Contrairement aux éthiques classiques (kantienne ou utilitariste), limitées au présent ou aux intentions, sa réflexion intègre les conséquences à long terme, imprévisibles et collectives, sur la vie humaine et la planète. Face aux risques inconnus (nucléaire, génétique, environnementaux), il prône une &quot;heuristique de la peur&quot; : anticiper le pire scénario (in dubio pro malo) pour guider l'action, sans paralyser le progrès mais en le subordonnant à la préservation de la vie. Le savoir devient un devoir moral prioritaire, élargissant l'éthique à la nature et aux générations absentes.&lt;/p&gt;  &lt;/p&gt; &lt;p&gt;  &lt;audio controls title=&quot; Hans Jonas. Pour une éthique de la société technologique par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/22267-14.06.2021-ITEMA_22702122-2014C12410E0357.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
+    <hyperlink ref="E67" r:id="rId34" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Karl-Otto_Apel&quot; title=&quot; Wikipedia&quot;&gt;Karl-Otto APEL&lt;/a&gt; était un philosophe allemand majeur de l’après-guerre, surtout connu pour avoir développé, avec Jürgen Habermas, l’éthique du discours et pour sa « pragmatique transcendantale », une tentative de refonder la philosophie à partir des présupposés normatifs de l’argumentation. &lt;/p&gt; &lt;p&gt; Il est souvent crédité d’avoir opéré la « linguistification » de la philosophie transcendantale kantienne : au lieu de partir de la conscience ou du sujet (comme chez Kant ou Husserl), il part du fait que toute connaissance et toute action s’inscrivent dans un langage commun et une communauté de communication. Pour lui, les conditions de possibilité de la connaissance ne sont pas d’abord dans la structure de la conscience, mais dans les règles implicites de l’usage du langage et de l’argumentation. &lt;/p&gt; &lt;p&gt;  &lt;a href=&quot;https://www.youtube.com/watch?v=R9jQv_akxFE&quot; &gt;Sa notion centrale &lt;/a&gt; est celle d’a priori de la communauté de communication : le simple fait d’argumenter présuppose déjà un cadre normatif inévitable (recherche de vérité, reconnaissance mutuelle des interlocuteurs, exigence de cohérence, etc.). Quiconque tente de nier ces présupposés tombe dans une auto-contradiction performative : en les contestant par la parole, il les utilise déjà. Il en tire l’idée d’une fondation ultime de la rationalité et de l’éthique à partir de la structure même de l’argumentation. &lt;/p&gt; &lt;p&gt; À partir de cette base, il développe une éthique du discours : seules sont moralement justifiées les normes qui pourraient être acceptées par tous les concernés dans un discours pratique idéal, où chacun est reconnu comme partenaire égal de l’argumentation. Cette éthique vise à fournir un fondement universel à la morale, sans retomber dans un absolutisme dogmatique ni dans un relativisme pur : l’universalité vient des conditions mêmes de l’argumentation rationnelle. Elle influence profondément Habermas, même si il insiste davantage sur la dimension de fondation ultime et sur l’obligation morale inconditionnelle qui en découle. &lt;/p&gt; &#10;"/>
+    <hyperlink ref="H67" r:id="rId35" display="https://www.laphilo.fr/pho/koapel-mini.webp"/>
+    <hyperlink ref="E69" r:id="rId36" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Reiner_Sch%C3%BCrmann&quot;  title=&quot; Wikipedia&quot;&gt;Reiner SCHÜRMANN&lt;/a&gt; est un philosophe allemand d’expression française, né à Amsterdam et mort à New York, où il a enseigné à la New School for Social Research à partir de 1975. Très marqué par la phénoménologie et la pensée de Heidegger, il se distingue par une réflexion exigeante sur la métaphysique, l’histoire de la philosophie et l’agir humain, développée dans trois grands ouvrages : Maître Eckhart et la joie errante (1972), Le principe d’anarchie (1982) et Des hégémonies brisées (posthume, 1996). &lt;/p&gt;&lt;p&gt; Dans Maître Eckhart et la joie errante, Schürmann reprend la pensée du mystique allemand du XIVᵉ siècle pour explorer la possibilité d’une vie spirituelle détachée de toute identité fixe ou de tout fondement stable. Il met en avant ce qu’il appelle une « joie errante » : une forme de liberté intérieure où le sujet ne se réclame plus d’une essence, d’un Dieu garanti ou d’une identité nationale, mais accepte de vivre dans une errance originaire et sans fondement. &lt;/p&gt; &lt;p&gt; Dans Le principe d’anarchie (souvent considéré comme son chef‑d’œuvre), Schürmann interprète Heidegger comme une pensée qui conduit à la ruine de tout principe premier (« archè ») sur lequel la tradition occidentale aurait voulu fonder la connaissance, la morale et la politique. Il en tire une théorie de l’« anarchie » non pas comme désordre, mais comme conscience lucide de l’absence de fondement ultime : l’agir humain doit alors se penser comme une praxis ouverte, responsable et créative, sans recours à une règle suprême. &lt;/p&gt; &lt;p&gt; Dans Des hégémonies brisées, Schürmann entreprend une vaste reconstruction de l’histoire de la philosophie occidentale comme succession d’« hégémonies » (modèles de vérité, de métaphysique, de politique) qui s’imposent, puis se défont. Il montre comment la modernité et la déconstruction heideggérienne ont dissous les grands systèmes de pensée, ouvrant à ce qu’il nomme une « philosophie tragique » où l’être se donne comme événement contingent, marqué par une distance, une fracture intérieure, plutôt que par une harmonie ou une cohérence totale. &lt;/p&gt; &#10;&#10;"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Fiches — 72 fiches nouvelles : Max WEBER, Johann Friedrich HERBART, Paul TILLICH, Dietrich BONHOEFFER, Jane ADDAMS, George Herbert MEAD et 66 autre(s)
Publié depuis l'éditeur des fiches.
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -2572,7 +2572,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD71"/>
+  <dimension ref="A1:XFD75"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.93"/>
@@ -5613,6 +5613,216 @@
         </is>
       </c>
       <c r="O71"/>
+    </row>
+    <row r="72" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0">
+        <v>1864</v>
+      </c>
+      <c r="B72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1920</t>
+        </is>
+      </c>
+      <c r="C72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1864 – 1920</t>
+        </is>
+      </c>
+      <c r="D72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max WEBER</t>
+        </is>
+      </c>
+      <c r="E72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Max_Weber" title=" Wikipedia"&gt;Max WEBER&lt;/a&gt; est un sociologue, économiste et philosophe allemand, l’un des fondateurs de la sociologie. Né à Erfurt en 1864, il étudie le droit et l’histoire, puis enseigne l’économie à Fribourg et à Heidelberg. En 1898, une grave dépression l’oblige à renoncer à l’enseignement pendant de longues années. Il se consacre alors à la recherche, et son œuvre, immense, couvre l’économie, le droit, les religions du monde, la musique et la politique. Il meurt à Munich en 1920, emporté par une pneumonie.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;L’Éthique protestante et l’esprit du capitalisme&lt;/em&gt; (1905), il montre que le calvinisme a favorisé l’essor du capitalisme : le croyant, inquiet de son salut, cherche dans le travail méthodique et la réussite le signe de son élection, sans jouir de sa richesse. Il fonde une sociologie « compréhensive », qui cherche à comprendre le sens que les individus donnent à leurs actions, à l’aide d’« idéaux-types », des modèles simplifiés qui servent à analyser la réalité. Il exige du savant la « neutralité axiologique » : séparer les faits des jugements de valeur.&lt;/p&gt; &lt;p&gt;Il décrit la modernité comme un « désenchantement du monde » : la science et la rationalisation chassent la magie et les dieux, et enferment l’homme dans une « cage d’acier » bureaucratique. Il définit l’État par le « monopole de la violence physique légitime » et distingue trois formes de domination : traditionnelle, charismatique et légale-rationnelle. Dans &lt;em&gt;Le Savant et le Politique&lt;/em&gt; (1919), il oppose l’éthique de conviction, fidèle à ses principes, à l’éthique de responsabilité, attentive aux conséquences des actes.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/maxweber-mini.webp</t>
+        </is>
+      </c>
+      <c r="J72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">politique ; epistemologie</t>
+        </is>
+      </c>
+      <c r="K72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Individualisme méthodologique ; Néo-kantisme</t>
+        </is>
+      </c>
+      <c r="L72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sociologue et philosophe allemand, théoricien du désenchantement du monde et de la domination légitime.</t>
+        </is>
+      </c>
+      <c r="N72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O72">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="0">
+        <v>1776</v>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1841</t>
+        </is>
+      </c>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1776 – 1841</t>
+        </is>
+      </c>
+      <c r="D73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Johann Friedrich HERBART</t>
+        </is>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Johann_Friedrich_Herbart" title=" Wikipedia"&gt;Johann Friedrich HERBART&lt;/a&gt; est un philosophe, psychologue et pédagogue allemand. Né à Oldenbourg en 1776, il étudie à Iéna auprès de Fichte, dont il s’éloigne vite. Précepteur en Suisse, il rend visite au pédagogue Pestalozzi, qui l’inspire durablement. Il enseigne à Göttingen, puis succède en 1809 à Kant dans sa chaire de Königsberg, où il fonde un séminaire de pédagogie avec une école d’application. Il revient à Göttingen en 1833 et y meurt en 1841.&lt;/p&gt; &lt;p&gt;Contre l’idéalisme allemand de Fichte, Schelling et Hegel, il défend un réalisme : le monde est fait d’une multitude d’êtres simples, qu’il appelle les « réels ». La philosophie doit clarifier nos concepts et en éliminer les contradictions. Il veut faire de la psychologie une science exacte : l’esprit est le lieu de « représentations » qui s’attirent ou se repoussent, avec des forces que l’on pourrait mesurer. Les plus faibles sont refoulées sous le « seuil de la conscience », sans disparaître : il annonce ainsi l’idée d’inconscient. En morale, il dégage cinq idées pratiques : la liberté intérieure, la perfection, la bienveillance, le droit et l’équité.&lt;/p&gt; &lt;p&gt;Dans sa &lt;em&gt;Pédagogie générale&lt;/em&gt; (1806), il fonde la pédagogie sur l’éthique, qui fixe le but, et sur la psychologie, qui donne les moyens. L’enseignement doit éveiller chez l’élève un intérêt aux multiples facettes. Ses disciples en tirent des étapes de leçon qui ont marqué les écoles du monde entier.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/herbart-mini.webp</t>
+        </is>
+      </c>
+      <c r="J73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">epistemologie ; ethique</t>
+        </is>
+      </c>
+      <c r="K73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Réalisme</t>
+        </is>
+      </c>
+      <c r="L73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe et psychologue allemand, fondateur de la pédagogie scientifique.</t>
+        </is>
+      </c>
+      <c r="N73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O73"/>
+    </row>
+    <row r="74" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="0">
+        <v>1886</v>
+      </c>
+      <c r="B74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1965</t>
+        </is>
+      </c>
+      <c r="C74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1886 – 1965</t>
+        </is>
+      </c>
+      <c r="D74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paul TILLICH</t>
+        </is>
+      </c>
+      <c r="E74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Paul_Tillich" title=" Wikipedia"&gt;Paul TILLICH&lt;/a&gt; est un théologien et philosophe protestant allemand, naturalisé américain. Né en 1886 dans le Brandebourg, fils de pasteur, il est aumônier pendant la Première Guerre mondiale, une expérience qui le marque profondément. Engagé dans le « socialisme religieux », il enseigne à Francfort, où il dirige la thèse d’habilitation d’Adorno. En 1933, il est l’un des premiers professeurs non juifs chassés par les nazis. Il émigre aux États-Unis, où il enseigne à New York, à Harvard puis à Chicago, où il meurt en 1965.&lt;/p&gt; &lt;p&gt;Sa méthode de « corrélation » met en relation les questions que pose l’existence humaine et les réponses de la foi chrétienne. Dans &lt;em&gt;Dynamique de la foi&lt;/em&gt; (1957), il définit la foi comme la « préoccupation ultime », ce qui nous concerne de manière absolue. Chacun a une préoccupation ultime, mais elle devient une idole quand elle vise une réalité limitée, comme la nation ou l’argent. Dieu n’est pas un être parmi d’autres, même le plus grand : il est « l’être même », le fondement de tout ce qui existe.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Le Courage d’être&lt;/em&gt; (1952), il décrit, en dialogue avec l’&lt;a href="https://fr.wikipedia.org/wiki/Existentialisme" title=" Wikipedia"&gt;existentialisme&lt;/a&gt;, les trois angoisses de l’homme moderne : celle de la mort, celle de la culpabilité et celle du non-sens. Le courage d’être consiste à s’affirmer malgré elles, en s’appuyant sur le « Dieu au-dessus de Dieu ». Sa &lt;em&gt;Théologie systématique&lt;/em&gt; et sa théologie de la culture ont eu un grand écho.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/tillich-mini.webp</t>
+        </is>
+      </c>
+      <c r="J74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spiritualite ; metaphysique</t>
+        </is>
+      </c>
+      <c r="K74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Existentialisme ; Réforme-protestante</t>
+        </is>
+      </c>
+      <c r="L74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">théologien et philosophe protestant germano-américain, pour qui la foi est la « préoccupation ultime ».</t>
+        </is>
+      </c>
+      <c r="N74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O74">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="0">
+        <v>1906</v>
+      </c>
+      <c r="B75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1945</t>
+        </is>
+      </c>
+      <c r="C75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1906 – 1945</t>
+        </is>
+      </c>
+      <c r="D75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dietrich BONHOEFFER</t>
+        </is>
+      </c>
+      <c r="E75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Dietrich_Bonhoeffer" title=" Wikipedia"&gt;Dietrich BONHOEFFER&lt;/a&gt; est un théologien et pasteur luthérien allemand. Né à Breslau en 1906 dans une famille de la grande bourgeoisie, il obtient son doctorat de théologie à 21 ans. Pendant un séjour à New York, il découvre les Églises noires de Harlem. Dès 1933, il s’oppose au nazisme et à sa politique antisémite, et rejoint l’Église confessante. Il dirige un séminaire clandestin de pasteurs, fermé par la Gestapo en 1937. Dans &lt;em&gt;Le Prix de la grâce&lt;/em&gt; (1937), il oppose la « grâce à bon marché », qui excuse tout sans rien demander, à la « grâce qui coûte », celle du disciple qui suit réellement le Christ.&lt;/p&gt; &lt;p&gt;Pendant la guerre, il s’engage dans la résistance et participe, par l’intermédiaire de son beau-frère, à la conspiration contre Hitler. Arrêté en 1943, il écrit en prison les lettres publiées après sa mort sous le titre &lt;em&gt;Résistance et soumission&lt;/em&gt;. Il y constate que le monde est « devenu majeur » : il n’a plus besoin de Dieu pour expliquer la nature ou guider la politique. Il ne faut pas faire de Dieu un « bouche-trou » pour combler les lacunes de notre savoir.&lt;/p&gt; &lt;p&gt;Il appelle à un christianisme « non religieux », vécu au milieu du monde, dans l’engagement pour les autres : « Devant Dieu et avec Dieu, nous vivons sans Dieu. » Le chrétien doit accepter de se salir les mains et d’assumer la responsabilité de ses actes. Il est pendu au camp de Flossenbürg le 9 avril 1945, sur ordre d’Hitler. Son témoignage a profondément marqué la &lt;a href="https://fr.wikipedia.org/wiki/R%C3%A9forme_protestante" title=" Wikipedia"&gt;pensée protestante&lt;/a&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/bonhoeffer-mini.webp</t>
+        </is>
+      </c>
+      <c r="J75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spiritualite ; ethique ; politique</t>
+        </is>
+      </c>
+      <c r="K75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Réforme-protestante</t>
+        </is>
+      </c>
+      <c r="L75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">théologien protestant allemand, résistant au nazisme, penseur d’un christianisme « non religieux ».</t>
+        </is>
+      </c>
+      <c r="N75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O75">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Fiches — 12 fiches nouvelles : Hans REICHENBACH, BASILE de Césarée, GRÉGOIRE de Nazianze, IRÉNÉE de Lyon, CLÉMENT d'Alexandrie, JUSTIN de Naplouse et 6 autre(s)
Publié depuis l'éditeur des fiches.
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -2572,7 +2572,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD75"/>
+  <dimension ref="A1:XFD76"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.93"/>
@@ -5823,6 +5823,57 @@
       <c r="O75">
         <v>2</v>
       </c>
+    </row>
+    <row r="76" customFormat="false" ht="214.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="0">
+        <v>1891</v>
+      </c>
+      <c r="B76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1953</t>
+        </is>
+      </c>
+      <c r="C76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1891 – 1953</t>
+        </is>
+      </c>
+      <c r="D76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hans REICHENBACH</t>
+        </is>
+      </c>
+      <c r="E76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Hans_Reichenbach" title=" Wikipedia"&gt;Hans REICHENBACH&lt;/a&gt; est un philosophe des sciences allemand. Né à Hambourg en 1891, il étudie la physique, les mathématiques et la philosophie, et suit à Berlin les cours d’Einstein sur la relativité. En 1928, il fonde à Berlin un cercle de philosophie scientifique, proche du cercle de Vienne, et dirige avec Rudolf Carnap la revue &lt;em&gt;Erkenntnis&lt;/em&gt;. Chassé de l’université en 1933 par les nazis, il enseigne à Istanbul, puis à partir de 1938 à l’université de Californie à Los Angeles. Il y meurt en 1953.&lt;/p&gt; &lt;p&gt;Il est l’un des principaux représentants du &lt;a href="https://fr.wikipedia.org/wiki/Empirisme_logique" title=" Wikipedia"&gt;positivisme logique&lt;/a&gt;. Dans &lt;em&gt;Philosophie de l’espace et du temps&lt;/em&gt; (1928), il tire les leçons de la relativité : la géométrie de l’espace physique n’est pas connue a priori, comme le pensait Kant, et certains de ses aspects reposent sur des conventions, comme la définition de la simultanéité de deux événements éloignés. Il distingue le « contexte de la découverte », la manière dont un savant trouve une idée, du « contexte de la justification », la manière dont on la prouve : seul le second intéresse le philosophe.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Expérience et prédiction&lt;/em&gt; (1938), il définit la probabilité comme la fréquence limite d’un événement et propose une justification pragmatique de l’induction : si une méthode peut réussir à prévoir l’avenir, c’est l’induction. Il imagine aussi une logique à trois valeurs pour la mécanique quantique, et étudie la direction du temps.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/reichenbach-mini.webp</t>
+        </is>
+      </c>
+      <c r="J76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">epistemologie ; logique</t>
+        </is>
+      </c>
+      <c r="K76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivisme Logique ; Empirisme</t>
+        </is>
+      </c>
+      <c r="L76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe des sciences allemand, figure de l’empirisme logique, théoricien de l’espace, du temps et de la probabilité.</t>
+        </is>
+      </c>
+      <c r="N76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O76"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Fiches — 13 fiches nouvelles : Juan Bautista ALBERDI, Domingo Faustino SARMIENTO, Simón RODRÍGUEZ, ZENGZI, HASAN al-Basri, RABIA al-Adawiyya et 7 autre(s) ; 290 fiches modifiées : Eduard BERNSTEIN, Rudolf EUCKEN, Max WEBER, Johann Friedrich HERBART, Paul TILLICH, Dietrich BONHOEFFER et 284 autre(s) ; 1 fiche retirée : Juan Bautista ALBERTI ; 3 images
Publié depuis l'éditeur des fiches.
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-allemands.xlsx
+++ b/data/frise-philosophes-allemands.xlsx
@@ -5526,8 +5526,16 @@
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Eduard_Bernstein" title=" Wikipedia"&gt;Eduard BERNSTEIN&lt;/a&gt; est un théoricien et homme politique allemand, le père du « révisionnisme » et l’un des fondateurs de la &lt;a href="https://fr.wikipedia.org/wiki/Social-d%C3%A9mocratie" title=" Wikipedia"&gt;social-démocratie&lt;/a&gt; moderne. Né à Berlin en 1850 dans une famille juive modeste, fils d’un mécanicien de locomotive, il est employé de banque quand il adhère en 1872 au parti social-démocrate. Les lois antisocialistes de Bismarck le contraignent à l’exil : en Suisse, où il dirige le journal du parti, puis à Londres, où il devient l’ami et le collaborateur de Friedrich Engels, qui fait de lui l’un de ses exécuteurs testamentaires.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Les Présupposés du socialisme&lt;/em&gt; (1899), il soumet le marxisme à l’épreuve des faits. Le capitalisme ne s’effondre pas, les classes moyennes ne disparaissent pas, la misère ouvrière ne s’aggrave pas : la théorie de la catastrophe finale est démentie. Le socialisme ne viendra pas d’une révolution, mais de réformes progressives, conquises par les syndicats, les coopératives et le suffrage universel. Il est l’héritier du libéralisme, et doit s’appuyer sur une éthique d’inspiration kantienne plutôt que sur une prétendue nécessité de l’histoire. « Ce qu’on appelle d’ordinaire le but final du socialisme n’est rien pour moi, le mouvement est tout. »&lt;/p&gt; &lt;p&gt;Ce « révisionnisme » déclenche une violente controverse. Karl Kautsky le combat au nom de l’orthodoxie, et &lt;a href="https://fr.wikipedia.org/wiki/Rosa_Luxemburg" title=" Wikipedia"&gt;Rosa Luxemburg&lt;/a&gt; lui répond par &lt;em&gt;Réforme sociale ou révolution ?&lt;/em&gt; (1899). Officiellement condamné par le parti, Bernstein inspire pourtant sa pratique réelle. Député au Reichstag, il vote en 1915 contre les crédits de guerre. Il meurt à Berlin en décembre 1932, peu avant l’arrivée de Hitler au pouvoir. En 1959, le programme de Bad Godesberg, par lequel le SPD renonce au marxisme, consacre ses idées.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F70" s="0"/>
-      <c r="G70" s="0"/>
+      <c r="F70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vna_Rp5aQ_s</t>
+        </is>
+      </c>
+      <c r="G70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Eduard Bernstein: Challenging Marxist Thought｜Philosopher Biography" par VIS PHILO.</t>
+        </is>
+      </c>
       <c r="H70" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/bernstein-mini.webp</t>
@@ -5587,6 +5595,16 @@
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Rudolf_Christoph_Eucken" title=" Wikipedia"&gt;Rudolf EUCKEN&lt;/a&gt; est un philosophe allemand. Né en 1846 à Aurich, en Frise orientale, il étudie à Göttingen et à Berlin, où il suit l’enseignement de Friedrich Adolf Trendelenburg, spécialiste d’Aristote. Professeur à Bâle, puis à Iéna de 1874 à 1920, il attire des étudiants du monde entier. En 1908, il reçoit le prix Nobel de littérature, l’un des rares philosophes à l’avoir obtenu, pour « sa recherche sincère de la vérité » et sa « vision idéaliste de la vie ».&lt;/p&gt; &lt;p&gt;Sa philosophie, qu’il appelle « activisme », est une réaction contre le matérialisme et le naturalisme de son temps. Selon lui, l’être humain n’est pas seulement un produit de la nature : il participe à une « vie de l’esprit » indépendante, universelle, qui le dépasse et qu’il doit conquérir par l’effort et l’action. Le sens de la vie ne se trouve ni dans le plaisir ni dans le seul progrès technique, mais dans cette élévation de l’individu vers une vie spirituelle, où la religion, la morale et la culture trouvent leur source. Cette vie de l’esprit n’est pas donnée d’avance : chaque époque et chaque personne doivent la reconquérir contre la dispersion et la routine.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Le Sens et la valeur de la vie&lt;/em&gt; (1908) et &lt;em&gt;Les Grands Courants de la pensée contemporaine&lt;/em&gt;, il veut donner à son époque une orientation spirituelle et défendre une religion débarrassée de ses dogmes. Très lu avant 1914, traduit dans de nombreuses langues, il s’engage pendant la guerre pour la cause allemande. Son &lt;a href="https://fr.wikipedia.org/wiki/Spiritualisme_%28philosophie%29" title=" Wikipedia"&gt;spiritualisme&lt;/a&gt; tombe ensuite dans l’oubli. Il meurt à Iéna en 1926.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tdu3BI-7i_Q</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"The Forgotten Philosopher who won the 1908 Nobel Prize for Literature | Rudolf Eucken" par Old Substack Writer</t>
+        </is>
+      </c>
       <c r="H71" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/eucken-mini.webp</t>
@@ -5638,6 +5656,16 @@
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Max_Weber" title=" Wikipedia"&gt;Max WEBER&lt;/a&gt; est un sociologue, économiste et philosophe allemand, l’un des fondateurs de la sociologie. Né à Erfurt en 1864, il étudie le droit et l’histoire, puis enseigne l’économie à Fribourg et à Heidelberg. En 1898, une grave dépression l’oblige à renoncer à l’enseignement pendant de longues années. Il se consacre alors à la recherche, et son œuvre, immense, couvre l’économie, le droit, les religions du monde, la musique et la politique. Il meurt à Munich en 1920, emporté par une pneumonie.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;L’Éthique protestante et l’esprit du capitalisme&lt;/em&gt; (1905), il montre que le calvinisme a favorisé l’essor du capitalisme : le croyant, inquiet de son salut, cherche dans le travail méthodique et la réussite le signe de son élection, sans jouir de sa richesse. Il fonde une sociologie « compréhensive », qui cherche à comprendre le sens que les individus donnent à leurs actions, à l’aide d’« idéaux-types », des modèles simplifiés qui servent à analyser la réalité. Il exige du savant la « neutralité axiologique » : séparer les faits des jugements de valeur.&lt;/p&gt; &lt;p&gt;Il décrit la modernité comme un « désenchantement du monde » : la science et la rationalisation chassent la magie et les dieux, et enferment l’homme dans une « cage d’acier » bureaucratique. Il définit l’État par le « monopole de la violence physique légitime » et distingue trois formes de domination : traditionnelle, charismatique et légale-rationnelle. Dans &lt;em&gt;Le Savant et le Politique&lt;/em&gt; (1919), il oppose l’éthique de conviction, fidèle à ses principes, à l’éthique de responsabilité, attentive aux conséquences des actes.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">krUYFtq9Jww</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Max Weber et "la violence légitime de l'État" - #CulturePrime" par France Culture</t>
+        </is>
+      </c>
       <c r="H72" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/maxweber-mini.webp</t>
@@ -5691,6 +5719,16 @@
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Johann_Friedrich_Herbart" title=" Wikipedia"&gt;Johann Friedrich HERBART&lt;/a&gt; est un philosophe, psychologue et pédagogue allemand. Né à Oldenbourg en 1776, il étudie à Iéna auprès de Fichte, dont il s’éloigne vite. Précepteur en Suisse, il rend visite au pédagogue Pestalozzi, qui l’inspire durablement. Il enseigne à Göttingen, puis succède en 1809 à Kant dans sa chaire de Königsberg, où il fonde un séminaire de pédagogie avec une école d’application. Il revient à Göttingen en 1833 et y meurt en 1841.&lt;/p&gt; &lt;p&gt;Contre l’idéalisme allemand de Fichte, Schelling et Hegel, il défend un réalisme : le monde est fait d’une multitude d’êtres simples, qu’il appelle les « réels ». La philosophie doit clarifier nos concepts et en éliminer les contradictions. Il veut faire de la psychologie une science exacte : l’esprit est le lieu de « représentations » qui s’attirent ou se repoussent, avec des forces que l’on pourrait mesurer. Les plus faibles sont refoulées sous le « seuil de la conscience », sans disparaître : il annonce ainsi l’idée d’inconscient. En morale, il dégage cinq idées pratiques : la liberté intérieure, la perfection, la bienveillance, le droit et l’équité.&lt;/p&gt; &lt;p&gt;Dans sa &lt;em&gt;Pédagogie générale&lt;/em&gt; (1806), il fonde la pédagogie sur l’éthique, qui fixe le but, et sur la psychologie, qui donne les moyens. L’enseignement doit éveiller chez l’élève un intérêt aux multiples facettes. Ses disciples en tirent des étapes de leçon qui ont marqué les écoles du monde entier.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1gKEHwOzuM0</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Johann Friedrich Herbart: Unraveling Reality｜Philosopher Biography" par VIS PHILO.</t>
+        </is>
+      </c>
       <c r="H73" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/herbart-mini.webp</t>
@@ -5742,6 +5780,16 @@
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Paul_Tillich" title=" Wikipedia"&gt;Paul TILLICH&lt;/a&gt; est un théologien et philosophe protestant allemand, naturalisé américain. Né en 1886 dans le Brandebourg, fils de pasteur, il est aumônier pendant la Première Guerre mondiale, une expérience qui le marque profondément. Engagé dans le « socialisme religieux », il enseigne à Francfort, où il dirige la thèse d’habilitation d’Adorno. En 1933, il est l’un des premiers professeurs non juifs chassés par les nazis. Il émigre aux États-Unis, où il enseigne à New York, à Harvard puis à Chicago, où il meurt en 1965.&lt;/p&gt; &lt;p&gt;Sa méthode de « corrélation » met en relation les questions que pose l’existence humaine et les réponses de la foi chrétienne. Dans &lt;em&gt;Dynamique de la foi&lt;/em&gt; (1957), il définit la foi comme la « préoccupation ultime », ce qui nous concerne de manière absolue. Chacun a une préoccupation ultime, mais elle devient une idole quand elle vise une réalité limitée, comme la nation ou l’argent. Dieu n’est pas un être parmi d’autres, même le plus grand : il est « l’être même », le fondement de tout ce qui existe.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Le Courage d’être&lt;/em&gt; (1952), il décrit, en dialogue avec l’&lt;a href="https://fr.wikipedia.org/wiki/Existentialisme" title=" Wikipedia"&gt;existentialisme&lt;/a&gt;, les trois angoisses de l’homme moderne : celle de la mort, celle de la culpabilité et celle du non-sens. Le courage d’être consiste à s’affirmer malgré elles, en s’appuyant sur le « Dieu au-dessus de Dieu ». Sa &lt;em&gt;Théologie systématique&lt;/em&gt; et sa théologie de la culture ont eu un grand écho.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RmqRTLSsYQU</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"« Paul Tillich, prédicateur ». André Gounelle" par Regards protestants</t>
+        </is>
+      </c>
       <c r="H74" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/tillich-mini.webp</t>
@@ -5795,6 +5843,16 @@
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Dietrich_Bonhoeffer" title=" Wikipedia"&gt;Dietrich BONHOEFFER&lt;/a&gt; est un théologien et pasteur luthérien allemand. Né à Breslau en 1906 dans une famille de la grande bourgeoisie, il obtient son doctorat de théologie à 21 ans. Pendant un séjour à New York, il découvre les Églises noires de Harlem. Dès 1933, il s’oppose au nazisme et à sa politique antisémite, et rejoint l’Église confessante. Il dirige un séminaire clandestin de pasteurs, fermé par la Gestapo en 1937. Dans &lt;em&gt;Le Prix de la grâce&lt;/em&gt; (1937), il oppose la « grâce à bon marché », qui excuse tout sans rien demander, à la « grâce qui coûte », celle du disciple qui suit réellement le Christ.&lt;/p&gt; &lt;p&gt;Pendant la guerre, il s’engage dans la résistance et participe, par l’intermédiaire de son beau-frère, à la conspiration contre Hitler. Arrêté en 1943, il écrit en prison les lettres publiées après sa mort sous le titre &lt;em&gt;Résistance et soumission&lt;/em&gt;. Il y constate que le monde est « devenu majeur » : il n’a plus besoin de Dieu pour expliquer la nature ou guider la politique. Il ne faut pas faire de Dieu un « bouche-trou » pour combler les lacunes de notre savoir.&lt;/p&gt; &lt;p&gt;Il appelle à un christianisme « non religieux », vécu au milieu du monde, dans l’engagement pour les autres : « Devant Dieu et avec Dieu, nous vivons sans Dieu. » Le chrétien doit accepter de se salir les mains et d’assumer la responsabilité de ses actes. Il est pendu au camp de Flossenbürg le 9 avril 1945, sur ordre d’Hitler. Son témoignage a profondément marqué la &lt;a href="https://fr.wikipedia.org/wiki/R%C3%A9forme_protestante" title=" Wikipedia"&gt;pensée protestante&lt;/a&gt;.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lsbd2sH_yK0</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Dietrich Bonhoeffer, le courage d'une conviction" par Regards protestants</t>
+        </is>
+      </c>
       <c r="H75" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/bonhoeffer-mini.webp</t>
@@ -5846,6 +5904,16 @@
       <c r="E76" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Hans_Reichenbach" title=" Wikipedia"&gt;Hans REICHENBACH&lt;/a&gt; est un philosophe des sciences allemand. Né à Hambourg en 1891, il étudie la physique, les mathématiques et la philosophie, et suit à Berlin les cours d’Einstein sur la relativité. En 1928, il fonde à Berlin un cercle de philosophie scientifique, proche du cercle de Vienne, et dirige avec Rudolf Carnap la revue &lt;em&gt;Erkenntnis&lt;/em&gt;. Chassé de l’université en 1933 par les nazis, il enseigne à Istanbul, puis à partir de 1938 à l’université de Californie à Los Angeles. Il y meurt en 1953.&lt;/p&gt; &lt;p&gt;Il est l’un des principaux représentants du &lt;a href="https://fr.wikipedia.org/wiki/Empirisme_logique" title=" Wikipedia"&gt;positivisme logique&lt;/a&gt;. Dans &lt;em&gt;Philosophie de l’espace et du temps&lt;/em&gt; (1928), il tire les leçons de la relativité : la géométrie de l’espace physique n’est pas connue a priori, comme le pensait Kant, et certains de ses aspects reposent sur des conventions, comme la définition de la simultanéité de deux événements éloignés. Il distingue le « contexte de la découverte », la manière dont un savant trouve une idée, du « contexte de la justification », la manière dont on la prouve : seul le second intéresse le philosophe.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Expérience et prédiction&lt;/em&gt; (1938), il définit la probabilité comme la fréquence limite d’un événement et propose une justification pragmatique de l’induction : si une méthode peut réussir à prévoir l’avenir, c’est l’induction. Il imagine aussi une logique à trois valeurs pour la mécanique quantique, et étudie la direction du temps.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">doQCNi2putc</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Hans Reichenbach on the Direction of Time" par Nick Nielsen</t>
         </is>
       </c>
       <c r="H76" s="0" t="inlineStr">

</xml_diff>